<commit_message>
Ajouter lien vers bulletin officiel sur nom du speaker
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -41,25 +41,127 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
+    <t xml:space="preserve">364841</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20251202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ständerat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hegglin Peter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat hat uns für 2026 einen Voranschlag mit einem schuldenbremsenkonformen Budget mit einem Handlungsspielraum von 108 Millionen Franken unterbreitet. Dabei darf aber nicht übersehen werden, dass wir 2026 trotzdem ein Finanzierungsdefizit von 845 Millionen Franken haben, zumal sich der Bund dann in diesem Umfang neu verschulden muss. Dieses Ergebnis kommt aber auch nur dank umfangreichen Bereinigungsmassnahmen in den Jahren 2024 und 2025, der guten Einnahmenentwicklung und einer teilwei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat hat uns für 2026 einen Voranschlag mit einem schuldenbremsenkonformen Budget mit einem Handlungsspielraum von 108 Millionen Franken unterbreitet. Dabei darf aber nicht übersehen werden, dass wir 2026 trotzdem ein Finanzierungsdefizit von 845 Millionen Franken haben, zumal sich der Bund dann in diesem Umfang neu verschulden muss. Dieses Ergebnis kommt aber auch nur dank umfangreichen Bereinigungsmassnahmen in den Jahren 2024 und 2025, der guten Einnahmenentwicklung und einer teilweisen Verbuchung der Ausgaben zugunsten der Schutzsuchenden aus der Ukraine im ausserordentlichen Haushalt zustande.
+Für die Jahre 2027 und 2028 werden die Vorgaben der Schuldenbremse ebenfalls eingehalten, wenn wir das Entlastungspaket 2027 so umsetzen, wie es uns der Bundesrat vorgeschlagen hat. Leider wird dem nicht so sein, denn nach den Beratungen des EP 27 in unserer Finanzkommission [PAGE 1098] dürfte der finanzielle Fehlbetrag in den Jahren 2027 und 2028 schon über 600 Millionen Franken betragen. Im Jahr 2029 würde der Bereinigungsbedarf bei 2 Milliarden Franken zu liegen kommen. Das sind beträchtliche Summen, die in den kommenden Jahren nicht einfach bei den ungebundenen Ausgaben eingespart werden dürfen. Die zusätzlichen Einnahmen aus dem Kanton Genf sind zwar erfreulich, verbessern die Ergebnisse 2025 und 2026, sind aber für die Jahre 2027 bis 2029 nicht hilfreich. Die Erträge werden dannzumal tiefer ausfallen und den Sanierungsbedarf zusätzlich erhöhen.
+Wie können wir darauf reagieren? Aus meiner Sicht gibt es mehrere Möglichkeiten. 
+1.[NB]Wir müssen schon im Voranschlag 2026 zusätzliche Einsparungen erwirken oder dürfen zumindest nicht mehr Ausgaben beschliessen, um die Lage der Ausgaben nicht zu verschlechtern.
+2.[NB]Es sind auch unkonventionelle Ideen einzubringen und zu prüfen, etwa ob öffentlich-rechtliche Körperschaften, die vor allem oder nur privatwirtschaftliche Dienstleistungen erbringen, der Steuerpflicht unterstellt werden sollen oder ob z.[NB]B. SBB Immobilien einen höheren Anteil zur Finanzierung der Bahninfrastruktur leisten soll.
+3.[NB]Es sind heute auch nicht substanziell höhere Mittel für Rüstungsgüter zu beschliessen. Davor müssten zumindest die strategischen Ziele des Bundesrates zur Sicherheitspolitik bekannt sein.
+4.[NB]Die Schuldenbremse ist nach wie vor unter allen Umständen einzuhalten. Stabile Finanzen sind ein wichtiger Pfeiler der Sicherheitspolitik. Wenn alle Massnahmen letztlich nicht reichen, müsste zumindest das Volk darüber befinden können, ob es Rüstungsbeschaffungen als notwendig erachtet oder bereit ist, dafür mehr Steuern zu bezahlen.
+Gerne gehe ich auf einzelne Aspekte näher ein. Im Budgetjahr 2026 haben wir eine Ausgabensteigerung von 5,2 Prozent. Über die ganze Finanzplanperiode sind es immer noch 3,1 Prozent, und dies erst noch unter Einhaltung des Entlastungsprogramms 2027 und gegenüber den Zahlen des Voranschlages 2025. Haupttreiber für diese Kostensteigerung sind die Bereiche Bildung und Forschung, soziale Wohlfahrt und Sicherheit. Diese haben Wachstumsraten zwischen 5 und 8 Prozent.
+Auf der Einnahmenseite sollen die Fiskalerträge für das nächste Jahr ebenfalls um 5 Prozent steigen, über die kommenden vier Jahre immer noch um 3,2 Prozent. Angesichts der wirtschaftlichen Situation in unseren Nachbarstaaten, aber auch auf den Absatzmärkten, angesichts der wirtschaftlichen Konflikte mit anderen Ländern, vor allem auch in Übersee, sind das ambitionierte Annahmen. Es wäre aber vermessen, wenn das Parlament die Schätzungen des Eidgenössischen Finanzdepartements und der Eidgenössischen Steuerverwaltung verändern würde. Ich glaube, sie haben in der Vergangenheit gezeigt, dass diese doch ziemlich genau sind. Ich gehe auch davon aus, dass die Kenngrössen, die aufgeführt sind, im nächsten Jahr erreicht werden können. Schwieriger dürfte es in den Finanzdebatten der späteren Jahre werden. Vorsorgen ist deshalb angesagt, um dann nicht bei den ungebundenen Ausgaben übermässig korrigieren zu müssen.
+Ich beziehe mich heute deshalb vor allem auch auf den Eigenbereich. Das sind vornehmlich Personal- und Sachkosten. Über das Entlastungspaket 2027 plant der Bundesrat, im Eigenbereich 300 Millionen Franken einzusparen. Das ist respektabel und verdient Unterstützung. Trotzdem soll es erlaubt sein, im Budgetprozess zusätzliche Ausgabenpositionen zu hinterfragen. Dazu gehört sicher die Anzahl der Beschäftigten bei der Verwaltung; diese steigt unaufhörlich. Im Jahr 2015 lag sie noch bei 36[NB]522. Sie soll von diesem Jahr auf das nächste Jahr um weitere 378 Vollzeitstellen auf 39[NB]453 anwachsen, allein beim VBS um 232 Stellen. Bald werden wir die vierzigtausendste Vollzeitstelle bei der Verwaltung feiern können.
+Wir sind an dieser Entwicklung nicht ganz unschuldig. Mit Beschlüssen für laufend neue Aufgaben für den Bund sind wir einerseits Treiber dieser Entwicklung, andererseits versuchen wir, durch die Digitalisierung Effizienzgewinne zu realisieren. Leider aber bleiben die Effizienzsteigerungen in einem bescheidenen Rahmen. Das Projekt Dazit ist diesbezüglich eine erwähnenswerte Ausnahme. Dieses Projekt spielte über 300 Personalstellen frei. 
+Wie können wir nun korrigierend eingreifen? Mit dem Neuen Führungsmodell des Bundes beschliessen wir nicht über Personalstellen, sondern nur über die Budgethöhe. Der Bundesrat wünscht keine Kürzungen nach der Rasenmähermethode, sondern erwartet konkrete Hinweise von uns. Die[NB]Mehrheit[NB]der[NB]Kommission schlägt solche Massnahmen vor. 
+So will sie erstens beim Bundesverwaltungsgericht das Wachstum des Funktionsaufwandes - das sind Personalstellen und Sachaufwände - auf 2 Millionen Franken begrenzen. Die Erwartung, die ich als Kommissionsmitglied auch teile, ist, dass das Bundesverwaltungsgericht seine drängenden organisatorischen Probleme löst, seine Effizienz steigert und die Abteilungen sich bei der Pendenzenlast gegenseitig unterstützen. So wurde es auch in einem anonymen Schreiben aus dieser Institution an die Kommissionsmitglieder verlangt. 
+Eine zweite Kürzung betrifft den Kommunikationsbereich. Die Massnahme soll im Verhältnis zu den Kommunikationsaufwänden umgesetzt werden. Gemäss der vorliegenden Jahresrechnung 2024 gab es in der Verwaltung allein für die Öffentlichkeitsarbeit über 420 Vollzeitstellen, was Kosten von über 100 Millionen Franken verursachte. Mit einem Absenkpfad sollen diese Stellen und die Aufwände schrittweise reduziert werden.
+Das sind kleine Versuche, das Personalstellenwachstum zu bremsen. Die Finanzkommission und auch ich sind aber bereit, bei Bedarf zusätzliche Stellen zuzulassen, so zum Beispiel beim Fedpol. Für dieses ist ein Bericht der Eidgenössischen Finanzkontrolle vorliegend, der besagt, dass dort mehr Personal notwendig sei. Dort sind 63 zusätzliche Stellen beantragt, die nicht infrage gestellt sind.
+Ein weiterer Bereich im Eigenbereich ist die Teuerung. Eingestellt sind 0,5 Prozent Teuerungsausgleich, das entspricht 34 Millionen Franken. Während der Debatte, während der Arbeit in der Kommission sank die Teuerungsrate immer mehr, auf 0,3, auf 0,2 bis auf aktuell 0,1 Prozent. Auch in Anbetracht der guten Besoldungshöhe, die verschiedene Gutachten belegen, ist es vertretbar, auf einen Teuerungsausgleich, eine generelle Lohnerhöhung, zu verzichten. Eine individuelle Lohnentwicklung ist aber unabhängig davon möglich, und diese möchte ich explizit nicht infrage stellen. Das soll nach wie vor möglich sein.
+Mit einer Anpassung der Bundespersonalverordnung hat der Bundesrat auf Anfang 2026 ein neues Lohnmodell eingeführt und dabei auch den Ortszuschlag integriert. Als Finanzkommission waren wir, abgesehen von einer Information im November 2022, nicht eingebunden. Wir haben über Umwege bei den Budgetvorbesprechungen davon erfahren. Nach den Kompetenzregelungen wäre auch die SPK unseres Rates zuständig gewesen. Wie ich aber informiert bin, liess auch sie sich nicht konsultieren, wahrscheinlich war sie über den Vorgang gar nicht informiert. Es besteht in diesem Bereich auch keine Konsultationspflicht des Bundesrates gegenüber den eidgenössischen Räten.
+Gemäss den Aussagen des Eidgenössischen Personalamtes sollen aus den neuen Personalregelungen keine höheren Kosten entstehen. Das kann ich aber schwerlich nachvollziehen: Einerseits gibt es höhere Einstiegslöhne, ein anderes Lohnband, andererseits haben uns die eidgenössischen Gerichte in den Budgetbesprechungen darauf hingewiesen, dass sie die Lohnsteigerungen, die ab Lohnklasse 33 rund 10 Prozent betragen können, ab 2027 nicht werden kompensieren können. Es braucht in diesem Bereich, ich glaube, vor allem seitens der eidgenössischen Gerichte, also noch Korrekturmassnahmen. In Zeiten des Sparprogramms hätte ich hier mehr Sensibilität oder auch einen Einbezug unserer Kommissionen gewünscht.
+Das waren jetzt zwei Schienen, auf welchen man, meine ich, korrigieren kann, sogar korrigieren soll: einerseits das Stellenwachstum - aber über das Budget, nicht über die Anzahl Stellen -, andererseits die Teuerungszulage. [PAGE 1099] 
+Nicht unerwähnt lassen möchte ich bei den Eigenausgaben noch die Spesen - diese wachsen ja auch beträchtlich. 2021 waren es noch 98 Millionen Franken, im vergangenen Jahr waren es über die gesamte Verwaltung hinweg 132 Millionen Franken. Ich meine, auch in diesem Bereich wäre es möglich, gewisse Einsparungen vorzunehmen - ohne eine konkrete Massnahme anzustossen.
+Damit komme ich zum Schluss. Ich glaube, insgesamt können wir einen guten Voranschlag beraten. Ich danke dem Bundesrat und der Verwaltung für die grosse Vorarbeit und bitte Sie, jeweils der Mehrheit Ihrer Kommission oder dem Bundesrat zu folgen und dem Voranschlag in der Gesamtabstimmung zuzustimmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binder-Keller Marianne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Einschätzung, dass das Fedpol mehr Mittel braucht, ist nicht aus der Luft gegriffen. Der Bundesrat hat die Ressourcensituation selbst analysiert, dies aufgrund eines Postulates, wie das auch der Vertreter der Minderheit II erwähnt hat. Die EFK überprüfte das dann und kam zum klaren Schluss, dass das Fedpol seinen Auftrag mit den aktuellen Mitteln nicht erfüllen kann.[NB]Es[NB]wurden[NB]auch strukturelle Defizite festgestellt - auch das wurde erwähnt -, die analysiert und angegangen worden si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Einschätzung, dass das Fedpol mehr Mittel braucht, ist nicht aus der Luft gegriffen. Der Bundesrat hat die Ressourcensituation selbst analysiert, dies aufgrund eines Postulates, wie das auch der Vertreter der Minderheit II erwähnt hat. Die EFK überprüfte das dann und kam zum klaren Schluss, dass das Fedpol seinen Auftrag mit den aktuellen Mitteln nicht erfüllen kann.[NB]Es[NB]wurden[NB]auch strukturelle Defizite festgestellt - auch das wurde erwähnt -, die analysiert und angegangen worden sind.
+Nichtsdestotrotz braucht das Fedpol mehr Mittel. Die Sicherheitslage eskaliert generell. Wir haben einen Krieg in Europa, darauf muss ich ja wohl nicht weiter eingehen. Die Eidgenössische Finanzkontrolle kam klar zum Schluss, dass die personellen Ressourcen in den Bereichen Terrorismus, organisierte Kriminalität, Wirtschaftskriminalität und Cyberkriminalität nicht ausreichen. Das führt dazu, dass Strafverfahren verzögert oder gar nicht eröffnet werden, und unter diesen Umständen verstehe ich eine Kürzung wirklich nicht. Das hat massive Auswirkungen auf die innere Sicherheit, und dass diese geschützt werden muss, steht klar in Artikel 2 der Bundesverfassung, dem Zweckartikel.
+Als Präsidentin der Subkommission Gerichte/BA habe ich mir die Problematik vom Bundesanwalt und von der Aufsichtsbehörde über die Bundesanwaltschaft eingehend schildern lassen; Kollege Zopfi hat mich darauf angesprochen. Ebenso haben wir die Probleme in der Sicherheitspolitischen Kommission analysiert.
+Ich erachte eine Erhöhung der Mittel aufgrund der allgemein eskalierenden sicherheitspolitischen Lage für mehr als gerechtfertigt. Es ist eine Zeitfrage. Die Zeit läuft uns davon, was die Finanzierung der Armee und die Verteidigungsfähigkeit betrifft, und das ist sträflich. Die Zeit läuft uns aber auch davon, was die innere Sicherheit betrifft, und diese beiden Anliegen sind miteinander verzahnt. Wir können in solch eskalierenden Zeiten nicht zu einer internationalen Drehscheibe werden.
+Deshalb werde ich die Minderheit II (Zopfi) unterstützen. [PAGE 1113] 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zopfi Mathias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Antrag meiner Minderheit II dürfte vielen von Ihnen bekannt vorkommen. Diejenigen von Ihnen, die in der GPK sind, haben sich damit schon beschäftigt, und diejenigen von Ihnen, die in der SiK sind, haben sich auch bereits mit dieser Problematik beschäftigt. Die Minderheit II will mit ihrem Konzept, das sich dann auch im Finanzplan niederschlägt, jährlich zehn bis zwanzig Stellen beim Fedpol aufbauen, insbesondere im Bereich der Bundeskriminalpolizei. 
+Ich habe Ihnen gesagt, dass sich viele vo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Antrag meiner Minderheit II dürfte vielen von Ihnen bekannt vorkommen. Diejenigen von Ihnen, die in der GPK sind, haben sich damit schon beschäftigt, und diejenigen von Ihnen, die in der SiK sind, haben sich auch bereits mit dieser Problematik beschäftigt. Die Minderheit II will mit ihrem Konzept, das sich dann auch im Finanzplan niederschlägt, jährlich zehn bis zwanzig Stellen beim Fedpol aufbauen, insbesondere im Bereich der Bundeskriminalpolizei. 
+Ich habe Ihnen gesagt, dass sich viele von Ihnen bereits damit auseinandergesetzt haben. Ich sage nur so viel: Bei der Anhörung in der Kommission und an verschiedenen anderen Orten hörte ich immer wieder, dass wir uns in Richtung von Ländern mit sehr hoher organisierter Kriminalität bewegen. Ich nenne ein Land, das ein enormes Problem hat. Sie denken vielleicht an Italien, Sie denken vielleicht an Albanien. Nein, ich nenne Schweden als Beispiel. Schweden ist heute im Bereich der organisierten Kriminalität absolut problematisch unterwegs. Wenn ich höre, dass wir auch in der Schweiz in diese Richtung unterwegs sind und es sich um Jahre, vielleicht sogar nur um Monate handelt, bis sich solche Entwicklungen auch bei uns ergeben, dann lässt mich das aufhorchen. 
+Ich höre, dass wir vierzig Fälle nicht behandeln können, weil die Ressourcen bei der Bundeskriminalpolizei schlicht und einfach fehlen. Das lässt mich aufhorchen. Bei diesen vierzig Fällen handelt es sich nicht etwa um Bagatellfälle. Es sind Fälle organisierter Kriminalität, das müssen Sie einfach sehen. Es geht nicht um ein gestohlenes Portemonnaie oder so etwas. 
+Letztlich geht es darum, dass das Fedpol eine wichtige Aufgabe für die Sicherheit unseres Landes übernimmt, insbesondere, um unser Land vor organisierter Kriminalität zu bewahren oder möglichst gut zu schützen. Dass es dabei auch um Terrorismus und um Terrorismusfinanzierung usw. geht, wissen Sie bereits. 
+Vor Kurzem habe ich ein sehr interessantes Interview mit einem Spezialisten gelesen. Ich weiss nicht mehr, ob es in der "NZZ" oder im "Tages-Anzeiger" war. Er hat bestätigt, dass sich die organisierte Kriminalität, die wir vielleicht immer noch in Süditalien vermuten, in ganz Europa massiv ausgebreitet hat. Wir haben heute an vielen Orten Zustände, die nichts mehr mit einer heilen Welt zu tun haben oder mit Aussagen wie "Bei uns ist es ja nicht so schlimm" erklärt werden können. 
+Ich sage Ihnen das, und Sie hören mir einigermassen aufmerksam zu. Aber ich kann Ihnen sagen: Nicht nur ich sage Ihnen das. Ich habe bereits erwähnt, dass diejenigen von Ihnen, die in der GPK sind, sich damit auseinandergesetzt haben. Die GPK hat ein Schreiben an die Finanzkommission verfasst. Ich zitiere daraus nur einen Satz: "Auch die GPK kommt ebenfalls zum Schluss, dass die personellen Ressourcen der BKP rasch erhöht werden müssen." Die GPK, die sich mit der Sache auseinandergesetzt hat, ist offenbar zum Schluss gekommen, dass wir rasch etwas tun müssen. Auch in der generellen Stellungnahme der Bundesanwaltschaft steht zum Beispiel: "Der Mangel an Ermittlerressourcen bei der BKP ist eine allseits unbestrittene Erkenntnis." 
+Und was sagt die Eidgenössische Finanzkontrolle? Sie ist ihres Zeichens nicht unbedingt dafür bekannt, ausufernde Stellenbegehren gutzuheissen oder den Ausbau des Staates zu forcieren. Vielmehr nimmt sie auch für die Finanzkommission die Rolle ein, genau hinzuschauen und eher kritisch zu sein. Auch die EFK kommt in ihrem Bericht zum Schluss, dass es beim Fedpol neben Effizienzmassnahmen - die notabene vom Fedpol schon teilweise umgesetzt werden; deren Potenzial wurde bestätigt - mehr Ressourcen für die Ermittlung braucht. Die EFK sieht das also genau gleich. [PAGE 1112] 
+Zuletzt spreche ich noch diejenigen von Ihnen an, die in der SiK sitzen. Sie haben ohne Gegenstimme und mit klarer Mehrheit eine Motion beschlossen. Diese wird am 11.[NB]Dezember 2025 in diesem Rat behandelt. Die Motion fordert eigentlich nichts anderes als das, was meine Minderheit[NB]II ebenfalls fordert. Wir können schon noch zuwarten, oder wir können heute irgendwas entscheiden. Am 11.[NB]Dezember kann uns dann die Berichterstatterin - es ist die ehemalige Präsidentin der SiK, Kollegin Andrea Gmür-Schönenberger - erläutern, weshalb es wichtig ist, dass wir diese Motion wie die SiK möglichst ohne Gegenstimme annehmen. Aber dann ist es mit dem Voranschlag schon gelaufen, dann haben wir dieses Thema hier schon behandelt. Sie merken es, ich spreche die Mitglieder der SiK an, und ich habe es ihnen bereits gesagt: Die Musik spielt beim Voranschlag, die Musik spielt genau jetzt. 
+Natürlich ist es wichtig, dass wir die Finanzen im Griff behalten. Da stimme ich meinem Vorredner zu. Es ist wichtig, dass wir nicht einfach ausufernde Stellenbegehren gutheissen, nur weil ein bisschen Druck gemacht wird. Aber hier haben wir es mit einem Problem zu tun. Sie haben es von allen Seiten gehört.
+Jetzt könnten Sie, wenn Sie den Entwurf des Bundesrates und den Antrag der Minderheit I anschauen, zur Auffassung kommen, dass der Bundesrat ja bereits etwas unternimmt, denn die Minderheit I (Mühlemann) will hier kürzen. Dazu müssen Sie aber berücksichtigen: Diese 51 Stellen, die gemäss Antrag des Bundesrates geschaffen werden sollen, dienen nicht dem Aufbau der Bundeskriminalpolizei, um dieser erhöhten Bedrohungs- und Sicherheitslage Herr zu werden. Sondern 44 dieser 51 Stellen werden benötigt, um Projekte, die wir bewilligt haben - zum Beispiel die Schengen-Weiterentwicklungen, die Weiterentwicklung des automatisierten Fingerabdrucksystems usw. -, umzusetzen. Mit dem Antrag des Bundesrates setzen Sie also gerade einmal das um, was wir beschlossen haben, Sie schaffen aber keine zusätzlichen Ressourcen bei der Bundeskriminalpolizei für die Themen, die ich soeben erwähnt habe. Die übrigen 7 dieser 51 Stellen werden benötigt, um am Verwaltungszentrum Guisanplatz, wo ein neues Gebäude in Betrieb genommen worden ist, die Loge zu betreiben. Das wird dann vom VBS wieder rückerstattet und ist in dem Sinn also kostenneutral. Aber Sie werden sich auch vorstellen können, dass die 7[NB]Personen,[NB]die[NB]die[NB]Loge[NB]betreiben, nicht unbedingt der Bundeskriminalpolizei zur Bekämpfung der organisierten Kriminalität ausserhalb des Sichtradius der Loge zur Verfügung stehen. 
+Damit will ich Ihnen sagen: Die Variante Bundesrat bedeutet im Bereich der Bundeskriminalpolizei überhaupt keine Aufstockung, sondern Bewahrung des Status quo. Wenn Sie berücksichtigen wollen, was Ihnen die GPK, die SiK und alle anderen empfehlen, dann müssen Sie hier mit der Minderheit II stimmen. 
+Wenn Sie mit der Minderheit I stimmen, wovon ich Ihnen trotz klarer Sympathie natürlich wärmstens abrate, dann werden Sie die zusätzlichen Stellen, die für die Umsetzung dieser Projekte notwendig sind, beim laufenden Betrieb bei der Bundeskriminalpolizei und an anderen Orten kompensieren müssen, was dazu führt, dass im Resultat sogar weniger Ressourcen zur Verfügung stehen werden, um der genannten Herausforderungen Herr zu werden. 
+Wenn man jetzt die Zahl der Meldungen ins Spiel bringt und sagt, es werde halt zu viel gemeldet, dann kommt mir das folgendermassen vor: Es gibt eine Sicherheitslage, in der sich die Kriminalität erhöht, in der die Leute nach mehr Polizei rufen und in der das Sicherheitsgefühl sinkt. Sie sehen, dass es ein Problem gibt, aber anstatt mehr Polizei anzustellen, sagen Sie zu den Menschen: Gebt halt weniger Strafanzeigen auf, dann haben wir das Problem gelöst. So schaffen Sie einfach eine Dunkelziffer, ein Dunkelfeld. 
+Ich sage damit nicht, dass der Effekt, den Kollege Mühlemann beschrieben hat, nicht ein Stück weit eintreten kann. Aber die Tatsache ist, dass wir es hier mit organisierter Kriminalität zu tun haben, und daher ist es wichtig, dass wir nicht in die Vogel-Strauss-Politik verfallen und sagen: Gebt halt weniger Anzeigen auf, ihr macht zu viele Anzeigen; wenn wir weniger davon wissen, dann wird es weniger schlimm sein. Das wäre das Prinzip "Augen zu und durch", und dazu rate ich Ihnen im Namen unserer Sicherheit nicht.
+Ich bitte Sie deshalb, mit der Minderheit II zu stimmen und zu berücksichtigen, was bereits die GPK, die SiK und viele andere empfehlen und empfohlen haben, und hier entsprechend konsequent zu sein. Dann können Sie am 11.[NB]Dezember auch der erwähnten Motion zustimmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wenn man Kollege Zopfi zuhört, könnte man meinen, wir hätten in den vergangenen Jahren zu wenig oder nichts getan. Das stimmt einfach nicht. Betrachten Sie die Personalstellen beim Fedpol: Im Jahr 2019 lag der Personalbestand bei 899 Vollzeitstellen. Im Jahr 2026 soll er auf 1060 Stellen aufgestockt werden. Im Jahr 2026 sollen im Vergleich zum Vorjahr 63 Stellen hinzukommen. Die Frage ist, wo sie eingesetzt werden. Aber wir beschliessen ja über das Gesamtbudget. Der Bundesrat hat die Verantwortu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wenn man Kollege Zopfi zuhört, könnte man meinen, wir hätten in den vergangenen Jahren zu wenig oder nichts getan. Das stimmt einfach nicht. Betrachten Sie die Personalstellen beim Fedpol: Im Jahr 2019 lag der Personalbestand bei 899 Vollzeitstellen. Im Jahr 2026 soll er auf 1060 Stellen aufgestockt werden. Im Jahr 2026 sollen im Vergleich zum Vorjahr 63 Stellen hinzukommen. Die Frage ist, wo sie eingesetzt werden. Aber wir beschliessen ja über das Gesamtbudget. Der Bundesrat hat die Verantwortung und die Aufgabe, die zur Verfügung gestellten Mittel sachgerecht einzusetzen.
+Ich habe gesagt, dass 63 zusätzliche Stellen vorgesehen sind - das entspricht einem Wachstum von 6,3 Prozent. Das ist ein sehr viel stärkeres Wachstum als in der übrigen Bundesverwaltung. Über den Zeithorizont von 2019 bis 2026 lag das Personalwachstum beim Fedpol bei 2,9 Prozent im Jahr, also bei fast 3 Prozent. In der Bundesverwaltung lag es im gleichen Zeitraum bei 0,8 Prozent im Jahr. Das Fedpol wächst also im Vergleich zur übrigen Bundesverwaltung überdurchschnittlich. Von daher kommen wir den Empfehlungen der EFK nach, und wir kommen mit dem Antrag der Mehrheit Ihrer Finanzkommission auch dem Anliegen und[NB]dem[NB]Auftrag in diesem Sektor nach. Denn die Sicherheit und die Bekämpfung der kriminellen Organisationen sind wichtig.
+Ich empfehle Ihnen also, der Mehrheit Ihrer Kommission zu folgen und damit, wie gesagt, den Rahmen dafür zu schaffen, dass 63 zusätzliche Stellen geschaffen werden können.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">365198</t>
   </si>
   <si>
-    <t xml:space="preserve">20251202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conseil des Etats</t>
-  </si>
-  <si>
     <t xml:space="preserve">Engler Stefan</t>
   </si>
   <si>
-    <t xml:space="preserve">M-E</t>
-  </si>
-  <si>
     <t xml:space="preserve">GR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR</t>
   </si>
   <si>
     <t xml:space="preserve">Angenommen - Adopté
@@ -585,97 +687,32 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">365062</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ständerat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Binder-Keller Marianne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Einschätzung, dass das Fedpol mehr Mittel braucht, ist nicht aus der Luft gegriffen. Der Bundesrat hat die Ressourcensituation selbst analysiert, dies aufgrund eines Postulates, wie das auch der Vertreter der Minderheit II erwähnt hat. Die EFK überprüfte das dann und kam zum klaren Schluss, dass das Fedpol seinen Auftrag mit den aktuellen Mitteln nicht erfüllen kann.[NB]Es[NB]wurden[NB]auch strukturelle Defizite festgestellt - auch das wurde erwähnt -, die analysiert und angegangen worden si</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Einschätzung, dass das Fedpol mehr Mittel braucht, ist nicht aus der Luft gegriffen. Der Bundesrat hat die Ressourcensituation selbst analysiert, dies aufgrund eines Postulates, wie das auch der Vertreter der Minderheit II erwähnt hat. Die EFK überprüfte das dann und kam zum klaren Schluss, dass das Fedpol seinen Auftrag mit den aktuellen Mitteln nicht erfüllen kann.[NB]Es[NB]wurden[NB]auch strukturelle Defizite festgestellt - auch das wurde erwähnt -, die analysiert und angegangen worden sind.
-Nichtsdestotrotz braucht das Fedpol mehr Mittel. Die Sicherheitslage eskaliert generell. Wir haben einen Krieg in Europa, darauf muss ich ja wohl nicht weiter eingehen. Die Eidgenössische Finanzkontrolle kam klar zum Schluss, dass die personellen Ressourcen in den Bereichen Terrorismus, organisierte Kriminalität, Wirtschaftskriminalität und Cyberkriminalität nicht ausreichen. Das führt dazu, dass Strafverfahren verzögert oder gar nicht eröffnet werden, und unter diesen Umständen verstehe ich eine Kürzung wirklich nicht. Das hat massive Auswirkungen auf die innere Sicherheit, und dass diese geschützt werden muss, steht klar in Artikel 2 der Bundesverfassung, dem Zweckartikel.
-Als Präsidentin der Subkommission Gerichte/BA habe ich mir die Problematik vom Bundesanwalt und von der Aufsichtsbehörde über die Bundesanwaltschaft eingehend schildern lassen; Kollege Zopfi hat mich darauf angesprochen. Ebenso haben wir die Probleme in der Sicherheitspolitischen Kommission analysiert.
-Ich erachte eine Erhöhung der Mittel aufgrund der allgemein eskalierenden sicherheitspolitischen Lage für mehr als gerechtfertigt. Es ist eine Zeitfrage. Die Zeit läuft uns davon, was die Finanzierung der Armee und die Verteidigungsfähigkeit betrifft, und das ist sträflich. Die Zeit läuft uns aber auch davon, was die innere Sicherheit betrifft, und diese beiden Anliegen sind miteinander verzahnt. Wir können in solch eskalierenden Zeiten nicht zu einer internationalen Drehscheibe werden.
-Deshalb werde ich die Minderheit II (Zopfi) unterstützen. [PAGE 1113] 
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">365066</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zopfi Mathias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Der Antrag meiner Minderheit II dürfte vielen von Ihnen bekannt vorkommen. Diejenigen von Ihnen, die in der GPK sind, haben sich damit schon beschäftigt, und diejenigen von Ihnen, die in der SiK sind, haben sich auch bereits mit dieser Problematik beschäftigt. Die Minderheit II will mit ihrem Konzept, das sich dann auch im Finanzplan niederschlägt, jährlich zehn bis zwanzig Stellen beim Fedpol aufbauen, insbesondere im Bereich der Bundeskriminalpolizei. 
-Ich habe Ihnen gesagt, dass sich viele vo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Der Antrag meiner Minderheit II dürfte vielen von Ihnen bekannt vorkommen. Diejenigen von Ihnen, die in der GPK sind, haben sich damit schon beschäftigt, und diejenigen von Ihnen, die in der SiK sind, haben sich auch bereits mit dieser Problematik beschäftigt. Die Minderheit II will mit ihrem Konzept, das sich dann auch im Finanzplan niederschlägt, jährlich zehn bis zwanzig Stellen beim Fedpol aufbauen, insbesondere im Bereich der Bundeskriminalpolizei. 
-Ich habe Ihnen gesagt, dass sich viele von Ihnen bereits damit auseinandergesetzt haben. Ich sage nur so viel: Bei der Anhörung in der Kommission und an verschiedenen anderen Orten hörte ich immer wieder, dass wir uns in Richtung von Ländern mit sehr hoher organisierter Kriminalität bewegen. Ich nenne ein Land, das ein enormes Problem hat. Sie denken vielleicht an Italien, Sie denken vielleicht an Albanien. Nein, ich nenne Schweden als Beispiel. Schweden ist heute im Bereich der organisierten Kriminalität absolut problematisch unterwegs. Wenn ich höre, dass wir auch in der Schweiz in diese Richtung unterwegs sind und es sich um Jahre, vielleicht sogar nur um Monate handelt, bis sich solche Entwicklungen auch bei uns ergeben, dann lässt mich das aufhorchen. 
-Ich höre, dass wir vierzig Fälle nicht behandeln können, weil die Ressourcen bei der Bundeskriminalpolizei schlicht und einfach fehlen. Das lässt mich aufhorchen. Bei diesen vierzig Fällen handelt es sich nicht etwa um Bagatellfälle. Es sind Fälle organisierter Kriminalität, das müssen Sie einfach sehen. Es geht nicht um ein gestohlenes Portemonnaie oder so etwas. 
-Letztlich geht es darum, dass das Fedpol eine wichtige Aufgabe für die Sicherheit unseres Landes übernimmt, insbesondere, um unser Land vor organisierter Kriminalität zu bewahren oder möglichst gut zu schützen. Dass es dabei auch um Terrorismus und um Terrorismusfinanzierung usw. geht, wissen Sie bereits. 
-Vor Kurzem habe ich ein sehr interessantes Interview mit einem Spezialisten gelesen. Ich weiss nicht mehr, ob es in der "NZZ" oder im "Tages-Anzeiger" war. Er hat bestätigt, dass sich die organisierte Kriminalität, die wir vielleicht immer noch in Süditalien vermuten, in ganz Europa massiv ausgebreitet hat. Wir haben heute an vielen Orten Zustände, die nichts mehr mit einer heilen Welt zu tun haben oder mit Aussagen wie "Bei uns ist es ja nicht so schlimm" erklärt werden können. 
-Ich sage Ihnen das, und Sie hören mir einigermassen aufmerksam zu. Aber ich kann Ihnen sagen: Nicht nur ich sage Ihnen das. Ich habe bereits erwähnt, dass diejenigen von Ihnen, die in der GPK sind, sich damit auseinandergesetzt haben. Die GPK hat ein Schreiben an die Finanzkommission verfasst. Ich zitiere daraus nur einen Satz: "Auch die GPK kommt ebenfalls zum Schluss, dass die personellen Ressourcen der BKP rasch erhöht werden müssen." Die GPK, die sich mit der Sache auseinandergesetzt hat, ist offenbar zum Schluss gekommen, dass wir rasch etwas tun müssen. Auch in der generellen Stellungnahme der Bundesanwaltschaft steht zum Beispiel: "Der Mangel an Ermittlerressourcen bei der BKP ist eine allseits unbestrittene Erkenntnis." 
-Und was sagt die Eidgenössische Finanzkontrolle? Sie ist ihres Zeichens nicht unbedingt dafür bekannt, ausufernde Stellenbegehren gutzuheissen oder den Ausbau des Staates zu forcieren. Vielmehr nimmt sie auch für die Finanzkommission die Rolle ein, genau hinzuschauen und eher kritisch zu sein. Auch die EFK kommt in ihrem Bericht zum Schluss, dass es beim Fedpol neben Effizienzmassnahmen - die notabene vom Fedpol schon teilweise umgesetzt werden; deren Potenzial wurde bestätigt - mehr Ressourcen für die Ermittlung braucht. Die EFK sieht das also genau gleich. [PAGE 1112] 
-Zuletzt spreche ich noch diejenigen von Ihnen an, die in der SiK sitzen. Sie haben ohne Gegenstimme und mit klarer Mehrheit eine Motion beschlossen. Diese wird am 11.[NB]Dezember 2025 in diesem Rat behandelt. Die Motion fordert eigentlich nichts anderes als das, was meine Minderheit[NB]II ebenfalls fordert. Wir können schon noch zuwarten, oder wir können heute irgendwas entscheiden. Am 11.[NB]Dezember kann uns dann die Berichterstatterin - es ist die ehemalige Präsidentin der SiK, Kollegin Andrea Gmür-Schönenberger - erläutern, weshalb es wichtig ist, dass wir diese Motion wie die SiK möglichst ohne Gegenstimme annehmen. Aber dann ist es mit dem Voranschlag schon gelaufen, dann haben wir dieses Thema hier schon behandelt. Sie merken es, ich spreche die Mitglieder der SiK an, und ich habe es ihnen bereits gesagt: Die Musik spielt beim Voranschlag, die Musik spielt genau jetzt. 
-Natürlich ist es wichtig, dass wir die Finanzen im Griff behalten. Da stimme ich meinem Vorredner zu. Es ist wichtig, dass wir nicht einfach ausufernde Stellenbegehren gutheissen, nur weil ein bisschen Druck gemacht wird. Aber hier haben wir es mit einem Problem zu tun. Sie haben es von allen Seiten gehört.
-Jetzt könnten Sie, wenn Sie den Entwurf des Bundesrates und den Antrag der Minderheit I anschauen, zur Auffassung kommen, dass der Bundesrat ja bereits etwas unternimmt, denn die Minderheit I (Mühlemann) will hier kürzen. Dazu müssen Sie aber berücksichtigen: Diese 51 Stellen, die gemäss Antrag des Bundesrates geschaffen werden sollen, dienen nicht dem Aufbau der Bundeskriminalpolizei, um dieser erhöhten Bedrohungs- und Sicherheitslage Herr zu werden. Sondern 44 dieser 51 Stellen werden benötigt, um Projekte, die wir bewilligt haben - zum Beispiel die Schengen-Weiterentwicklungen, die Weiterentwicklung des automatisierten Fingerabdrucksystems usw. -, umzusetzen. Mit dem Antrag des Bundesrates setzen Sie also gerade einmal das um, was wir beschlossen haben, Sie schaffen aber keine zusätzlichen Ressourcen bei der Bundeskriminalpolizei für die Themen, die ich soeben erwähnt habe. Die übrigen 7 dieser 51 Stellen werden benötigt, um am Verwaltungszentrum Guisanplatz, wo ein neues Gebäude in Betrieb genommen worden ist, die Loge zu betreiben. Das wird dann vom VBS wieder rückerstattet und ist in dem Sinn also kostenneutral. Aber Sie werden sich auch vorstellen können, dass die 7[NB]Personen,[NB]die[NB]die[NB]Loge[NB]betreiben, nicht unbedingt der Bundeskriminalpolizei zur Bekämpfung der organisierten Kriminalität ausserhalb des Sichtradius der Loge zur Verfügung stehen. 
-Damit will ich Ihnen sagen: Die Variante Bundesrat bedeutet im Bereich der Bundeskriminalpolizei überhaupt keine Aufstockung, sondern Bewahrung des Status quo. Wenn Sie berücksichtigen wollen, was Ihnen die GPK, die SiK und alle anderen empfehlen, dann müssen Sie hier mit der Minderheit II stimmen. 
-Wenn Sie mit der Minderheit I stimmen, wovon ich Ihnen trotz klarer Sympathie natürlich wärmstens abrate, dann werden Sie die zusätzlichen Stellen, die für die Umsetzung dieser Projekte notwendig sind, beim laufenden Betrieb bei der Bundeskriminalpolizei und an anderen Orten kompensieren müssen, was dazu führt, dass im Resultat sogar weniger Ressourcen zur Verfügung stehen werden, um der genannten Herausforderungen Herr zu werden. 
-Wenn man jetzt die Zahl der Meldungen ins Spiel bringt und sagt, es werde halt zu viel gemeldet, dann kommt mir das folgendermassen vor: Es gibt eine Sicherheitslage, in der sich die Kriminalität erhöht, in der die Leute nach mehr Polizei rufen und in der das Sicherheitsgefühl sinkt. Sie sehen, dass es ein Problem gibt, aber anstatt mehr Polizei anzustellen, sagen Sie zu den Menschen: Gebt halt weniger Strafanzeigen auf, dann haben wir das Problem gelöst. So schaffen Sie einfach eine Dunkelziffer, ein Dunkelfeld. 
-Ich sage damit nicht, dass der Effekt, den Kollege Mühlemann beschrieben hat, nicht ein Stück weit eintreten kann. Aber die Tatsache ist, dass wir es hier mit organisierter Kriminalität zu tun haben, und daher ist es wichtig, dass wir nicht in die Vogel-Strauss-Politik verfallen und sagen: Gebt halt weniger Anzeigen auf, ihr macht zu viele Anzeigen; wenn wir weniger davon wissen, dann wird es weniger schlimm sein. Das wäre das Prinzip "Augen zu und durch", und dazu rate ich Ihnen im Namen unserer Sicherheit nicht.
-Ich bitte Sie deshalb, mit der Minderheit II zu stimmen und zu berücksichtigen, was bereits die GPK, die SiK und viele andere empfehlen und empfohlen haben, und hier entsprechend konsequent zu sein. Dann können Sie am 11.[NB]Dezember auch der erwähnten Motion zustimmen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">365070</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hegglin Peter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wenn man Kollege Zopfi zuhört, könnte man meinen, wir hätten in den vergangenen Jahren zu wenig oder nichts getan. Das stimmt einfach nicht. Betrachten Sie die Personalstellen beim Fedpol: Im Jahr 2019 lag der Personalbestand bei 899 Vollzeitstellen. Im Jahr 2026 soll er auf 1060 Stellen aufgestockt werden. Im Jahr 2026 sollen im Vergleich zum Vorjahr 63 Stellen hinzukommen. Die Frage ist, wo sie eingesetzt werden. Aber wir beschliessen ja über das Gesamtbudget. Der Bundesrat hat die Verantwortu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wenn man Kollege Zopfi zuhört, könnte man meinen, wir hätten in den vergangenen Jahren zu wenig oder nichts getan. Das stimmt einfach nicht. Betrachten Sie die Personalstellen beim Fedpol: Im Jahr 2019 lag der Personalbestand bei 899 Vollzeitstellen. Im Jahr 2026 soll er auf 1060 Stellen aufgestockt werden. Im Jahr 2026 sollen im Vergleich zum Vorjahr 63 Stellen hinzukommen. Die Frage ist, wo sie eingesetzt werden. Aber wir beschliessen ja über das Gesamtbudget. Der Bundesrat hat die Verantwortung und die Aufgabe, die zur Verfügung gestellten Mittel sachgerecht einzusetzen.
-Ich habe gesagt, dass 63 zusätzliche Stellen vorgesehen sind - das entspricht einem Wachstum von 6,3 Prozent. Das ist ein sehr viel stärkeres Wachstum als in der übrigen Bundesverwaltung. Über den Zeithorizont von 2019 bis 2026 lag das Personalwachstum beim Fedpol bei 2,9 Prozent im Jahr, also bei fast 3 Prozent. In der Bundesverwaltung lag es im gleichen Zeitraum bei 0,8 Prozent im Jahr. Das Fedpol wächst also im Vergleich zur übrigen Bundesverwaltung überdurchschnittlich. Von daher kommen wir den Empfehlungen der EFK nach, und wir kommen mit dem Antrag der Mehrheit Ihrer Finanzkommission auch dem Anliegen und[NB]dem[NB]Auftrag in diesem Sektor nach. Denn die Sicherheit und die Bekämpfung der kriminellen Organisationen sind wichtig.
-Ich empfehle Ihnen also, der Mehrheit Ihrer Kommission zu folgen und damit, wie gesagt, den Rahmen dafür zu schaffen, dass 63 zusätzliche Stellen geschaffen werden können.
+    <t xml:space="preserve">365786</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20251208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundesrat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keller-Sutter Karin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgrund eines Einstellungsfehlers in der Veranlagungssoftware konnte die kantonale Steuerverwaltung Genf für rund 60 Unternehmen, die in den vorangegangenen Steuerperioden noch nicht definitiv veranlagt worden waren, keine provisorischen Rechnungen gemäss Artikel 162 des Bundesgesetzes über die direkte Bundessteuer ausstellen. Dieser technische Fehler konnte mittlerweile behoben werden, sodass nun ordnungsgemäss provisorische Rechnungen ausgestellt werden können.
+Der Gesetzgeber hat die Finanza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgrund eines Einstellungsfehlers in der Veranlagungssoftware konnte die kantonale Steuerverwaltung Genf für rund 60 Unternehmen, die in den vorangegangenen Steuerperioden noch nicht definitiv veranlagt worden waren, keine provisorischen Rechnungen gemäss Artikel 162 des Bundesgesetzes über die direkte Bundessteuer ausstellen. Dieser technische Fehler konnte mittlerweile behoben werden, sodass nun ordnungsgemäss provisorische Rechnungen ausgestellt werden können.
+Der Gesetzgeber hat die Finanzaufsicht über die direkte Bundessteuer den 26 kantonalen Finanzkontrollen übertragen. Sie sind gehalten, jährlich die Ordnungs- und Rechtmässigkeit der Erhebung der direkten Bundessteuer und der Ablieferung des Bundesanteils zu prüfen und der Eidgenössischen Steuerverwaltung sowie der Eidgenössischen Finanzkontrolle darüber Bericht zu erstatten. Als Oberaufsicht hat die Eidgenössische Steuerverwaltung hierzu eine Richtlinie sowie ein verbindliches Prüfraster zuhanden der kantonalen Finanzkontrollen erlassen. Der erwähnte Softwarefehler wurde von der kantonalen Finanzkontrolle nicht festgestellt. Die Eidgenössische Steuerverwaltung ist derzeit daran, die Zusammenarbeit mit den kantonalen Finanzkontrollen zu intensivieren, und prüft übergeordnet, gemeinsam mit der Eidgenössischen Finanzverwaltung, weitergehende Massnahmen im Bereich der Rechnungsstellung für die direkte Bundessteuer. 
+Was die finanziellen Auswirkungen anbelangt, so steht der sogenannte Vergütungszins im Vordergrund. Dieser ist geschuldet, wenn Steuerpflichtige höhere Vorauszahlungen machen, als ihnen in Rechnung gestellt wurden. In welchem Ausmass dies tatsächlich erfolgte, kann erst bei der Erstellung der definitiven Veranlagung berechnet werden. Zu berücksichtigen ist jedoch, dass der Zinssatz für die Vergütungen tief ist: Für die primär betroffenen Kalenderjahre 2019 bis 2023 lag er bei 0,00 Prozent, für 2024 bei 1,25 Prozent und für 2025 bei 0,75 Prozent.
 </t>
   </si>
   <si>
     <t xml:space="preserve">366164</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20251208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bundesrat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keller-Sutter Karin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SG</t>
   </si>
   <si>
     <t xml:space="preserve">Ich äussere mich zu ausgewählten Minderheiten, da wir ja auch mit der Zeit etwas sorgsam umgehen sollten. Ich beginne beim Staatssekretariat für Migration (SEM) mit dem Ziel "Erfüllung der Qualitätsstandards im Bereich Unterbringung"; der Bundesrat ist hier einverstanden.
@@ -697,45 +734,16 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">366073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conseil national</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nicolet Jacques</t>
+    <t xml:space="preserve">365999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nationalrat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bürgi Roman</t>
   </si>
   <si>
     <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ce deuxième bloc traite de la sécurité, de la justice et de la migration. Treize propositions vous sont soumises. Je vais traiter les premières et Peter Schilliger commentera les dernières.
-Concernant le DFJP, dans l'unité administrative 402, l'Office fédéral de la justice, à la position "Valeurs patrimoniales confisquées", à la page A11 du dépliant, il s'agit de valeurs qui peuvent être confisquées à des bandes criminelles organisées. Tenant compte du résultat des comptes 2024 et du fait de l'a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ce deuxième bloc traite de la sécurité, de la justice et de la migration. Treize propositions vous sont soumises. Je vais traiter les premières et Peter Schilliger commentera les dernières.
-Concernant le DFJP, dans l'unité administrative 402, l'Office fédéral de la justice, à la position "Valeurs patrimoniales confisquées", à la page A11 du dépliant, il s'agit de valeurs qui peuvent être confisquées à des bandes criminelles organisées. Tenant compte du résultat des comptes 2024 et du fait de l'augmentation des effectifs de l'Office fédéral de la police, Fedpol, la majorité de la commission propose de majorer de 12,8 millions de francs les valeurs patrimoniales confisquées afin de les porter à 100 millions. Une minorité Farinelli propose d'en rester au montant de 87 millions, comme le prévoit le Conseil fédéral, jugé plus réaliste. Cette proposition vaut également pour le plan financier 2027-2029. Par 13 voix contre 11 et 0 abstention, la Commission des finances vous demande de suivre la proposition de la majorité, à 100 millions.
-Toujours à la page A11, à la position "Subventions de construction pour la détention administrative", le Conseil des États a décidé, par 40 voix contre 2 et 1 abstention, d'une coupe de 10 millions de francs. Il s'agit d'une réduction de 10 millions pour le centre de détention administrative en vue d'expulsion de l'aéroport de Zurich. Ces contributions méritent d'être réexaminées sous l'angle de leur nécessité et de leur envergure, et, pour l'heure, en attendant des éclaircissements, par 15 voix contre 10, la commission vous demande de suivre la position du Conseil des États, soit une coupe de 10 millions. La minorité Fehlmann Rielle demande d'en rester au montant proposé par le Conseil fédéral.
-Pour l'unité administrative 403, Fedpol, à la page A11, à la position "Charges de fonctionnement", une minorité Bürgi Roman propose d'en rester au montant de 294,5 millions de francs, comme le propose le Conseil fédéral. La question du nombre de postes pour Fedpol en général, et à la police judiciaire plus particulièrement, n'est pas nouvelle. Tant l'examen des ressources de Fedpol que le rapport du Contrôle fédéral des finances l'attestent. Bien que plus de 50 postes soient prévus, 15 autres postes doivent être supprimés dans le cadre des mesures d'allégement 2027. Cette proposition vaut également pour le plan financier 2027-2029. La commission, par 16 voix contre 8 et 0 abstention, propose de majorer de 1,8 million les moyens pour Fedpol.
-Pour l'unité administrative 420, le Secrétariat d'État aux migrations (SEM), à la page A11, dans le domaine des dépenses courantes, estimant qu'il faut impérativement faire des économies dans le domaine migratoire, une minorité Sollberger propose de réduire de 600 millions de francs cette position budgétaire pour la ramener à 3,36 milliards. La commission, par 16 voix contre 8 et 0 abstention, estime qu'il n'est pas adéquat de faire une demande de coupe et propose d'en rester au montant de 3,96 milliards demandé par le Conseil fédéral.
-Toujours pour le SEM, à la page A12, dans le domaine de l'aide sociale pour les requérants admis à titre provisoire comme réfugiés, le Conseil fédéral a porté au budget un montant de 2,089 milliards de francs ainsi que de 600 millions dans la contribution aux cantons pour l'Ukraine. La majorité de notre commission propose un transfert comptable de 130 millions, qui seraient prélevés dans la contribution aux cantons pour l'Ukraine, dans les dépenses extraordinaires, pour les réaffecter aux dépenses ordinaires dans le domaine de l'aide sociale pour les requérants d'asile admis à titre provisoire. Cela permettra de soulager de 130 millions les dépenses extraordinaires. Dans le même temps, la majorité propose de diminuer de 130 millions aussi les indemnités versées aux cantons au titre de l'aide sociale dans le domaine de la migration, cela en raison des prévisions à la baisse concernant les demandes d'asile en 2026. Cette proposition a été soutenue par 14 voix contre 11. La minorité Funiciello souhaite en rester aux propositions initiales du Conseil fédéral, soit renoncer au transfert de 130 millions et maintenir 2,089 milliards en dépenses ordinaires et 600 millions en dépenses extraordinaires. Cette proposition a été refusée par 14 voix contre[NB]11.
-La minorité II (Sollberger) souhaite rapatrier les 600 millions de francs de la contribution des cantons à l'Ukraine dans l'aide sociale pour les personnes admises à titre provisoire, portant cette position à 2,69 milliards de francs, cela afin que l'ensemble des dépenses soient comptabilisées dans les dépenses ordinaires.
-Estimant qu'il y a un risque important que la Confédération doive tout de même indemniser obligatoirement les cantons, cette proposition a été rejetée, par 15 voix contre 8 et 1 abstention.
-À la page C2, s'agissant des objectifs et de la valeur-cible du Secrétariat d'État aux migrations, la commission, sans avis contraire, propose, en ce qui concerne les procédures d'asile, de porter les objectifs en matière de respect des normes de qualité dans le domaine de l'hébergement à 95 pour cent, contre 90 pour cent pour le Conseil fédéral.
-S'agissant des indicateurs relatifs aux demandes pendantes en première instance depuis plus d'un an, la minorité Kälin a été retirée.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">365999</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nationalrat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bürgi Roman</t>
   </si>
   <si>
     <t xml:space="preserve">SZ</t>
@@ -758,6 +766,9 @@
   </si>
   <si>
     <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
   </si>
   <si>
     <t xml:space="preserve">Ja, dieser wichtige EFK-Bericht ist der Finanzkommission natürlich bekannt. Ich würde Ihnen antworten: das eine tun, das andere nicht lassen. Ich bin mit Ihnen natürlich völlig einig, dass die Ressourcen möglichst effizient eingesetzt werden müssen. Aber wenn man genau hinschaut, auch bei den anderen Staatsebenen, sieht man, dass es sich tatsächlich um ein substanzielles Ressourcenproblem handelt. Entsprechend helfen wir da mit.
@@ -829,6 +840,9 @@
   </si>
   <si>
     <t xml:space="preserve">367062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conseil des Etats</t>
   </si>
   <si>
     <t xml:space="preserve">Juillard Charles</t>
@@ -944,6 +958,9 @@
   </si>
   <si>
     <t xml:space="preserve">Parmelin Guy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VD</t>
   </si>
   <si>
     <t xml:space="preserve">Les temps actuels sont caractérisés par une forte incertitude et de grands défis, surtout sur le plan international, avec les tensions géopolitiques, la politique commerciale des États-Unis, des actualités comme l'imposition minimale de l'OCDE et j'en oublie. La réduction des droits de douane américains est un élément important, mais la situation va rester volatile. Avec toutes les actualités internationales, il est essentiel de ne pas perdre le focus sur notre pays, notre économie, nos travaill</t>
@@ -1006,10 +1023,42 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">367979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20251217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rösti Albert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte einleitend klar festhalten, dass der Bundesrat und auch ich persönlich zur Dekarbonisierung und zum Fahrplan, den unser Volk verabschiedet hat, stehen. Da besteht kein Zweifel. Ich erinnere aber gleichzeitig daran, dass wir diese Debatte - und ich danke dafür, dass wir sie führen können, es ist eine wichtige Debatte - rund einen Monat nach der Klimakonferenz in Belém abhalten. In Belém ist es nicht gelungen, international mindestens einen Fahrplan, eine Roadmap mit verbindlichen Punkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte einleitend klar festhalten, dass der Bundesrat und auch ich persönlich zur Dekarbonisierung und zum Fahrplan, den unser Volk verabschiedet hat, stehen. Da besteht kein Zweifel. Ich erinnere aber gleichzeitig daran, dass wir diese Debatte - und ich danke dafür, dass wir sie führen können, es ist eine wichtige Debatte - rund einen Monat nach der Klimakonferenz in Belém abhalten. In Belém ist es nicht gelungen, international mindestens einen Fahrplan, eine Roadmap mit verbindlichen Punkten, wo wann was zu geschehen hat, aufzustellen; es ist nicht gelungen, auch nur zu sagen, dass sich die Länder für eine Roadmap entscheiden und eine solche aufstellen sollen. Die wichtigsten Produzenten von fossiler Energie, die grossen Mächte China, USA, Indien und Saudi-Arabien, waren nicht bereit, in diese Richtung zu gehen. Das muss man wissen. Unsere Debatte hier findet auch einen Tag nachdem die Europäische Union das Verbrennerverbot rückgängig gemacht hat, statt.
+Wir müssen einfach auch vom Umfeld sprechen. Denn eines möchte ich am Anfang in aller Klarheit sagen: Wir stehen zur Dekarbonisierung. Aber sie bringt der Schweiz nur etwas, wenn sie weltweit geschieht. Sie wissen es alle haargenau: Die Schweiz alleine wird das Klima nicht ändern, kein Jota ändern. Deshalb bin ich jetzt schon erstaunt, wenn man hier hört, dass sich der Bundesrat weigere, Verantwortung zu übernehmen.
+Ihre Initiative für den Klimaschutz, die 0,5 bis 1 Prozent des Bruttoinlandproduktes für Klimamassnahmen verwenden will, bedeutet, dass der Bund die Verantwortung alleine übernehmen und jährlich 3,5 bis über 7 Milliarden Franken für den Klimaschutz einsetzen soll. Es ist absolut legitim, das zu fordern. Aber jetzt sage ich Ihnen, was wir heute machen, auch wenn Sie es als fehlende Verantwortung quantifizieren oder darstellen: Der Bund bezahlt jährlich, das wurde von Ihnen entschieden, 2 Milliarden Franken für die Dekarbonisierung und den Klimaschutz. Dazu kommen 600 Millionen Franken für die Biodiversität und noch 800 Millionen Franken für den internationalen Klimaschutz. Das heisst, die Schweiz, die gemäss Ihren Voten und den Interpellationen offenbar nichts tut, investiert bereits heute jährlich 3,4 Milliarden Franken, dies kombiniert mit Anreizmassnahmen, mit Abbaupfaden, mit Sanktionen für die Autohersteller, mit einem Emissionshandelssystem. Es ist eine Kombination verschiedener Massnahmen. Es wird nicht einfach nur der Bund in die Verantwortung gestellt. Ich kann durchaus nachvollziehen, dass man das in der Debatte so bringt, aber ich möchte es schon klar zurückweisen, dass der Bundesrat die Verantwortung verweigert. 
+Wir haben die Interpellationen entsprechend beantwortet. Ich danke Ihnen für die entsprechenden Fragen und werde mich gesamthaft dazu äussern, weil wir nicht allzu viel Zeit haben. 
+Zur Interpellation der Fraktionen der SP und der Grünen: Die Klimaszenarien zeigen, dass die Schweiz vom Klimawandel betroffen ist, das ist unbestritten. Die Szenarien verdeutlichen die Notwendigkeit globaler - nochmals: globaler - Anstrengungen zur Verminderung der Treibhausgasemissionen und auch der Anpassung der Klimamassnahmen. Die Klimaszenarien bilden auch für den Bundesrat die Grundlage für seine Strategie zur Dekarbonisierung und zur Anpassung an den Klimawandel. 
+Der Bundesrat anerkennt den Investitionsbedarf; vorhin habe ich bereits die jährlichen Investitionen erwähnt. In den letzten Jahren haben Sie mit wichtigen Gesetzesvorlagen - dafür danke ich - klare Vorgaben gemacht. Anfang dieses Jahres haben wir vier Vorlagen unverzüglich durch Verordnungen in Kraft gesetzt: das Klima- und Innovationsgesetz, das revidierte CO2-Gesetz für die Periode 2025-2030, das Bundesgesetz über eine sichere Stromversorgung mit erneuerbaren Energien sowie das Umweltschutzgesetz zur Stärkung der Kreislaufmassnahmen. Bei Letzterem sind zwar noch einige Punkte nicht vollständig umgesetzt, doch wir sind daran, sie anzugehen. Es sind also vier Gesetze, die Sie in Kraft gesetzt haben und die der Bundesrat unverzüglich mit Verordnungen umsetzt, ebenso wie Investitionen in der Höhe von jährlich 3,4 Milliarden Franken in den Klimaschutz und die Erneuerung unseres Energiesystems. Und Sie sagen, der Bundesrat verweigere hier die Verantwortung? Mit Verlaub, das kann ich so einfach nicht stehenlassen.
+Nochmals zur Erinnerung: Heute stellt der Bund jährlich 2 Milliarden Franken für den Klimaschutz und den Umbau des Energiesystems bereit. Diese Zahl berücksichtigt bereits die Kürzungen infolge des Entlastungspaketes. Sie werden über die rund 400 Millionen Franken diskutieren und demokratisch entscheiden, die wir als Gegenpart einsparen wollen. Wenn Sie diese 400 Millionen Franken nicht einsparen, liegen wir nicht bei 3,4 Milliarden, sondern bei 3,8 Milliarden Franken. Dieser Betrag ist also bereits eingerechnet. 
+Ehrlich gesagt bin ich mir nicht sicher, ob die Schweiz ihre Klimaziele bis 2030 erreichen kann. Es braucht zusätzliche Investitionen, und diese fallen in ein finanzpolitisches Umfeld, das es uns nicht leichtmacht, angesichts der Bedürfnisse in der Armee und im Sozialbereich. Der Bundesrat wird diesbezüglich am Ball bleiben, alles analysieren und sich 2027 dazu äussern, wo wir stehen. Ich meine, heute, ein Jahr nach Inkrafttreten des revidierten CO2-Gesetzes, ist es noch zu früh, um über die Zielerreichung zu sprechen.
+Das Klima- und Innovationsgesetz verpflichtet den Bundesrat, dem Parlament rechtzeitig Vorschläge zur Weiterentwicklung der Klimapolitik vorzulegen. Das Parlament behält jederzeit die Kompetenz, hier auch zu intervenieren. Zur Weiterentwicklung der Klimapolitik hat der Bundesrat denn auch verzugslos gehandelt. Am 12.[NB]September dieses Jahres haben wir zwei Aussprachen geführt. Zum einen haben wir über die Revision des CO2-Gesetzes ab 2031 bis 2040 diskutiert und bereits Eckwerte festgehalten, die dann in eine Vernehmlassung auf Mitte nächstes Jahr einfliessen, bei der Sie Stellung nehmen können, sodass wir Ihnen 2027 auch rechtzeitig eine Botschaft werden vorlegen können. Dann werden wir sicher auch Bilanz ziehen, wo wir stehen. Zukünftig sollen gemäss diesen Eckwerten CO2-Emissionen aus Gebäuden und aus dem Verkehr respektive Brenn- und Treibstoffe in ein neues Emissionshandelssystem eingebunden werden. Dadurch können gemäss unseren Überlegungen deutlich mehr Mittel generiert werden, ohne Steuern zu erhöhen. Mehr Mittel können natürlich aus den heute bestehenden Abgaben generiert werden, indem man diese dann auch effektiv für Klimamassnahmen einsetzen kann. Der Bundesrat anerkennt das und will auf diesem Pfad weitergehen. Die Einnahmen sollen, wie gesagt, zur Dekarbonisierung in den bekannten Sektoren Gebäude, Verkehr und Industrie eingesetzt werden. Wir sind als UVEK jetzt beauftragt, für den Bundesrat bis [PAGE 2390] spätestens Sommer 2026 eine Vernehmlassungsvorlage vorzulegen.
+Ich habe vorhin die globale Situation angesprochen, und die ist wirklich schwierig und aktuell in einigen Bereichen blockiert. Deshalb bin ich dankbar, dass Frau Nationalrätin Wismer eine Interpellation zu den Anpassungsmassnahmen eingereicht hat. Es ist so: Wir brauchen zusätzliche Anpassungsmassnahmen, wir kommen nicht darum herum. Auch wenn das 1,5-Grad-Ziel erreicht wird, braucht es Anpassungsmassnahmen. Wenn es nicht erreicht wird, braucht es entsprechend mehr Anpassungsmassnahmen.
+Aber bereits heute setzen Bund, Kantone und Gemeinden jährlich 600 Millionen Franken ein. Wir stellen fest, dass diese Summe aktuell ausreicht. Mit diesen Mitteln wollen wir in Zukunft mehr erreichen, indem sie risikobasiert eingesetzt werden. Indem wir eine risikobasierte, bessere Planung machen, über die Raumplanung die Risiken auch abschwächen, wollen wir den einzelnen Franken also effizienter einsetzen. Das haben Sie letztes Jahr mit der Änderung des Wasserbaugesetzes so entschieden. Die Kantone sind zudem seit dem 1.[NB]August dieses Jahres verpflichtet, bei der Gefahrenbeurteilung und Massnahmenplanung den Klimawandel zu berücksichtigen. Gemeinsam mit dem Bund setzen die Kantone auch die nationale Strategie zur Anpassung an den Klimawandel um. Diese wird derzeit aktualisiert. 
+Zudem wurden in der Herbstsession das Postulat Wandfluh 25.3489, "Naturgefahren. Kriterien für eine differenzierte Nutzung von Gefahrengebieten", und das Postulat 25.3669 der FDP-Liberalen Fraktion, "Überprüfung und allfällige Ergänzung der gesetzlichen Grundlagen für eine rasche Katastrophenhilfe des Bundes", angenommen. Wir werden diese Postulate detailliert beantworten, dazu Bericht erstatten und daraus allfällige Schlussfolgerungen ziehen, ob es im Anpassungsbereich zusätzliche Massnahmen braucht. 
+Der Bundesrat nimmt die Erkenntnisse aus den Klimaszenarien ernst. Sie verdeutlichen den Handlungsbedarf bei der Verminderung der Treibhausgasemissionen und der Anpassung an den Klimawandel. 
+Ich möchte nun nochmals auf das Sparprogramm eingehen und erklären, weshalb die Massnahmen, die wir vorgesehen haben, für den Bundesrat und für mich verantwortbar und durchaus kohärent zum jetzt von mir Gesagten sind. Im Bericht Gaillard wurde vorgeschlagen, die 400 Millionen Franken, über die vom Volk in der Abstimmung über das Klima- und Innovationsgesetz entschieden wurde, einzusparen. Der Bundesrat hat schliesslich gesagt: Wir wollen das nicht einsparen, wir brauchen diese Mittel für den Ölheizungsersatz in Mehrparteiengebäuden, und wir brauchen sie für Innovationen. Und hier ist für mich eben die internationale Komponente sehr wichtig: dass wir mit Innovationen nicht nur in der Schweiz zur Dekarbonisierung beitragen, sondern auch international. 
+Ich war aber gezwungen, im Gegenzug zu sagen, wo wir stattdessen sparen, denn jeder Bereich musste einen Beitrag leisten. Was haben wir also genommen? Wir haben den Gebäudebereich genommen, da das Gebäudeprogramm schon sehr lange läuft und alle, die rasch ihre Heizung umstellen wollten, die Subventionen und Unterstützung längst abgeholt haben. Und bei jenen, die nicht "first movers" waren, die das noch nicht gemacht haben, kommt genau der Mitnahmeeffekt ins Spiel: Sie machen den Ersatz auch, aber erst dann, wenn ihre Heizung abgeschrieben ist; dann nehmen sie einfach die Subvention, aber das ist ohne Wirkung, weil sie die Heizung sowieso ersetzen müssen. Das ist der Mitnahmeeffekt. Wir haben in einem Bericht der Eidgenössischen Finanzkontrolle und in verschiedenen Studien gesehen, wie gross dieser Mitnahmeeffekt in etwa ist: Je nach Studie - es ist schwierig zu berechnen - sind es 40 bis 70 Prozent. Sie wollen doch nicht, dass der Bund Leuten Geld sozusagen schenkt, die es einfach nehmen, weil es der Bund anbietet, die aber ihre Heizung ohnehin umstellen würden. Das einfach zu den Sparmassnahmen. 
+Es wurden auch die 200 Millionen Franken Einsparung beim Bahninfrastrukturfonds erwähnt. Sie haben dazu bereits eine Motion angenommen, damit hier in Zukunft, ab 2029, wieder mehr Geld zur Verfügung steht. Wenn wir die Finanzierung mit dem Mehrwertsteuerpromille weiterführen, sind es 400 Millionen Franken, die jährlich dazukommen. Ich habe das ausgeführt, um einfach etwas die Relationen hier in diesem Bereich aufzuzeigen.
+Ich danke Ihnen für die Debatte und dafür, dass ich die Haltung des Bundesrates hier transparent darstellen durfte.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">368245</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20251217</t>
   </si>
   <si>
     <t xml:space="preserve">Das ist ein bisschen ein Streit um des Kaisers Bart. Der Präsident der Finanzkommission hat es gesagt: Es geht um ein Rahmengesetz. An sich wollte der Bundesrat im Gesetz klarer festhalten, dass die Empfänger von Finanzhilfen ihre Aufgaben soweit möglich selbst finanzieren; das war auch immer ein Wunsch der Eidgenössischen Finanzkontrolle (EFK). Der Herr Präsident hat es gesagt: Es kamen dann Ängste aus dem Kultur- und dem Umweltbereich, dass durchgehend nur noch 50 Prozent Subventionen ausbezah</t>
@@ -1017,6 +1066,23 @@
   <si>
     <t xml:space="preserve">Das ist ein bisschen ein Streit um des Kaisers Bart. Der Präsident der Finanzkommission hat es gesagt: Es geht um ein Rahmengesetz. An sich wollte der Bundesrat im Gesetz klarer festhalten, dass die Empfänger von Finanzhilfen ihre Aufgaben soweit möglich selbst finanzieren; das war auch immer ein Wunsch der Eidgenössischen Finanzkontrolle (EFK). Der Herr Präsident hat es gesagt: Es kamen dann Ängste aus dem Kultur- und dem Umweltbereich, dass durchgehend nur noch 50 Prozent Subventionen ausbezahlt würden. Das wäre nicht der Fall gewesen.
 Wenn Sie das streichen, ist das nicht gravierend, weil auch das aktuelle Recht davon ausgeht, und das ist wichtig, dass Subventionsempfänger nach Kräften und ihrer wirtschaftlichen Leistungsfähigkeit mitbeteiligt werden. In der Regel, nach ständiger Praxis der Eidgenössischen Finanzverwaltung, sind das 50 Prozent, aber das muss im Einzelfall festgelegt werden. Ich verzichte hier auf eine Abstimmung, wir können mit dem geltenden Recht leben, es war der Versuch einer Präzisierung. In der Sache wird das nicht viel daran ändern, dass man immer noch darum feilschen wird, welcher Subventionssatz im Einzelfall angewendet wird.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">368193</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stark Jakob</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und dabei ist zu beachten, dass das eine ureigene Aufgabe der Kantone ist und dass sich der Bund mit Spezialgesetzen im Ausländerrecht, in der ALV und IV hier schon engagiert. Aus diesem Grund beantragt der Bundesrat, die Bestimmungen aufzuheben. Die Entlastungswirkung ist bei 19,8 Millionen Franken.
+Diese drei Anträge, die Sie hier vor sich haben, sehen alle vor, auf die Gesetzesänderung zu verzichten, mit Verweis auf die Kann-Bestimmung in Artikel 12 Absatz 1 WeBiG. Es ist also ohne Weiteres möglich, das Gesetz so zu belassen und bei der entsprechenden Position im Voranschlag den Betrag anzupassen. Die Kommissionsmehrheit möchte die volle Entlastungswirkung beibehalten, also die gut 19 Millionen Franken. Die Minderheit I (Herzog Eva) möchte die Entlastungswirkung knapp halbieren, sie möchte hier weiterhin 10[NB]Millionen[NB]Franken budgetieren. Die Minderheit II (Maillard Pierre-Yves) empfiehlt Ihnen, auf eine Kürzung ganz zu verzichten.
 </t>
   </si>
   <si>
@@ -1053,6 +1119,29 @@
 Die Ruag-Affäre ist dabei nur die Spitze des Eisbergs. Die Eidgenössische Finanzkontrolle hat gravierende Missstände aufgezeigt: fehlende Compliance, Mängel in der Governance, sogar Betrugsverdacht. Dass ein bundeseigenes Unternehmen mit Leopard-Panzern dubiose Geschäfte tätigen wollte, zeigt, dass Kontrolle und Verantwortung nicht funktionieren. Wir haben es hier nicht mit kleinen Schönheitsfehlern zu tun, sondern mit wiederkehrenden Mustern - Beschaffung ohne Reife, Kostenüberschreitungen, jahrelange Verzögerungen. Es ist immer dasselbe Muster: Verantwortung wird abgeschoben, niemand ist zuständig. 
 Ja, das Parlament hat mit GPK und FinDel starke Aufsichtsorgane. Aber sie stossen hier an ihre Grenzen. Nur eine PUK hat die vollen Rechte und ausreichend Ressourcen. Sie kann Bundesratsprotokolle einsehen, Zeugen vorladen und die ganze Führungskette unter die Lupe nehmen. Genau das braucht es, wenn wir verlorenes Vertrauen zurückgewinnen wollen. Es geht nicht darum, das VBS zu schwächen, sondern darum, es endlich zu stärken: durch Transparenz, klare Verantwortlichkeiten und eine Kultur, die Fehler nicht vertuscht, sondern aus ihnen lernt. Unser Ziel ist es, die Struktur zu verbessern, damit die Armee ihren Auftrag zuverlässig erfüllen kann, ohne dass Milliarden versickern. Die Schweiz kennt die Lehren aus der Mirage-Affäre von 1964. [PAGE 2478] Nur eine PUK kann das Vertrauen in das VBS wiederherstellen. Heute stehen wir an einem ähnlichen Punkt. Wenn wir jetzt nicht handeln, drohen neue Skandale. Die Zeche zahlen am Schluss die Steuerzahlenden und die Sicherheit unseres Landes. 
 Ich bitte Sie deshalb, diesen parlamentarischen Initiativen Folge zu geben. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">368811</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Büchel Roland Rino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Büro des Nationalrates hat die parlamentarischen Initiativen 25.407 und 25.414 an seiner Sitzung vom 22.[NB]August 2025 vorgeprüft. Diese waren von der Sozialdemokratischen Fraktion am 10.[NB]März 2025 bzw. von der Grünen Fraktion am[NB]21.[NB]März 2025 eingereicht worden. Sie fordern je die Einsetzung einer PUK mit dem Zweck, die Probleme bei der Rüstungsbeschaffung sowie die Führungs-, Kontroll- und Aufsichtsstrukturen innerhalb des VBS zu untersuchen. Sie haben es gehört von Herrn Bendaha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Büro des Nationalrates hat die parlamentarischen Initiativen 25.407 und 25.414 an seiner Sitzung vom 22.[NB]August 2025 vorgeprüft. Diese waren von der Sozialdemokratischen Fraktion am 10.[NB]März 2025 bzw. von der Grünen Fraktion am[NB]21.[NB]März 2025 eingereicht worden. Sie fordern je die Einsetzung einer PUK mit dem Zweck, die Probleme bei der Rüstungsbeschaffung sowie die Führungs-, Kontroll- und Aufsichtsstrukturen innerhalb des VBS zu untersuchen. Sie haben es gehört von Herrn Bendahan: Er denkt, dass eigentlich 15 PUK das Richtige wären - dazu gibt es aber keinen Antrag. Konkret geht es um zwei PUK, die verlangt werden.
+Das Büro des Nationalrates beantragt mit 9 zu 3 Stimmen, beiden Initiativen keine Folge zu geben. Die Minderheiten beantragen - Sie haben es gehört -, diesen Folge zu geben.
+Eine parlamentarische Untersuchungskommission einzusetzen, um die Missstände im Bereich der Ruag und Probleme bei der Rüstungsbeschaffung zu untersuchen, ist für die Minderheiten das richtige Vorgehen. Auch die Probleme bei den Führungs-, Kontroll- und Aufsichtsstrukturen innerhalb des VBS könnten von einer PUK besser untersucht werden als von der GPK und der FinDel.
+In Bezug auf die Oberaufsicht beim VBS liess sich das Büro von den GPK und der FinDel als zuständige Organe über deren laufende Arbeiten informieren. In beiden GPK gibt es je eine ständige Subkommission zur parlamentarischen Kontrolle der Geschäftsführung des VBS. Aktuelle Schwerpunktthemen sind die Inspektion zum Fixpreis des F-35A und die [PAGE 2479] Untersuchung der Governance der Ruag MRO durch den Eigner. Die beiden Berichte werden voraussichtlich im kommenden Jahr veröffentlicht.
+Mit ihrer Inspektion zum Fixpreis des F-35A will die GPK-N unter anderem klären, ob bei der Aushandlung der Verträge rückblickend Mängel in der Geschäftsführung des Bundesrates festgestellt werden können. Die GPK-S nimmt vertiefte Abklärungen zur Aufsicht und Steuerung der Ruag MRO durch den Bundesrat vor. Auslöser für diese Untersuchungen waren Unstimmigkeiten beim versuchten Verkauf - auf der anderen Seite auch beim Kauf - von 96 Leopard-1-Panzern an Deutschland im Jahr 2023, aber auch weiter zurückreichende Betrugsvorwürfe, welche von der Eidgenössischen Finanzkontrolle aufgedeckt worden waren.
+Die GPK beschäftigen sich zudem wiederkehrend und teils über Jahre hinweg mit der Mehrheit der Top-Projekte des VBS. Beispiele dafür sind das ehemalige Munitionslager Mitholz, das Aufklärungsdrohnensystem ADS 15, die Neue Digitalisierungsplattform und das Sicherheitsfunknetz Polycom. Weitere wichtige Projekte des VBS werden von den beiden GPK im Rahmen ihrer Oberaufsicht begleitet. Dabei handelt es sich unter anderem um die Planung der Rüstungsbeschaffung oder um den Schutz kritischer Infrastrukturen und um die Berechnung des Armeebestandes. An einer speziellen Sitzung befassen sich die beiden GPK jährlich mit den Berichten des Bundesrates über die Zielerreichung der Ruag MRO und der Ruag International. Dort müssen neben den Spitzen von VBS und EFD auch die beiden Unternehmungen Red und Antwort stehen.
+Aber auch die FinDel befasst sich im Rahmen ihrer Finanzoberaufsicht mit den Schlüssel- und Top-Projekten des VBS. Weil es sich beim VBS um das Departement - das wurde zu Recht erwähnt - mit den grössten finanziellen Risiken handelt und das Parlament die Rüstungsausgaben für 2025 aufgestockt hat, wird die FinDel die Finanz- und Investitionsplanung im Rüstungsbereich richtigerweise verstärkt beaufsichtigen.
+Aufgrund dieser Informationen zu den laufenden Arbeiten in den GPK und der FinDel kommt das Büro zum Schluss, dass die aufgeworfenen Problemstellungen im VBS von den entsprechenden Aufsichtsorganen des Parlamentes bereits im Detail beaufsichtigt werden.
+Für die beiden Minderheiten Widmer Céline und Glättli handelt es sich bei den aufgezählten Missständen im VBS um ein Systemversagen. Für sie kann nur eine PUK das verlorene Vertrauen in das VBS wiederherstellen; die Minderheitssprecherin hat das noch einmal unterstrichen. Für das Büro hingegen sollten die GPK und die FinDel mit ihren weitreichenden Kompetenzen und den ordentlichen Mitteln in der Lage sein, ihre Aufsichtspflicht gegenüber dem VBS wahrzunehmen. Zudem würde die Konstituierung einer PUK einen zu hohen finanziellen und zeitlichen Aufwand bedeuten, ohne einen wirklichen Mehrwert zu generieren.
+Aus diesen Gründen beantragt Ihnen das Büro, wie eingangs gesagt, den beiden Initiativen keine Folge zu geben.
+[VS]
 </t>
   </si>
 </sst>
@@ -1101,8 +1190,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I23" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I27" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I27"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1469,592 +1558,704 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>30</v>
       </c>
-      <c r="F5" t="s">
+      <c r="I5" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
       </c>
       <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" t="s">
         <v>36</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7"/>
-      <c r="F7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" t="s">
-        <v>49</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="E8"/>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" t="s">
         <v>49</v>
-      </c>
-      <c r="F9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" t="s">
-        <v>57</v>
-      </c>
-      <c r="I9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>15</v>
       </c>
-      <c r="G10" t="s">
-        <v>25</v>
-      </c>
       <c r="H10" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="I11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
         <v>65</v>
       </c>
-      <c r="G12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H12" t="s">
-        <v>69</v>
-      </c>
       <c r="I12" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13"/>
+        <v>67</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
       <c r="F13" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
         <v>72</v>
       </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" t="s">
-        <v>13</v>
-      </c>
+      <c r="E14"/>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="G14" t="s">
         <v>15</v>
       </c>
       <c r="H14" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I14" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H15" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="I15" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="D16" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="E16" t="s">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G16" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="H16" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I16" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
       </c>
       <c r="F17" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="G17" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="F18" t="s">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I18" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>105</v>
-      </c>
-      <c r="E19"/>
+        <v>97</v>
+      </c>
+      <c r="E19" t="s">
+        <v>98</v>
+      </c>
       <c r="F19" t="s">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="G19" t="s">
         <v>15</v>
       </c>
       <c r="H19" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I19" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>105</v>
       </c>
       <c r="E20"/>
       <c r="F20" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="G20" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="H20" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I20" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E21"/>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G21" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" t="s">
+        <v>115</v>
+      </c>
+      <c r="E22"/>
+      <c r="F22" t="s">
         <v>116</v>
       </c>
-      <c r="B22" t="s">
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
         <v>117</v>
       </c>
-      <c r="C22" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="I22" t="s">
         <v>118</v>
-      </c>
-      <c r="E22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" t="s">
-        <v>25</v>
-      </c>
-      <c r="H22" t="s">
-        <v>119</v>
-      </c>
-      <c r="I22" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23"/>
+      <c r="F23" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>120</v>
+      </c>
+      <c r="I23" t="s">
         <v>121</v>
       </c>
-      <c r="B23" t="s">
-        <v>117</v>
-      </c>
-      <c r="C23" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
         <v>122</v>
       </c>
-      <c r="E23" t="s">
+      <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>123</v>
+      </c>
+      <c r="E24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>125</v>
+      </c>
+      <c r="I24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" t="s">
+        <v>128</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>130</v>
+      </c>
+      <c r="I25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" t="s">
         <v>84</v>
       </c>
-      <c r="F23" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" t="s">
-        <v>25</v>
-      </c>
-      <c r="H23" t="s">
-        <v>123</v>
-      </c>
-      <c r="I23" t="s">
-        <v>124</v>
+      <c r="F26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>134</v>
+      </c>
+      <c r="I26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" t="s">
+        <v>128</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>138</v>
+      </c>
+      <c r="I27" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrections filtres débats: conseil N/S, session, layout objet
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -20,7 +20,7 @@
     <t xml:space="preserve">MeetingDate</t>
   </si>
   <si>
-    <t xml:space="preserve">CouncilName</t>
+    <t xml:space="preserve">MeetingCouncilAbbreviation</t>
   </si>
   <si>
     <t xml:space="preserve">SpeakerFullName</t>
@@ -47,7 +47,7 @@
     <t xml:space="preserve">20251202</t>
   </si>
   <si>
-    <t xml:space="preserve">Ständerat</t>
+    <t xml:space="preserve">S</t>
   </si>
   <si>
     <t xml:space="preserve">Hegglin Peter</t>
@@ -693,7 +693,7 @@
     <t xml:space="preserve">20251208</t>
   </si>
   <si>
-    <t xml:space="preserve">Bundesrat</t>
+    <t xml:space="preserve">N</t>
   </si>
   <si>
     <t xml:space="preserve">Keller-Sutter Karin</t>
@@ -709,6 +709,83 @@
     <t xml:space="preserve">Aufgrund eines Einstellungsfehlers in der Veranlagungssoftware konnte die kantonale Steuerverwaltung Genf für rund 60 Unternehmen, die in den vorangegangenen Steuerperioden noch nicht definitiv veranlagt worden waren, keine provisorischen Rechnungen gemäss Artikel 162 des Bundesgesetzes über die direkte Bundessteuer ausstellen. Dieser technische Fehler konnte mittlerweile behoben werden, sodass nun ordnungsgemäss provisorische Rechnungen ausgestellt werden können.
 Der Gesetzgeber hat die Finanzaufsicht über die direkte Bundessteuer den 26 kantonalen Finanzkontrollen übertragen. Sie sind gehalten, jährlich die Ordnungs- und Rechtmässigkeit der Erhebung der direkten Bundessteuer und der Ablieferung des Bundesanteils zu prüfen und der Eidgenössischen Steuerverwaltung sowie der Eidgenössischen Finanzkontrolle darüber Bericht zu erstatten. Als Oberaufsicht hat die Eidgenössische Steuerverwaltung hierzu eine Richtlinie sowie ein verbindliches Prüfraster zuhanden der kantonalen Finanzkontrollen erlassen. Der erwähnte Softwarefehler wurde von der kantonalen Finanzkontrolle nicht festgestellt. Die Eidgenössische Steuerverwaltung ist derzeit daran, die Zusammenarbeit mit den kantonalen Finanzkontrollen zu intensivieren, und prüft übergeordnet, gemeinsam mit der Eidgenössischen Finanzverwaltung, weitergehende Massnahmen im Bereich der Rechnungsstellung für die direkte Bundessteuer. 
 Was die finanziellen Auswirkungen anbelangt, so steht der sogenannte Vergütungszins im Vordergrund. Dieser ist geschuldet, wenn Steuerpflichtige höhere Vorauszahlungen machen, als ihnen in Rechnung gestellt wurden. In welchem Ausmass dies tatsächlich erfolgte, kann erst bei der Erstellung der definitiven Veranlagung berechnet werden. Zu berücksichtigen ist jedoch, dass der Zinssatz für die Vergütungen tief ist: Für die primär betroffenen Kalenderjahre 2019 bis 2023 lag er bei 0,00 Prozent, für 2024 bei 1,25 Prozent und für 2025 bei 0,75 Prozent.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bürgi Roman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich begründe meinen Minderheitsantrag zum Funktionsaufwand des Bundesamts für Polizei. Der Bundesrat beantragt ein Globalbudget von 294 Millionen Franken. Die Mehrheit der Kommission möchte diesen Betrag nun um weitere 1,8 Millionen Franken erhöhen. Die SVP-Fraktion lehnt diese Aufstockung ab und beantragt, dem Bundesrat zu folgen. 
+Aus Sicht der SVP-Fraktion ist unbestritten, dass die Bundeskriminalpolizei zusätzliche Manpower an der Front benötigt. Das steht aber nicht zur Diskussion. Die Frag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich begründe meinen Minderheitsantrag zum Funktionsaufwand des Bundesamts für Polizei. Der Bundesrat beantragt ein Globalbudget von 294 Millionen Franken. Die Mehrheit der Kommission möchte diesen Betrag nun um weitere 1,8 Millionen Franken erhöhen. Die SVP-Fraktion lehnt diese Aufstockung ab und beantragt, dem Bundesrat zu folgen. 
+Aus Sicht der SVP-Fraktion ist unbestritten, dass die Bundeskriminalpolizei zusätzliche Manpower an der Front benötigt. Das steht aber nicht zur Diskussion. Die Frage ist vielmehr, ob wir eine strukturelle Budgeterhöhung sprechen sollen, bevor klar ist, wo und wie das Fedpol die zusätzlichen Stellen tatsächlich einsetzt. 
+Die Beratungen haben deutlich gezeigt, dass das Fedpol in der Vergangenheit primär hinsichtlich der Verwaltung und in der Kommunikation und nicht bei der operativen Kriminalpolizei ausgebaut wurde. Das Fedpol hat in den letzten Jahren Ressourcen erhalten, aber eben nicht für die Bereiche, in denen der eigentliche Bedarf besteht. Auch der EFK-Bericht bestätigt, dass intern bereits Effizienzsteigerungen im Gang und Kompensationen vorgenommen worden sind. Gleichzeitig aber bleibt unklar, weshalb genau jetzt externe Mittel über zusätzliche Stellen gesprochen werden müssen, bevor das Fedpol intern das vorhandene Potenzial ausgeschöpft hat. 
+Die Bundeskriminalpolizei verfügt heute über rund 700 Stellen, und der Bundesrat plant bereits 51 neue Stellen im Jahr 2026. Doch gemäss den Unterlagen entfallen davon nur sehr wenige auf die Ermittlungsarbeit, während der Rest für neue Projekte, für die IT-Weiterentwicklung und für die Bewirtschaftung des Verwaltungszentrums vorgesehen ist. Das hat mit der eigentlichen Kriminalbekämpfung wenig zu tun. 
+Bevor wir also zusätzliche Mittel bewilligen, erwarten wir zwei Dinge: Erstens muss das Fedpol intern jene Stellenprozente kompensieren, die es gemäss eigenen Aussagen einsparen kann, und zweitens braucht es ein klares Konzept, das detailliert aufzeigt, wo die zusätzlichen Ermittlungsstellen tatsächlich eingesetzt werden sollen. Wir fragten zu Recht, weshalb das Fedpol im ordentlichen Voranschlag nicht selbst mehr Ermittlungsstellen beantragte und weshalb im Entwicklungsrahmen zwar mehr Stellen gefordert wurden, diese dann aber nicht priorisiert wurden. Solange diese Fragen nicht beantwortet sind, ist eine Erhöhung des Budgets um 1,8 Millionen Franken nicht nachvollziehbar. Ich möchte betonen: Es geht nicht darum, die Sicherheit zu schwächen oder die Bedrohungslage zu verharmlosen. Es geht darum, dass wir zuerst sicherstellen müssen, dass die Bundesverwaltung ihre Mittel richtig einsetzt. Wenn das Fedpol erklärt, dass es intern noch Kompensationspotenzial hat, und gleichzeitig bestimmte Stellenpriorisierungen nicht vorgenommen wurden, ist es nicht sachgerecht, jetzt zusätzliches Geld zu sprechen. [PAGE 2100] 
+Der Bundesrat hat diese Abwägung gemacht und ist zum Schluss gekommen, dass 294 Millionen Franken ausreichend sind. Die SVP-Fraktion folgt dieser Einschätzung.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">366005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja, dieser wichtige EFK-Bericht ist der Finanzkommission natürlich bekannt. Ich würde Ihnen antworten: das eine tun, das andere nicht lassen. Ich bin mit Ihnen natürlich völlig einig, dass die Ressourcen möglichst effizient eingesetzt werden müssen. Aber wenn man genau hinschaut, auch bei den anderen Staatsebenen, sieht man, dass es sich tatsächlich um ein substanzielles Ressourcenproblem handelt. Entsprechend helfen wir da mit.
+Es ist eine spezielle Situation, dass Ihre Fraktion, die Law-and-Or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja, dieser wichtige EFK-Bericht ist der Finanzkommission natürlich bekannt. Ich würde Ihnen antworten: das eine tun, das andere nicht lassen. Ich bin mit Ihnen natürlich völlig einig, dass die Ressourcen möglichst effizient eingesetzt werden müssen. Aber wenn man genau hinschaut, auch bei den anderen Staatsebenen, sieht man, dass es sich tatsächlich um ein substanzielles Ressourcenproblem handelt. Entsprechend helfen wir da mit.
+Es ist eine spezielle Situation, dass Ihre Fraktion, die Law-and-Order-Fraktion, hier kritisch ist, wo es um mehr Polizei geht, und wir mit der Kommissionsmehrheit dafür sind. Das ist eine interessante Ausgangslage. Aber ich würde auf jeden Fall meinen: das eine tun, das andere nicht lassen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">366006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fischer Benjamin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geschätzter Kollege Andrey, ist Ihnen der EFK-Prüfbericht zur Ressourcensituation des Fedpol bekannt? Darin stellt die Eidgenössische Finanzkontrolle Mängel fest und hält auch klar fest, dass es ein Ressourcenproblem, aber auch ein grosses Potenzial gebe und[NB]man[NB]zuerst[NB]intern diese Ressourcen freispielen müsse, bevor das Parlament für das Fedpol wieder zusätzliche Gelder spricht. [PAGE 2103] 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">366067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bürgin Yvonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich spreche für die Mitte-Fraktion. Die Mitte. EVP zu Block 2, "Justiz, Sicherheit und Migration". Dieser Block betrifft zentrale Aufgaben unseres Staates, den Schutz des Rechtsstaats, die innere Sicherheit, die Cyberresilienz und die Steuerung der Migration. Unsere Haltung ist klar und ziemlich einfach. Wir unterstützen alle Mehrheitsanträge der Finanzkommission und lehnen alle Minderheitsanträge ab.
+Ein Punkt ist uns besonders wichtig. Neue Stellen betrachten wir grundsätzlich kritisch. Die Ve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich spreche für die Mitte-Fraktion. Die Mitte. EVP zu Block 2, "Justiz, Sicherheit und Migration". Dieser Block betrifft zentrale Aufgaben unseres Staates, den Schutz des Rechtsstaats, die innere Sicherheit, die Cyberresilienz und die Steuerung der Migration. Unsere Haltung ist klar und ziemlich einfach. Wir unterstützen alle Mehrheitsanträge der Finanzkommission und lehnen alle Minderheitsanträge ab.
+Ein Punkt ist uns besonders wichtig. Neue Stellen betrachten wir grundsätzlich kritisch. Die Verwaltung wächst seit Jahren. Es braucht Prioritäten und Effizienz, nicht reflexartige Aufstockungen. Gleichzeitig gilt: Wo Sicherheit und Funktionsfähigkeit des Staates gefährdet sind, müssen wir handeln. Das betrifft insbesondere das Fedpol und das Bundesamt für Cybersicherheit (BACS). Dort unterstützen wir zusätzliche Stellen ausdrücklich. Und ich möchte auch noch eine Antwort auf die Frage von vorhin von Herrn Fischer an Herrn Andrey geben: Ja, intern wurde schon sehr viel gemacht, aber das Fedpol braucht mehr Stellen.
+Beim Budget müssen aber auch die Einnahmen betrachtet werden. Wir unterstützen eine Erhöhung, und zwar mithilfe der eingezogenen Vermögenswerte beim Bundesamt für Justiz. Die realisierten Werte lagen in den letzten Jahren regelmässig über dem Budget. Mit diesem Durchschnittswert der Vergangenheit ist eine realistische Planung möglich.
+Beim Staatssekretariat für Migration sehen wir die bekannten Dynamiken. Die Sozialhilfekosten im Asylbereich hängen direkt von den Zugangszahlen ab. Bei den Beiträgen an die Kantone bezüglich der Ukraine-Flüchtlinge sind die Zahlen stabil, aber ein Teil der Kosten wird immer noch ausserordentlich verbucht. Wir unterstützen den Ansatz, dass diese Finanzierung schrittweise ins ordentliche Budget zu überführen ist. Gleich auf null zu gehen, geht uns zu weit. Wir möchten den Antrag unterstützen, dies entsprechend dem Beschluss des Ständerates schneller zu tun, d.[NB]h., nur 470 Millionen statt 600 Millionen Franken ausserordentlich zu verbuchen. Die dadurch ordentlich verbuchten 130 Millionen Franken kompensieren wir beim Kredit "Sozialhilfe Asylsuchende, vorläufig Aufgenommene, Flüchtlinge"; dies ist aufgrund der Erwartung tieferer Zugangszahlen möglich.
+Kern dieses Blocks ist die Sicherheit. Beim Fedpol zeigt sich klar: Wir wollen nicht einfach kürzen, wir wollen dort stärken, wo es nötig ist. Der Personalbestand, besonders bei der Bundeskriminalpolizei, ist zu tief. Das belegen der EFK-Bericht, die Antwort auf das Postulat der Finanzkommission und weitere Unterlagen eindeutig. Die Bekämpfung der Schwerstkriminalität ist gefährdet. Operativ ist eine Aufstockung schon 2026 möglich. Der Bundesrat plant sie erst ab 2027. Wir, die Mitte-Fraktion. Die Mitte. EVP, unterstützen die Erhöhung um 1,8 Millionen Franken für 10 zusätzliche Ermittlerstellen bereits ab nächstem Jahr sowie einen gestaffelten Ausbau ab 2027 zur Stärkung der inneren Sicherheit. Ein Zuwarten wäre fahrlässig. 
+Ähnlich ist es beim BACS. Die Cyberbedrohungslage verschärft sich massiv, und zentrale Wirtschaftssektoren benötigen Unterstützung. Auch hier zeigt ein Zusatzbericht klar Handlungsbedarf. Wir unterstützen auch hier eine Aufstockung um zusätzliche 10 Millionen Franken im Funktionsaufwand zur Stärkung der Cyberresilienz.
+Bei der Verteidigung geht es um die Umsetzung des parlamentarischen Auftrags des letzten Jahres: mehr Rüstungsinvestitionen und tiefere Betriebsausgaben durch Effizienzmassnahmen. Wir unterstützen den Antrag, bei der Position "Rüstungsaufwand und -investitionen" 50 Millionen Franken mehr zu sprechen und 25 Millionen Franken bei der Position "Funktionsaufwand (Globalbudget)" zu kompensieren oder zu sparen. Der Ständerat möchte weiter gehen. Er möchte 70 Millionen Franken zusätzlich investieren. Hier liegt nun auch der Einzelantrag Nause vor. Angesichts der sicherheitspolitischen Lage und Bedrohung - Stichwort Drohnen über Belgien, Deutschland, Dänemark und sogar auch über der Schweiz, über dem Flugplatz Meiringen - müssen wir bei den Investitionen tatsächlich einen Zacken zulegen. Wir unterstützen den Einzelantrag Nause, zusätzliche 70 Millionen Franken bereits in diesem Budget einzustellen. Der Pfad, 1 Prozent des BIP bis 2032 für die Armee aufzuwenden, bleibt unverändert.
+Die Mitte-Fraktion steht für eine verantwortungsvolle Finanzpolitik. Wir sparen dort, wo es möglich ist, und investieren dort, wo es für Sicherheit und Stabilität notwendig ist.
 </t>
   </si>
   <si>
@@ -734,157 +811,10 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">365999</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nationalrat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bürgi Roman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich begründe meinen Minderheitsantrag zum Funktionsaufwand des Bundesamts für Polizei. Der Bundesrat beantragt ein Globalbudget von 294 Millionen Franken. Die Mehrheit der Kommission möchte diesen Betrag nun um weitere 1,8 Millionen Franken erhöhen. Die SVP-Fraktion lehnt diese Aufstockung ab und beantragt, dem Bundesrat zu folgen. 
-Aus Sicht der SVP-Fraktion ist unbestritten, dass die Bundeskriminalpolizei zusätzliche Manpower an der Front benötigt. Das steht aber nicht zur Diskussion. Die Frag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich begründe meinen Minderheitsantrag zum Funktionsaufwand des Bundesamts für Polizei. Der Bundesrat beantragt ein Globalbudget von 294 Millionen Franken. Die Mehrheit der Kommission möchte diesen Betrag nun um weitere 1,8 Millionen Franken erhöhen. Die SVP-Fraktion lehnt diese Aufstockung ab und beantragt, dem Bundesrat zu folgen. 
-Aus Sicht der SVP-Fraktion ist unbestritten, dass die Bundeskriminalpolizei zusätzliche Manpower an der Front benötigt. Das steht aber nicht zur Diskussion. Die Frage ist vielmehr, ob wir eine strukturelle Budgeterhöhung sprechen sollen, bevor klar ist, wo und wie das Fedpol die zusätzlichen Stellen tatsächlich einsetzt. 
-Die Beratungen haben deutlich gezeigt, dass das Fedpol in der Vergangenheit primär hinsichtlich der Verwaltung und in der Kommunikation und nicht bei der operativen Kriminalpolizei ausgebaut wurde. Das Fedpol hat in den letzten Jahren Ressourcen erhalten, aber eben nicht für die Bereiche, in denen der eigentliche Bedarf besteht. Auch der EFK-Bericht bestätigt, dass intern bereits Effizienzsteigerungen im Gang und Kompensationen vorgenommen worden sind. Gleichzeitig aber bleibt unklar, weshalb genau jetzt externe Mittel über zusätzliche Stellen gesprochen werden müssen, bevor das Fedpol intern das vorhandene Potenzial ausgeschöpft hat. 
-Die Bundeskriminalpolizei verfügt heute über rund 700 Stellen, und der Bundesrat plant bereits 51 neue Stellen im Jahr 2026. Doch gemäss den Unterlagen entfallen davon nur sehr wenige auf die Ermittlungsarbeit, während der Rest für neue Projekte, für die IT-Weiterentwicklung und für die Bewirtschaftung des Verwaltungszentrums vorgesehen ist. Das hat mit der eigentlichen Kriminalbekämpfung wenig zu tun. 
-Bevor wir also zusätzliche Mittel bewilligen, erwarten wir zwei Dinge: Erstens muss das Fedpol intern jene Stellenprozente kompensieren, die es gemäss eigenen Aussagen einsparen kann, und zweitens braucht es ein klares Konzept, das detailliert aufzeigt, wo die zusätzlichen Ermittlungsstellen tatsächlich eingesetzt werden sollen. Wir fragten zu Recht, weshalb das Fedpol im ordentlichen Voranschlag nicht selbst mehr Ermittlungsstellen beantragte und weshalb im Entwicklungsrahmen zwar mehr Stellen gefordert wurden, diese dann aber nicht priorisiert wurden. Solange diese Fragen nicht beantwortet sind, ist eine Erhöhung des Budgets um 1,8 Millionen Franken nicht nachvollziehbar. Ich möchte betonen: Es geht nicht darum, die Sicherheit zu schwächen oder die Bedrohungslage zu verharmlosen. Es geht darum, dass wir zuerst sicherstellen müssen, dass die Bundesverwaltung ihre Mittel richtig einsetzt. Wenn das Fedpol erklärt, dass es intern noch Kompensationspotenzial hat, und gleichzeitig bestimmte Stellenpriorisierungen nicht vorgenommen wurden, ist es nicht sachgerecht, jetzt zusätzliches Geld zu sprechen. [PAGE 2100] 
-Der Bundesrat hat diese Abwägung gemacht und ist zum Schluss gekommen, dass 294 Millionen Franken ausreichend sind. Die SVP-Fraktion folgt dieser Einschätzung.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">366005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andrey Gerhard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ja, dieser wichtige EFK-Bericht ist der Finanzkommission natürlich bekannt. Ich würde Ihnen antworten: das eine tun, das andere nicht lassen. Ich bin mit Ihnen natürlich völlig einig, dass die Ressourcen möglichst effizient eingesetzt werden müssen. Aber wenn man genau hinschaut, auch bei den anderen Staatsebenen, sieht man, dass es sich tatsächlich um ein substanzielles Ressourcenproblem handelt. Entsprechend helfen wir da mit.
-Es ist eine spezielle Situation, dass Ihre Fraktion, die Law-and-Or</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ja, dieser wichtige EFK-Bericht ist der Finanzkommission natürlich bekannt. Ich würde Ihnen antworten: das eine tun, das andere nicht lassen. Ich bin mit Ihnen natürlich völlig einig, dass die Ressourcen möglichst effizient eingesetzt werden müssen. Aber wenn man genau hinschaut, auch bei den anderen Staatsebenen, sieht man, dass es sich tatsächlich um ein substanzielles Ressourcenproblem handelt. Entsprechend helfen wir da mit.
-Es ist eine spezielle Situation, dass Ihre Fraktion, die Law-and-Order-Fraktion, hier kritisch ist, wo es um mehr Polizei geht, und wir mit der Kommissionsmehrheit dafür sind. Das ist eine interessante Ausgangslage. Aber ich würde auf jeden Fall meinen: das eine tun, das andere nicht lassen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">366006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fischer Benjamin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geschätzter Kollege Andrey, ist Ihnen der EFK-Prüfbericht zur Ressourcensituation des Fedpol bekannt? Darin stellt die Eidgenössische Finanzkontrolle Mängel fest und hält auch klar fest, dass es ein Ressourcenproblem, aber auch ein grosses Potenzial gebe und[NB]man[NB]zuerst[NB]intern diese Ressourcen freispielen müsse, bevor das Parlament für das Fedpol wieder zusätzliche Gelder spricht. [PAGE 2103] 
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">366067</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bürgin Yvonne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich spreche für die Mitte-Fraktion. Die Mitte. EVP zu Block 2, "Justiz, Sicherheit und Migration". Dieser Block betrifft zentrale Aufgaben unseres Staates, den Schutz des Rechtsstaats, die innere Sicherheit, die Cyberresilienz und die Steuerung der Migration. Unsere Haltung ist klar und ziemlich einfach. Wir unterstützen alle Mehrheitsanträge der Finanzkommission und lehnen alle Minderheitsanträge ab.
-Ein Punkt ist uns besonders wichtig. Neue Stellen betrachten wir grundsätzlich kritisch. Die Ve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich spreche für die Mitte-Fraktion. Die Mitte. EVP zu Block 2, "Justiz, Sicherheit und Migration". Dieser Block betrifft zentrale Aufgaben unseres Staates, den Schutz des Rechtsstaats, die innere Sicherheit, die Cyberresilienz und die Steuerung der Migration. Unsere Haltung ist klar und ziemlich einfach. Wir unterstützen alle Mehrheitsanträge der Finanzkommission und lehnen alle Minderheitsanträge ab.
-Ein Punkt ist uns besonders wichtig. Neue Stellen betrachten wir grundsätzlich kritisch. Die Verwaltung wächst seit Jahren. Es braucht Prioritäten und Effizienz, nicht reflexartige Aufstockungen. Gleichzeitig gilt: Wo Sicherheit und Funktionsfähigkeit des Staates gefährdet sind, müssen wir handeln. Das betrifft insbesondere das Fedpol und das Bundesamt für Cybersicherheit (BACS). Dort unterstützen wir zusätzliche Stellen ausdrücklich. Und ich möchte auch noch eine Antwort auf die Frage von vorhin von Herrn Fischer an Herrn Andrey geben: Ja, intern wurde schon sehr viel gemacht, aber das Fedpol braucht mehr Stellen.
-Beim Budget müssen aber auch die Einnahmen betrachtet werden. Wir unterstützen eine Erhöhung, und zwar mithilfe der eingezogenen Vermögenswerte beim Bundesamt für Justiz. Die realisierten Werte lagen in den letzten Jahren regelmässig über dem Budget. Mit diesem Durchschnittswert der Vergangenheit ist eine realistische Planung möglich.
-Beim Staatssekretariat für Migration sehen wir die bekannten Dynamiken. Die Sozialhilfekosten im Asylbereich hängen direkt von den Zugangszahlen ab. Bei den Beiträgen an die Kantone bezüglich der Ukraine-Flüchtlinge sind die Zahlen stabil, aber ein Teil der Kosten wird immer noch ausserordentlich verbucht. Wir unterstützen den Ansatz, dass diese Finanzierung schrittweise ins ordentliche Budget zu überführen ist. Gleich auf null zu gehen, geht uns zu weit. Wir möchten den Antrag unterstützen, dies entsprechend dem Beschluss des Ständerates schneller zu tun, d.[NB]h., nur 470 Millionen statt 600 Millionen Franken ausserordentlich zu verbuchen. Die dadurch ordentlich verbuchten 130 Millionen Franken kompensieren wir beim Kredit "Sozialhilfe Asylsuchende, vorläufig Aufgenommene, Flüchtlinge"; dies ist aufgrund der Erwartung tieferer Zugangszahlen möglich.
-Kern dieses Blocks ist die Sicherheit. Beim Fedpol zeigt sich klar: Wir wollen nicht einfach kürzen, wir wollen dort stärken, wo es nötig ist. Der Personalbestand, besonders bei der Bundeskriminalpolizei, ist zu tief. Das belegen der EFK-Bericht, die Antwort auf das Postulat der Finanzkommission und weitere Unterlagen eindeutig. Die Bekämpfung der Schwerstkriminalität ist gefährdet. Operativ ist eine Aufstockung schon 2026 möglich. Der Bundesrat plant sie erst ab 2027. Wir, die Mitte-Fraktion. Die Mitte. EVP, unterstützen die Erhöhung um 1,8 Millionen Franken für 10 zusätzliche Ermittlerstellen bereits ab nächstem Jahr sowie einen gestaffelten Ausbau ab 2027 zur Stärkung der inneren Sicherheit. Ein Zuwarten wäre fahrlässig. 
-Ähnlich ist es beim BACS. Die Cyberbedrohungslage verschärft sich massiv, und zentrale Wirtschaftssektoren benötigen Unterstützung. Auch hier zeigt ein Zusatzbericht klar Handlungsbedarf. Wir unterstützen auch hier eine Aufstockung um zusätzliche 10 Millionen Franken im Funktionsaufwand zur Stärkung der Cyberresilienz.
-Bei der Verteidigung geht es um die Umsetzung des parlamentarischen Auftrags des letzten Jahres: mehr Rüstungsinvestitionen und tiefere Betriebsausgaben durch Effizienzmassnahmen. Wir unterstützen den Antrag, bei der Position "Rüstungsaufwand und -investitionen" 50 Millionen Franken mehr zu sprechen und 25 Millionen Franken bei der Position "Funktionsaufwand (Globalbudget)" zu kompensieren oder zu sparen. Der Ständerat möchte weiter gehen. Er möchte 70 Millionen Franken zusätzlich investieren. Hier liegt nun auch der Einzelantrag Nause vor. Angesichts der sicherheitspolitischen Lage und Bedrohung - Stichwort Drohnen über Belgien, Deutschland, Dänemark und sogar auch über der Schweiz, über dem Flugplatz Meiringen - müssen wir bei den Investitionen tatsächlich einen Zacken zulegen. Wir unterstützen den Einzelantrag Nause, zusätzliche 70 Millionen Franken bereits in diesem Budget einzustellen. Der Pfad, 1 Prozent des BIP bis 2032 für die Armee aufzuwenden, bleibt unverändert.
-Die Mitte-Fraktion steht für eine verantwortungsvolle Finanzpolitik. Wir sparen dort, wo es möglich ist, und investieren dort, wo es für Sicherheit und Stabilität notwendig ist.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">367087</t>
+    <t xml:space="preserve">367075</t>
   </si>
   <si>
     <t xml:space="preserve">20251211</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jans Beat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mit dieser Motion ist ja vorgesehen, dass die Bundeskriminalpolizei (BKP) personell etappenweise verstärkt wird. Aus unserer Sicht ist das zwingend nötig. Sie und der Nationalrat sehen das erfreulicherweise gleich. Sie haben an der diesjährigen Budgetberatung in beiden Räten beschlossen, dass das Fedpol für das Jahr 2026 vorbehältlich der Schlussabstimmung 1,8 Millionen Franken mehr personelle Mittel bekommt; das entspricht zehn Ermittlerinnen und Ermittlern für die BKP. Das ist ein wichtiger Sc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mit dieser Motion ist ja vorgesehen, dass die Bundeskriminalpolizei (BKP) personell etappenweise verstärkt wird. Aus unserer Sicht ist das zwingend nötig. Sie und der Nationalrat sehen das erfreulicherweise gleich. Sie haben an der diesjährigen Budgetberatung in beiden Räten beschlossen, dass das Fedpol für das Jahr 2026 vorbehältlich der Schlussabstimmung 1,8 Millionen Franken mehr personelle Mittel bekommt; das entspricht zehn Ermittlerinnen und Ermittlern für die BKP. Das ist ein wichtiger Schritt hin zu einer wirksameren Bekämpfung der Schwerkriminalität. 
-Der Bundesrat will für den Aufbau der Bundeskriminalpolizei aber eben die ordentlichen Prozesse nutzen. Das heisst, eine solche personelle Verstärkung müssen wir als EJPD in den ordentlichen Budgetprozess eingeben und eine Genehmigung beantragen. Deshalb empfiehlt der Bundesrat die vorliegende Motion zur Ablehnung. Das heisst aber auch, Herr Salzmann, dass der Bundesrat dann Anfang 2026 über Prioritäten entscheiden muss; denn es ist jetzt schon klar, dass die verfügbaren Ressourcen bei Weitem nicht genügen, um alle Stellenanträge der Departemente zu erfüllen. Sollte der Bundesrat eine Erhöhung der Stellen bei der BKP genehmigen, wie wir das als EJPD beantragen - auch aufgrund der verschiedenen Berichte, die uns zugrunde liegen -, so würden die entsprechenden Mittel aber in jedem Fall frühestens 2027 zur Verfügung stehen. Mit zusätzlichen Ressourcen für das Fedpol und namentlich für die BKP, gestaffelt über die nächsten Jahre, können gezielt Stellen geschaffen werden - dort, wo die Not am grössten ist und wo sie den grössten Beitrag zur Sicherheit leisten. Mir als Departementsvorsteher ist es ein wichtiges Anliegen, dass wir klar darlegen können, wofür genau es diese Stellen braucht, welchen Nutzen sie haben und wie wir die Prioritäten entsprechend setzen. Wir sind gemeinsam auf diesem Weg, die innere Sicherheit dort, wo es ihrer bedarf, zu stärken. 
-Ich möchte mich aber gegen die Vorwürfe, dass strategisches oder konzeptionelles Vorgehen fehlt, doch ein bisschen wehren, Herr Hegglin. Der EFK-Bericht war für mich zwingend. Bevor ich überhaupt Stellen beantrage, wollte ich diesen Bericht hören und sehen. Ich gehöre nicht zu den Departementsvorstehern, die in den letzten Jahren einfach gesagt haben: "Wir brauchen, wir brauchen, und wir stellen ein", sondern ich habe gesagt, dass wir das anders machen müssen, dass wir das abstützen müssen, dass wir das strategisch korrekt machen müssen. Da haben wir eben von der EFK klar - und das gibt es selten - den Hinweis erhalten, dass die BKP zusätzliche Mittel braucht, um in der aktuellen Situation die Aufgaben zu erfüllen; das ist klar. Sie sagt aber auch, dass wir eine Reorganisation machen müssen, dass wir auch Stellen im Bereich Kopf wegnehmen müssen und in den Bereich der Ermittler bringen. Auch das gehen wir an, die neue Fedpol-Leitung ist an diesem Vorhaben dran. Das sind nicht einfache Entscheide, das wissen Sie auch; man kann Leute nicht einfach von einem Tag auf den anderen zu Spezialisten machen. Das sind anstrengende, wichtige Prozesse, die wir sehr ernst nehmen. Also wir sind da unterwegs. 
-Aber was ich wirklich wichtig finde, ist, dass wir das alle sehen, auch Sie bitte, Herr Rieder: Der Bedarf ist da, und das ist nicht nur mit diesen neuesten Statistiken zu erfassen. Wir haben heute ein ganz anderes Lagebild, das sagt uns Europol in all ihren Untersuchungen. Wir haben verschiedene Länder, die es verpasst haben, rechtzeitig gegen die organisierte Kriminalität vorzugehen. Diese haben auch Unterlassungen gemacht und sind in ihren Strafverfahren zu wenig [PAGE 1322] streng gewesen. Das hat dazu geführt, dass sie heute zum Teil - ich rede jetzt von Holland, ich rede von Dänemark und von Schweden - offene Bandenkriminalität in ihren Städten bekämpfen müssen.
-Wenn Sie damit zu spät anfangen oder spät anfangen, kann es sein, dass Sie dann zu spät sind. Das ist das, was mir die EU-Innenminister letzte Woche alle gesagt haben. Da müssen wir rechtzeitig sein, und da müssen wir genau hinschauen. Die Schweiz ist als Finanzplatz für die organisierte Kriminalität exponiert. Wir werden mit dieser Strategie kommen, und zwar schon sehr bald: erstens mit der Sicherheitsstrategie und darin eingebettet mit der Strategie für organisierte Kriminalität. Wir werden zweitens - das ist Teil dieser Strategie - Gesetzesänderungen vorschlagen, um den Strafverfolgungsbehörden auch bessere Instrumente an die Hand zu geben, nicht nur mehr Personal. Das ist etwas, das wir feststellen: Die Fälle insbesondere zur Bekämpfung der organisierten Kriminalität sind auch sehr viel komplizierter geworden.
-Der Bundesanwalt, mit dem ich heute Morgen noch telefonieren konnte, begrüsst es sehr, dass es für Fälle, die er zum Teil heute einfach nicht bewältigen kann, mehr Ermittler geben soll, Fälle, bei denen er zum Teil bis zu 20 oder sogar mehr Ermittler braucht - das für einen einzigen Fall. Sie stellen sich wahrscheinlich immer vor, ein Fall, ein Ermittler. Das ist leider nicht so. Die Fälle sind unglaublich kompliziert, und gerade die Netzwerke der organisierten Kriminalität nehmen ihre Verteidigungsrechte, die sie mit der Strafprozessordnung neu erhalten haben, sehr exzessiv wahr. Die machen mit einem Heer von besten Anwälten alles, um die Prozesse zu verlängern und komplizierter zu machen, um weitere Berichte und Untersuchungen einzufordern. Das ist die Realität, der wir uns stellen müssen. Diese wurde noch durch die Tatsache verschärft - das ist ganz wichtig, was Frau Gmür-Schönenberger gesagt hat -, dass die organisierte Kriminalität im Internet stattfindet. Dort müssen wir besser werden. Es ist enorm kompliziert und aufwendig, die grenzüberschreitend im virtuellen Bereich tätigen Banden zu knacken. Aber es ist wegen des Risikos für die Sicherheit unserer Bevölkerung, aber auch wegen des Image unseres Landes, wegen der Reputation, die auf der Kippe steht, unglaublich wichtig. 
-Deshalb ist es wichtig, dass wir hier vorangehen und dass wir schrittweise vorgehen. Der Bundesrat braucht diese Motion nicht dafür, wir werden diese Entscheide schrittweise im Rahmen der ordentlichen Budgetprozesse fällen, aber es ist wichtig, das möchte ich doch noch sagen, dass Sie den Handlungsbedarf wirklich erkennen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">367062</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conseil des Etats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juillard Charles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je vais m'exprimer en tant que membre de la Commission de la politique de sécurité, mais aussi en tant que membre et ancien président de la Commission de gestion, puisque nous avons abordé la question des effectifs de Fedpol à plusieurs reprises lors des séances de la Commission de gestion, et que nous sommes arrivés à la conclusion qu'il y avait un vrai problème d'effectifs concernant les enquêteurs de Fedpol. C'est aussi dans cet esprit que nous avons écrit au Conseil fédéral pour qu'il envisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je vais m'exprimer en tant que membre de la Commission de la politique de sécurité, mais aussi en tant que membre et ancien président de la Commission de gestion, puisque nous avons abordé la question des effectifs de Fedpol à plusieurs reprises lors des séances de la Commission de gestion, et que nous sommes arrivés à la conclusion qu'il y avait un vrai problème d'effectifs concernant les enquêteurs de Fedpol. C'est aussi dans cet esprit que nous avons écrit au Conseil fédéral pour qu'il envisage l'augmentation des effectifs, ce qui va dans le même sens que cette motion. Je dois cependant vous dire que nous n'avons pas examiné dans le détail si ces postes supplémentaires, - ces postes d'enquêteurs, parce que c'est surtout là qu'il y a un problème -, pouvaient être en tout ou partie compensés par une réorganisation de Fedpol - qui s'impose, selon le Contrôle fédéral des finances -, et s'il serait possible de diminuer les postes dans le domaine administratif pour les concentrer sur le terrain, là où les besoins se font particulièrement sentir, si l'on écoute aussi le Ministère public de la Confédération. Je voulais vous donner ces informations.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">367096</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommaruga Carlo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je prends la parole en tant que président de la sous-commission de la Commission de gestion qui s'occupe du DFJP et de la Chancellerie fédérale. Ce sujet, nous l'avons traité à plusieurs reprises et le faisons depuis fort longtemps. Nous avons entendu le procureur général de la Confédération, nous avons entendu l'ancienne et la nouvelle directrice de Fedpol et différentes autres personnes. Sur cette base-là, nous avons pu constater de manière claire que les personnes entendues relevaient qu'il y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je prends la parole en tant que président de la sous-commission de la Commission de gestion qui s'occupe du DFJP et de la Chancellerie fédérale. Ce sujet, nous l'avons traité à plusieurs reprises et le faisons depuis fort longtemps. Nous avons entendu le procureur général de la Confédération, nous avons entendu l'ancienne et la nouvelle directrice de Fedpol et différentes autres personnes. Sur cette base-là, nous avons pu constater de manière claire que les personnes entendues relevaient qu'il y a aujourd'hui un déficit de personnel pour assurer la sécurité de la Suisse au niveau des infractions qui sont de la compétence fédérale et donc de la compétence du DFJP.
-J'entends bien les chiffres de notre collègue Rieder, mais ces chiffres ne reflètent pas la réalité qui nous est décrite par le procureur général de la Confédération et dont les termes ont été rappelés par notre collègue Dittli, à savoir que, aujourd'hui, il y a des procédures pénales concernant surtout la criminalité organisée internationale qui ne peuvent pas être ouvertes parce qu'il n'y a pas assez de personnel spécialisé. Je pense que cet élément doit être pris en compte.
-Si cette motion est aujourd'hui sur la table, c'est parce qu'il y a non seulement le rapport du Contrôle fédéral des finances, mais également des rapports de la Commission de gestion. Ce sont des éléments essentiels, et j'avoue que je suis surpris que l'on conteste les travaux faits par la Commission de gestion, et au Conseil national et au Conseil des États, sur la situation au niveau du procureur général et au niveau de Fedpol.
-J'aimerais juste dire que l'élément central qui a été évoqué par notre collègue, ce n'est pas la stabilité des plaintes ou des procédures qui ont été ouvertes de manière générale, c'est la criminalité organisée. Il a confirmé qu'il y avait une augmentation de 8 pour cent des affaires. Or, ce ne sont pas seulement les chiffres qu'il faut regarder, mais aussi la complexité des procédures qui sont ouvertes. Aujourd'hui, elles sont de plus en plus complexes dans le cadre de la poursuite pénale.
-J'aimerais juste relever que ce ne sont pas seulement des gigabits ou des mégabits qu'il faut examiner dans le cadre de toutes ces saisies de données faites en rapport avec la criminalité organisée, mais aussi les boîtes mail et les téléphones cryptés, et que cela nécessite des spécialistes. Aujourd'hui, le problème est immédiat. Il n'y a pas lieu d'attendre ou de compter sur le fait que des personnes vont partir à la retraite, même dans d'autres domaines, pour pouvoir engager du personnel.
-Je prends juste un exemple[NB]: il n'y a pas très longtemps, Fedpol a dû s'occuper d'un cas très particulier, celui des bombes qui avaient été placées pour faire chanter Patek Philippe. Pour rappel, cela s'est passé à Genève. Des bombes artisanales ont été mises dans des boîtes aux lettres et il y a eu des blessés. Il a fallu déployer des moyens extrêmement importants, non seulement à Genève, mais également au niveau de Fedpol qui disposait de spécialiste, pour enfin trouver la personne responsable de ces actes. J'aimerais relever que ce sont aussi des procédures qui, en général, demandent beaucoup, beaucoup de ressources humaines, et des ressources humaines spécialisées.
-Dès lors, je veux simplement vous dire que si l'on veut avoir une sécurité de la Suisse non seulement extérieure mais aussi intérieure, je crois qu'il faut entendre le message qui nous est donné par Fedpol, par le procureur général et par la Commission de gestion.
-Je vous invite donc à accepter cette motion, comme le propose la majorité de la commission.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">367075</t>
   </si>
   <si>
     <t xml:space="preserve">Gmür-Schönenberger Andrea</t>
@@ -925,6 +855,28 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">367087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jans Beat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit dieser Motion ist ja vorgesehen, dass die Bundeskriminalpolizei (BKP) personell etappenweise verstärkt wird. Aus unserer Sicht ist das zwingend nötig. Sie und der Nationalrat sehen das erfreulicherweise gleich. Sie haben an der diesjährigen Budgetberatung in beiden Räten beschlossen, dass das Fedpol für das Jahr 2026 vorbehältlich der Schlussabstimmung 1,8 Millionen Franken mehr personelle Mittel bekommt; das entspricht zehn Ermittlerinnen und Ermittlern für die BKP. Das ist ein wichtiger Sc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit dieser Motion ist ja vorgesehen, dass die Bundeskriminalpolizei (BKP) personell etappenweise verstärkt wird. Aus unserer Sicht ist das zwingend nötig. Sie und der Nationalrat sehen das erfreulicherweise gleich. Sie haben an der diesjährigen Budgetberatung in beiden Räten beschlossen, dass das Fedpol für das Jahr 2026 vorbehältlich der Schlussabstimmung 1,8 Millionen Franken mehr personelle Mittel bekommt; das entspricht zehn Ermittlerinnen und Ermittlern für die BKP. Das ist ein wichtiger Schritt hin zu einer wirksameren Bekämpfung der Schwerkriminalität. 
+Der Bundesrat will für den Aufbau der Bundeskriminalpolizei aber eben die ordentlichen Prozesse nutzen. Das heisst, eine solche personelle Verstärkung müssen wir als EJPD in den ordentlichen Budgetprozess eingeben und eine Genehmigung beantragen. Deshalb empfiehlt der Bundesrat die vorliegende Motion zur Ablehnung. Das heisst aber auch, Herr Salzmann, dass der Bundesrat dann Anfang 2026 über Prioritäten entscheiden muss; denn es ist jetzt schon klar, dass die verfügbaren Ressourcen bei Weitem nicht genügen, um alle Stellenanträge der Departemente zu erfüllen. Sollte der Bundesrat eine Erhöhung der Stellen bei der BKP genehmigen, wie wir das als EJPD beantragen - auch aufgrund der verschiedenen Berichte, die uns zugrunde liegen -, so würden die entsprechenden Mittel aber in jedem Fall frühestens 2027 zur Verfügung stehen. Mit zusätzlichen Ressourcen für das Fedpol und namentlich für die BKP, gestaffelt über die nächsten Jahre, können gezielt Stellen geschaffen werden - dort, wo die Not am grössten ist und wo sie den grössten Beitrag zur Sicherheit leisten. Mir als Departementsvorsteher ist es ein wichtiges Anliegen, dass wir klar darlegen können, wofür genau es diese Stellen braucht, welchen Nutzen sie haben und wie wir die Prioritäten entsprechend setzen. Wir sind gemeinsam auf diesem Weg, die innere Sicherheit dort, wo es ihrer bedarf, zu stärken. 
+Ich möchte mich aber gegen die Vorwürfe, dass strategisches oder konzeptionelles Vorgehen fehlt, doch ein bisschen wehren, Herr Hegglin. Der EFK-Bericht war für mich zwingend. Bevor ich überhaupt Stellen beantrage, wollte ich diesen Bericht hören und sehen. Ich gehöre nicht zu den Departementsvorstehern, die in den letzten Jahren einfach gesagt haben: "Wir brauchen, wir brauchen, und wir stellen ein", sondern ich habe gesagt, dass wir das anders machen müssen, dass wir das abstützen müssen, dass wir das strategisch korrekt machen müssen. Da haben wir eben von der EFK klar - und das gibt es selten - den Hinweis erhalten, dass die BKP zusätzliche Mittel braucht, um in der aktuellen Situation die Aufgaben zu erfüllen; das ist klar. Sie sagt aber auch, dass wir eine Reorganisation machen müssen, dass wir auch Stellen im Bereich Kopf wegnehmen müssen und in den Bereich der Ermittler bringen. Auch das gehen wir an, die neue Fedpol-Leitung ist an diesem Vorhaben dran. Das sind nicht einfache Entscheide, das wissen Sie auch; man kann Leute nicht einfach von einem Tag auf den anderen zu Spezialisten machen. Das sind anstrengende, wichtige Prozesse, die wir sehr ernst nehmen. Also wir sind da unterwegs. 
+Aber was ich wirklich wichtig finde, ist, dass wir das alle sehen, auch Sie bitte, Herr Rieder: Der Bedarf ist da, und das ist nicht nur mit diesen neuesten Statistiken zu erfassen. Wir haben heute ein ganz anderes Lagebild, das sagt uns Europol in all ihren Untersuchungen. Wir haben verschiedene Länder, die es verpasst haben, rechtzeitig gegen die organisierte Kriminalität vorzugehen. Diese haben auch Unterlassungen gemacht und sind in ihren Strafverfahren zu wenig [PAGE 1322] streng gewesen. Das hat dazu geführt, dass sie heute zum Teil - ich rede jetzt von Holland, ich rede von Dänemark und von Schweden - offene Bandenkriminalität in ihren Städten bekämpfen müssen.
+Wenn Sie damit zu spät anfangen oder spät anfangen, kann es sein, dass Sie dann zu spät sind. Das ist das, was mir die EU-Innenminister letzte Woche alle gesagt haben. Da müssen wir rechtzeitig sein, und da müssen wir genau hinschauen. Die Schweiz ist als Finanzplatz für die organisierte Kriminalität exponiert. Wir werden mit dieser Strategie kommen, und zwar schon sehr bald: erstens mit der Sicherheitsstrategie und darin eingebettet mit der Strategie für organisierte Kriminalität. Wir werden zweitens - das ist Teil dieser Strategie - Gesetzesänderungen vorschlagen, um den Strafverfolgungsbehörden auch bessere Instrumente an die Hand zu geben, nicht nur mehr Personal. Das ist etwas, das wir feststellen: Die Fälle insbesondere zur Bekämpfung der organisierten Kriminalität sind auch sehr viel komplizierter geworden.
+Der Bundesanwalt, mit dem ich heute Morgen noch telefonieren konnte, begrüsst es sehr, dass es für Fälle, die er zum Teil heute einfach nicht bewältigen kann, mehr Ermittler geben soll, Fälle, bei denen er zum Teil bis zu 20 oder sogar mehr Ermittler braucht - das für einen einzigen Fall. Sie stellen sich wahrscheinlich immer vor, ein Fall, ein Ermittler. Das ist leider nicht so. Die Fälle sind unglaublich kompliziert, und gerade die Netzwerke der organisierten Kriminalität nehmen ihre Verteidigungsrechte, die sie mit der Strafprozessordnung neu erhalten haben, sehr exzessiv wahr. Die machen mit einem Heer von besten Anwälten alles, um die Prozesse zu verlängern und komplizierter zu machen, um weitere Berichte und Untersuchungen einzufordern. Das ist die Realität, der wir uns stellen müssen. Diese wurde noch durch die Tatsache verschärft - das ist ganz wichtig, was Frau Gmür-Schönenberger gesagt hat -, dass die organisierte Kriminalität im Internet stattfindet. Dort müssen wir besser werden. Es ist enorm kompliziert und aufwendig, die grenzüberschreitend im virtuellen Bereich tätigen Banden zu knacken. Aber es ist wegen des Risikos für die Sicherheit unserer Bevölkerung, aber auch wegen des Image unseres Landes, wegen der Reputation, die auf der Kippe steht, unglaublich wichtig. 
+Deshalb ist es wichtig, dass wir hier vorangehen und dass wir schrittweise vorgehen. Der Bundesrat braucht diese Motion nicht dafür, wir werden diese Entscheide schrittweise im Rahmen der ordentlichen Budgetprozesse fällen, aber es ist wichtig, das möchte ich doch noch sagen, dass Sie den Handlungsbedarf wirklich erkennen.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">367106</t>
   </si>
   <si>
@@ -948,13 +900,49 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">367062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juillard Charles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je vais m'exprimer en tant que membre de la Commission de la politique de sécurité, mais aussi en tant que membre et ancien président de la Commission de gestion, puisque nous avons abordé la question des effectifs de Fedpol à plusieurs reprises lors des séances de la Commission de gestion, et que nous sommes arrivés à la conclusion qu'il y avait un vrai problème d'effectifs concernant les enquêteurs de Fedpol. C'est aussi dans cet esprit que nous avons écrit au Conseil fédéral pour qu'il envisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je vais m'exprimer en tant que membre de la Commission de la politique de sécurité, mais aussi en tant que membre et ancien président de la Commission de gestion, puisque nous avons abordé la question des effectifs de Fedpol à plusieurs reprises lors des séances de la Commission de gestion, et que nous sommes arrivés à la conclusion qu'il y avait un vrai problème d'effectifs concernant les enquêteurs de Fedpol. C'est aussi dans cet esprit que nous avons écrit au Conseil fédéral pour qu'il envisage l'augmentation des effectifs, ce qui va dans le même sens que cette motion. Je dois cependant vous dire que nous n'avons pas examiné dans le détail si ces postes supplémentaires, - ces postes d'enquêteurs, parce que c'est surtout là qu'il y a un problème -, pouvaient être en tout ou partie compensés par une réorganisation de Fedpol - qui s'impose, selon le Contrôle fédéral des finances -, et s'il serait possible de diminuer les postes dans le domaine administratif pour les concentrer sur le terrain, là où les besoins se font particulièrement sentir, si l'on écoute aussi le Ministère public de la Confédération. Je voulais vous donner ces informations.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">367096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sommaruga Carlo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je prends la parole en tant que président de la sous-commission de la Commission de gestion qui s'occupe du DFJP et de la Chancellerie fédérale. Ce sujet, nous l'avons traité à plusieurs reprises et le faisons depuis fort longtemps. Nous avons entendu le procureur général de la Confédération, nous avons entendu l'ancienne et la nouvelle directrice de Fedpol et différentes autres personnes. Sur cette base-là, nous avons pu constater de manière claire que les personnes entendues relevaient qu'il y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je prends la parole en tant que président de la sous-commission de la Commission de gestion qui s'occupe du DFJP et de la Chancellerie fédérale. Ce sujet, nous l'avons traité à plusieurs reprises et le faisons depuis fort longtemps. Nous avons entendu le procureur général de la Confédération, nous avons entendu l'ancienne et la nouvelle directrice de Fedpol et différentes autres personnes. Sur cette base-là, nous avons pu constater de manière claire que les personnes entendues relevaient qu'il y a aujourd'hui un déficit de personnel pour assurer la sécurité de la Suisse au niveau des infractions qui sont de la compétence fédérale et donc de la compétence du DFJP.
+J'entends bien les chiffres de notre collègue Rieder, mais ces chiffres ne reflètent pas la réalité qui nous est décrite par le procureur général de la Confédération et dont les termes ont été rappelés par notre collègue Dittli, à savoir que, aujourd'hui, il y a des procédures pénales concernant surtout la criminalité organisée internationale qui ne peuvent pas être ouvertes parce qu'il n'y a pas assez de personnel spécialisé. Je pense que cet élément doit être pris en compte.
+Si cette motion est aujourd'hui sur la table, c'est parce qu'il y a non seulement le rapport du Contrôle fédéral des finances, mais également des rapports de la Commission de gestion. Ce sont des éléments essentiels, et j'avoue que je suis surpris que l'on conteste les travaux faits par la Commission de gestion, et au Conseil national et au Conseil des États, sur la situation au niveau du procureur général et au niveau de Fedpol.
+J'aimerais juste dire que l'élément central qui a été évoqué par notre collègue, ce n'est pas la stabilité des plaintes ou des procédures qui ont été ouvertes de manière générale, c'est la criminalité organisée. Il a confirmé qu'il y avait une augmentation de 8 pour cent des affaires. Or, ce ne sont pas seulement les chiffres qu'il faut regarder, mais aussi la complexité des procédures qui sont ouvertes. Aujourd'hui, elles sont de plus en plus complexes dans le cadre de la poursuite pénale.
+J'aimerais juste relever que ce ne sont pas seulement des gigabits ou des mégabits qu'il faut examiner dans le cadre de toutes ces saisies de données faites en rapport avec la criminalité organisée, mais aussi les boîtes mail et les téléphones cryptés, et que cela nécessite des spécialistes. Aujourd'hui, le problème est immédiat. Il n'y a pas lieu d'attendre ou de compter sur le fait que des personnes vont partir à la retraite, même dans d'autres domaines, pour pouvoir engager du personnel.
+Je prends juste un exemple[NB]: il n'y a pas très longtemps, Fedpol a dû s'occuper d'un cas très particulier, celui des bombes qui avaient été placées pour faire chanter Patek Philippe. Pour rappel, cela s'est passé à Genève. Des bombes artisanales ont été mises dans des boîtes aux lettres et il y a eu des blessés. Il a fallu déployer des moyens extrêmement importants, non seulement à Genève, mais également au niveau de Fedpol qui disposait de spécialiste, pour enfin trouver la personne responsable de ces actes. J'aimerais relever que ce sont aussi des procédures qui, en général, demandent beaucoup, beaucoup de ressources humaines, et des ressources humaines spécialisées.
+Dès lors, je veux simplement vous dire que si l'on veut avoir une sécurité de la Suisse non seulement extérieure mais aussi intérieure, je crois qu'il faut entendre le message qui nous est donné par Fedpol, par le procureur général et par la Commission de gestion.
+Je vous invite donc à accepter cette motion, comme le propose la majorité de la commission.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">367621</t>
   </si>
   <si>
     <t xml:space="preserve">20251215</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conseil fédéral</t>
   </si>
   <si>
     <t xml:space="preserve">Parmelin Guy</t>
@@ -1058,6 +1046,23 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">368193</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stark Jakob</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und dabei ist zu beachten, dass das eine ureigene Aufgabe der Kantone ist und dass sich der Bund mit Spezialgesetzen im Ausländerrecht, in der ALV und IV hier schon engagiert. Aus diesem Grund beantragt der Bundesrat, die Bestimmungen aufzuheben. Die Entlastungswirkung ist bei 19,8 Millionen Franken.
+Diese drei Anträge, die Sie hier vor sich haben, sehen alle vor, auf die Gesetzesänderung zu verzichten, mit Verweis auf die Kann-Bestimmung in Artikel 12 Absatz 1 WeBiG. Es ist also ohne Weiteres möglich, das Gesetz so zu belassen und bei der entsprechenden Position im Voranschlag den Betrag anzupassen. Die Kommissionsmehrheit möchte die volle Entlastungswirkung beibehalten, also die gut 19 Millionen Franken. Die Minderheit I (Herzog Eva) möchte die Entlastungswirkung knapp halbieren, sie möchte hier weiterhin 10[NB]Millionen[NB]Franken budgetieren. Die Minderheit II (Maillard Pierre-Yves) empfiehlt Ihnen, auf eine Kürzung ganz zu verzichten.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">368245</t>
   </si>
   <si>
@@ -1066,23 +1071,6 @@
   <si>
     <t xml:space="preserve">Das ist ein bisschen ein Streit um des Kaisers Bart. Der Präsident der Finanzkommission hat es gesagt: Es geht um ein Rahmengesetz. An sich wollte der Bundesrat im Gesetz klarer festhalten, dass die Empfänger von Finanzhilfen ihre Aufgaben soweit möglich selbst finanzieren; das war auch immer ein Wunsch der Eidgenössischen Finanzkontrolle (EFK). Der Herr Präsident hat es gesagt: Es kamen dann Ängste aus dem Kultur- und dem Umweltbereich, dass durchgehend nur noch 50 Prozent Subventionen ausbezahlt würden. Das wäre nicht der Fall gewesen.
 Wenn Sie das streichen, ist das nicht gravierend, weil auch das aktuelle Recht davon ausgeht, und das ist wichtig, dass Subventionsempfänger nach Kräften und ihrer wirtschaftlichen Leistungsfähigkeit mitbeteiligt werden. In der Regel, nach ständiger Praxis der Eidgenössischen Finanzverwaltung, sind das 50 Prozent, aber das muss im Einzelfall festgelegt werden. Ich verzichte hier auf eine Abstimmung, wir können mit dem geltenden Recht leben, es war der Versuch einer Präzisierung. In der Sache wird das nicht viel daran ändern, dass man immer noch darum feilschen wird, welcher Subventionssatz im Einzelfall angewendet wird.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">368193</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stark Jakob</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Der Bundesrat beantragt, auf Finanzhilfen des Bundes im Bereich der Weiterbildung zu verzichten. Die Gründe sind folgende: Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert. Es gibt in diesem Bereich sehr namhafte Mitnahmeeffekte. Mehrfach schon gab es Kritik der Eidgenössischen Finanzkontrolle daran, wie und wofür diese Beiträge an die Organisationen der Weiterbildung gehen und wie ihre Wirkung ist. Schwergewichtig geht es hier ja um die Förderung der Grundkompetenzen, und dabei ist zu beachten, dass das eine ureigene Aufgabe der Kantone ist und dass sich der Bund mit Spezialgesetzen im Ausländerrecht, in der ALV und IV hier schon engagiert. Aus diesem Grund beantragt der Bundesrat, die Bestimmungen aufzuheben. Die Entlastungswirkung ist bei 19,8 Millionen Franken.
-Diese drei Anträge, die Sie hier vor sich haben, sehen alle vor, auf die Gesetzesänderung zu verzichten, mit Verweis auf die Kann-Bestimmung in Artikel 12 Absatz 1 WeBiG. Es ist also ohne Weiteres möglich, das Gesetz so zu belassen und bei der entsprechenden Position im Voranschlag den Betrag anzupassen. Die Kommissionsmehrheit möchte die volle Entlastungswirkung beibehalten, also die gut 19 Millionen Franken. Die Minderheit I (Herzog Eva) möchte die Entlastungswirkung knapp halbieren, sie möchte hier weiterhin 10[NB]Millionen[NB]Franken budgetieren. Die Minderheit II (Maillard Pierre-Yves) empfiehlt Ihnen, auf eine Kürzung ganz zu verzichten.
 </t>
   </si>
   <si>
@@ -1195,7 +1183,7 @@
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
-    <tableColumn id="3" name="CouncilName"/>
+    <tableColumn id="3" name="MeetingCouncilAbbreviation"/>
     <tableColumn id="4" name="SpeakerFullName"/>
     <tableColumn id="5" name="ParlGroupAbbreviation"/>
     <tableColumn id="6" name="CantonAbbreviation"/>
@@ -1730,75 +1718,77 @@
         <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9"/>
+        <v>48</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
         <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
         <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I11" t="s">
         <v>61</v>
@@ -1812,22 +1802,22 @@
         <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G12" t="s">
         <v>15</v>
       </c>
       <c r="H12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I12" t="s">
         <v>65</v>
@@ -1841,235 +1831,233 @@
         <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="E13"/>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="G13" t="s">
         <v>15</v>
       </c>
       <c r="H13" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13" t="s">
         <v>68</v>
-      </c>
-      <c r="I13" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
         <v>70</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
         <v>71</v>
       </c>
-      <c r="C14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
         <v>72</v>
-      </c>
-      <c r="E14"/>
-      <c r="F14" t="s">
-        <v>73</v>
       </c>
       <c r="G14" t="s">
         <v>15</v>
       </c>
       <c r="H14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" t="s">
         <v>74</v>
-      </c>
-      <c r="I14" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
         <v>13</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="H15" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I15" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" t="s">
         <v>82</v>
-      </c>
-      <c r="B16" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" t="s">
-        <v>77</v>
-      </c>
-      <c r="D16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" t="s">
-        <v>59</v>
-      </c>
-      <c r="H16" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E17" t="s">
-        <v>13</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G17" t="s">
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="I17" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
         <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="E18" t="s">
         <v>13</v>
       </c>
       <c r="F18" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="H18" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
         <v>11</v>
       </c>
       <c r="D19" t="s">
+        <v>95</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" t="s">
+        <v>55</v>
+      </c>
+      <c r="H19" t="s">
         <v>97</v>
       </c>
-      <c r="E19" t="s">
+      <c r="I19" t="s">
         <v>98</v>
-      </c>
-      <c r="F19" t="s">
-        <v>99</v>
-      </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
-        <v>100</v>
-      </c>
-      <c r="I19" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E20"/>
       <c r="F20" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G20" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="I20" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D21" t="s">
         <v>43</v>
@@ -2082,168 +2070,168 @@
         <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="I21" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C22" t="s">
         <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E22"/>
       <c r="F22" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G22" t="s">
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I22" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23"/>
+        <v>116</v>
+      </c>
+      <c r="E23" t="s">
+        <v>49</v>
+      </c>
       <c r="F23" t="s">
-        <v>44</v>
+        <v>117</v>
       </c>
       <c r="G23" t="s">
         <v>15</v>
       </c>
       <c r="H23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C24" t="s">
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
-      </c>
-      <c r="E24" t="s">
-        <v>53</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="E24"/>
       <c r="F24" t="s">
-        <v>124</v>
+        <v>44</v>
       </c>
       <c r="G24" t="s">
         <v>15</v>
       </c>
       <c r="H24" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I24" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E25" t="s">
         <v>25</v>
       </c>
       <c r="F25" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G25" t="s">
         <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I25" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B26" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E26" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="F26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G26" t="s">
         <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I26" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B27" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D27" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E27" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F27" t="s">
         <v>44</v>
@@ -2252,10 +2240,10 @@
         <v>15</v>
       </c>
       <c r="H27" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="I27" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Régénération JSON avec recherche italien: 163 débats (+3)
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="672">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -904,6 +904,45 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">338578</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giacometti Anna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il 27 marzo 2024 il Consiglio federale ha adottato il messaggio concernente il consuntivo della Confederazione svizzera per il 2023 a mano del Parlamento. La Commissione delle finanze ha esaminato il consuntivo nelle sue quattro sottocommissioni e nelle riunioni plenarie.
+La Commissione delle finanze ha preso atto del rapporto del Controllo federale delle finanze che raccomanda di approvare i conti annuali della Confederazione e dei due fondi FIF e Fostra.
+La modifica della legge federale sulle </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il 27 marzo 2024 il Consiglio federale ha adottato il messaggio concernente il consuntivo della Confederazione svizzera per il 2023 a mano del Parlamento. La Commissione delle finanze ha esaminato il consuntivo nelle sue quattro sottocommissioni e nelle riunioni plenarie.
+La Commissione delle finanze ha preso atto del rapporto del Controllo federale delle finanze che raccomanda di approvare i conti annuali della Confederazione e dei due fondi FIF e Fostra.
+La modifica della legge federale sulle finanze della Confederazione (LFC) che semplifica e ottimizza la gestione delle finanze pubbliche, è entrata in vigore il 1° gennaio 2022 ed è stata applicata per la prima volta nel preventivo 2023. Il consuntivo 2023 è quindi la prima chiusura dei conti secondo la nuova legislazione. Le novità principali riguardano la soppressione del conto di finanziamento come conto autonomo, una gestione delle finanze pubbliche improntata al principio della conformità temporale - la costituzione e lo scioglimento di accantonamenti e delimitazioni sottostanno ora al freno all'indebitamento - e una nuova definizione del debito netto. La modifica della LFC ha richiesto un [PAGE 821] adeguamento una tantum del conto di compensazione e del conto di ammortamento.
+Per la seconda volta consecutiva e per la terza volta dal 2005, la Confederazione registra un deficit strutturale nel suo bilancio ordinario. Il consuntivo 2023 chiude con un deficit di finanziamento pari a 1,4 miliardi di franchi; questo significa che le entrate non sono bastate per finanziare le uscite e gli investimenti netti. 
+Circa la metà del deficit proviene dal bilancio ordinario e il resto da quello straordinario.
+Il freno all'indebitamento limita le uscite ordinarie al livello delle entrate ordinarie, tenendo conto della situazione economica. Per il 2023 il freno all'indebitamento avrebbe consentito alle uscite di superare le entrate di 238 milioni di franchi, pari allo 0,3 per cento delle entrate ordinarie. Il deficit ordinario di finanziamento per il 2023 ammonta però a 672 milioni di franchi. I rimanenti 434 milioni di deficit sono pertanto di natura strutturale e vengono addebitati al conto di compensazione. Il saldo al 31 dicembre 2023 è di 20,043 miliardi di franchi.
+Sul conto di ammortamento vengono addebitate le uscite e accreditate le entrate supplementari. A causa delle uscite legate alla pandemia di Covid-19, il conto di ammortamento presenta un saldo fortemente negativo. Il disavanzo del conto di ammortamento al 31 dicembre 2023 ammonta a 27,216 miliardi di franchi.
+L'economia svizzera è cresciuta dell'1,3 per cento in termini reali e del 2,3 per cento in termini nominali registrando, in entrambi i casi, un andamento meno dinamico di quello ipotizzato nel preventivo. Il calo degli investimenti e la crescita negativa a livello mondiale hanno neutralizzato gli impulsi positivi generati dai consumi privati. Per contro, l'indice nazionale dei prezzi al consumo è aumentato più del previsto, attestandosi al 2,1 per cento.
+Il debito netto è dato dal capitale di terzi al netto dei beni patrimoniali. Nel 2023 l'indebitamento netto è aumentato di 2,7 miliardi di franchi, attestandosi a 142 miliardi; questo è dovuto al deficit di finanziamento e a transazioni imputate direttamente al capitale proprio.
+Nel 2023 sono state contabilizzate entrate pari a 79,6 miliardi di franchi, il che corrisponde a una progressione del 5,2 per cento rispetto all'esercizio 2022. Le entrate della Confederazione sono aumentate sensibilmente, nonostante la mancata distribuzione degli utili della Banca nazionale svizzera. L'incremento è riconducibile principalmente alle maggiori entrate dall'imposta federale diretta e dall'imposta preventiva. Il reddito fiscale dell'imposta sul valore aggiunto è aumentato di 0,6 miliardi di franchi. Nell'ambito dell'imposta federale diretta è aumentato soprattutto il gettito dell'imposta sull'utile delle persone giuridiche, più 2,2 miliardi di franchi. Per[NB]quanto[NB]riguarda[NB]l'imposta preventiva, il forte aumento è riconducibile alla correzione di alcune stime riguardanti gli anni precedenti.
+Le entrate straordinarie ammontano a 310 milioni di franchi. La vendita di alcune unità operative di Ruag International Holding SA ha generato entrate straordinarie pari a 200 milioni di franchi. Altre entrate straordinarie derivano dai premi di rischio versati da Credit Suisse per i mutui a sostegno della liquidità, coperti da una garanzia della Confederazione.
+Le uscite complessive della Confederazione nel 2023 ammontano a 81 miliardi di franchi, rimanendo quindi stabili rispetto all'anno precedente. Già per il quarto anno consecutivo è stato necessario far valere un fabbisogno finanziario eccezionale. Rispetto agli esercizi precedenti, caratterizzati dalle uscite legate alla pandemia, esso è però sensibilmente inferiore.
+Le uscite ordinarie sono cresciute di 2,2 miliardi di franchi, dunque in maniera più marcata rispetto al PIL nominale pari al 2,3 per cento. Il contributo della Confederazione a favore della previdenza per la vecchiaia è aumentato di 459 milioni rispetto all'anno precedente, e quello destinato all'assicurazione per l'invalidità di 90 milioni di franchi. Sono aumentate anche le uscite per le riduzioni dei premi nell'assicurazione malattie e per le prestazioni complementari. Si osservano maggiori uscite per il settore della migrazione sebbene le uscite a favore delle persone provenienti dall'Ucraina siano state contabilizzate a titolo straordinario. 
+Le uscite legate alle finanze e alle imposte sono cresciute del 10 per cento, questo a causa dell'aumento dei tassi d'interesse e della partecipazione dei cantoni alle entrate dell'imposta federale diretta e dell'imposta preventiva. Infine, rispetto al 2022, la Confederazione ha speso 310 milioni di franchi in più per il Settore educazione e ricerca. Le uscite per le relazioni con l'estero e la cooperazione internazionale sono aumentate di 208 milioni di franchi, pari al 5,4 per cento.
+Per quanto concerne le uscite straordinarie, i contributi ai cantoni per le persone in cerca di protezione provenienti dall'Ucraina ammontano a 1,1 miliardi di franchi. Il piano di salvataggio per il Settore energia elettrica di 4 miliardi di franchi è rimasto inutilizzato e ha quindi potuto essere revocato.
+La vostra Commissione delle finanze propone, con 16 voti contro 8, di approvare il consuntivo 2023 e, all'unanimità, di approvare i conti speciali "Fondo per l'infrastruttura ferroviaria" e "Fondo per le strade nazionali e il traffico d'agglomerato". In tal modo segue la raccomandazione del Controllo federale delle finanze che, nel suo ruolo di revisore, si era espresso a favore dell'approvazione del conto annuale 2023 della Confederazione, dei sorpassi di credito per 2,25 miliardi di franchi e della costituzione di nuove riserve per 174 milioni di franchi.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">339510</t>
   </si>
   <si>
@@ -1010,9 +1049,6 @@
   </si>
   <si>
     <t xml:space="preserve">Wehrli Laurent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL</t>
   </si>
   <si>
     <t xml:space="preserve">Dans sa séance plénière de mai 2024, en présence du président et du secrétaire général du Tribunal fédéral, votre Commission de gestion a pris connaissance et étudié le rapport de gestion du Tribunal fédéral pour l'année 2023. Votre sous-commission de gestion, en charge notamment du suivi des tribunaux fédéraux et du Ministère public de la Confédération, l'avait précédemment fait lors de sa séance, qui a eu lieu à Lausanne le 8 mai 2024, en présence du président et de divers autres responsables.</t>
@@ -1105,9 +1141,6 @@
     <t xml:space="preserve">Engler Stefan</t>
   </si>
   <si>
-    <t xml:space="preserve">GR</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bei der Beratung dieses Geschäfts können wir uns kurzhalten. Ihre Staatspolitische Kommission hat die Motion Farinelli 23.3592, "Alle Berichte sollen zumindest eine Zusammenfassung in den drei Amtssprachen enthalten", vorgeprüft und ist zum Schluss gekommen, Ihnen die Annahme dieser Motion zu beantragen. Dasselbe hat der Nationalrat getan, und dasselbe will auch der Bundesrat tun, allerdings mit der Einschränkung, dass es sich um Berichte des Bundesrates und der Bundesverwaltung handeln müsse, d</t>
   </si>
   <si>
@@ -1118,6 +1151,27 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">341085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regazzi Fabio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visto che parliamo di un tema legato al multilinguismo permettetemi di rivolgermi a voi in italiano per qualche breve riflessione.
+Come ticinese so bene quanto sia importante sentirsi parte del tessuto nazionale svizzero a pieno titolo. Per questo sostengo con convinzione la mozione Farinelli, e ho sentito con piacere che anche la commissione competente la sostiene. L'autore della mozione chiede che tutti i rapporti presentati dall'amministrazione e dal Consiglio federale includano un breve rias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visto che parliamo di un tema legato al multilinguismo permettetemi di rivolgermi a voi in italiano per qualche breve riflessione.
+Come ticinese so bene quanto sia importante sentirsi parte del tessuto nazionale svizzero a pieno titolo. Per questo sostengo con convinzione la mozione Farinelli, e ho sentito con piacere che anche la commissione competente la sostiene. L'autore della mozione chiede che tutti i rapporti presentati dall'amministrazione e dal Consiglio federale includano un breve riassunto nelle tre lingue ufficiali della Svizzera. Questa proposta, che mi sembra ragionevole, è un buon compromesso. Non solo promuove la diversità linguistica del nostro paese, ma rafforza anche la trasparenza e l'accessibilità delle informazioni. Attualmente i riassunti dei rapporti, come l'ha ricordato il relatore, sono spesso disponibili solo in una o due lingue ufficiali, escludendo quindi una parte significativa della popolazione. Ricordo che quando si parla di Svizzera italiana non si deve pensare solo al canton Ticino o al Grigioni italiano, ma a quasi 700[NB]000 persone che in tutta la Svizzera parlano la lingua di Dante.
+Il modello adottato dal Controllo federale delle finanze, che include sempre una versione riassuntiva nelle lingue ufficiali, ha dimostrato l'efficacia di questa pratica. Estendere questo approccio a tutti i rapporti dell'amministrazione e del Consiglio federale standardizzerebbe e migliorerebbe ulteriormente la comunicazione istituzionale.
+In sintesi, sostenere questa mozione significa promuovere multilinguismo, trasparenza ed efficienza comunicativa. È un impegno concreto per una maggiore accessibilità delle informazioni governative e rappresenta una misura equa e rispettosa della diversità linguistica della Svizzera.
+Per questo motivo vi invito ad approvare la presente mozione.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">341480</t>
   </si>
   <si>
@@ -1140,9 +1194,6 @@
   </si>
   <si>
     <t xml:space="preserve">Chiesa Marco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TI</t>
   </si>
   <si>
     <t xml:space="preserve">Künftig darf der medizinisch-technische Fortschritt nicht nur Berücksichtigung finden, wenn es zu teuer wird. Wie auch sonst im Markt müssen die Effizienzgewinne der Kundschaft bzw. den Kostenträgern, den Prämienzahlern und der öffentlichen Hand, weitergegeben werden. Die Tarifpartner müssen diesbezüglich aktiv werden und Lösungen finden, auch wenn dies nicht allen Beteiligten passt. Der Bundesrat muss subsidiär, regelmässig und zeitnah eingreifen, wenn die Tarifpartner den präzisierten gesetzli</t>
@@ -1402,9 +1453,6 @@
   </si>
   <si>
     <t xml:space="preserve">20240924</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regazzi Fabio</t>
   </si>
   <si>
     <t xml:space="preserve">Ich danke dem Bundesrat für die Stellungnahme zu meiner Interpellation. Ich bin damit aber nicht zufrieden, daher möchte ich den Bundesrat um eine Klarstellung bitten. Es hat nämlich den Anschein, als ob der Kostenrahmen nur scheinbar eingehalten wird. Die Stellungnahme vermittelt den Eindruck, dass das Projekt inhaltlich und finanziell im Rahmen liegt, nur weil bisher nicht das gesamte Budget aufgewendet wurde. Der Verweis darauf, dass 71,8 Prozent der veranlagten Kosten verwendet wurden, sagt </t>
@@ -2859,6 +2907,29 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">356868</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farinelli Alex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A nome della Commissione delle finanze vi presento le considerazioni emerse durante l'esame del consuntivo 2024. Non ripeterò tutte le cifre già citate dalla collega. Vi posso dire che l'esame si è svolto in diverse sedute e ha incluso l'audizione del Consiglio federale, dei vari uffici federali rispettivamente del Controllo federale delle finanze e delle autorità della Confederazione. 
+Nel 2024, il consuntivo chiude con un disavanzo di finanziamento contenuto pari a 80 milioni di franchi. È il </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A nome della Commissione delle finanze vi presento le considerazioni emerse durante l'esame del consuntivo 2024. Non ripeterò tutte le cifre già citate dalla collega. Vi posso dire che l'esame si è svolto in diverse sedute e ha incluso l'audizione del Consiglio federale, dei vari uffici federali rispettivamente del Controllo federale delle finanze e delle autorità della Confederazione. 
+Nel 2024, il consuntivo chiude con un disavanzo di finanziamento contenuto pari a 80 milioni di franchi. È il miglior risultato dal 2019 con un'eccedenza strutturale di 1,3 miliardi di franchi nel bilancio ordinario. Le entrate hanno superato le previsioni soprattutto grazie ad un forte incremento del gettito dell'imposta federale diretta e dell'IVA - questo è dovuto sia a fattori straordinari che strutturali -, mentre le spese sono rimaste sotto controllo. 
+La commissione prende atto con soddisfazione che i principi della legge sul freno all'indebitamento sono stati rispettati. Tuttavia desidera richiamare l'attenzione su alcuni elementi critici messi in evidenza dal Controllo federale delle finanze nei suoi rapporti di revisione. 
+Primo: il fondo dell'infrastruttura ferroviaria mostra segnali di squilibrio a medio termine. Le uscite previste supereranno le entrate già nel 2027. In assenza di misure correttive, le riserve minime legali non potranno più essere rispettate entro il 2028. Anche se non è oggetto diretto dalla revisione, la commissione sostiene la raccomandazione del Controllo federale delle finanze di monitorare attentamente l'evoluzione per garantire la sostenibilità finanziaria del fondo. 
+Secondo: persistono incertezze nella contabilizzazione delle entrate, in particolare riguardante la tassa sul traffico pesante commisurata alle prestazioni e l'e-vignetta, dove la mancanza di giustificativi completi limita la tracciabilità. Il Controllo federale delle finanze ha riconosciuto gli sforzi dell'amministrazione per contenere i rischi, ma ritiene necessaria una soluzione strutturale entro la fine di quest'anno. 
+Terzo: continuano ad essere presenti poste di bilancio segnate da un'elevata incertezza delle stime, come le riserve per i test Covid, i crediti Covid alle imprese o i costi di bonifica del deposito di munizioni di Mitholz. In tutti questi casi le stime sono state confermate come plausibili, ma devono essere sempre oggetto di un riesame continuo. 
+La commissione riconosce inoltre l'importanza della gestione prudente delle spese straordinarie legate al conflitto in Ucraina. Tale spese, ammesse nel bilancio straordinario per il 2024, dovranno progressivamente rientrare nel bilancio ordinario. A partire dal 2027, dovranno essere completamente assorbite da quest'ultimo. Si condivide quindi l'osservazione del Controllo federale delle finanze, che la classificazione delle spese straordinarie deve rimanere eccezionale e rigorosa, per non compromettere la credibilità del freno all'indebitamento e la stabilità delle finanze federali.
+Nel complesso, la commissione ritiene che il conto di Stato della Confederazione 2024 presenti un'immagine conforme alla legge. Pertanto, sostiene la raccomandazione del Controllo federale delle finanze di approvare la contabilità dello Stato. Propone a questo consiglio, con 17 voti favorevoli, 0 contrari e 8 astensioni, di approvare il consuntivo 2024. 
+Per quanto riguarda invece i fondi infrastrutturali legati all'infrastruttura ferroviaria e a quella stradale, ossia il FIF e il Fostra, essi sono stati approvati all'unanimità dei 25 consiglieri presenti in sala.
+In conclusione, mi permetto di ringraziare anch'io il Consiglio federale e la presidente della Confederazione per l'ottima collaborazione e il lavoro svolto, l'amministrazione federale delle finanze per averci supportato, il segretariato commissionale che è sempre a disposizione e il Controllo federale delle finanze che ci supporta in tutto quello che riguarda il controllo dei conti della Confederazione. 
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">357753</t>
   </si>
   <si>
@@ -4286,8 +4357,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I161" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I161"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I164" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I164"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -5643,42 +5714,42 @@
         <v>177</v>
       </c>
       <c r="B38" t="s">
+        <v>167</v>
+      </c>
+      <c r="C38" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" t="s">
         <v>178</v>
       </c>
-      <c r="C38" t="s">
-        <v>19</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>179</v>
       </c>
-      <c r="E38" t="s">
-        <v>28</v>
-      </c>
       <c r="F38" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="G38" t="s">
-        <v>22</v>
+        <v>181</v>
       </c>
       <c r="H38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B39" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C39" t="s">
         <v>19</v>
       </c>
       <c r="D39" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E39" t="s">
         <v>28</v>
@@ -5690,147 +5761,147 @@
         <v>22</v>
       </c>
       <c r="H39" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="I39" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B40" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D40" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E40" t="s">
         <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>188</v>
+        <v>117</v>
       </c>
       <c r="G40" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H40" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I40" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B41" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C41" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D41" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41"/>
+        <v>194</v>
+      </c>
+      <c r="E41" t="s">
+        <v>28</v>
+      </c>
       <c r="F41" t="s">
-        <v>21</v>
+        <v>195</v>
       </c>
       <c r="G41" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H41" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="I41" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B42" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C42" t="s">
         <v>19</v>
       </c>
       <c r="D42" t="s">
-        <v>122</v>
-      </c>
-      <c r="E42" t="s">
-        <v>37</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E42"/>
       <c r="F42" t="s">
-        <v>98</v>
+        <v>21</v>
       </c>
       <c r="G42" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H42" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="I42" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B43" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C43" t="s">
         <v>19</v>
       </c>
       <c r="D43" t="s">
-        <v>200</v>
+        <v>122</v>
       </c>
       <c r="E43" t="s">
-        <v>201</v>
+        <v>37</v>
       </c>
       <c r="F43" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="G43" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H43" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="I43" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B44" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D44" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E44" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="F44" t="s">
-        <v>207</v>
+        <v>117</v>
       </c>
       <c r="G44" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H44" t="s">
         <v>208</v>
@@ -5853,39 +5924,39 @@
         <v>212</v>
       </c>
       <c r="E45" t="s">
-        <v>78</v>
+        <v>179</v>
       </c>
       <c r="F45" t="s">
-        <v>73</v>
+        <v>213</v>
       </c>
       <c r="G45" t="s">
         <v>14</v>
       </c>
       <c r="H45" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I45" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B46" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C46" t="s">
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E46" t="s">
         <v>78</v>
       </c>
       <c r="F46" t="s">
-        <v>218</v>
+        <v>73</v>
       </c>
       <c r="G46" t="s">
         <v>14</v>
@@ -5905,33 +5976,33 @@
         <v>222</v>
       </c>
       <c r="C47" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D47" t="s">
-        <v>60</v>
+        <v>223</v>
       </c>
       <c r="E47" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F47" t="s">
-        <v>48</v>
+        <v>180</v>
       </c>
       <c r="G47" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H47" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I47" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B48" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C48" t="s">
         <v>11</v>
@@ -5940,13 +6011,13 @@
         <v>227</v>
       </c>
       <c r="E48" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F48" t="s">
         <v>228</v>
       </c>
       <c r="G48" t="s">
-        <v>14</v>
+        <v>181</v>
       </c>
       <c r="H48" t="s">
         <v>229</v>
@@ -5960,36 +6031,36 @@
         <v>231</v>
       </c>
       <c r="B49" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D49" t="s">
-        <v>232</v>
+        <v>60</v>
       </c>
       <c r="E49" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F49" t="s">
+        <v>48</v>
+      </c>
+      <c r="G49" t="s">
+        <v>22</v>
+      </c>
+      <c r="H49" t="s">
         <v>233</v>
       </c>
-      <c r="G49" t="s">
-        <v>14</v>
-      </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>234</v>
-      </c>
-      <c r="I49" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>235</v>
+      </c>
+      <c r="B50" t="s">
         <v>236</v>
-      </c>
-      <c r="B50" t="s">
-        <v>226</v>
       </c>
       <c r="C50" t="s">
         <v>11</v>
@@ -5998,13 +6069,13 @@
         <v>237</v>
       </c>
       <c r="E50" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>117</v>
+        <v>228</v>
       </c>
       <c r="G50" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H50" t="s">
         <v>238</v>
@@ -6018,19 +6089,19 @@
         <v>240</v>
       </c>
       <c r="B51" t="s">
+        <v>236</v>
+      </c>
+      <c r="C51" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" t="s">
         <v>241</v>
       </c>
-      <c r="C51" t="s">
-        <v>19</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
+        <v>78</v>
+      </c>
+      <c r="F51" t="s">
         <v>242</v>
-      </c>
-      <c r="E51" t="s">
-        <v>201</v>
-      </c>
-      <c r="F51" t="s">
-        <v>43</v>
       </c>
       <c r="G51" t="s">
         <v>14</v>
@@ -6047,46 +6118,48 @@
         <v>245</v>
       </c>
       <c r="B52" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="C52" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D52" t="s">
-        <v>20</v>
-      </c>
-      <c r="E52"/>
+        <v>246</v>
+      </c>
+      <c r="E52" t="s">
+        <v>11</v>
+      </c>
       <c r="F52" t="s">
-        <v>21</v>
+        <v>117</v>
       </c>
       <c r="G52" t="s">
         <v>22</v>
       </c>
       <c r="H52" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I52" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B53" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C53" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D53" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E53" t="s">
-        <v>28</v>
+        <v>179</v>
       </c>
       <c r="F53" t="s">
-        <v>251</v>
+        <v>43</v>
       </c>
       <c r="G53" t="s">
         <v>14</v>
@@ -6103,10 +6176,10 @@
         <v>254</v>
       </c>
       <c r="B54" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C54" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D54" t="s">
         <v>20</v>
@@ -6139,24 +6212,24 @@
         <v>259</v>
       </c>
       <c r="E55" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F55" t="s">
-        <v>79</v>
+        <v>260</v>
       </c>
       <c r="G55" t="s">
         <v>14</v>
       </c>
       <c r="H55" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I55" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B56" t="s">
         <v>258</v>
@@ -6165,36 +6238,34 @@
         <v>11</v>
       </c>
       <c r="D56" t="s">
-        <v>259</v>
-      </c>
-      <c r="E56" t="s">
-        <v>11</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E56"/>
       <c r="F56" t="s">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="G56" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H56" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I56" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B57" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C57" t="s">
         <v>11</v>
       </c>
       <c r="D57" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="E57" t="s">
         <v>11</v>
@@ -6206,99 +6277,103 @@
         <v>14</v>
       </c>
       <c r="H57" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="I57" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B58" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C58" t="s">
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>154</v>
-      </c>
-      <c r="E58"/>
+        <v>268</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
       <c r="F58" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="G58" t="s">
         <v>14</v>
       </c>
       <c r="H58" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="I58" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B59" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C59" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D59" t="s">
-        <v>20</v>
-      </c>
-      <c r="E59"/>
+        <v>268</v>
+      </c>
+      <c r="E59" t="s">
+        <v>11</v>
+      </c>
       <c r="F59" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="G59" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H59" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I59" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B60" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C60" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D60" t="s">
-        <v>20</v>
+        <v>154</v>
       </c>
       <c r="E60"/>
       <c r="F60" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G60" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H60" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I60" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B61" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C61" t="s">
         <v>19</v>
@@ -6311,36 +6386,34 @@
         <v>21</v>
       </c>
       <c r="G61" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H61" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="I61" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B62" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D62" t="s">
-        <v>284</v>
-      </c>
-      <c r="E62" t="s">
-        <v>78</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E62"/>
       <c r="F62" t="s">
-        <v>228</v>
+        <v>21</v>
       </c>
       <c r="G62" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H62" t="s">
         <v>285</v>
@@ -6354,77 +6427,75 @@
         <v>287</v>
       </c>
       <c r="B63" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C63" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D63" t="s">
-        <v>217</v>
-      </c>
-      <c r="E63" t="s">
-        <v>78</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E63"/>
       <c r="F63" t="s">
-        <v>218</v>
+        <v>21</v>
       </c>
       <c r="G63" t="s">
         <v>14</v>
       </c>
       <c r="H63" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I63" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B64" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C64" t="s">
         <v>11</v>
       </c>
       <c r="D64" t="s">
-        <v>291</v>
+        <v>227</v>
       </c>
       <c r="E64" t="s">
         <v>78</v>
       </c>
       <c r="F64" t="s">
-        <v>163</v>
+        <v>228</v>
       </c>
       <c r="G64" t="s">
         <v>14</v>
       </c>
       <c r="H64" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="I64" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B65" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C65" t="s">
         <v>11</v>
       </c>
       <c r="D65" t="s">
-        <v>295</v>
+        <v>223</v>
       </c>
       <c r="E65" t="s">
         <v>78</v>
       </c>
       <c r="F65" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="G65" t="s">
         <v>14</v>
@@ -6441,7 +6512,7 @@
         <v>298</v>
       </c>
       <c r="B66" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C66" t="s">
         <v>11</v>
@@ -6450,10 +6521,10 @@
         <v>299</v>
       </c>
       <c r="E66" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F66" t="s">
-        <v>73</v>
+        <v>163</v>
       </c>
       <c r="G66" t="s">
         <v>14</v>
@@ -6470,7 +6541,7 @@
         <v>302</v>
       </c>
       <c r="B67" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C67" t="s">
         <v>11</v>
@@ -6482,7 +6553,7 @@
         <v>78</v>
       </c>
       <c r="F67" t="s">
-        <v>98</v>
+        <v>195</v>
       </c>
       <c r="G67" t="s">
         <v>14</v>
@@ -6499,7 +6570,7 @@
         <v>306</v>
       </c>
       <c r="B68" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C68" t="s">
         <v>11</v>
@@ -6508,39 +6579,39 @@
         <v>307</v>
       </c>
       <c r="E68" t="s">
-        <v>28</v>
+        <v>179</v>
       </c>
       <c r="F68" t="s">
+        <v>73</v>
+      </c>
+      <c r="G68" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" t="s">
         <v>308</v>
       </c>
-      <c r="G68" t="s">
-        <v>14</v>
-      </c>
-      <c r="H68" t="s">
+      <c r="I68" t="s">
         <v>309</v>
-      </c>
-      <c r="I68" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B69" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C69" t="s">
         <v>11</v>
       </c>
       <c r="D69" t="s">
-        <v>217</v>
+        <v>311</v>
       </c>
       <c r="E69" t="s">
         <v>78</v>
       </c>
       <c r="F69" t="s">
-        <v>218</v>
+        <v>98</v>
       </c>
       <c r="G69" t="s">
         <v>14</v>
@@ -6557,48 +6628,48 @@
         <v>314</v>
       </c>
       <c r="B70" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C70" t="s">
         <v>11</v>
       </c>
       <c r="D70" t="s">
-        <v>284</v>
+        <v>315</v>
       </c>
       <c r="E70" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F70" t="s">
-        <v>228</v>
+        <v>316</v>
       </c>
       <c r="G70" t="s">
         <v>14</v>
       </c>
       <c r="H70" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I70" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B71" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
       <c r="C71" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D71" t="s">
-        <v>319</v>
+        <v>223</v>
       </c>
       <c r="E71" t="s">
         <v>78</v>
       </c>
       <c r="F71" t="s">
-        <v>73</v>
+        <v>180</v>
       </c>
       <c r="G71" t="s">
         <v>14</v>
@@ -6615,36 +6686,36 @@
         <v>322</v>
       </c>
       <c r="B72" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
       <c r="C72" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D72" t="s">
+        <v>227</v>
+      </c>
+      <c r="E72" t="s">
+        <v>78</v>
+      </c>
+      <c r="F72" t="s">
+        <v>228</v>
+      </c>
+      <c r="G72" t="s">
+        <v>14</v>
+      </c>
+      <c r="H72" t="s">
         <v>323</v>
       </c>
-      <c r="E72" t="s">
-        <v>28</v>
-      </c>
-      <c r="F72" t="s">
-        <v>218</v>
-      </c>
-      <c r="G72" t="s">
-        <v>14</v>
-      </c>
-      <c r="H72" t="s">
+      <c r="I72" t="s">
         <v>324</v>
-      </c>
-      <c r="I72" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
+        <v>325</v>
+      </c>
+      <c r="B73" t="s">
         <v>326</v>
-      </c>
-      <c r="B73" t="s">
-        <v>318</v>
       </c>
       <c r="C73" t="s">
         <v>19</v>
@@ -6653,10 +6724,10 @@
         <v>327</v>
       </c>
       <c r="E73" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F73" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="G73" t="s">
         <v>14</v>
@@ -6673,7 +6744,7 @@
         <v>330</v>
       </c>
       <c r="B74" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C74" t="s">
         <v>19</v>
@@ -6682,10 +6753,10 @@
         <v>331</v>
       </c>
       <c r="E74" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F74" t="s">
-        <v>73</v>
+        <v>180</v>
       </c>
       <c r="G74" t="s">
         <v>14</v>
@@ -6702,7 +6773,7 @@
         <v>334</v>
       </c>
       <c r="B75" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C75" t="s">
         <v>19</v>
@@ -6711,154 +6782,156 @@
         <v>335</v>
       </c>
       <c r="E75" t="s">
-        <v>78</v>
+        <v>179</v>
       </c>
       <c r="F75" t="s">
+        <v>43</v>
+      </c>
+      <c r="G75" t="s">
+        <v>14</v>
+      </c>
+      <c r="H75" t="s">
         <v>336</v>
       </c>
-      <c r="G75" t="s">
-        <v>14</v>
-      </c>
-      <c r="H75" t="s">
+      <c r="I75" t="s">
         <v>337</v>
-      </c>
-      <c r="I75" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
+        <v>338</v>
+      </c>
+      <c r="B76" t="s">
+        <v>326</v>
+      </c>
+      <c r="C76" t="s">
+        <v>19</v>
+      </c>
+      <c r="D76" t="s">
         <v>339</v>
       </c>
-      <c r="B76" t="s">
-        <v>318</v>
-      </c>
-      <c r="C76" t="s">
-        <v>19</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" t="s">
+        <v>73</v>
+      </c>
+      <c r="G76" t="s">
+        <v>14</v>
+      </c>
+      <c r="H76" t="s">
         <v>340</v>
       </c>
-      <c r="E76" t="s">
+      <c r="I76" t="s">
         <v>341</v>
-      </c>
-      <c r="F76" t="s">
-        <v>13</v>
-      </c>
-      <c r="G76" t="s">
-        <v>14</v>
-      </c>
-      <c r="H76" t="s">
-        <v>342</v>
-      </c>
-      <c r="I76" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
+        <v>342</v>
+      </c>
+      <c r="B77" t="s">
+        <v>326</v>
+      </c>
+      <c r="C77" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77" t="s">
+        <v>343</v>
+      </c>
+      <c r="E77" t="s">
+        <v>78</v>
+      </c>
+      <c r="F77" t="s">
         <v>344</v>
       </c>
-      <c r="B77" t="s">
-        <v>318</v>
-      </c>
-      <c r="C77" t="s">
-        <v>19</v>
-      </c>
-      <c r="D77" t="s">
+      <c r="G77" t="s">
+        <v>14</v>
+      </c>
+      <c r="H77" t="s">
         <v>345</v>
       </c>
-      <c r="E77"/>
-      <c r="F77" t="s">
-        <v>29</v>
-      </c>
-      <c r="G77" t="s">
-        <v>14</v>
-      </c>
-      <c r="H77" t="s">
+      <c r="I77" t="s">
         <v>346</v>
-      </c>
-      <c r="I77" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
+        <v>347</v>
+      </c>
+      <c r="B78" t="s">
+        <v>326</v>
+      </c>
+      <c r="C78" t="s">
+        <v>19</v>
+      </c>
+      <c r="D78" t="s">
         <v>348</v>
       </c>
-      <c r="B78" t="s">
-        <v>318</v>
-      </c>
-      <c r="C78" t="s">
-        <v>19</v>
-      </c>
-      <c r="D78" t="s">
-        <v>55</v>
-      </c>
       <c r="E78" t="s">
-        <v>37</v>
+        <v>349</v>
       </c>
       <c r="F78" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="G78" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H78" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I78" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B79" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C79" t="s">
         <v>19</v>
       </c>
       <c r="D79" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E79"/>
       <c r="F79" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="G79" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H79" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="I79" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B80" t="s">
-        <v>356</v>
+        <v>326</v>
       </c>
       <c r="C80" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D80" t="s">
-        <v>303</v>
+        <v>55</v>
       </c>
       <c r="E80" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="F80" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="G80" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H80" t="s">
         <v>357</v>
@@ -6872,48 +6945,46 @@
         <v>359</v>
       </c>
       <c r="B81" t="s">
+        <v>326</v>
+      </c>
+      <c r="C81" t="s">
+        <v>19</v>
+      </c>
+      <c r="D81" t="s">
         <v>360</v>
       </c>
-      <c r="C81" t="s">
-        <v>19</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="E81"/>
+      <c r="F81" t="s">
+        <v>117</v>
+      </c>
+      <c r="G81" t="s">
+        <v>22</v>
+      </c>
+      <c r="H81" t="s">
         <v>361</v>
       </c>
-      <c r="E81" t="s">
-        <v>201</v>
-      </c>
-      <c r="F81" t="s">
-        <v>73</v>
-      </c>
-      <c r="G81" t="s">
-        <v>14</v>
-      </c>
-      <c r="H81" t="s">
+      <c r="I81" t="s">
         <v>362</v>
-      </c>
-      <c r="I81" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
+        <v>363</v>
+      </c>
+      <c r="B82" t="s">
         <v>364</v>
       </c>
-      <c r="B82" t="s">
-        <v>360</v>
-      </c>
       <c r="C82" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D82" t="s">
-        <v>36</v>
+        <v>311</v>
       </c>
       <c r="E82" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="F82" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="G82" t="s">
         <v>14</v>
@@ -6939,10 +7010,10 @@
         <v>369</v>
       </c>
       <c r="E83" t="s">
-        <v>28</v>
+        <v>179</v>
       </c>
       <c r="F83" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="G83" t="s">
         <v>14</v>
@@ -6962,16 +7033,16 @@
         <v>368</v>
       </c>
       <c r="C84" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D84" t="s">
-        <v>217</v>
+        <v>36</v>
       </c>
       <c r="E84" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="F84" t="s">
-        <v>218</v>
+        <v>22</v>
       </c>
       <c r="G84" t="s">
         <v>14</v>
@@ -6988,48 +7059,48 @@
         <v>375</v>
       </c>
       <c r="B85" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C85" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D85" t="s">
-        <v>187</v>
+        <v>377</v>
       </c>
       <c r="E85" t="s">
         <v>28</v>
       </c>
       <c r="F85" t="s">
-        <v>188</v>
+        <v>98</v>
       </c>
       <c r="G85" t="s">
         <v>14</v>
       </c>
       <c r="H85" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="I85" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B86" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C86" t="s">
         <v>11</v>
       </c>
       <c r="D86" t="s">
-        <v>379</v>
+        <v>223</v>
       </c>
       <c r="E86" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F86" t="s">
-        <v>380</v>
+        <v>180</v>
       </c>
       <c r="G86" t="s">
         <v>14</v>
@@ -7046,46 +7117,48 @@
         <v>383</v>
       </c>
       <c r="B87" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="C87" t="s">
         <v>11</v>
       </c>
       <c r="D87" t="s">
-        <v>103</v>
-      </c>
-      <c r="E87"/>
+        <v>194</v>
+      </c>
+      <c r="E87" t="s">
+        <v>28</v>
+      </c>
       <c r="F87" t="s">
-        <v>104</v>
+        <v>195</v>
       </c>
       <c r="G87" t="s">
         <v>14</v>
       </c>
       <c r="H87" t="s">
+        <v>384</v>
+      </c>
+      <c r="I87" t="s">
         <v>385</v>
-      </c>
-      <c r="I87" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B88" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="C88" t="s">
         <v>11</v>
       </c>
       <c r="D88" t="s">
+        <v>387</v>
+      </c>
+      <c r="E88" t="s">
+        <v>179</v>
+      </c>
+      <c r="F88" t="s">
         <v>388</v>
-      </c>
-      <c r="E88" t="s">
-        <v>201</v>
-      </c>
-      <c r="F88" t="s">
-        <v>341</v>
       </c>
       <c r="G88" t="s">
         <v>14</v>
@@ -7102,133 +7175,133 @@
         <v>391</v>
       </c>
       <c r="B89" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C89" t="s">
         <v>11</v>
       </c>
       <c r="D89" t="s">
-        <v>187</v>
-      </c>
-      <c r="E89" t="s">
-        <v>28</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E89"/>
       <c r="F89" t="s">
-        <v>188</v>
+        <v>104</v>
       </c>
       <c r="G89" t="s">
         <v>14</v>
       </c>
       <c r="H89" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I89" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B90" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C90" t="s">
         <v>11</v>
       </c>
       <c r="D90" t="s">
-        <v>303</v>
+        <v>396</v>
       </c>
       <c r="E90" t="s">
-        <v>78</v>
+        <v>179</v>
       </c>
       <c r="F90" t="s">
-        <v>98</v>
+        <v>349</v>
       </c>
       <c r="G90" t="s">
         <v>14</v>
       </c>
       <c r="H90" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="I90" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B91" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C91" t="s">
         <v>11</v>
       </c>
       <c r="D91" t="s">
-        <v>126</v>
+        <v>194</v>
       </c>
       <c r="E91" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F91" t="s">
-        <v>21</v>
+        <v>195</v>
       </c>
       <c r="G91" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H91" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I91" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B92" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C92" t="s">
         <v>11</v>
       </c>
       <c r="D92" t="s">
-        <v>401</v>
+        <v>311</v>
       </c>
       <c r="E92" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F92" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="G92" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H92" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="I92" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B93" t="s">
-        <v>405</v>
+        <v>392</v>
       </c>
       <c r="C93" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D93" t="s">
-        <v>345</v>
-      </c>
-      <c r="E93"/>
+        <v>126</v>
+      </c>
+      <c r="E93" t="s">
+        <v>78</v>
+      </c>
       <c r="F93" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G93" t="s">
         <v>22</v>
@@ -7245,16 +7318,16 @@
         <v>408</v>
       </c>
       <c r="B94" t="s">
-        <v>405</v>
+        <v>392</v>
       </c>
       <c r="C94" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D94" t="s">
+        <v>409</v>
+      </c>
+      <c r="E94" t="s">
         <v>179</v>
-      </c>
-      <c r="E94" t="s">
-        <v>28</v>
       </c>
       <c r="F94" t="s">
         <v>117</v>
@@ -7263,60 +7336,60 @@
         <v>22</v>
       </c>
       <c r="H94" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I94" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B95" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C95" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D95" t="s">
-        <v>103</v>
+        <v>353</v>
       </c>
       <c r="E95"/>
       <c r="F95" t="s">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="G95" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H95" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="I95" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B96" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C96" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D96" t="s">
-        <v>134</v>
+        <v>186</v>
       </c>
       <c r="E96" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F96" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="G96" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H96" t="s">
         <v>417</v>
@@ -7336,16 +7409,14 @@
         <v>11</v>
       </c>
       <c r="D97" t="s">
-        <v>126</v>
-      </c>
-      <c r="E97" t="s">
-        <v>78</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E97"/>
       <c r="F97" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="G97" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H97" t="s">
         <v>421</v>
@@ -7362,14 +7433,16 @@
         <v>424</v>
       </c>
       <c r="C98" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D98" t="s">
-        <v>84</v>
-      </c>
-      <c r="E98"/>
+        <v>134</v>
+      </c>
+      <c r="E98" t="s">
+        <v>78</v>
+      </c>
       <c r="F98" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="G98" t="s">
         <v>14</v>
@@ -7386,48 +7459,46 @@
         <v>427</v>
       </c>
       <c r="B99" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="C99" t="s">
         <v>11</v>
       </c>
       <c r="D99" t="s">
-        <v>401</v>
+        <v>126</v>
       </c>
       <c r="E99" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F99" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="G99" t="s">
         <v>22</v>
       </c>
       <c r="H99" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I99" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B100" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C100" t="s">
         <v>19</v>
       </c>
       <c r="D100" t="s">
-        <v>432</v>
-      </c>
-      <c r="E100" t="s">
-        <v>341</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E100"/>
       <c r="F100" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="G100" t="s">
         <v>14</v>
@@ -7444,49 +7515,51 @@
         <v>435</v>
       </c>
       <c r="B101" t="s">
+        <v>432</v>
+      </c>
+      <c r="C101" t="s">
+        <v>11</v>
+      </c>
+      <c r="D101" t="s">
+        <v>409</v>
+      </c>
+      <c r="E101" t="s">
+        <v>179</v>
+      </c>
+      <c r="F101" t="s">
+        <v>117</v>
+      </c>
+      <c r="G101" t="s">
+        <v>22</v>
+      </c>
+      <c r="H101" t="s">
         <v>436</v>
       </c>
-      <c r="C101" t="s">
-        <v>19</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="I101" t="s">
         <v>437</v>
-      </c>
-      <c r="E101" t="s">
-        <v>341</v>
-      </c>
-      <c r="F101" t="s">
-        <v>29</v>
-      </c>
-      <c r="G101" t="s">
-        <v>14</v>
-      </c>
-      <c r="H101" t="s">
-        <v>438</v>
-      </c>
-      <c r="I101" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
+        <v>438</v>
+      </c>
+      <c r="B102" t="s">
+        <v>439</v>
+      </c>
+      <c r="C102" t="s">
+        <v>19</v>
+      </c>
+      <c r="D102" t="s">
         <v>440</v>
       </c>
-      <c r="B102" t="s">
-        <v>436</v>
-      </c>
-      <c r="C102" t="s">
-        <v>19</v>
-      </c>
-      <c r="D102" t="s">
-        <v>20</v>
-      </c>
-      <c r="E102"/>
+      <c r="E102" t="s">
+        <v>349</v>
+      </c>
       <c r="F102" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="G102" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H102" t="s">
         <v>441</v>
@@ -7500,76 +7573,76 @@
         <v>443</v>
       </c>
       <c r="B103" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C103" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D103" t="s">
-        <v>84</v>
-      </c>
-      <c r="E103"/>
+        <v>445</v>
+      </c>
+      <c r="E103" t="s">
+        <v>349</v>
+      </c>
       <c r="F103" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="G103" t="s">
         <v>14</v>
       </c>
       <c r="H103" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="I103" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B104" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C104" t="s">
         <v>19</v>
       </c>
       <c r="D104" t="s">
-        <v>345</v>
+        <v>20</v>
       </c>
       <c r="E104"/>
       <c r="F104" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G104" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H104" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I104" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B105" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="C105" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D105" t="s">
-        <v>55</v>
-      </c>
-      <c r="E105" t="s">
-        <v>37</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E105"/>
       <c r="F105" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="G105" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H105" t="s">
         <v>452</v>
@@ -7583,75 +7656,75 @@
         <v>454</v>
       </c>
       <c r="B106" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="C106" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D106" t="s">
-        <v>295</v>
-      </c>
-      <c r="E106" t="s">
-        <v>78</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="E106"/>
       <c r="F106" t="s">
-        <v>188</v>
+        <v>29</v>
       </c>
       <c r="G106" t="s">
         <v>14</v>
       </c>
       <c r="H106" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I106" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B107" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C107" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D107" t="s">
-        <v>20</v>
-      </c>
-      <c r="E107"/>
+        <v>55</v>
+      </c>
+      <c r="E107" t="s">
+        <v>37</v>
+      </c>
       <c r="F107" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="G107" t="s">
         <v>22</v>
       </c>
       <c r="H107" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="I107" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B108" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C108" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D108" t="s">
-        <v>462</v>
+        <v>303</v>
       </c>
       <c r="E108" t="s">
-        <v>341</v>
+        <v>78</v>
       </c>
       <c r="F108" t="s">
-        <v>43</v>
+        <v>195</v>
       </c>
       <c r="G108" t="s">
         <v>14</v>
@@ -7668,225 +7741,223 @@
         <v>465</v>
       </c>
       <c r="B109" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="C109" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D109" t="s">
-        <v>467</v>
-      </c>
-      <c r="E109" t="s">
-        <v>201</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E109"/>
       <c r="F109" t="s">
-        <v>468</v>
+        <v>21</v>
       </c>
       <c r="G109" t="s">
         <v>22</v>
       </c>
       <c r="H109" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="I109" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
+        <v>468</v>
+      </c>
+      <c r="B110" t="s">
+        <v>469</v>
+      </c>
+      <c r="C110" t="s">
+        <v>19</v>
+      </c>
+      <c r="D110" t="s">
+        <v>470</v>
+      </c>
+      <c r="E110" t="s">
+        <v>349</v>
+      </c>
+      <c r="F110" t="s">
+        <v>43</v>
+      </c>
+      <c r="G110" t="s">
+        <v>14</v>
+      </c>
+      <c r="H110" t="s">
         <v>471</v>
       </c>
-      <c r="B110" t="s">
+      <c r="I110" t="s">
         <v>472</v>
-      </c>
-      <c r="C110" t="s">
-        <v>11</v>
-      </c>
-      <c r="D110" t="s">
-        <v>187</v>
-      </c>
-      <c r="E110" t="s">
-        <v>28</v>
-      </c>
-      <c r="F110" t="s">
-        <v>188</v>
-      </c>
-      <c r="G110" t="s">
-        <v>14</v>
-      </c>
-      <c r="H110" t="s">
-        <v>473</v>
-      </c>
-      <c r="I110" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
+        <v>473</v>
+      </c>
+      <c r="B111" t="s">
+        <v>474</v>
+      </c>
+      <c r="C111" t="s">
+        <v>19</v>
+      </c>
+      <c r="D111" t="s">
         <v>475</v>
       </c>
-      <c r="B111" t="s">
+      <c r="E111" t="s">
+        <v>179</v>
+      </c>
+      <c r="F111" t="s">
         <v>476</v>
       </c>
-      <c r="C111" t="s">
-        <v>19</v>
-      </c>
-      <c r="D111" t="s">
+      <c r="G111" t="s">
+        <v>22</v>
+      </c>
+      <c r="H111" t="s">
         <v>477</v>
       </c>
-      <c r="E111" t="s">
-        <v>11</v>
-      </c>
-      <c r="F111" t="s">
-        <v>29</v>
-      </c>
-      <c r="G111" t="s">
-        <v>14</v>
-      </c>
-      <c r="H111" t="s">
+      <c r="I111" t="s">
         <v>478</v>
-      </c>
-      <c r="I111" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
+        <v>479</v>
+      </c>
+      <c r="B112" t="s">
         <v>480</v>
       </c>
-      <c r="B112" t="s">
-        <v>476</v>
-      </c>
       <c r="C112" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D112" t="s">
+        <v>194</v>
+      </c>
+      <c r="E112" t="s">
+        <v>28</v>
+      </c>
+      <c r="F112" t="s">
+        <v>195</v>
+      </c>
+      <c r="G112" t="s">
+        <v>14</v>
+      </c>
+      <c r="H112" t="s">
         <v>481</v>
       </c>
-      <c r="E112" t="s">
-        <v>201</v>
-      </c>
-      <c r="F112" t="s">
-        <v>163</v>
-      </c>
-      <c r="G112" t="s">
-        <v>14</v>
-      </c>
-      <c r="H112" t="s">
+      <c r="I112" t="s">
         <v>482</v>
-      </c>
-      <c r="I112" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
+        <v>483</v>
+      </c>
+      <c r="B113" t="s">
         <v>484</v>
       </c>
-      <c r="B113" t="s">
-        <v>476</v>
-      </c>
       <c r="C113" t="s">
         <v>19</v>
       </c>
       <c r="D113" t="s">
-        <v>168</v>
+        <v>485</v>
       </c>
       <c r="E113" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="F113" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="G113" t="s">
         <v>14</v>
       </c>
       <c r="H113" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I113" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B114" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="C114" t="s">
         <v>19</v>
       </c>
       <c r="D114" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="E114" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="F114" t="s">
-        <v>29</v>
+        <v>163</v>
       </c>
       <c r="G114" t="s">
         <v>14</v>
       </c>
       <c r="H114" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="I114" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B115" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="C115" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D115" t="s">
-        <v>206</v>
+        <v>168</v>
       </c>
       <c r="E115" t="s">
-        <v>201</v>
+        <v>37</v>
       </c>
       <c r="F115" t="s">
-        <v>207</v>
+        <v>79</v>
       </c>
       <c r="G115" t="s">
         <v>14</v>
       </c>
       <c r="H115" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="I115" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B116" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="C116" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D116" t="s">
-        <v>495</v>
+        <v>485</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
       </c>
       <c r="F116" t="s">
-        <v>468</v>
+        <v>29</v>
       </c>
       <c r="G116" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H116" t="s">
         <v>496</v>
@@ -7900,20 +7971,22 @@
         <v>498</v>
       </c>
       <c r="B117" t="s">
+        <v>484</v>
+      </c>
+      <c r="C117" t="s">
+        <v>19</v>
+      </c>
+      <c r="D117" t="s">
         <v>499</v>
       </c>
-      <c r="C117" t="s">
-        <v>19</v>
-      </c>
-      <c r="D117" t="s">
-        <v>154</v>
-      </c>
-      <c r="E117"/>
+      <c r="E117" t="s">
+        <v>179</v>
+      </c>
       <c r="F117" t="s">
-        <v>29</v>
+        <v>228</v>
       </c>
       <c r="G117" t="s">
-        <v>14</v>
+        <v>181</v>
       </c>
       <c r="H117" t="s">
         <v>500</v>
@@ -7927,104 +8000,102 @@
         <v>502</v>
       </c>
       <c r="B118" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C118" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D118" t="s">
-        <v>154</v>
-      </c>
-      <c r="E118"/>
+        <v>212</v>
+      </c>
+      <c r="E118" t="s">
+        <v>179</v>
+      </c>
       <c r="F118" t="s">
-        <v>29</v>
+        <v>213</v>
       </c>
       <c r="G118" t="s">
         <v>14</v>
       </c>
       <c r="H118" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I118" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B119" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C119" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D119" t="s">
-        <v>200</v>
+        <v>507</v>
       </c>
       <c r="E119" t="s">
-        <v>201</v>
+        <v>11</v>
       </c>
       <c r="F119" t="s">
-        <v>117</v>
+        <v>476</v>
       </c>
       <c r="G119" t="s">
         <v>22</v>
       </c>
       <c r="H119" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="I119" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B120" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C120" t="s">
         <v>19</v>
       </c>
       <c r="D120" t="s">
-        <v>510</v>
-      </c>
-      <c r="E120" t="s">
-        <v>37</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="E120"/>
       <c r="F120" t="s">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="G120" t="s">
         <v>14</v>
       </c>
       <c r="H120" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="I120" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B121" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C121" t="s">
         <v>19</v>
       </c>
       <c r="D121" t="s">
-        <v>514</v>
-      </c>
-      <c r="E121" t="s">
-        <v>28</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="E121"/>
       <c r="F121" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="G121" t="s">
         <v>14</v>
@@ -8041,36 +8112,36 @@
         <v>517</v>
       </c>
       <c r="B122" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C122" t="s">
         <v>19</v>
       </c>
       <c r="D122" t="s">
+        <v>207</v>
+      </c>
+      <c r="E122" t="s">
+        <v>179</v>
+      </c>
+      <c r="F122" t="s">
+        <v>117</v>
+      </c>
+      <c r="G122" t="s">
+        <v>22</v>
+      </c>
+      <c r="H122" t="s">
         <v>518</v>
       </c>
-      <c r="E122" t="s">
-        <v>11</v>
-      </c>
-      <c r="F122" t="s">
-        <v>73</v>
-      </c>
-      <c r="G122" t="s">
-        <v>14</v>
-      </c>
-      <c r="H122" t="s">
+      <c r="I122" t="s">
         <v>519</v>
-      </c>
-      <c r="I122" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
+        <v>520</v>
+      </c>
+      <c r="B123" t="s">
         <v>521</v>
-      </c>
-      <c r="B123" t="s">
-        <v>509</v>
       </c>
       <c r="C123" t="s">
         <v>19</v>
@@ -8079,13 +8150,13 @@
         <v>522</v>
       </c>
       <c r="E123" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="F123" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="G123" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H123" t="s">
         <v>523</v>
@@ -8099,440 +8170,440 @@
         <v>525</v>
       </c>
       <c r="B124" t="s">
+        <v>521</v>
+      </c>
+      <c r="C124" t="s">
+        <v>19</v>
+      </c>
+      <c r="D124" t="s">
         <v>526</v>
       </c>
-      <c r="C124" t="s">
-        <v>19</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="E124" t="s">
+        <v>28</v>
+      </c>
+      <c r="F124" t="s">
+        <v>73</v>
+      </c>
+      <c r="G124" t="s">
+        <v>14</v>
+      </c>
+      <c r="H124" t="s">
         <v>527</v>
       </c>
-      <c r="E124" t="s">
-        <v>37</v>
-      </c>
-      <c r="F124" t="s">
-        <v>43</v>
-      </c>
-      <c r="G124" t="s">
-        <v>14</v>
-      </c>
-      <c r="H124" t="s">
+      <c r="I124" t="s">
         <v>528</v>
-      </c>
-      <c r="I124" t="s">
-        <v>529</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
+        <v>529</v>
+      </c>
+      <c r="B125" t="s">
+        <v>521</v>
+      </c>
+      <c r="C125" t="s">
+        <v>19</v>
+      </c>
+      <c r="D125" t="s">
         <v>530</v>
-      </c>
-      <c r="B125" t="s">
-        <v>531</v>
-      </c>
-      <c r="C125" t="s">
-        <v>19</v>
-      </c>
-      <c r="D125" t="s">
-        <v>532</v>
       </c>
       <c r="E125" t="s">
         <v>11</v>
       </c>
       <c r="F125" t="s">
-        <v>468</v>
+        <v>73</v>
       </c>
       <c r="G125" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H125" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="I125" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B126" t="s">
-        <v>536</v>
+        <v>521</v>
       </c>
       <c r="C126" t="s">
         <v>19</v>
       </c>
       <c r="D126" t="s">
-        <v>345</v>
-      </c>
-      <c r="E126"/>
+        <v>534</v>
+      </c>
+      <c r="E126" t="s">
+        <v>11</v>
+      </c>
       <c r="F126" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="G126" t="s">
         <v>22</v>
       </c>
       <c r="H126" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="I126" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
+        <v>537</v>
+      </c>
+      <c r="B127" t="s">
+        <v>538</v>
+      </c>
+      <c r="C127" t="s">
+        <v>19</v>
+      </c>
+      <c r="D127" t="s">
         <v>539</v>
       </c>
-      <c r="B127" t="s">
+      <c r="E127" t="s">
+        <v>37</v>
+      </c>
+      <c r="F127" t="s">
+        <v>43</v>
+      </c>
+      <c r="G127" t="s">
+        <v>14</v>
+      </c>
+      <c r="H127" t="s">
         <v>540</v>
       </c>
-      <c r="C127" t="s">
-        <v>19</v>
-      </c>
-      <c r="D127" t="s">
-        <v>84</v>
-      </c>
-      <c r="E127"/>
-      <c r="F127" t="s">
-        <v>13</v>
-      </c>
-      <c r="G127" t="s">
-        <v>14</v>
-      </c>
-      <c r="H127" t="s">
+      <c r="I127" t="s">
         <v>541</v>
-      </c>
-      <c r="I127" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
+        <v>542</v>
+      </c>
+      <c r="B128" t="s">
         <v>543</v>
       </c>
-      <c r="B128" t="s">
-        <v>540</v>
-      </c>
       <c r="C128" t="s">
         <v>19</v>
       </c>
       <c r="D128" t="s">
-        <v>84</v>
-      </c>
-      <c r="E128"/>
+        <v>544</v>
+      </c>
+      <c r="E128" t="s">
+        <v>11</v>
+      </c>
       <c r="F128" t="s">
-        <v>13</v>
+        <v>476</v>
       </c>
       <c r="G128" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H128" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="I128" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B129" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="C129" t="s">
         <v>19</v>
       </c>
       <c r="D129" t="s">
-        <v>547</v>
-      </c>
-      <c r="E129" t="s">
-        <v>28</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="E129"/>
       <c r="F129" t="s">
-        <v>308</v>
+        <v>29</v>
       </c>
       <c r="G129" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H129" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="I129" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B130" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="C130" t="s">
         <v>19</v>
       </c>
       <c r="D130" t="s">
-        <v>550</v>
-      </c>
-      <c r="E130" t="s">
-        <v>11</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E130"/>
       <c r="F130" t="s">
-        <v>308</v>
+        <v>13</v>
       </c>
       <c r="G130" t="s">
         <v>14</v>
       </c>
       <c r="H130" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="I130" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B131" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="C131" t="s">
         <v>19</v>
       </c>
       <c r="D131" t="s">
-        <v>547</v>
-      </c>
-      <c r="E131" t="s">
-        <v>28</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E131"/>
       <c r="F131" t="s">
-        <v>308</v>
+        <v>13</v>
       </c>
       <c r="G131" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H131" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="I131" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B132" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="C132" t="s">
         <v>19</v>
       </c>
       <c r="D132" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="E132" t="s">
         <v>28</v>
       </c>
       <c r="F132" t="s">
-        <v>117</v>
+        <v>316</v>
       </c>
       <c r="G132" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H132" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="I132" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B133" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="C133" t="s">
+        <v>19</v>
+      </c>
+      <c r="D133" t="s">
+        <v>562</v>
+      </c>
+      <c r="E133" t="s">
         <v>11</v>
       </c>
-      <c r="D133" t="s">
-        <v>217</v>
-      </c>
-      <c r="E133" t="s">
-        <v>78</v>
-      </c>
       <c r="F133" t="s">
-        <v>218</v>
+        <v>316</v>
       </c>
       <c r="G133" t="s">
         <v>14</v>
       </c>
       <c r="H133" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="I133" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B134" t="s">
+        <v>552</v>
+      </c>
+      <c r="C134" t="s">
+        <v>19</v>
+      </c>
+      <c r="D134" t="s">
         <v>559</v>
       </c>
-      <c r="C134" t="s">
-        <v>11</v>
-      </c>
-      <c r="D134" t="s">
-        <v>20</v>
-      </c>
-      <c r="E134"/>
+      <c r="E134" t="s">
+        <v>28</v>
+      </c>
       <c r="F134" t="s">
-        <v>21</v>
+        <v>316</v>
       </c>
       <c r="G134" t="s">
         <v>22</v>
       </c>
       <c r="H134" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="I134" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B135" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="C135" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D135" t="s">
-        <v>495</v>
+        <v>568</v>
       </c>
       <c r="E135" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F135" t="s">
-        <v>468</v>
+        <v>117</v>
       </c>
       <c r="G135" t="s">
         <v>22</v>
       </c>
       <c r="H135" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="I135" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B136" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C136" t="s">
         <v>11</v>
       </c>
       <c r="D136" t="s">
-        <v>303</v>
+        <v>223</v>
       </c>
       <c r="E136" t="s">
         <v>78</v>
       </c>
       <c r="F136" t="s">
-        <v>98</v>
+        <v>180</v>
       </c>
       <c r="G136" t="s">
         <v>14</v>
       </c>
       <c r="H136" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="I136" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B137" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C137" t="s">
         <v>11</v>
       </c>
       <c r="D137" t="s">
-        <v>212</v>
-      </c>
-      <c r="E137" t="s">
-        <v>78</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E137"/>
       <c r="F137" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="G137" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H137" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="I137" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B138" t="s">
-        <v>570</v>
+        <v>578</v>
       </c>
       <c r="C138" t="s">
         <v>11</v>
       </c>
       <c r="D138" t="s">
-        <v>577</v>
+        <v>507</v>
       </c>
       <c r="E138" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="F138" t="s">
-        <v>341</v>
+        <v>476</v>
       </c>
       <c r="G138" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H138" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="I138" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B139" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="C139" t="s">
         <v>11</v>
       </c>
       <c r="D139" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="E139" t="s">
         <v>78</v>
@@ -8544,485 +8615,491 @@
         <v>14</v>
       </c>
       <c r="H139" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="I139" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B140" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="C140" t="s">
         <v>11</v>
       </c>
       <c r="D140" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E140" t="s">
         <v>78</v>
       </c>
       <c r="F140" t="s">
-        <v>218</v>
+        <v>73</v>
       </c>
       <c r="G140" t="s">
         <v>14</v>
       </c>
       <c r="H140" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="I140" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B141" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="C141" t="s">
         <v>11</v>
       </c>
       <c r="D141" t="s">
-        <v>217</v>
+        <v>589</v>
       </c>
       <c r="E141" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="F141" t="s">
-        <v>218</v>
+        <v>349</v>
       </c>
       <c r="G141" t="s">
         <v>14</v>
       </c>
       <c r="H141" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="I141" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B142" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="C142" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D142" t="s">
-        <v>103</v>
-      </c>
-      <c r="E142"/>
+        <v>311</v>
+      </c>
+      <c r="E142" t="s">
+        <v>78</v>
+      </c>
       <c r="F142" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="G142" t="s">
         <v>14</v>
       </c>
       <c r="H142" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="I142" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="B143" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="C143" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D143" t="s">
-        <v>594</v>
+        <v>223</v>
       </c>
       <c r="E143" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F143" t="s">
-        <v>251</v>
+        <v>180</v>
       </c>
       <c r="G143" t="s">
         <v>14</v>
       </c>
       <c r="H143" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="I143" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B144" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="C144" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D144" t="s">
-        <v>36</v>
+        <v>223</v>
       </c>
       <c r="E144" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="F144" t="s">
-        <v>22</v>
+        <v>180</v>
       </c>
       <c r="G144" t="s">
         <v>14</v>
       </c>
       <c r="H144" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="I144" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B145" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="C145" t="s">
         <v>19</v>
       </c>
       <c r="D145" t="s">
-        <v>601</v>
-      </c>
-      <c r="E145" t="s">
-        <v>28</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E145"/>
       <c r="F145" t="s">
-        <v>43</v>
+        <v>104</v>
       </c>
       <c r="G145" t="s">
         <v>14</v>
       </c>
       <c r="H145" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="I145" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B146" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="C146" t="s">
         <v>19</v>
       </c>
       <c r="D146" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E146" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F146" t="s">
-        <v>43</v>
+        <v>260</v>
       </c>
       <c r="G146" t="s">
         <v>14</v>
       </c>
       <c r="H146" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I146" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B147" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="C147" t="s">
         <v>19</v>
       </c>
       <c r="D147" t="s">
-        <v>103</v>
-      </c>
-      <c r="E147"/>
+        <v>36</v>
+      </c>
+      <c r="E147" t="s">
+        <v>37</v>
+      </c>
       <c r="F147" t="s">
-        <v>104</v>
+        <v>22</v>
       </c>
       <c r="G147" t="s">
         <v>14</v>
       </c>
       <c r="H147" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I147" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="B148" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="C148" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D148" t="s">
-        <v>291</v>
+        <v>613</v>
       </c>
       <c r="E148" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F148" t="s">
-        <v>163</v>
+        <v>43</v>
       </c>
       <c r="G148" t="s">
         <v>14</v>
       </c>
       <c r="H148" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="I148" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B149" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="C149" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D149" t="s">
-        <v>303</v>
+        <v>616</v>
       </c>
       <c r="E149" t="s">
         <v>78</v>
       </c>
       <c r="F149" t="s">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="G149" t="s">
         <v>14</v>
       </c>
       <c r="H149" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="I149" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B150" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="C150" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D150" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="E150"/>
       <c r="F150" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="G150" t="s">
         <v>14</v>
       </c>
       <c r="H150" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="I150" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B151" t="s">
-        <v>611</v>
+        <v>623</v>
       </c>
       <c r="C151" t="s">
         <v>11</v>
       </c>
       <c r="D151" t="s">
-        <v>206</v>
+        <v>299</v>
       </c>
       <c r="E151" t="s">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="F151" t="s">
-        <v>207</v>
+        <v>163</v>
       </c>
       <c r="G151" t="s">
         <v>14</v>
       </c>
       <c r="H151" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="I151" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
+        <v>626</v>
+      </c>
+      <c r="B152" t="s">
         <v>623</v>
-      </c>
-      <c r="B152" t="s">
-        <v>611</v>
       </c>
       <c r="C152" t="s">
         <v>11</v>
       </c>
       <c r="D152" t="s">
-        <v>126</v>
+        <v>311</v>
       </c>
       <c r="E152" t="s">
         <v>78</v>
       </c>
       <c r="F152" t="s">
-        <v>21</v>
+        <v>98</v>
       </c>
       <c r="G152" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H152" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="I152" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B153" t="s">
-        <v>611</v>
+        <v>623</v>
       </c>
       <c r="C153" t="s">
         <v>11</v>
       </c>
       <c r="D153" t="s">
-        <v>495</v>
-      </c>
-      <c r="E153" t="s">
-        <v>11</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E153"/>
       <c r="F153" t="s">
-        <v>468</v>
+        <v>13</v>
       </c>
       <c r="G153" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H153" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="I153" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="B154" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="C154" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D154" t="s">
-        <v>352</v>
-      </c>
-      <c r="E154"/>
+        <v>212</v>
+      </c>
+      <c r="E154" t="s">
+        <v>179</v>
+      </c>
       <c r="F154" t="s">
-        <v>117</v>
+        <v>213</v>
       </c>
       <c r="G154" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H154" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="I154" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B155" t="s">
-        <v>634</v>
+        <v>623</v>
       </c>
       <c r="C155" t="s">
         <v>11</v>
       </c>
       <c r="D155" t="s">
-        <v>103</v>
-      </c>
-      <c r="E155"/>
+        <v>126</v>
+      </c>
+      <c r="E155" t="s">
+        <v>78</v>
+      </c>
       <c r="F155" t="s">
-        <v>104</v>
+        <v>21</v>
       </c>
       <c r="G155" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H155" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="I155" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B156" t="s">
-        <v>638</v>
+        <v>623</v>
       </c>
       <c r="C156" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D156" t="s">
-        <v>345</v>
-      </c>
-      <c r="E156"/>
+        <v>507</v>
+      </c>
+      <c r="E156" t="s">
+        <v>11</v>
+      </c>
       <c r="F156" t="s">
-        <v>29</v>
+        <v>476</v>
       </c>
       <c r="G156" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H156" t="s">
         <v>639</v>
@@ -9036,36 +9113,34 @@
         <v>641</v>
       </c>
       <c r="B157" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="C157" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D157" t="s">
-        <v>187</v>
-      </c>
-      <c r="E157" t="s">
-        <v>28</v>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="E157"/>
       <c r="F157" t="s">
-        <v>188</v>
+        <v>117</v>
       </c>
       <c r="G157" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H157" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="I157" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B158" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="C158" t="s">
         <v>11</v>
@@ -9081,59 +9156,57 @@
         <v>14</v>
       </c>
       <c r="H158" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="I158" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="B159" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C159" t="s">
         <v>19</v>
       </c>
       <c r="D159" t="s">
-        <v>649</v>
-      </c>
-      <c r="E159" t="s">
-        <v>37</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="E159"/>
       <c r="F159" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="G159" t="s">
         <v>14</v>
       </c>
       <c r="H159" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="I159" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B160" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C160" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D160" t="s">
-        <v>653</v>
+        <v>194</v>
       </c>
       <c r="E160" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F160" t="s">
-        <v>43</v>
+        <v>195</v>
       </c>
       <c r="G160" t="s">
         <v>14</v>
@@ -9150,17 +9223,15 @@
         <v>656</v>
       </c>
       <c r="B161" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C161" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D161" t="s">
-        <v>657</v>
-      </c>
-      <c r="E161" t="s">
-        <v>28</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E161"/>
       <c r="F161" t="s">
         <v>104</v>
       </c>
@@ -9168,10 +9239,97 @@
         <v>14</v>
       </c>
       <c r="H161" t="s">
+        <v>657</v>
+      </c>
+      <c r="I161" t="s">
         <v>658</v>
       </c>
-      <c r="I161" t="s">
+    </row>
+    <row r="162">
+      <c r="A162" t="s">
         <v>659</v>
+      </c>
+      <c r="B162" t="s">
+        <v>660</v>
+      </c>
+      <c r="C162" t="s">
+        <v>19</v>
+      </c>
+      <c r="D162" t="s">
+        <v>661</v>
+      </c>
+      <c r="E162" t="s">
+        <v>37</v>
+      </c>
+      <c r="F162" t="s">
+        <v>43</v>
+      </c>
+      <c r="G162" t="s">
+        <v>14</v>
+      </c>
+      <c r="H162" t="s">
+        <v>662</v>
+      </c>
+      <c r="I162" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s">
+        <v>664</v>
+      </c>
+      <c r="B163" t="s">
+        <v>660</v>
+      </c>
+      <c r="C163" t="s">
+        <v>19</v>
+      </c>
+      <c r="D163" t="s">
+        <v>665</v>
+      </c>
+      <c r="E163" t="s">
+        <v>11</v>
+      </c>
+      <c r="F163" t="s">
+        <v>43</v>
+      </c>
+      <c r="G163" t="s">
+        <v>14</v>
+      </c>
+      <c r="H163" t="s">
+        <v>666</v>
+      </c>
+      <c r="I163" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>668</v>
+      </c>
+      <c r="B164" t="s">
+        <v>660</v>
+      </c>
+      <c r="C164" t="s">
+        <v>19</v>
+      </c>
+      <c r="D164" t="s">
+        <v>669</v>
+      </c>
+      <c r="E164" t="s">
+        <v>28</v>
+      </c>
+      <c r="F164" t="s">
+        <v>104</v>
+      </c>
+      <c r="G164" t="s">
+        <v>14</v>
+      </c>
+      <c r="H164" t="s">
+        <v>670</v>
+      </c>
+      <c r="I164" t="s">
+        <v>671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-03-03
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -113,6 +113,25 @@
   </si>
   <si>
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik. Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">369583</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guggisberg Lars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
 </sst>
@@ -161,8 +180,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -576,6 +595,35 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-04
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -132,6 +132,208 @@
   </si>
   <si>
     <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">369707</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Pierre-André</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ziff. 34
+Antrag der Mehrheit [GZ]
+Art. 10b Titel [GZ]
+Zusammenarbeit des EFD, der FINMA und der Nationalbank zur Abwendung und Bewältigung des Ausfalls einer systemrelevanten Bank
+Art. 10b Text [GZ]
+Schätzt die FINMA, insbesondere nach Beurteilung der Risiken bei einer systemrelevanten Bank, die Anordnung einer Massnahme nach Artikel 25 Absatz 1 als voraussichtlich notwendig ein, teilt sie ihre Einschätzung unverzüglich dem EFD und der Nationalbank mit. Nach Benachrichtigung durch die FINMA teil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ziff. 34
+Antrag der Mehrheit [GZ]
+Art. 10b Titel [GZ]
+Zusammenarbeit des EFD, der FINMA und der Nationalbank zur Abwendung und Bewältigung des Ausfalls einer systemrelevanten Bank
+Art. 10b Text [GZ]
+Schätzt die FINMA, insbesondere nach Beurteilung der Risiken bei einer systemrelevanten Bank, die Anordnung einer Massnahme nach Artikel 25 Absatz 1 als voraussichtlich notwendig ein, teilt sie ihre Einschätzung unverzüglich dem EFD und der Nationalbank mit. Nach Benachrichtigung durch die FINMA teilt die Nationalbank dem EFD ihre Einschätzung insbesondere in Bezug auf die Risiken für die Schweizer Volkswirtschaft und das schweizerische Finanzsystem mit.
+Art. 30b Abs. 3 Bst. a[GZ]
+a. privilegierte Forderungen der ersten und zweiten Klasse nach Artikel 219 Absatz 4 SchKG sowie Forderungen nach Artikel 32c Absatz 1: im Umfang ihrer Privilegierung;
+Elfter a. Abschnitt Titel[GZ]
+Gewährung von Ausfallgarantien des Bundes für Liquiditätshilfe-Darlehen der Nationalbank an systemrelevante Banken
+Art. 32a Titel [GZ]
+Ausfallgarantien
+Art. 32a Abs. 1 [GZ]
+Der Bund kann der Nationalbank subsidiäre Ausfallgarantien gewähren für Liquiditätshilfe-Darlehen an Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, sofern:
+a. das Verfahren zur Sanierung der Darlehensnehmerin eingeleitet worden ist oder dessen Einleitung bevorsteht; und
+b. ohne Gewährung solcher Darlehen eine erhebliche Schädigung der Schweizer Volkswirtschaft und des schweizerischen Finanzsystems droht.
+Art. 32a Abs. 2 [GZ]
+Der Bund erhebt von den Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, jährlich eine Pauschale für das Risiko einer allfälligen Bereitstellung einer Ausfallgarantie. Die Pauschale entspricht dem Produkt aus einem einheitlichen Bemessungssatz und einer für jede Bank berechneten Bemessungsgrundlage. 
+Art. 32a Abs. 3 [GZ]
+Der Bund hat Anspruch auf eine Prämie für die Bereitstellung einer Ausfallgarantie. Die Bereitstellungsprämie bemisst sich nach der Höhe der Ausfallgarantie. 
+32a Abs. 4 [GZ]
+Der Bund und die Nationalbank haben Anspruch auf je eine Risikoprämie zur Abgeltung der mit einem Liquiditätshilfe-Darlehen mit Ausfallgarantie übernommenen Risiken. Die Risikoprämien bemessen sich nach der Höhe der ausbezahlten Liquiditätshilfe-Darlehen mit Ausfallgarantie. 
+Art. 32a Abs. 5 [GZ]
+Die Nationalbank hat Anspruch auf Zinsen auf Liquiditätshilfe-Darlehen mit Ausfallgarantie.
+Art. 32a Abs. 6 [GZ]
+Kosten für Leistungen Dritter, die im Zusammenhang mit Liquiditätshilfe-Darlehen mit Ausfallgarantie beim Bund, der Nationalbank oder der FINMA entstehen, werden der Darlehensnehmerin auferlegt.
+Art. 32a Abs. 7 [GZ]
+Der Bundesrat regelt namentlich:
+a. welche Massnahmen die Darlehensnehmerin ausgeschöpft haben muss, um sich Finanzierungsquellen zu erschliessen oder Sicherheiten zu beschaffen;
+b. den Bemessungssatz und die Berechnungsgrundlage der Pauschale sowie die Bemessung und Berechnung der Bereitstellungsprämie, der Risikoprämien und der Zinsen und deren jeweilige Erhebung;
+c. wann und in welchem Umfang der Anspruch der Nationalbank auf Übernahme eines definitiven Verlusts aus den von ihr gewährten Liquiditätshilfe-Darlehen mit Ausfallgarantie entsteht und unter welchen Voraussetzungen fällig wird;
+d. die weiteren Voraussetzungen zur Inanspruchnahme von Liquiditätshilfe-Darlehens mit Ausfallgarantie, namentlich notwendige Bestätigungen der FINMA und der Nationalbank;
+e. die Pflichten der FINMA und der Nationalbank im Zusammenhang mit der Risikoreduktion, Überwachung und Berichterstattung.
+Art. 32b Titel [GZ]
+Pflichten der Darlehensnehmerin als Folge von Liquiditätshilfe-Darlehen mit Ausfallgarantie
+Art. 32b Abs. 1 [GZ]
+Der Darlehensnehmerin und ihren direkten oder indirekten Tochtergesellschaften sind nicht erlaubt:
+a. die Beschlussfassung über und die Auszahlung von Dividenden und Tantiemen an Personen inner- und ausserhalb des Konzerns der Darlehensnehmerin
+b. die Rückerstattung von hartem Kernkapital, zusätzlichem Kernkapital, Ergänzungskapital und zusätzlichen verlustabsorbierenden Mitteln;
+c. die Gewährung von Darlehen an die und die Rückzahlung von Darlehen der Eigentümer der Konzernobergesellschaft.
+Art. 32b Abs. 2 [GZ]
+Die Darlehensnehmerin und die mit ihr direkt oder indirekt verbundenen Konzerngesellschaften dürfen weder Handlungen vornehmen, die die Rückzahlung der Liquiditätshilfe-Darlehen mit Ausfallgarantie und die vollständige Begleichung der Zinsen und Prämien nach Artikel 32a verzögern oder gefährden könnten, noch dürfen sie Handlungen unterlassen, die der Rückzahlung dieser Darlehen und der vollständigen Begleichung dieser Zinsen und Prämien dienlich sind. 
+Art. 32b Abs. 3 [GZ]
+Die Darlehensnehmerin muss die Liquiditätshilfe-Darlehen mit Ausfallgarantie vor anderen Liquiditätshilfe-Darlehen, die die Nationalbank ihr gewährt hat, zurückzahlen.
+Art. 32b Abs. 4 [GZ]
+Der Bundesrat regelt die Pflichten der Darlehensnehmerin einschliesslich der Ausnahmen:
+a. von den Pflichten der Darlehensnehmerin nach den Absätzen 1 und 2, insbesondere für die Fälle:
+1. vorbestehender ordentlicher Zahlungspflichten in Bezug auf Zinsen oder Amortisationen in Zusammenhang mit Geschäften nach Absatz 1 Buchstaben b oder c; und
+2. wenn die Darlehensnehmerin oder die Finanzgruppe von einer Drittgesellschaft übernommen und die Darlehensnehmerin oder die Finanzgruppe von einer Einheit der Drittgesellschaft absorbiert wird.
+b. von der Pflicht zur vorrangigen Rückzahlung der Liquiditätshilfe-Darlehen mit Ausfallgarantie.
+Art. 32c Titel [GZ]
+Konkursprivileg für Forderungen aus Liquiditätshilfe-Darlehen mit Ausfallgarantie
+Art. 32c Abs. 1 [GZ]
+Forderungen der Nationalbank aus Liquiditätshilfe-Darlehen mit Ausfallgarantie, die aufgelaufenen Prämien der Nationalbank und des Bundes und die aufgelaufenen Zinsen werden der dritten Klasse nach Artikel 219 Absatz 4 SchKG zugewiesen. 
+Art. 32c Abs. 2 [GZ]
+Sofern solche Forderungen bestehen, sind in Abweichung von Artikel 220 Absatz 1 SchKG die Forderungen innerhalb der dritten Klasse nach folgender Rangordnung zu befriedigen:
+a. Forderungen aus Freizügigkeitskonten in Form der reinen Sparlösung, die vom Bundesrat gestützt auf Artikel 26 Absatz 1 des Freizügigkeitsgesetzes vom 17. Dezember 1993 vorgesehen werden, und Forderungen aus Spareinlagen auf Konten der gebundenen Selbstvorsorge nach Artikel 82 Absatz 1 Buchstabe b des Bundesgesetzes vom 25. Juni 1982 über die berufliche Alters-, Hinterlassenen- und Invalidenvorsorge; 
+b. Forderungen der Nationalbank aus Liquiditätshilfe-Darlehen mit Ausfallgarantie, die aufgelaufenen Prämien der Nationalbank und des Bundes und die aufgelaufenen Zinsen; 
+c. alle übrigen Forderungen der dritten Klasse.
+Art. 32d Titel [GZ]
+Datenbearbeitung und Informationsaustausch 
+Art. 32d Abs. 1 [GZ]
+Das EFD, die FINMA, die Nationalbank und die Eidgenössische Finanzkontrolle sowie die für den Vollzug dieses Abschnitts beigezogenen Dritten dürfen Personendaten und Daten juristischer Personen, einschliesslich besonders schützenswerter Daten nach Artikel 5 Buchstabe c Ziffern 1, 2, 5 und 6 des Datenschutzgesetzes vom 25. September 2020 und besonders schützenswerter Daten juristischer Personen nach Artikel 57r Absatz 2 des Regierungs- und Verwaltungsorganisationsgesetzes vom 21. März 1997, und andere Informationen bearbeiten und einander bekanntgeben, soweit dies für den Vollzug dieses Abschnitts, namentlich für die Gewährung, Verwaltung, Überwachung, Prüfung und Abwicklung von Liquiditätshilfe-Darlehen und Ausfallgarantien sowie von Sicherheiten oder für die Marktbeobachtung notwendig ist. 
+Art. 32d Abs. 2 [GZ]
+Der Bundesrat regelt für die Zwecke der Liquiditätshilfedarlehen mit Ausfallgarantie den Austausch nicht öffentlich zugänglicher Informationen zwischen dem EFD, der FINMA, der Nationalbank und ausserdem:
+a. zur Bewertung der Risiken für den eidgenössischen Haushalt: die von der FINMA und der Nationalbank an das EFD zu erteilenden Informationen; und
+b. zur Beurteilung der Liquiditätshilfe-Darlehen, der Ausfallgarantien sowie der damit zusammenhängenden finanziellen Verpflichtungen des Bundes: die vom EFD der Eidgenössischen Finanzkontrolle zu übermittelnden Unterlagen und Informationen.
+Art. 32e Titel [GZ]
+Überprüfung dieses Abschnitts
+Art. 32e Text [GZ]
+Der Bundesrat muss spätestens fünf Jahre nach Inkrafttreten der Änderung vom ... die Bestimmungen dieses Abschnitts sowie der Ausführungsbestimmungen prüfen. Er erstattet der Bundesversammlung darüber Bericht und zeigt den allfälligen Aufhebungs- oder Anpassungsbedarf auf Gesetzesstufe auf.
+Art. 34 Abs. 1 [GZ]
+... Abweichende Bestimmungen des vorliegenden Gesetzes bleiben vorbehalten.
+Art. 36 Abs. 1bis [GZ]
+Die Rangordnung der Gläubiger und die Befriedigung ihrer Forderungen innerhalb der Rangklassen nach dem Artikel 32c sind im Kollokationsplan zu berücksichtigen.
+Art. 46 Abs. 1 Bst. d [GZ]
+d. die Pflichten nach Artikel 32b verletzt.
+[VS]
+Antrag der Minderheit I [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Gemäss Mehrheit
+[VS]
+Antrag der Minderheit II [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Streichen
+[VS]
+Antrag Aeschi [GZ]
+Streichen
+Schriftliche Begründung [GZ]
+Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat z. H. des Parlaments verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, Ständeräte hielten in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrsession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB ins Entlastungspaket 27:
+1. Die in der Fahne zum Entlastungspaket vorgeschlagene Regelung weicht in zentralen Punkten deutlich vom PLB-Gesetzesvorschlag des Bundesrates ab. So enthält der PLB-Vorschlag gemäss Entlastungspaket bloss die Hälfte der Bestimmungen, die der Bundesrat bei der PLB-Vorlage unterbreitet hatte. Eine fundierte und seriöse Analyse der konkreten Abweichungen war sowohl für die Mitglieder der FK-N als auch für die übrigen Mitglieder des Nationalrats im gegebenen Zeitrahmen nicht möglich. Umso problematischer ist, dass die Gründe für diese erheblichen Differenzen nicht transparent dargelegt wurden. Eine solche Intransparenz erschwert eine sachgerechte parlamentarische Beurteilung und untergräbt die notwendige Nachvollziehbarkeit des Gesetzgebungsprozesses.
+2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
+[VS]
+Proposition de la majorité [GZ]
+Art. 10b titre [GZ]
+Collaboration du DFF, de la FINMA et de la Banque nationale en vue de prévenir ou de maîtriser la défaillance d'une banque d'importance systémique
+Art. 10b texte [GZ]
+Si la FINMA estime, notamment après avoir évalué les risques encourus par une banque d'importance systémique, qu'il pourrait être nécessaire d'ordonner une des mesures visées à l'article 25 alinéa 1, la FINMA communique immédiatement son évaluation au DFF et à la Banque nationale. Une fois avisée par la FINMA, la Banque nationale communique son évaluation au DFF, notamment en ce qui concerne les risques pour l'économie et le système financier suisses.
+Art. 30b al. 3 let. a[GZ]
+a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés ;
+Chapitre XIa titre[GZ]
+Octroi par la Confédération de garanties du risque de défaillance pour les prêts d'aide sous forme de liquidités de la Banque nationale à des banques d'importance systémique
+Art. 32a titre [GZ]
+Garanties du risque de défaillance
+Art. 32a al. 1 [GZ]
+La Confédération peut octroyer à la Banque nationale des garanties du risque de défaillance subsidiaires pour les prêts d'aide sous forme de liquidités qui ont été accordés à des banques d'importance systémique ou faisant partie d'un groupe financier d'importance systémique, si
+a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être; et
+b. sans l'octroi de tels prêts, l'économie et le système financier suisses risquent de subir des dommages considérables.
+Art. 32a al. 2 [GZ]
+Une fois par année, la Confédération prélève auprès des banques qui sont d'importance systémique ou font partie d'un groupe financier d'importance systémique un forfait pour risque lié à une éventuelle mise à disposition d'une garantie du risque de défaillance. Le forfait équivaut au produit d'un taux de calcul unique et d'une base de calcul déterminée pour chacune des banques.
+Art. 32a al. 3 [GZ]
+La Confédération peut prétendre à une prime pour la mise à disposition d'une garantie du risque de défaillance. La prime de mise à disposition dépend du montant de la garantie.
+Art. 32a al. 4 [GZ]
+La Confédération et la Banque nationale peuvent chacune prétendre à une prime de risque au titre de compensation des risques qu'elles courent du fait de l'octroi d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance. Les primes de risque dépendent du montant versé au titre d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance.
+Art. 32a al. 5 [GZ]
+La Banque nationale peut prétendre à des intérêts sur les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance.
+Art. 32a al. 6 [GZ]
+Les frais pour des prestations de tiers liés aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance de la Confédération, de la Banque nationale ou de la FINMA sont mis à la charge de l'emprunteur.
+Art. 32a al. 7 [GZ]
+Le Conseil fédéral règle notamment :
+a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties ;
+b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts ;
+c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible ;
+d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale ;
+e. les obligations de la FINMA et de la Banque nationale en matière de réduction des risques, de surveillance et de rapports.
+Art. 32b titre [GZ]
+Obligations de l'emprunteur liées aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
+Art. 32b al. 1 [GZ]
+L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes :
+a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur ;
+b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes ;
+c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe ;
+Art. 32b al. 2 [GZ]
+L'emprunteur et les sociétés du groupe qui y sont directement ou indirectement liées n'effectuent pas d'acte qui pourrait retarder ou compromettre le remboursement des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ou le paiement de la totalité des primes et des intérêts visés à l'article 32a, ni n'omettent d'acte qui favoriserait le remboursement des prêts ainsi que le paiement de la totalité de ces primes et intérêts
+Art. 32b al. 3 [GZ]
+L'emprunteur est tenu de rembourser les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance avant les autres prêts d'aide sous forme de liquidités que la Banque nationale lui a octroyés.
+Art. 32b al. 4 [GZ]
+Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
+a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier :
+1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
+2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
+b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
+Art. 32c titre [GZ]
+Privilège des créances découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
+Art. 32c al. 1 [GZ]
+Les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus sont attribués à la troisième classe au sens de l'article 219 alinéa 4 LP.
+Art. 32c al. 2 [GZ]
+S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant :
+a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité ;
+b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus ;
+c. toutes les autres créances de la troisième classe.
+Art. 32d titre [GZ]
+Traitement des données et échange d'informations
+Art. 32d al. 1 [GZ]
+Le DFF, la FINMA, la Banque nationale, le CDF et les tiers chargés de l'exécution des dispositions du présent chapitre peuvent traiter et se communiquer mutuellement des données personnelles et des données concernant des personnes morales, y compris des données sensibles au sens de l'article 5 lettre c chiffres 1, 2, 5 et 6, de la loi du 25 septembre 2020 sur la protection des données et des données sensibles concernant des personnes morales au sens de l'article 57r alinéa 2 de la loi du 21 mars 1997 sur l'organisation du gouvernement et de l'administration, ainsi que d'autres informations, dans la mesure où cela est nécessaire à l'exécution des dispositions du présent chapitre, notamment pour l'octroi, l'administration, la surveillance, le contrôle et le traitement des prêts d'aide sous forme de liquidités et des garanties du risque de défaillance ainsi que des sûretés, ou pour l'observation du marché.
+Art. 32d al. 2 [GZ]
+Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre :
+a. pour l'évaluation des risques pour le budget de la Confédération : les informations par que la FINMA et la Banque nationale doivent fournir au DFF ; et
+b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés : les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
+Art. 32e titre [GZ]
+Examen des dispositions du présent chapitre
+Art. 32e texte [GZ]
+Cinq ans au plus tard après l'entrée en vigueur de la modification du ..., le Conseil fédéral réexamine les dispositions du présent chapitre ainsi que les dispositions d'exécution. Il fait rapport à l'Assemblée fédérale et détermine les dispositions législatives qu'il y a lieu éventuellement de modifier ou d'abroger.
+Art. 34 al. 1 [GZ]
+... Les dispositions dérogatoires de la présente loi sont réservées.
+Art. 36 al. 1bis [GZ]
+L'ordre des créanciers et le paiement de leurs créances selon l'ordre visé à l'article 32c sont pris en compte dans l'état de collocation.
+Art. 46 al. 1 let d[GZ]
+d. contrevient aux obligations prévues à l'article 32b.
+[VS]
+Proposition de la minorité I [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Selon majorité
+[VS]
+Proposition de la minorité II [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Biffer
+[VS]
+Proposition Aeschi [GZ]
+Biffer
+[VS]
+Le président (Page Pierre-André, président): La majorité et la minorité I proposent différentes modifications du plan financier. Les votes valent également pour l'arrêté fédéral IIa concernant les mesures d'allègement du budget 2027 arrêtées dans le plan financier pour les années 2027-2029.
 </t>
   </si>
 </sst>
@@ -180,8 +382,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -624,6 +826,35 @@
         <v>36</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-05
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -172,7 +172,7 @@
 Der Bund erhebt von den Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, jährlich eine Pauschale für das Risiko einer allfälligen Bereitstellung einer Ausfallgarantie. Die Pauschale entspricht dem Produkt aus einem einheitlichen Bemessungssatz und einer für jede Bank berechneten Bemessungsgrundlage. 
 Art. 32a Abs. 3 [GZ]
 Der Bund hat Anspruch auf eine Prämie für die Bereitstellung einer Ausfallgarantie. Die Bereitstellungsprämie bemisst sich nach der Höhe der Ausfallgarantie. 
-32a Abs. 4 [GZ]
+Art. 32a Abs. 4 [GZ]
 Der Bund und die Nationalbank haben Anspruch auf je eine Risikoprämie zur Abgeltung der mit einem Liquiditätshilfe-Darlehen mit Ausfallgarantie übernommenen Risiken. Die Risikoprämien bemessen sich nach der Höhe der ausbezahlten Liquiditätshilfe-Darlehen mit Ausfallgarantie. 
 Art. 32a Abs. 5 [GZ]
 Die Nationalbank hat Anspruch auf Zinsen auf Liquiditätshilfe-Darlehen mit Ausfallgarantie.
@@ -361,6 +361,31 @@
 Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">370058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds der AHV, IV und EO, sodass keine Belastung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds der AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
+Ziel des Vorhabens ist die umfassende Modernisierung der Organisation, der Geschäftsprozesse und der Informatiksysteme der ZAS, die als operatives Rückgrat der ersten Säule zentrale Register führt, die Finanzflüsse steuert und weltweit über eine Million Renten auszahlt. Die bestehenden Systeme seien technisch überaltert und stark fragmentiert, was die Automatisierung hemme, die Anpassung an gesetzliche Änderungen verteuere und die Datensicherheit gefährde. Ohne eine tiefgreifende Transformation wäre die ZAS laut eigenen Aussagen künftig nicht mehr in der Lage, Qualität und Effizienz ihrer Leistungen sicherzustellen. 
+Das Programm ist ein Schlüsselprojekt der Bundesverwaltung und als solches eingestuft. Es umfasst rund zehn miteinander verknüpfte Projekte, die in drei Phasen bis ins Jahr 2032 laufen. Kernpunkte sind die Umgestaltung der Prozesse hin zu vier bereichsübergreifenden Querschnittsprozessen, die Migration auf die standardisierte IT-Architektur, die Integration marktgängiger Lösungen und die Einführung eines neuen Betriebsmodells. Damit sollen die Silostrukturen aufgebrochen, die Automatisierung vorangetrieben und die Interoperabilität mit anderen Projekten der ersten Säule gewährleistet werden.
+Die Transformation soll es ermöglichen, das wachsende Arbeitsvolumen ohne zusätzliche Stellen zu bewältigen. Das Einsparpotenzial wird auf bis zu 80 Vollzeitäquivalente über zehn Jahre geschätzt, wobei die tatsächliche Wirkung vom Automatisierungsgrad und der Stabilität der Prozesse abhängen wird. Neben Effizienzgewinnen werden kürzere Bearbeitungszeiten, eine höhere Datensicherheit und eine bessere Anpassungsfähigkeit an gesetzliche Änderungen erwartet. 
+Ihre Finanzkommission hat die Vorlage eingehend beraten. In der Eintretensdebatte wurde die strategische Bedeutung des Projekts unumstritten anerkannt. Angesichts der demografischen Entwicklung, der steigenden Mobilität und der veralteten Infrastruktur wurde die Notwendigkeit einer Modernisierung von allen Seiten bestätigt. Diskutiert wurden Fragen zur Kontrolle der Effizienzgewinne, zu Teuerungsannahmen sowie zur Vermeidung von Anbieterabhängigkeit. Die Kommission begrüsst die geplante Standardisierung und die Reuse-Strategie, um bestehende Lösungen innerhalb der Bundesverwaltung zu nutzen. Auch die Governance-Struktur mit der Einbindung der Bundeskanzlei und der Begleitung durch die Eidgenössische Finanzkontrolle wurde positiv bewertet. 
+Die Kommission hat sich über die Konsequenzen des neuen Bundesgesetz über den Einsatz elektronischer Mittel zur Erfüllung von Behördenaufgaben (EMBAG) informiert, das die Veröffentlichung des Quellcodes solcher behördlicher Software verlangt. Der Kommission wurde versichert, dass es diesbezüglich keine Probleme gebe, weil die Rechte der bestehenden Software weitgehend beim Bund liegen und sich das mit dem neuen Programm nicht ändern werde. 
+Ihre Finanzkommission sieht im Programm eine notwendige Investition in die Zukunftsfähigkeit der ersten Säule und empfiehlt dem Rat einstimmig, auf die Vorlage einzutreten und den Verpflichtungskredit zu bewilligen.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -407,8 +432,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -909,6 +934,35 @@
         <v>45</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-06
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -241,9 +241,9 @@
 Antrag Aeschi [GZ]
 Streichen
 Schriftliche Begründung [GZ]
-Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat z. H. des Parlaments verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, Ständeräte hielten in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrsession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB ins Entlastungspaket 27:
+Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat zuhanden des Parlamentes verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, hielten Ständeräte in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrssession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB in das Entlastungspaket 27:
 1. Die in der Fahne zum Entlastungspaket vorgeschlagene Regelung weicht in zentralen Punkten deutlich vom PLB-Gesetzesvorschlag des Bundesrates ab. So enthält der PLB-Vorschlag gemäss Entlastungspaket bloss die Hälfte der Bestimmungen, die der Bundesrat bei der PLB-Vorlage unterbreitet hatte. Eine fundierte und seriöse Analyse der konkreten Abweichungen war sowohl für die Mitglieder der FK-N als auch für die übrigen Mitglieder des Nationalrats im gegebenen Zeitrahmen nicht möglich. Umso problematischer ist, dass die Gründe für diese erheblichen Differenzen nicht transparent dargelegt wurden. Eine solche Intransparenz erschwert eine sachgerechte parlamentarische Beurteilung und untergräbt die notwendige Nachvollziehbarkeit des Gesetzgebungsprozesses.
-2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
+2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine Ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
 [VS]
 Ch. 34[GZ]
 Proposition de la majorité [GZ]

</xml_diff>

<commit_message>
Update debates data - 2026-03-09
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -89,10 +89,10 @@
     <t xml:space="preserve">DE</t>
   </si>
   <si>
-    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
+    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ih</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
 Mein Antrag lautet also: Überweisung an die zuständige Kommission.
 </t>
   </si>
@@ -112,7 +112,8 @@
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzresso</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik. Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+    <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik.
+Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-03-10
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -403,6 +403,29 @@
     <t xml:space="preserve">Monsieur le conseiller national Amoos, Sipacfutur est un projet clé de la Confédération. À ce titre, il a été accompagné par le Contrôle fédéral des finances, qui a publié six rapports à son propos. Les recommandations des cinq premiers rapports ont été mises en oeuvre, ce qui a été attesté dans le sixième et dernier rapport. Ce dernier attirait encore l'attention sur la phase de migration entre l'ancien et le nouveau système. La migration a donc fait l'objet d'une attention particulière et a été effectuée sans problèmes notables. Des dysfonctionnements importants sont apparus par la suite et ont causé du retard dans certains paiements, ce qui est regrettable. Depuis février, le système est nettement plus stable. Actuellement, on travaille à la résorption du retard et à l'amélioration de la performance du système - voir aussi les questions 26.7131 et 26.7133 Mahaim.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">370837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans cette affaire, je ne peux que répéter une nouvelle fois mon plaidoyer en faveur d'une action efficace et rapide. Aux yeux du Conseil fédéral, un accord reste la façon la plus simple et la plus directe d'y parvenir. Lancer maintenant un processus législatif nous ferait perdre un temps précieux, d'autant plus que la consultation publique a montré que la majorité des participants approuvent l'accord et la démarche du Conseil fédéral. Je reviendrai plus tard sur les résultats de la consultation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans cette affaire, je ne peux que répéter une nouvelle fois mon plaidoyer en faveur d'une action efficace et rapide. Aux yeux du Conseil fédéral, un accord reste la façon la plus simple et la plus directe d'y parvenir. Lancer maintenant un processus législatif nous ferait perdre un temps précieux, d'autant plus que la consultation publique a montré que la majorité des participants approuvent l'accord et la démarche du Conseil fédéral. Je reviendrai plus tard sur les résultats de la consultation.
+Le Conseil fédéral est certain d'avoir choisi la bonne voie. Lors de la visite de la première ministre Ioulia Sviridenko en Suisse fin août, elle a explicitement souligné l'efficacité des instruments suisses pour inclure le secteur privé. Elle considère l'approche suisse comme un modèle pour d'autres pays. L'Ukraine elle-même recherche, en complément des instruments classiques de la coopération internationale, des investissements privés afin de stabiliser son économie. Le Conseil fédéral prend ce besoin très au sérieux et a fait de l'implication de l'économie privée suisse dans la reconstruction de l'Ukraine une priorité en allouant un montant de 500 millions de francs pour les quatre prochaines années. Le fait que nous ne pouvons simplement pas attendre est particulièrement évident au vu des derniers développements en Ukraine. Compte tenu de la grave crise énergétique sur place et à la suite d'une demande du gouvernement ukrainien, le Conseil fédéral a décidé le 11 février dernier d'adopter un plan d'aide humanitaire pour la livraison de produits énergétiques de première nécessité avec un plafond de 32 millions de francs. Ce plan d'aide va permettre d'acquérir, de livrer et d'installer 18 modules électriques fonctionnant au gaz naturel et jusqu'à 80 générateurs diesel de différentes puissances des fournisseurs suisses.
+Depuis le dépôt de la motion, quels sont les derniers développements ? Cette motion de la Commission de politique extérieure du Conseil des États a été acceptée par ce dernier, par 33 voix contre 12. C'était le 19 mars de l'année passée. Vous, le Conseil national, en revanche, avez rejeté le 20 mars 2025, par 105 voix contre 74 et 12 abstentions, une motion de votre Commission de politique extérieure dont le contenu était exactement le même. Je vous demande de rester cohérents et d'en rester à votre position. Parallèlement, lors de la consultation du mandat de négociation pour un traité international avec l'Ukraine, les Commissions de politique extérieure des deux conseils ont accepté ce mandat. C'était en février et en avril dernier. Ainsi, elles ont accepté la démarche du Conseil fédéral concernant la base légale pour l'aide à l'Ukraine. Cela nous a permis de faire avancer les travaux pour la négociation d'un traité avec l'Ukraine. Les négociations entre la Suisse et l'Ukraine se sont déroulées de manière très constructive et le résultat des négociations correspond aux objectifs de la Suisse. Tous ces échanges nous ont permis d'établir une relation de confiance entre notre pays et l'Ukraine. La collaboration est étroite. Nous devons bâtir sur cette confiance. Si la motion devait être adoptée, ce travail se poursuivrait, mais cela marquerait tout de même un sérieux coup dans nos relations avec l'Ukraine et cela freinerait ce mouvement positif que nous connaissons actuellement.
+Concernant les prochaines étapes pour l'approbation de l'accord par l'Assemblée fédérale, le Conseil fédéral a soumis vendredi dernier, le 6 mars, son message au Parlement pour l'approbation du traité. Le traité fera également l'objet de la possibilité d'un référendum.
+J'en viens maintenant, comme je vous l'ai dit tout à l'heure, à une brève appréciation des résultats de la consultation publique concernant le traité. Celle-ci s'est terminée le 12 novembre dernier et nous avons reçu un total de 53 prises de position dont 24 cantons, 4 partis politiques, 5 associations faîtières de l'économie et 20 ONG. Je peux vous informer, et je suis heureux de pouvoir vous dire qu'une majorité des participants se sont exprimés en faveur de l'accord que le Conseil fédéral a signé. Les principales raisons qui motivent l'approbation de l'accord sont les suivantes.
+Les principales raisons qui motivent l'approbation de l'accord sont les suivantes. L'importance du soutien à l'Ukraine pour la stabilité en Europe et, par conséquent, l'engagement de la Suisse, sont reconnus. L'implication du secteur privé suisse est considérée comme indispensable pour la reconstruction en Ukraine. L'accord permet d'apporter une aide rapide à l'Ukraine. L'approche de partenariat dans le cadre de laquelle l'Ukraine et la Suisse collaborent étroitement pour choisir les projets est saluée. La protection juridique des moyens engagés par le biais du monitorage, de l'évaluation, du contrôle par le Contrôle fédéral des finances ainsi que par le respect des principes de l'état de droit et de la démocratie, des droits de l'homme et de la lutte contre la corruption ont été soulignés positivement.
+Le Conseil fédéral reste convaincu que l'accord négocié avec l'Ukraine représente une solution élégante et efficiente qui nous permet de résoudre les questions juridiques relatives aux aides financières prévues ainsi que de régler les obligations des deux parties. Alors que les arguments en faveur du traité international restent les mêmes, nous sommes aujourd'hui plus avancés et avons la preuve que notre approche rencontre un écho positif en Ukraine et en Suisse. Au moment de la clôture du premier appel d'offres, près de 80 propositions avaient été reçues, venant de 60 entreprises suisses. Douze projets ont été sélectionnés, et leur mise en oeuvre est en bonne route. Les projets couvrent des thèmes tels que l'approvisionnement énergétique, l'hébergement pour les personnes déplacées à l'intérieur du pays ou les chemins de fer. Le budget total des projets sélectionnés s'élève à plus de 112 millions de francs, dont 93 millions sont financés par la Suisse, le reste étant pris en charge par les entreprises et par leurs partenaires ukrainiens.
+Il convient également de mentionner la participation des ONG suisses dans le cadre de ces projets. Elles apportent en effet leur expertise au secteur privé, une piste qui pourrait être approfondie pour de futurs appels à propositions. Entre-temps, nous avons lancé un deuxième appel à propositions le 9 janvier et le délai pour soumettre les projets échoit cette semaine. Compte tenu des retours positifs du marché, nous attendons à nouveau un grand nombre de propositions de projets.
+En conclusion, je suis persuadé que nous, Parlement et Conseil fédéral, avons le même objectif : fournir une aide à l'Ukraine le plus vite possible, là où elle est nécessaire, en encourageant les entreprises suisses à livrer des biens et des services urgents pour sa reconstruction, dont l'Ukraine ne dispose pas actuellement. Nous pouvons ainsi créer un levier ou un effet de levier pour relancer l'économie ukrainienne. Grâce à l'accord que nous avons négocié et signé, nous pourrons atteindre cet objectif dès l'automne prochain. Je vous invite à continuer sur cette voie, qui est efficace et à ne pas en ouvrir une deuxième qui pourrait ralentir le processus de soutien et utiliserait des ressources aujourd'hui utiles à la mise en oeuvre du programme suisse pour l'Ukraine.
+Je vous invite dès lors à accepter la démarche que nous suivons et à rejeter une deuxième fois cette motion qui a, je le répète, les mêmes termes que la première motion.
+Si vous deviez l'accepter, le Conseil fédéral poursuivrait le processus de ratification de l'accord. Il élaborera en parallèle une loi, et nous pourrons ainsi faire de notre mieux pour que le soutien à l'Ukraine et les secteurs privés en Suisse puissent débuter l'année prochaine. Je le répète : il serait administrativement et politiquement extrêmement dommage que vous suiviez cet aspect. Je vous invite vivement à rejeter cette motion, pour des raisons d'efficacité.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -449,8 +472,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I10"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1007,6 +1030,33 @@
         <v>56</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-11
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -129,10 +129,10 @@
     <t xml:space="preserve">BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+    <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
   <si>
@@ -426,6 +426,24 @@
 Si vous deviez l'accepter, le Conseil fédéral poursuivrait le processus de ratification de l'accord. Il élaborera en parallèle une loi, et nous pourrons ainsi faire de notre mieux pour que le soutien à l'Ukraine et les secteurs privés en Suisse puissent débuter l'année prochaine. Je le répète : il serait administrativement et politiquement extrêmement dommage que vous suiviez cet aspect. Je vous invite vivement à rejeter cette motion, pour des raisons d'efficacité.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">371050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich vertrete hier meine Minderheit II, eine starke Minderheit zur Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz". Die Finanzkommission hat hier mit 13 zu 12 Stimmen entschieden.
+Wir beantragen Ihnen, dem Entwurf des Bundesrates zu folgen. 
+Das Weiterbildungsgesetz ist 2017 in Kraft getreten. Hier geht es in erster Linie um Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich vertrete hier meine Minderheit II, eine starke Minderheit zur Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz". Die Finanzkommission hat hier mit 13 zu 12 Stimmen entschieden.
+Wir beantragen Ihnen, dem Entwurf des Bundesrates zu folgen. 
+Das Weiterbildungsgesetz ist 2017 in Kraft getreten. Hier geht es in erster Linie um Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Auch ist gemäss einer Überprüfung der Eidgenössischen Finanzkontrolle aus dem Jahr 2021 unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Es sind also sozusagen Beiträge, die gemäss Bundesrat durchaus gekürzt werden können. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. 
+Daher unterstützen wir den Entwurf des Bundesrates, und wir empfehlen Ihnen, dies auch zu tun.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -472,8 +490,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1057,6 +1075,35 @@
         <v>60</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-13
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -93,7 +93,7 @@
   </si>
   <si>
     <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
-Mein Antrag lautet also: Überweisung an die zuständige Kommission.
+Mein Antrag lautet also: Zuweisung an die zuständige Kommission.
 </t>
   </si>
   <si>
@@ -113,7 +113,7 @@
   </si>
   <si>
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik.
-Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Zuweisung an die Kommission.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-03-16
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -133,7 +133,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. 
-Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt 1 Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. 
+Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. 
+Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
   <si>
@@ -254,7 +256,7 @@
 Art. 10b texte [GZ]
 Si la FINMA estime, notamment après avoir évalué les risques encourus par une banque d'importance systémique, qu'il pourrait être nécessaire d'ordonner une des mesures visées à l'article 25 alinéa 1, la FINMA communique immédiatement son évaluation au DFF et à la Banque nationale. Une fois avisée par la FINMA, la Banque nationale communique son évaluation au DFF, notamment en ce qui concerne les risques pour l'économie et le système financier suisses.
 Art. 30b al. 3 let. a[GZ]
-a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés ;
+a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés[NB];
 Chapitre XIa titre[GZ]
 Octroi par la Confédération de garanties du risque de défaillance pour les prêts d'aide sous forme de liquidités de la Banque nationale à des banques d'importance systémique
 Art. 32a titre [GZ]
@@ -274,26 +276,26 @@
 Art. 32a al. 6 [GZ]
 Les frais pour des prestations de tiers liés aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance de la Confédération, de la Banque nationale ou de la FINMA sont mis à la charge de l'emprunteur.
 Art. 32a al. 7 [GZ]
-Le Conseil fédéral règle notamment :
-a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties ;
-b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts ;
-c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible ;
-d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale ;
+Le Conseil fédéral règle notamment[NB]:
+a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties[NB];
+b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts[NB];
+c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible[NB];
+d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale[NB];
 e. les obligations de la FINMA et de la Banque nationale en matière de réduction des risques, de surveillance et de rapports.
 Art. 32b titre [GZ]
 Obligations de l'emprunteur liées aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
 Art. 32b al. 1 [GZ]
-L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes :
-a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur ;
-b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes ;
-c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe ;
+L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes[NB]:
+a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur[NB];
+b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes[NB];
+c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe[NB];
 Art. 32b al. 2 [GZ]
 L'emprunteur et les sociétés du groupe qui y sont directement ou indirectement liées n'effectuent pas d'acte qui pourrait retarder ou compromettre le remboursement des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ou le paiement de la totalité des primes et des intérêts visés à l'article 32a, ni n'omettent d'acte qui favoriserait le remboursement des prêts ainsi que le paiement de la totalité de ces primes et intérêts
 Art. 32b al. 3 [GZ]
 L'emprunteur est tenu de rembourser les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance avant les autres prêts d'aide sous forme de liquidités que la Banque nationale lui a octroyés.
 Art. 32b al. 4 [GZ]
 Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
-a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier :
+a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier[NB]:
 1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
 2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
 b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
@@ -302,18 +304,18 @@
 Art. 32c al. 1 [GZ]
 Les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus sont attribués à la troisième classe au sens de l'article 219 alinéa 4 LP.
 Art. 32c al. 2 [GZ]
-S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant :
-a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité ;
-b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus ;
+S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant[NB]:
+a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité[NB];
+b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus[NB];
 c. toutes les autres créances de la troisième classe.
 Art. 32d titre [GZ]
 Traitement des données et échange d'informations
 Art. 32d al. 1 [GZ]
 Le DFF, la FINMA, la Banque nationale, le CDF et les tiers chargés de l'exécution des dispositions du présent chapitre peuvent traiter et se communiquer mutuellement des données personnelles et des données concernant des personnes morales, y compris des données sensibles au sens de l'article 5 lettre c chiffres 1, 2, 5 et 6, de la loi du 25 septembre 2020 sur la protection des données et des données sensibles concernant des personnes morales au sens de l'article 57r alinéa 2 de la loi du 21 mars 1997 sur l'organisation du gouvernement et de l'administration, ainsi que d'autres informations, dans la mesure où cela est nécessaire à l'exécution des dispositions du présent chapitre, notamment pour l'octroi, l'administration, la surveillance, le contrôle et le traitement des prêts d'aide sous forme de liquidités et des garanties du risque de défaillance ainsi que des sûretés, ou pour l'observation du marché.
 Art. 32d al. 2 [GZ]
-Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre :
-a. pour l'évaluation des risques pour le budget de la Confédération : les informations par que la FINMA et la Banque nationale doivent fournir au DFF ; et
-b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés : les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
+Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre[NB]:
+a. pour l'évaluation des risques pour le budget de la Confédération[NB]: les informations par que la FINMA et la Banque nationale doivent fournir au DFF[NB]; et
+b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés[NB]: les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
 Art. 32e titre [GZ]
 Examen des dispositions du présent chapitre
 Art. 32e texte [GZ]

</xml_diff>

<commit_message>
Update debates data - 2026-03-17
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -350,17 +350,17 @@
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
 Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Entwurf des Bundesrates und also dem Be</t>
+Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem </t>
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
 Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Entwurf des Bundesrates und also dem Beschluss des Ständerates. Den Minderheitsantrag Funiciello lehnen wir ab.
+Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
 Bei der Massnahme 11, "Kürzung der Subventionen für ausserschulische Kinder- und Jugendförderung", folgen wir dem Entwurf des Bundesrates. Die Kürzung dieser 1,5 Millionen Franken ist verkraftbar. Die Minderheitsanträge I (Zybach) und II (Gredig) lehnen wir dementsprechend ab.
 Bei den Massnahmen 27 und 30 folgen wir der Mehrheit der Finanzkommission und dem Beschluss des Ständerates.
 Ich komme zu meinen Minderheiten in diesem Block.
-Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen" beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildung und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
-Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
+Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
+Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch, und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
 Bei der Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz", habe ich die Minderheit III eingereicht. Das Weiterbildungsgesetz ist seit 2017 in Kraft. Auch hier beantrage ich, dem Entwurf des Bundesrates zu folgen. Es geht in erster Linie um die Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Gemäss einer Überprüfung der EFK aus dem Jahr 2021 ist unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. Daher unterstützen wir hier ebenfalls den Entwurf des Bundesrates.
 Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
@@ -461,6 +461,33 @@
   </si>
   <si>
     <t xml:space="preserve">Artikel 76e Absatz 1 BPR schreibt vor, dass die Kontrolle über die Korrektheit der Angaben und Dokumente lediglich stichprobenweise erfolgt. Die Eidgenössische Finanzkontrolle ist die zuständige Kontrollbehörde. Sie nimmt ihre Aufgaben im Rahmen der gesetzlichen Vorschriften selbstständig und unabhängig wahr. Sie wählt die Akteure, die sie prüft, risikoorientiert aus. Sie veröffentlicht die Namen der geprüften Akteure auf ihrer Website.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amaudruz Céline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réunie le 8 janvier 2026, la Commission de la sécurité sociale et de la santé publique du Conseil national a procédé à l'examen préalable de la motion 25.3637, "Mesures contraignantes en cas de hausse excessive des coûts, y compris pour les tarifs 'officiels' définis dans la LAMal", qui avait été déposée le 17 juin 2025 par M. Stefan Engler. Cette motion a été adoptée par le Conseil des États le 18 septembre 2025, par 34 voix contre 8 contre et 1 abstention.
+Que vise cette motion ? Elle charge l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réunie le 8 janvier 2026, la Commission de la sécurité sociale et de la santé publique du Conseil national a procédé à l'examen préalable de la motion 25.3637, "Mesures contraignantes en cas de hausse excessive des coûts, y compris pour les tarifs 'officiels' définis dans la LAMal", qui avait été déposée le 17 juin 2025 par M. Stefan Engler. Cette motion a été adoptée par le Conseil des États le 18 septembre 2025, par 34 voix contre 8 contre et 1 abstention.
+Que vise cette motion ? Elle charge le Conseil fédéral de compléter la loi fédérale sur l'assurance-maladie afin que l'évolution des coûts dans le domaine des tarifs officiels fixés par la Confédération fasse également l'objet d'une surveillance en cas de hausse excessive, par analogie avec le mécanisme prévu à l'article 47c LAMal pour les tarifs négociés.
+La hausse des coûts de l'assurance-maladie reste une préoccupation majeure pour la population suisse. Les projections indiquent que les personnes payant des primes ainsi que les contribuables devront assumer des charges croissantes au cours des prochaines décennies. Plusieurs facteurs contribuent à cette évolution, notamment la cherté des médicaments, les thérapies coûteuses pour certaines maladies rares, l'évolution démographique, les prestations inappropriées ou excessives, ainsi que l'augmentation quantitative de certaines prestations. Dans ce contexte, les partenaires tarifaires sont désormais tenus de surveiller l'évolution des coûts dans les domaines relevant des tarifs négociés et de prendre des mesures en cas d'évolution inexpliquée. L'auteur de la motion estime qu'il serait cohérent d'étendre un mécanisme comparable aux tarifs officiels fixés par la Confédération, notamment pour les médicaments, les analyses ou la liste des moyens et appareils.
+Le Conseil fédéral estime que la surveillance de l'évolution des coûts des tarifs officiels est déjà possible en vertu du droit en vigueur et que des mesures correctives peuvent être prises si cela est nécessaire. Il reconnaît toutefois que certaines différences existent entre les règles applicables aux tarifs officiels et celles applicables aux tarifs négociés, notamment en matière de communication et de fourniture de données. Dans ce contexte, il se déclare disposé à procéder à un état des lieux concernant les bases de données disponibles et, le cas échéant, à proposer des adaptations législatives. Toutefois, le Conseil fédéral recommande le rejet de la motion.
+La commission estime qu'une surveillance systématique de l'évolution des coûts de la santé est indispensable, compte tenu de la charge toujours plus lourde que représentent les primes dans le budget des personnes assurées. Cela vaut également pour les prestations fournies dans le cadre des tarifs officiels. En 2024, le domaine ambulatoire, les médicaments utilisés, les analyses de laboratoire, ainsi que les moyens et appareils ont représenté près de trois dixièmes des coûts bruts de l'assurance obligatoire des soins. La commission constate que la Confédération surveille de manière générale l'évolution des coûts dans les domaines soumis à des tarifs officiels et qu'elle prend également des mesures pour les réduire. Cependant, elle considère que des mesures supplémentaires doivent être prises afin que la Confédération puisse surveiller plus efficacement l'évolution des coûts dans ces domaines et exploiter au maximum le potentiel d'économies. La commission relève que, pour une surveillance efficace, il est nécessaire de procéder à des analyses différenciées et de disposer de données détaillées. Le rapport d'audit "Processus destiné à assurer la réalité des coûts dans le domaine des tarifs médicaux" du Contrôle fédéral des finances (CDF), daté du 16 décembre 2024, le confirme. Le CDF indique qu'en ce qui concerne les tarifs officiels, les compétences de la Confédération en matière de communication et de fourniture des données sont moins étendues que pour les tarifs négociés, alors même que ces tarifs sont fixés par les autorités.
+Lors de ses délibérations, la commission a également été informée par l'administration que, dans le domaine des tarifs officiels, les autorités dépendent encore souvent de la coopération des fournisseurs de prestations pour obtenir certaines données nécessaires à l'adaptation des services. Plusieurs membres ont estimé que la motion pouvait contribuer à combler cette lacune et à renforcer la cohérence des instruments de surveillance des coûts. Pour avoir accès aux données nécessaires, les autorités dépendent donc du bon vouloir des fournisseurs de prestations et n'exigent pas non plus de possibilités d'adopter des sanctions.
+En conséquence, la commission salue la volonté du Conseil fédéral de dresser un état des lieux des bases de données. En adoptant la motion, elle entend encourager ces travaux, renforcer le rôle de la Confédération dans ce domaine et donc combler les éventuelles lacunes.
+Je vous recommande donc, au nom de la commission, d'adopter cette motion que nous avons acceptée, par 24 voix contre 0 et 1 abstention.
 </t>
   </si>
 </sst>
@@ -509,8 +536,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I13" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I13"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1150,6 +1177,35 @@
         <v>69</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-18
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -263,7 +263,7 @@
 Garanties du risque de défaillance
 Art. 32a al. 1 [GZ]
 La Confédération peut octroyer à la Banque nationale des garanties du risque de défaillance subsidiaires pour les prêts d'aide sous forme de liquidités qui ont été accordés à des banques d'importance systémique ou faisant partie d'un groupe financier d'importance systémique, si
-a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être; et
+a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être[NB]; et
 b. sans l'octroi de tels prêts, l'économie et le système financier suisses risquent de subir des dommages considérables.
 Art. 32a al. 2 [GZ]
 Une fois par année, la Confédération prélève auprès des banques qui sont d'importance systémique ou font partie d'un groupe financier d'importance systémique un forfait pour risque lié à une éventuelle mise à disposition d'une garantie du risque de défaillance. Le forfait équivaut au produit d'un taux de calcul unique et d'une base de calcul déterminée pour chacune des banques.
@@ -296,7 +296,7 @@
 Art. 32b al. 4 [GZ]
 Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
 a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier[NB]:
-1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
+1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c[NB]; et
 2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
 b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
 Art. 32c titre [GZ]
@@ -488,6 +488,77 @@
 Lors de ses délibérations, la commission a également été informée par l'administration que, dans le domaine des tarifs officiels, les autorités dépendent encore souvent de la coopération des fournisseurs de prestations pour obtenir certaines données nécessaires à l'adaptation des services. Plusieurs membres ont estimé que la motion pouvait contribuer à combler cette lacune et à renforcer la cohérence des instruments de surveillance des coûts. Pour avoir accès aux données nécessaires, les autorités dépendent donc du bon vouloir des fournisseurs de prestations et n'exigent pas non plus de possibilités d'adopter des sanctions.
 En conséquence, la commission salue la volonté du Conseil fédéral de dresser un état des lieux des bases de données. En adoptant la motion, elle entend encourager ces travaux, renforcer le rôle de la Confédération dans ce domaine et donc combler les éventuelles lacunes.
 Je vous recommande donc, au nom de la commission, d'adopter cette motion que nous avons acceptée, par 24 voix contre 0 et 1 abstention.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372428</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260318</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dittli Josef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aus dem Bereich der ständerätlichen Subkommission EDA/VBS berichte ich Ihnen heute über drei massgebliche Geschäfte, welche uns im Jahr 2025 intensiv beschäftigten: erstens die Inspektion der Parlamentarischen Verwaltungskontrolle über die Honorarkonsulate, zweitens die Steuerung der Ruag MRO durch das VBS und drittens die Cybersicherheit der Armee.
+Lassen Sie mich mit den Honorarkonsulaten beginnen. Diese ehrenamtlich geführten Vertretungen sind eine lokale Anlaufstelle für Schweizer Staatsange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aus dem Bereich der ständerätlichen Subkommission EDA/VBS berichte ich Ihnen heute über drei massgebliche Geschäfte, welche uns im Jahr 2025 intensiv beschäftigten: erstens die Inspektion der Parlamentarischen Verwaltungskontrolle über die Honorarkonsulate, zweitens die Steuerung der Ruag MRO durch das VBS und drittens die Cybersicherheit der Armee.
+Lassen Sie mich mit den Honorarkonsulaten beginnen. Diese ehrenamtlich geführten Vertretungen sind eine lokale Anlaufstelle für Schweizer Staatsangehörige und unterstützen unsere Interessensvertretungen im Ausland. Gleichzeitig sind damit jedoch Reputationsrisiken verbunden. Da sich die Zahl der Schweizer Honorarkonsulate im Ausland seit 1990 verdoppelt hat, beauftragten die Geschäftsprüfungskommissionen im Januar 2024 die Parlamentarische Verwaltungskontrolle mit einer Evaluation. Diese untersuchte sowohl den Umgang des EDA mit den Schweizer Vertretungen im Ausland als auch jenen mit den ausländischen Honorarkonsulaten in der Schweiz. 
+Die Evaluation hat gezeigt, dass die Schweizer Honorarkonsulate im Ausland einen Mehrwert erbringen und vom EDA insgesamt angemessen betreut werden. Allerdings hängt die Qualität der Führung stark von der jeweiligen Vertretung im Empfangsstaat ab. Zudem halten sich die Vertretungen bei der Ernennung zwar an die Vorgaben, prüfen aber die Interessenbindungen zu wenig systematisch. Hier empfiehlt die GPK zukünftig eine systematische Prüfung potenzieller Interessenkonflikte. Auch fehlten im Untersuchungszeitraum klare strategische Vorgaben des Bundesrates zum Einsatz der Honorarkonsulate im Ausland. Das EDA hat zwar Ende 2025 eine neue Konsularstrategie publiziert, deren Mehrwert werden wir jedoch im Rahmen der Stellungnahme des Bundesrates erst noch analysieren.
+Kritischer beurteilt die Kommission das Vorgehen gegenüber ausländischen Honorarkonsulaten in der Schweiz, wo sich das EDA aus Rücksicht auf die bilateralen Beziehungen zu stark zurückhält. Wir empfehlen hier ein stringenteres Vorgehen. Wir erwarten auch hier die Stellungnahmen des Bundesrates.
+Ich komme nun zum zweiten Schwerpunkt, der Steuerung der Ruag MRO. Die Abklärungen der GPK-S zur Steuerung durch das VBS als Eigner bestätigten verschiedene erhebliche Mängel. Ein zentraler Punkt betrifft den unzweckmässigen Umgang mit Hinweisen auf Probleme aus dem Jahre 2019. Aus Sicht der Kommission wurde eine damalige Whistleblower-Meldung bei der Ruag Holding AG durch den Eigner suboptimal behandelt. Das VBS reagierte zwar im Prinzip zuerst richtig, indem es eine Anfrage an den Verwaltungsrat stellte. Im Nachhinein zeigte sich jedoch, dass auf dessen Beschwichtigungen kein Verlass war. Es ist für uns nur schwer nachvollziehbar, dass das VBS 2019 nicht in der Lage war, zu erkennen, dass in der Stellungnahme der Geschäftsleitung die Entkräftung des wichtigsten Vorwurfs fehlte, nämlich die Veräusserung von Material deutlich unter Marktpreisen. 
+Ebenfalls kritisch beurteilen wir die verspätete Berücksichtigung der Compliance in den strategischen Zielen. Obwohl der Bundesrat nach der Postauto-Affäre entschieden hatte, dass bundesnahe Unternehmen ein Compliance-Management-System führen müssen, verzichtete er bei der Ruag MRO zunächst darauf. Erst für die Periode 2024 bis 2027 wurde ein entsprechendes Ziel aufgenommen, was aus Sicht der Kommission eindeutig zu spät war. Wir bekräftigen unsere Haltung, dass der Bundesrat dafür sorgen muss, dass die Eignerstellen solche Compliance-Themen regelmässig mit dem Unternehmen besprechen. 
+Ein weiterer Mangel betrifft die zu positive Berichterstattung. Der Verwaltungsrat erstattete zunächst zu optimistisch Bericht, und der Bundesrat hinterfragte diese Zielbeurteilung zu wenig kritisch. In der Folge fiel auch die Information an die parlamentarischen Aufsichtskommissionen zu positiv aus. Wir fordern hier künftig eine transparente und kritische Information der Oberaufsicht. Die Vorfälle rund um den geplanten Verkauf von 96 Leopard-1-Panzern im Jahre 2023 haben diese Fragen zur Aufsicht und Steuerung durch den Eigner massiv verschärft.
+Deshalb haben wir ein Postulat eingereicht, um das aktuelle System der Corporate Governance und das duale Steuerungsmodell grundlegend zu prüfen. Wir erwarten, dass der Bundesrat die anstehende Anpassung der Rechtsform der Ruag MRO strategisch nutzt, um die Erkenntnisse aus den Prüfungen konsequent umzusetzen. Da die forensischen Untersuchungen externer Kanzleien und weitere Prüfungen der Eidgenössischen Finanzkontrolle noch andauern, behält sich die Kommission vor, zu einem späteren Zeitpunkt auf die Ereignisse zurückzukommen. Es wurden verschiedene Empfehlungen ausgesprochen. Der Bundesrat wird zu diesen Empfehlungen Stellung nehmen, und die Subkommission wird zusammen mit der Kommission die Antworten überprüfen.
+Abschliessend zum dritten Schwerpunkt, der Cybersicherheit der Armee. Die GPK-S beschäftigt sich seit 2023 im Nachgang zum Cyberangriff auf den Dienstleister Xplain vertieft mit der zivilen Cybersicherheit der Bundesverwaltung. Im Berichtsjahr hat die Kommission nun auch die Cybersicherheit der Armee behandelt. Dazu liess sie sich vom Kommando Cyber über dessen Organisation, Aufgaben und Herausforderungen informieren. Dabei nahm die Kommission den Stand der Umsetzung der Gesamtkonzeption Cyber vom 13. April 2022 zur Kenntnis.
+Wir konnten feststellen, dass die Rechtsgrundlagen, die Finanzen und das Personal das Kommando Cyber derzeit befähigen, seine Ziele zu erreichen. Herausforderungen bestehen weiterhin, insbesondere im Umgang mit international unterschiedlichen Klassifizierungsstufen und bei möglichen kollateralen Auswirkungen von Störungsaktionen, die das Kommando Cyber betreffen. Dennoch konnte sich die Kommission davon überzeugen, dass der Austausch des Kommandos mit den betroffenen Akteuren zweckmässig ist. Im Umgang mit den erwähnten Klassifizierungsstufen verfolgt das Kommando Cyber nachvollziehbare Ziele.
+Zudem konnten wir feststellen, dass das Kommando das Risiko einer Abhängigkeit von Betreibern grosser Rechenzentren wie Microsoft, Google oder Meta in seinen Umsetzungsarbeiten so weit als möglich angemessen berücksichtigt.
+Ein besonderer Schwerpunkt unserer Befassung war die Rolle des Kommandos Cyber in diversen IT-Projekten, die das VBS als sogenannte Top-Projekte führt. Dazu gehören die Projekte Telekommunikation der Armee, Führungsnetz Schweiz, Neue Digitalisierungsplattform (NDP) sowie das sichere Datenverbundnetz plus (SDVN+). 
+Ein zweiter Schwerpunkt betraf die Zusammenarbeit des Kommandos Cyber mit dem Bundesamt für Cybersicherheit (BACS). Hier stellte die Kommission fest, dass der Informationsaustausch zwischen den Einheiten funktioniert und eine klare Bereitschaft zur gegenseitigen Amtshilfe vorhanden ist. Das Kommando Cyber und das BACS arbeiten zudem gemeinsam daran, die Leistung von Amtshilfe durch Milizeinheiten zugunsten des BACS zu vereinfachen. Das ist entscheidend, um die nötige Reaktionsgeschwindigkeit bei Cybervorfällen sicherstellen zu können. Da die Kommission im Berichtsjahr keinen weiteren Handlungsbedarf bei der Cybersicherheit der Armee auf allgemeiner Ebene feststellte, hat sie ihre Arbeiten zu diesem Thema vorerst abgeschlossen. Sie bleibt aber über die Begleitung der Top-Projekte weiterhin am Ball.
+Auch ich möchte mich zum Schluss beim Sekretariat für die tolle Unterstützung und die getätigten Arbeiten während des Jahres bedanken.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372719</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hegglin Peter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Motion beauftragt den Bundesrat, die Subventionsprüfung gemäss Subventionsgesetz so anzupassen, dass daraus ein Paket für den Abbau von schädlichen Subventionen hervorgeht. Als Begründung wird ausgeführt, dass Subventionen häufig in einem suboptimalen Kosten-Nutzen-Verhältnis stünden, was in der Regel mit Fehlanreizen und Marktverzerrungen einhergehe. Deshalb sei eine sorgfältige Subventionsüberprüfung essenziell. Insbesondere sei es angesichts des sich abzeichnenden strukturellen Defizits i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Motion beauftragt den Bundesrat, die Subventionsprüfung gemäss Subventionsgesetz so anzupassen, dass daraus ein Paket für den Abbau von schädlichen Subventionen hervorgeht. Als Begründung wird ausgeführt, dass Subventionen häufig in einem suboptimalen Kosten-Nutzen-Verhältnis stünden, was in der Regel mit Fehlanreizen und Marktverzerrungen einhergehe. Deshalb sei eine sorgfältige Subventionsüberprüfung essenziell. Insbesondere sei es angesichts des sich abzeichnenden strukturellen Defizits im Bundeshaushalt wichtig, dass der Bund die Subventionen und Aufgaben immer wieder fundiert prüfe. Die Motionäre äussern die Vermutung, dass es, obwohl alle sechs Jahre eine Subventionsüberprüfung durchgeführt werde, beachtliches Optimierungspotenzial gebe. Deshalb sei der Bundesrat zu beauftragen, verschiedene Prüfvarianten zu evaluieren, so einerseits den sechsjährigen Prüfzyklus zu verkürzen und andererseits das Format anzupassen und mit einem Massnahmenpaket zu verbinden. 
+Obwohl der Bundesrat das Anliegen der Motionärin teilt, lehnt er das Motionsbegehren ab. Mit dem Entlastungspaket 27 habe er bei zahlreichen Subventionen einen Verzicht oder eine Reduktion vorgeschlagen. Er hätte auch im Subventionsgesetz festschreiben wollen, dass Finanzhilfen künftig 50 Prozent der Kosten der unterstützten Aufgabe grundsätzlich nicht übersteigen dürfen. Das hätten die Räte dann aber abgelehnt. Aus Sicht des Bundesrates sind Entlastungspakete dann zielführend, wenn sich Defizite abzeichnen. Er erachtet es deshalb als nicht zielführend, die Subventionsüberprüfung zu einem systematischen Entlastungsprogramm umzubauen. 
+Bei der Beratung lag der Kommission ein Bericht der EFK zur Subventionsüberprüfung vor. Die EFK kommt zum Schluss, dass die Prüfung wenig bewirke. Die EFK habe in den zehn Jahren zwischen 2014 und 2024 lediglich vier Fälle gefunden, in denen aus der Überprüfung tatsächlich Einsparungen hervorgegangen seien. Eingespart wurden damit dann nur zwei Millionen Franken. 
+Die Kommissionsmehrheit beurteilt die aktuelle Subventionsprüfung nicht so negativ. Die Prüfresultate der aktuell geprüften Verwaltungseinheiten werden jedes Jahr in den Botschaften zur Jahresrechnung abgedruckt. Finanzdelegation und Finanzkommission haben Einblick und können entsprechende Resultate aufnehmen und korrigieren. Das Ziel der Überprüfung besteht eh darin, die Rechtmässigkeit der Subventionen sicherzustellen. Die Prüfung hat auch einen präventiven Charakter bei den verschiedenen Ämtern und Departementen.
+Die Kommissionsmehrheit ist im Weiteren der Ansicht, dass der Zweck der Subventionsprüfung nicht darin besteht, regelmässig, systematisch und in institutioneller Weise das Sparpotenzial bei den Subventionen aufzuzeigen. Das Streichen oder Kürzen von Subventionen ist ein politischer Entscheid, der in erster Linie dem Parlament obliegen soll. Von erforderlichen Entlastungspaketen einmal abgesehen, sollte sich der gesamte Prozess von der anfänglichen Überlegung bis hin zum definitiven Subventionsbeschluss in den Händen des Parlamentes befinden. Aus Sicht der Kommission hat das Parlament heute schon die Möglichkeit, Subventionen zu befristen und damit eine periodische Überprüfung durch das Parlament zu erwirken, um endlosen Subventionen entgegenzuwirken.
+Im Rahmen von Entlastungspaketen wie dem EP 27 haben generelle Überprüfungen aber ihre Berechtigung und sind erfolgreicher. Gemäss EFK sind die Subventionsüberprüfungen heute unvollständig. Aus ihrer Sicht sind eigentlich auch Steuererleichterungen Subventionen, die alle sechs Jahre überprüft werden müssten. Weil die Politik, also wir, ihr den Zugang zu diesen Daten verwehrt, liegt die letzte Überprüfung schon 15 Jahre zurück. Daran dürfte die Politik, denke ich, auch nichts ändern wollen. 
+Weiter ist der Ausdruck "schädliche Subventionen", wie er im Motionstext steht, nicht eindeutig. Je nach politischer Sichtweise kann man zu einer anderen Einschätzung kommen, was "schädlich" bedeutet. Auch eine andere Wortwahl, z. B. "unnütze" Subventionen, oder gar die Streichung des Adjektivs erachtete die Kommission als nicht zielführend. Wenn die Bundesverwaltung Subventionen regelmässig analysieren und kontrollieren sowie Vorschläge unterbreiten müsste, könnten erhebliche unnötige Kosten entstehen, wenn das Parlament dann im Nachgang identifizierte Sparpotenziale nicht umsetzen würde. So hat das Parlament zum Beispiel beim EP 27 nur rund 60 Prozent der bundesrätlichen Sparvorschläge angenommen - und das trotz ausgewiesenem Sparbedarf. 
+Die Kommission sieht aber durchaus Verbesserungspotenzial: So können wir Subventionsregelungen bei der Ausgestaltung enger fassen, die Subventionsbeträge tief halten, die Subventionen zeitlich begrenzen und sie auch im Budgetprozess hinterfragen. Weiter können natürlich auch Subventionen, die nicht als Kredite ausgestaltet werden, einbezogen werden. Dies betrifft Leistungen, die der Bund kostenlos oder zu reduzierten Kosten anbietet, so beispielsweise Leistungen der Armee für das WEF. Es betrifft aber auch Subventionen, die über Fonds wie den Tabakpräventionsfonds ausgerichtet werden. Auch diese Leistungen sollten zukünftig durch die EFK geprüft werden. 
+Aus all den genannten Gründen lehnt die Kommission den Vorstoss mit 8 zu 4 Stimmen bei 0 Enthaltungen ab. Es gibt eine Minderheit, die ihre Argumente selber vortragen wird. Ich empfehle Ihnen, die Motion abzulehnen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben eine gleichlautende Motion schon einmal behandelt, und zwar in der Dezembersession des letzten Jahres. Jene Motion haben Sie mit 27 zu 14 Stimmen bei 2 Enthaltungen abgelehnt. Ich möchte Sie im Namen des Bundesrates bitten, auch diese Motion abzulehnen. Dies nicht, weil der Bundesrat nicht auch der Meinung ist, dass man Subventionen überprüfen soll und dass man Subventionen, die ein schlechtes Kosten-Nutzen-Verhältnis aufweisen, abschaffen soll; nein, ganz im Gegenteil. Wir haben ja di</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben eine gleichlautende Motion schon einmal behandelt, und zwar in der Dezembersession des letzten Jahres. Jene Motion haben Sie mit 27 zu 14 Stimmen bei 2 Enthaltungen abgelehnt. Ich möchte Sie im Namen des Bundesrates bitten, auch diese Motion abzulehnen. Dies nicht, weil der Bundesrat nicht auch der Meinung ist, dass man Subventionen überprüfen soll und dass man Subventionen, die ein schlechtes Kosten-Nutzen-Verhältnis aufweisen, abschaffen soll; nein, ganz im Gegenteil. Wir haben ja diese Übung jetzt gemacht, ich komme darauf zurück. 
+Es gibt einen Subventionsüberprüfungsmechanismus, der greift und an und für sich gut eingespielt ist. Wir überprüfen jedes Jahr im Rahmen der Staatsrechnung die Subventionen in einem Departement. Dieses Jahr, mit der Staatsrechnung 2025, war das UVEK betroffen; Sie werden am Freitag die Botschaft bekommen und sehen, dass wir das UVEK überprüft und Massnahmen vorgeschlagen haben. Nächstes Jahr kommt das EDA dran. Die Eidgenössische Finanzkontrolle überprüft derzeit auch diesen Mechanismus und wird Bericht erstatten. Der Bundesrat wird dann die Empfehlungen der EFK selbstverständlich würdigen. Also wir machen das; das ist ein eingespielter Mechanismus.
+Zudem möchte ich Ihnen einfach in Erinnerung rufen, dass wir mit der Gruppe Gaillard eine gross angelegte Aufgaben- und Subventionsüberprüfung gemacht haben. Wir haben Ihnen die entsprechenden Anträge gestellt. So haben wir Ihnen beispielsweise beantragt, das Subventionsgesetz zu schärfen, was Sie aber im Rahmen dieses EP 27 abgelehnt haben. Und wir haben Ihnen fast 60 Massnahmen vorgelegt, insbesondere Subventionsabbau, wobei Sie aber - das ist Ihre Freiheit - rund einen Drittel davon nicht gutgeheissen haben. Der Bundesrat erachtet es deshalb im Moment nicht als nötig, noch einmal eine solche Überprüfung zu machen. Die Massnahmen, die Sie abgelehnt haben, liegen auf dem Tisch, die könnte man wieder hervornehmen. Ob sich aber deren Mehrheitsfähigkeit so schnell ändert, möchte ich bezweifeln.
+Jedenfalls bitte ich Sie, diese Motion abzulehnen. 
+Übrigens bin ich noch auf eine interessante Massnahme gestossen. In den Achtzigerjahren gab es ein Sparpaket und da hat der Bundesrat einfach die Subventionen befristet über drei Jahre um 10 Prozent reduziert hat. Ich finde das auch noch interessant. Aber Sie können sich vorstellen, was das auslösen würde.
 </t>
   </si>
 </sst>
@@ -536,8 +607,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I13" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I16"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1206,6 +1277,91 @@
         <v>75</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" t="s">
+        <v>85</v>
+      </c>
+      <c r="I15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G16" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-19
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -561,6 +561,60 @@
 Übrigens bin ich noch auf eine interessante Massnahme gestossen. In den Achtzigerjahren gab es ein Sparpaket, und da hat der Bundesrat einfach die Subventionen befristet über drei Jahre um 10 Prozent reduziert. Ich finde das auch noch interessant. Aber Sie können sich vorstellen, was das auslösen würde.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">373030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sormanni Daniel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La réponse ou les réponses du Conseil fédéral, à ce jour, sont insuffisantes. On nous parle d'un système "stable" et de 94,3 pour cent des montants versés, mais ces chiffres ne reflètent pas la réalité sur le terrain. La vérité, c'est que des personnes vivent aujourd'hui sans revenu depuis des semaines, depuis des mois. Certaines attendent leurs indemnités depuis septembre 2025, alors même que leurs droits sont reconnus et que toutes les démarches ont été accomplies. Dans ces conditions, parler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La réponse ou les réponses du Conseil fédéral, à ce jour, sont insuffisantes. On nous parle d'un système "stable" et de 94,3 pour cent des montants versés, mais ces chiffres ne reflètent pas la réalité sur le terrain. La vérité, c'est que des personnes vivent aujourd'hui sans revenu depuis des semaines, depuis des mois. Certaines attendent leurs indemnités depuis septembre 2025, alors même que leurs droits sont reconnus et que toutes les démarches ont été accomplies. Dans ces conditions, parler encore de "résorber un retard" est inacceptable. Pour les personnes concernées, ce retard est déjà insupportable.
+Autre problème majeur : le Conseil fédéral ne connaît pas le nombre exact de paiements tardifs. Dans un système financé par les cotisations, cela n'est pas acceptable. Sans transparence, il n'y a pas de confiance. On nous propose des avances, selon l'article 31 de l'ordonnance sur l'assurance-chômage, mais une avance n'est pas une solution ; c'est un palliatif. Encore faudrait-il que cela soit efficace. Les avances compliquent souvent les démarches pour des personnes déjà en difficulté et ne corrigent en rien le dysfonctionnement du système. D'ailleurs, il apparaît que l'octroi d'une avance, avec ce nouveau système, est presque aussi complexe que le traitement d'un dossier, selon certaines caisses de chômage.
+Le Contrôle fédéral des finances a publié six rapports à l'attention du SECO, avant la mise en service de ce nouveau système informatique. Toutes ses recommandations ont été acceptées, mais trop tard. Elles sont en cours d'exécution, mais on a mis en service le nouveau système. Aujourd'hui, il faut, semble-t-il, selon certaines caisses de chômage, environ 30 minutes pour créer un dossier contre 1 minute 30 dans l'ancien système. C'est une régression incompréhensible. L'argument juridique sur les délais de retard est lui aussi déconnecté de la réalité. Quand on dépend de ces prestations pour vivre, chaque jour compte. Les conséquences sont immédiates : loyers impayés, dettes, pression psychologique. Et pourtant, aucune compensation réelle n'existe. Les intérêts moratoires éventuels peuvent intervenir après des délais allant jusqu'à deux ans. Ce n'est pas une protection. Pendant ce temps, les personnes concernées doivent survivre. Comment ? Elles ne peuvent pas attendre décembre 2026 ni la fin d'un projet informatique. Je rappelle que des avertissements avaient été émis sur les risques du système. Aujourd'hui, nous en voyons les conséquences. Un seul mois de retard, vous le savez bien, peut déjà entraîner une résiliation de bail, selon la loi - un seul mois. Et pendant ce temps, au moindre manquement, un assuré est immédiatement sanctionné et perdra des jours d'indemnités. Où est l'égalité de traitement dans ce cas ? 
+Nous ne pouvons pas rester passifs. Ce qui est fait aujourd'hui est insuffisant. C'est pourquoi je demande instamment de simplifier et systématiser les avances pour répondre à l'urgence, en application de l'article 19 de la loi fédérale sur la partie générale du droit des assurances sociales (LGPA) ; de revenir provisoirement à l'ancien système Sipac - on me dit que c'est impossible, mais impossible n'est pas français ; de renforcer immédiatement les moyens humains - je pense qu'il faut des moyens provisoires humains pour résoudre ces problèmes informatiques qui ne peuvent plus attendre encore juin ou la fin de l'année ; d'envisager des indemnités dans les cas les plus graves, nonobstant l'article 26 de la LGPA ; et de présenter un rapport à la session de juin. C'est aujourd'hui qu'il faut que les assurés puissent toucher les prestations auxquelles ils ont droit, les anciens assurés comme les nouveaux, dans un contexte où le chômage augmente en Suisse, où 800 postes de travail ont été perdus dans l'Arc jurassien. 
+Au-delà de la technique, c'est la crédibilité de l'assurance-chômage qui est en jeu. La protection sociale ne doit pas dépendre d'un système informatique défaillant, elle doit être garantie pour toutes et tous, maintenant.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'aimerais tout d'abord commencer en vous assurant que le Conseil fédéral est conscient de la situation difficile dans laquelle se trouvent les personnes concernées et qu'il la déplore. La situation, de manière générale, se stabilise. Les caisses de chômage, soutenues par le SECO, travaillent sans relâche pour résorber le retard pris dans le traitement des dossiers de personnes nouvellement inscrites au chômage. Je vais maintenant répondre aux questions de manière groupée, par thématique.
+Tout d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'aimerais tout d'abord commencer en vous assurant que le Conseil fédéral est conscient de la situation difficile dans laquelle se trouvent les personnes concernées et qu'il la déplore. La situation, de manière générale, se stabilise. Les caisses de chômage, soutenues par le SECO, travaillent sans relâche pour résorber le retard pris dans le traitement des dossiers de personnes nouvellement inscrites au chômage. Je vais maintenant répondre aux questions de manière groupée, par thématique.
+Tout d'abord, le processus et la décision de déploiement : le projet Sipacfutur a fait l'objet d'une préparation minutieuse. Il était assorti d'un processus de validation formelle comprenant notamment la possibilité d'un retour à la version précédente - ce qu'on appelle un "rollback" -, ainsi que des procédures alternatives pour le déploiement du nouveau système de paiement. Celles-ci n'ont cependant pas dû être activées, puisque la mise en service échelonnée de Sipac 2.0 au début du mois de janvier de cette année s'est déroulée de manière stable sur le plan technique. Le 5 janvier, le comité de pilotage du projet a donc donné son feu vert pour une utilisation à l'échelon national dès le lendemain. Ce n'est qu'après le déploiement à l'échelon national que des dysfonctionnements, parfois importants, sont apparus. Les conséquences en ont été une prolongation des délais de traitement et une accumulation de tâches au sein des caisses de chômage, ce qui a causé des retards pour certains paiements. Ces dysfonctionnements techniques importants ont, depuis, été corrigés. Malgré les difficultés rencontrées après la mise en service, le système a fonctionné de bout en bout en février, et les paiements escomptés ont globalement pu être effectués. Le système est aujourd'hui stable. La vitesse de traitement n'a pas encore atteint le niveau souhaité, mais elle s'améliore progressivement. La lenteur du système crée une surcharge de travail pour les employés des caisses de chômage, qui doivent travailler souvent le soir ou le week-end pour assurer un paiement rapide des prestations. Je les remercie sincèrement pour cet engagement exceptionnel. Les optimisations techniques se poursuivront durant la phase dite de stabilisation - qu'on appelle "hypercare". Cette phase est prévue jusqu'au mois de juin de cette année.
+Concernant la gouvernance et les recommandations du Contrôle fédéral des finances (CDF) : le comité de pilotage du projet réunit des spécialistes du DEFR, du SECO et de ses prestataires externes, des représentants des caisses de chômage publiques et privées ainsi que des autorités cantonales. Sipacfutur étant un projet informatique clé de la Confédération, il a fait l'objet d'audits de la part du CDF, qui a publié, cela a été dit, au total six rapports à ce sujet. Le SECO a accepté toutes les recommandations et les a mises ou les met en oeuvre. Comme c'est généralement le cas pour les grands projets menés par la Confédération, une analyse structurée de la clôture du projet sera effectuée d'ici, probablement, la fin 2026.
+Quelle est la situation actuelle en matière de paiements ? Les paiements sont désormais en bonne voie. Pour garantir la rapidité des paiements, des mesures ont été mises en place pour les mois de janvier à avril 2026. Les caisses de chômage bénéficient d'une plus grande marge d'appréciation pour l'examen des dossiers. De plus, l'examen du droit des personnes récemment inscrites au chômage a été simplifié sur certains points. Depuis la mise en service de Sipac 2.0 le 6 janvier et jusqu'au 17 mars 2026, près de 1181 millions de francs ont été versés. Cela représente 95,7 pour cent du montant attendu selon les estimations. Il n'y a malheureusement pas de chiffres disponibles sur le nombre de personnes affectées par les délais de paiement plus longs. Chaque paiement dépend, en effet, d'un dossier individuel et de l'examen du droit aux indemnités. Indépendamment du système de paiement, l'expérience montre que l'examen, pour les nouvelles inscriptions, prend généralement plusieurs semaines et peut être nettement plus long dans des cas complexes. La raison en est que la personne assurée doit fournir de nombreux documents qui nécessitent, selon la situation, des clarifications auprès d'employeurs précédents, d'autres autorités ou de la personne assurée elle-même. Il existe donc des lenteurs qui sont liées au nouveau système de paiement, mais aussi d'autres durées de traitement plus longues qui ne sont pas liées au changement de système.
+Concernant les demandes de compensation, une caisse de chômage doit verser l'indemnité de chômage, en règle générale, dans le courant du mois suivant la période de contrôle écoulée, ainsi que le précise l'article 30 de l'ordonnance sur l'assurance-chômage (OACI).
+Toutefois, les caisses de chômage ont souvent effectué les versements plus vite que les exigences légales, ce qui reste d'ailleurs l'objectif. Par conséquent, au sens juridique, il n'est question de retard de paiement qu'au terme du mois suivant au plus tôt. La loi ne prévoit pas de compensation générale pour des lenteurs dans le système de versement de l'indemnité. Un versement tardif des prestations déclenche en premier lieu le mécanisme de l'intérêt moratoire. Ce droit à l'intérêt moratoire est réglé à l'article 26 de la loi fédérale sur la partie générale du droit des assurances sociales. Un tel intérêt moratoire n'est dû que lorsque deux années se sont écoulées depuis la naissance du droit.
+Concernant la possibilité des avances, le Conseil fédéral est conscient qu'un délai prolongé pour le traitement du versement de l'indemnité de chômage peut avoir des conséquences pour les personnes concernées et il le regrette. Selon l'article 31 de l'ordonnance sur l'assurance-chômage, une personne au chômage peut demander une avance à sa caisse de chômage si elle est confrontée à des difficultés financières avant le versement de son indemnité. 
+J'en viens maintenant au postulat Gysi 25.4737, "Combler durablement les lacunes dans les assurances sociales". L'objectif de ce postulat est de charger le Conseil fédéral d'exposer dans un rapport commun si une assurance générale du revenu permettrait de combler les lacunes du système suisse d'assurances sociales de manière durable et financièrement responsable. La raison invoquée est notamment la nécessité de combler les lacunes en matière de couverture en cas de maladie. Une assurance générale du revenu va toutefois bien au-delà des domaines de la maladie, des accidents et de l'invalidité : elle couvrirait également la perte de revenu due au chômage, à la maternité ou au service militaire. Le Conseil fédéral est conscient que les pertes de gain peuvent entraîner des charges personnelles et financières considérables pour les personnes concernées. Cela peut notamment être le cas lors de maladies chroniques ou d'évolution prolongée et difficilement prévisible de la maladie. À titre d'exemples, on peut mentionner le COVID long ou le syndrome de fatigue chronique.
+Pour le Conseil fédéral, il n'y a toutefois pas de lacune à combler dans le système suisse d'assurance sociale en matière de perte de gain en cas de maladie temporaire, car celle-ci est largement couverte par les assurances d'indemnités journalières. Comme l'ont montré divers avis et rapports, le système actuel, qui comprend différentes assurances sociales et assurances facultatives, garantit à une grande partie de la population active une protection suffisante en cas de maladie temporaire ou d'accident. Une modification de l'ordonnance sur l'assurance-accidents (OLAA) est en consultation. Elle vise à abaisser le seuil d'entrée afin de permettre à un plus grand nombre d'indépendants d'accéder à l'assurance-accidents facultative. 
+Les situations de perte de gain suite à des maladies chroniques ont quant à elles gagné en importance. Le Conseil fédéral est conscient que ces situations peuvent poser des défis majeurs pour les personnes concernées. Ici, l'assurance indemnités journalières en cas de maladie et l'assurance-invalidité (AI) jouent un rôle primordial. Il convient de relever que, dans une première phase, la perte de gain n'entraîne que peu d'incertitudes grâce à une bonne coordination des prestations, et ce, malgré l'absence d'assurance obligatoire d'indemnités journalières en cas de maladie.
+Il est en outre important qu'une annonce en temps utile soit faite auprès de l'AI. Cela permet de garantir que lorsque la perte de gain se prolonge de manière durable, les prestations de l'AI remplacent sans interruption celles de l'assurance d'indemnités journalières en cas de maladie si les conditions d'octroi sont remplies. De plus, le Conseil fédéral a été chargé, avec la motion von Falkenstein 23.3808, "Accélérer la procédure AI et garantir la sécurité financière des assurés durant celle-ci", de prendre des mesures pour accélérer la procédure AI et pour garantir la sécurité financière des personnes concernées. Sa mise en oeuvre est en cours d'examen.
+J'aborde maintenant la perte de revenu en cas de chômage. Les personnes ayant perdu leur emploi en raison d'une incapacité durable peuvent, en principe, être couvertes par l'assurance-chômage. Cette dernière garantit en effet une compensation convenable du manque à gagner. En cas d'annonce à l'AI ou auprès d'une autre assurance sociale, la personne peut bénéficier d'une indemnité pleine de l'assurance-chômage. Pour cela, elle doit notamment être disposée et en mesure de prendre un emploi convenable correspondant à 20 pour cent au moins d'un emploi à plein temps.
+Concernant les rapports disponibles et les travaux en cours, de nombreux documents de référence, analyses et rapports existent ou sont en cours d'élaboration concernant les supposées lacunes mentionnées par le présent postulat dans le domaine des indemnités journalières en cas de maladie. Il convient en outre de se référer à la motion Romano 21.4209, "Assurance perte de gain obligatoire en cas de maladie", adoptée par votre conseil et suspendue par la Commission de la sécurité sociale et de la santé publique du Conseil des États dans l'attente du rapport en réponse à son postulat visant un état des lieux en vue d'un développement de l'assurance perte de gain en cas de maladie.
+Le Conseil fédéral est, dans ce cadre, notamment chargé d'analyser les problèmes actuels, de discuter de différentes solutions possibles et d'en présenter les avantages et les inconvénients. Le rapport est en cours d'élaboration. Il sera adopté par le Conseil fédéral, vraisemblablement cet été.
+Enfin, le Conseil fédéral s'est récemment également penché à plusieurs reprises sur la couverture sociale de différents groupes professionnels. C'est le cas, par exemple, dans le rapport "Protection sociale des indépendants", en réponse au postulat Roduit 20.4141. En raison des travaux en cours dans ce domaine, ce rapport n'a pas approfondi la question de l'assurance d'indemnités journalières en cas de maladie. Aucune mesure n'a été jugée nécessaire dans les autres domaines de la sécurité sociale.
+En conclusion, on peut retenir que le système actuel d'assurance sociale, structuré de manière différenciée, garantit à une grande partie des personnes actives une protection suffisante en cas de perte de gain. Une assurance générale du revenu modifierait fondamentalement ce système et soulèverait d'importantes questions d'ordre systémique et financier, sans offrir de valeur ajoutée évidente. En ce qui concerne l'assurance d'indemnités journalières en cas de maladie, il convient de se référer au rapport existant et à ceux en cours d'élaboration. Tant que les résultats correspondants ne seront pas disponibles, le Conseil fédéral estime qu'un nouveau rapport ne serait pas pertinent.
+Au vu de ces considérations, je vous invite, au nom du Conseil fédéral, à rejeter ce postulat.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C'est pour cela, Monsieur le conseiller national Amoos, qu'à la fin de tout projet comme celui-ci, qui est un projet clé au niveau de la Confédération, il y aura une analyse de fond qui fera le point sur tout ce qui n'a pas bien fonctionné, que ce soit au SECO ou ailleurs dans les caisses de chômage. C'est ce que nous ferons à la fin, sur demande du Contrôle fédéral des finances, mais aussi certainement sur demande de la Délégation des finances.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -607,8 +661,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I19" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I19"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1362,6 +1416,89 @@
         <v>89</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>93</v>
+      </c>
+      <c r="I17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>99</v>
+      </c>
+      <c r="I19" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-20
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -349,20 +349,21 @@
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
-Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem </t>
+Bei der Massnahme 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
+Bei der Massnahme 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem En</t>
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
-Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
+Bei der Massnahme 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
+Bei der Massnahme 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
 Bei der Massnahme 11, "Kürzung der Subventionen für ausserschulische Kinder- und Jugendförderung", folgen wir dem Entwurf des Bundesrates. Die Kürzung dieser 1,5 Millionen Franken ist verkraftbar. Die Minderheitsanträge I (Zybach) und II (Gredig) lehnen wir dementsprechend ab.
 Bei den Massnahmen 27 und 30 folgen wir der Mehrheit der Finanzkommission und dem Beschluss des Ständerates.
 Ich komme zu meinen Minderheiten in diesem Block.
-Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
+Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 
+2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
 Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch, und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
 Bei der Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz", habe ich die Minderheit III eingereicht. Das Weiterbildungsgesetz ist seit 2017 in Kraft. Auch hier beantrage ich, dem Entwurf des Bundesrates zu folgen. Es geht in erster Linie um die Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Gemäss einer Überprüfung der EFK aus dem Jahr 2021 ist unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. Daher unterstützen wir hier ebenfalls den Entwurf des Bundesrates.
-Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
+Abschliessend kann ich sagen, dass die SVP-Fraktion in Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
   </si>
   <si>
@@ -378,10 +379,10 @@
     <t xml:space="preserve">G</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12.[NB]September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12.[NB]September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
 Ziel des Vorhabens ist die umfassende Modernisierung der Organisation, der Geschäftsprozesse und der Informatiksysteme der ZAS, die als operatives Rückgrat der ersten Säule zentrale Register führt, die Finanzflüsse steuert und weltweit über eine Million Renten auszahlt. Die bestehenden Systeme seien technisch überaltert und stark fragmentiert, was die Automatisierung hemme, die Anpassung an gesetzliche Änderungen verteuere und die Datensicherheit gefährde. Ohne eine tiefgreifende Transformation wäre die ZAS laut eigenen Aussagen künftig nicht mehr in der Lage, die Qualität und Effizienz ihrer Leistungen sicherzustellen. 
 Das Programm ist ein Schlüsselprojekt der Bundesverwaltung und als solches eingestuft. Es umfasst rund zehn miteinander verknüpfte Projekte, die in drei Phasen bis ins Jahr 2032 laufen. Kernpunkte sind die Umgestaltung der Prozesse hin zu vier bereichsübergreifenden Querschnittsprozessen, die Migration auf die standardisierte IT-Architektur, die Integration marktgängiger Lösungen und die Einführung eines neuen Betriebsmodells. Damit sollen die Silostrukturen aufgebrochen, die Automatisierung vorangetrieben und die Interoperabilität mit anderen Projekten der ersten Säule gewährleistet werden.
 Die Transformation soll es ermöglichen, das wachsende Arbeitsvolumen ohne zusätzliche Stellen zu bewältigen. Das Einsparpotenzial wird auf bis zu 80 Vollzeitäquivalente über zehn Jahre geschätzt, wobei die tatsächliche Wirkung vom Automatisierungsgrad und der Stabilität der Prozesse abhängen wird. Neben Effizienzgewinnen werden kürzere Bearbeitungszeiten, eine höhere Datensicherheit und eine bessere Anpassungsfähigkeit an gesetzliche Änderungen erwartet. 

</xml_diff>

<commit_message>
Update debates data - 2026-04-29
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -166,10 +166,10 @@
 La disposition proposée par la majorité vise donc à inscrire cette collaboration dans la loi et à lui donner un cadre contraignant bienvenu. Elle correspond en outre à la recommandation formulée dans le rapport du Contrôle fédéral des finances sur la numérisation dans le premier pilier.
 Je vous invite dès lors à suivre la majorité de la commission et à rejeter la proposition de minorité de Courten.
 Une autre minorité de Courten vise, quant à elle, la suppression des règles relatives à la transparence des coûts ainsi qu'à la standardisation et à l'interopérabilité des systèmes d'information. Il s'agit toutefois de conditions essentielles, là aussi, pour que la Confédération puisse exercer efficacement sa fonction de pilotage, mais aussi sa fonction de surveillance. Le Contrôle fédéral des finances a d'ailleurs invité l'OFAS à utiliser de manière plus systématique ces instruments de pilotage existants, notamment en ce qui concerne les coûts informatiques. Là aussi, je vous invite à suivre la majorité de votre commission.
-Enfin, la minorité Reichsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
+Enfin, la minorité Rechsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
 Das Anliegen ist nachvollziehbar. Der Antrag der Minderheit würde jedoch unserer Meinung nach zu weit gehen. Es würde der Militär- und der Unfallversicherung Zugang zu allen Daten der ersten Säule gewähren. Wir dürfen nicht vergessen, dass es sich dabei teilweise um besonders sensible Daten handelt, insbesondere um Daten zur Gesundheit oder zur Invalidität. Das BSV hat in Zusammenarbeit mit den betroffenen Versichern ein Projekt lanciert. Ziel ist es, die Datenflüsse zu analysieren und die notwendigen rechtlichen Grundlagen zu klären, um einen gezielten und nachvollziehbaren Datenaustausch zu ermöglichen.
 Cependant, nous l'avons indiqué en commission, ce projet de discussions n'est pas encore suffisamment avancé à l'heure actuelle. J'ai demandé à l'OFAS de mettre la priorité sur ces discussions. Je crois que tout le monde est intéressé à clarifier la nature des données à transmettre pour faciliter et favoriser le travail de concertation entre les assurances, mais aussi pour aller en faveur des assurés. L'objectif est de pouvoir présenter une disposition correspondante, donc d'être pragmatique, en faisant une proposition au Conseil des États.
-Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Reichsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
+Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Rechsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-02
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -41,157 +41,109 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
-    <t xml:space="preserve">373984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20260429</t>
+    <t xml:space="preserve">374600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260602</t>
   </si>
   <si>
     <t xml:space="preserve">N</t>
   </si>
   <si>
-    <t xml:space="preserve">Silberschmidt Andri</t>
+    <t xml:space="preserve">Götte Michael</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Depar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019.
+Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
+Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken. Hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
+Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
+Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
+Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
+Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf.
+Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
+Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
+Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
+Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
+Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">374870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schaffner Barbara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Ei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
+Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
+Das ist Steuersubventionitis, eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Sätze, Befreiungen oder Abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">374713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giacometti Anna</t>
   </si>
   <si>
     <t xml:space="preserve">RL</t>
   </si>
   <si>
-    <t xml:space="preserve">ZH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wir sprechen heute über das Bundesgesetz über Informationssysteme in den Sozialversicherungen (BISS), das es für die Digitalisierung der ersten Säule zwingend braucht. Vereinfacht gesagt geht es darum, dass Bürgerinnen und Bürger einen einfachen digitalen Zugriff auf die Informationen ihrer eigenen Sozialversicherungen erhalten, z. B. in der AHV. Heute besteht ein analoger Prozess, wenn man wissen will, wie viel man in die AHV einbezahlt hat, wie hoch die eigene Rente ausfallen wird und ob Beitr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wir sprechen heute über das Bundesgesetz über Informationssysteme in den Sozialversicherungen (BISS), das es für die Digitalisierung der ersten Säule zwingend braucht. Vereinfacht gesagt geht es darum, dass Bürgerinnen und Bürger einen einfachen digitalen Zugriff auf die Informationen ihrer eigenen Sozialversicherungen erhalten, z. B. in der AHV. Heute besteht ein analoger Prozess, wenn man wissen will, wie viel man in die AHV einbezahlt hat, wie hoch die eigene Rente ausfallen wird und ob Beitragslücken bestehen, die man noch begleichen will. Dieser Prozess dauert Tage, wenn nicht Wochen, und ist sehr komplex, weil sich die verschiedenen Durchführungsstellen untereinander abstimmen müssen. Dabei ist zu klären, wo eine Person überall AHV-Beiträge geleistet hat; anschliessend müssen die Daten zusammengeführt und der betroffenen Person in Form eines individuellen Kontoauszuges mitgeteilt werden. Mit dem BISS soll sich dies ändern. Künftig soll es in der ganzen Schweiz ein Portal geben, über das sich Bürgerinnen und Bürger bzw. versicherte Personen einloggen und per Knopfdruck alle relevanten Informationen abrufen können, d. h. etwa die voraussichtliche Rentenhöhe oder bestehende Beitragslücken.
-Weshalb braucht es nun dieses Gesetz? Grundsätzlich gilt, dass alles staatliche Handeln eine gesetzliche Grundlage benötigt. Die Regulierung der ersten Säule, d. h. der AHV, der IV, der EO und der Familienzulagen, liegt bereits heute beim Bund; die Leistungen sind national geregelt. Die Durchführung der ersten Säule ist jedoch bei den Kantonen und teilweise auch bei den Verbandsausgleichskassen angesiedelt. Es bestehen öffentliche und private Ausgleichskassen, die die erste Säule abwickeln. Für die Digitalisierung ergibt es jedoch wenig Sinn, wenn zehn oder zwanzig unterschiedliche Onlineportale bestehen. Dies hat auch die Eidgenössische Finanzkontrolle erkannt. Allen, die argumentieren, es brauche keine Lösung des Bundes, sondern eine der Kantone, sei der Bericht der EFK zur Lektüre empfohlen. Er fällt bezüglich der bisherigen Digitalisierungsanstrengungen der Ausgleichskassen leider wenig schmeichelhaft aus. Er zeigt, dass diese bisher hohe Kosten verursacht haben und dass keine gemeinsame Lösung erzielt werden konnte. Auch aus diesem Grund ist es im Interesse der Steuerzahler sinnvoller, ein einziges Portal statt mehrere Dutzend Portale zu betreiben.
-Übrigens machen wir im Gesundheitswesen derzeit genau das Gleiche: das Patientendossier, das neu "Gesundheitsdossier" heisst. Auch dort ist man zur Überzeugung gelangt, dass es in einem Land mit 9 Millionen Einwohnern keinen Wettbewerb bei der digitalen Grundinfrastruktur braucht. Bei der Autobahn und beim Schienennetz haben wir ja auch keinen Wettbewerb. So ist es auch hier sinnvoll, dass wir eine einheitliche Infrastruktur haben, die den Bürgerinnen und Bürgern einen einfachen Zugang zu ihren Vorsorgedaten gibt.
-Dieses relativ schlanke Bundesgesetz über Informationssysteme in den Sozialversicherungen setzt also gemeinsame Standards. Es übernimmt nicht die Aufgaben der Durchführungsstellen; es ist ganz klar und bewusst so gemacht, dass diese weiterhin bei den Kantonen bleiben. Aber es definiert in Zukunft Standards, wie man digital miteinander kommuniziert und wie die Versicherten entsprechend an die Informationen kommen, die sie betreffen. Wir haben jetzt gehört, dass dies langfristig weniger Kosten verursacht, weil der heutige papierlastige Prozess zwar nicht hinfällig, aber sicherlich abnehmen wird.
-Wir von der Mehrheit haben auch Folgendes gemacht: Wir haben selbstverständlich die Kritik aus der Vernehmlassung ernst genommen und wollen einen Passus ins Gesetz schreiben, mit dem den Durchführungsstellen explizit auch das Recht eingeräumt wird, in die Entwicklung dieser Plattform eingebunden zu werden. Das ist auch mir persönlich ein grosses Anliegen. Die Durchführungsstellen leisten in den Kantonen eine sehr wichtige und hervorragende Arbeit. Wir müssen sie einbeziehen, wenn auf nationaler Ebene eine solche Plattform entwickelt wird. Das soll nun explizit im Gesetz verankert werden. Ich danke auch den Durchführungsstellen, dass sie sich so engagiert haben.
-Das Bundesgesetz über Informationssysteme in den Sozialversicherungen ist auch eine Grundlage für ein digitales Vorsorgeportal. Wir regeln hier bewusst lediglich die staatliche Sozialversicherung und nicht die private, also nicht die zweite und die dritte Säule. Aber wenn wir einen guten digitalen Zugang zur ersten Säule ermöglichen, ist es viel einfacher, auch Portale zu bauen, die den Leuten eine Gesamtübersicht über die eigene Vorsorgesituation bieten. Dazu leistet dieses Gesetz ebenfalls einen wichtigen Beitrag.
-Ich bitte Sie, auf die Vorlage einzutreten und sie nicht an den Bundesrat zurückzuweisen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte gerne auf Artikel 22a und Artikel 22b eingehen, welche wir in der Kommission eingeführt haben. Es geht hier um das Steuerungs- und Mitwirkungsgremium. 
-Ich verstehe nicht, weshalb der Minderheitssprecher das ablehnt, zumal es der SVP-Fraktion in der Beratung ein Anliegen war, dass die kantonalen Durchführungsstellen in die Gesetzgebung einbezogen werden. Genau das stellen wir mit diesem Artikel 22a sicher. Wir stellen sicher, dass nicht ausschliesslich der Bund Standards festlegen kan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte gerne auf Artikel 22a und Artikel 22b eingehen, welche wir in der Kommission eingeführt haben. Es geht hier um das Steuerungs- und Mitwirkungsgremium. 
-Ich verstehe nicht, weshalb der Minderheitssprecher das ablehnt, zumal es der SVP-Fraktion in der Beratung ein Anliegen war, dass die kantonalen Durchführungsstellen in die Gesetzgebung einbezogen werden. Genau das stellen wir mit diesem Artikel 22a sicher. Wir stellen sicher, dass nicht ausschliesslich der Bund Standards festlegen kann, sondern dass ein Gremium mit Vertreterinnen und Vertretern des BSV, der ZAS sowie der Durchführungsstellen verbindlich die Standards festlegt, die Digitalisierungsprojekte priorisiert und die Umsetzungsmodalitäten festlegt. Genau das, was die Minderheitssprecher moniert haben, haben wir in diesen Artikel 22a aufgenommen. Die Durchführungsstellen werden nicht nur angehört, sondern sind Teil des Steuerungs- und Mitwirkungsgremiums. 
-Artikel 22b ist wie auch Artikel 22a inspiriert von der Analyse der Eidgenössischen Finanzkontrolle, deren Bericht ich wirklich zur Lektüre empfehlen kann. Hier verlangen wir, dass das BSV verbindliche Vorgaben bei der Standardisierung, bei der Interoperabilität wie auch bei der einheitlichen Erfassung der IKT-Kosten macht. Ich denke, Absatz 1 Buchstabe a wird man im Ständerat streichen können, weil das im AHVG bereits geregelt ist. Die Buchstaben b und c sowie Absatz 2 sind hingegen nach wie vor wichtig; deshalb unterstützen wir diese auch. 
-Ich möchte noch kurz auf den Antrag der Minderheit Rechsteiner Thomas zu sprechen kommen, welchen wir ebenfalls unterstützen. Wenn ich den Antrag dieser Minderheit lese, steht klar geschrieben, dass die Unfallversicherung wie auch die Militärversicherung nur dort Zugriff auf die Daten haben, wo das zur Koordinierung der Leistungen notwendig ist. Es ist also nicht ein Blankoscheck, wie vorhin erwähnt wurde. Unserer Meinung nach ist es richtig, dass die Unfallversicherung wie auch die Militärversicherung Teil dieser Plattform sein können, weil wir sonst wieder neue Medienbrüche haben. Deshalb ist es aus unserer Sicht sehr wichtig, dass wir diese Minderheit Rechsteiner Thomas unterstützen. Wie gesagt, es ist kein Blankoscheck; es steht im Gesetz klar, dass nur dort Zugriff gewährt wird, wo es zur Koordination der Leistungen notwendig ist. 
-Das Datenschutzgesetz findet natürlich auch im Bundesgesetz über die Informationssysteme in den Sozialversicherungen Anwendung. Wenn jetzt gesagt wird, es gebe ja noch ein Datenschutzgesetz, dann ist das in der Tat so. Das Gesetz, das wir beraten, setzt das Datenschutzgesetz nicht ausser Kraft. In diesem Sinne finde ich die Begründung dagegen ein bisschen überzogen. Ich denke, wir sollten diese Minderheit unterstützen. Wenn man dann in dieser Gruppe, wo man das jetzt definieren will, weitergekommen ist, kann man im Ständerat noch die eine oder andere Präzisierung vornehmen. Ich denke, es ist wichtig, dass wir in diesem Gesetz alle Sozialversicherungen einbeziehen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechsteiner Thomas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M-E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich informiere Sie über die Diskussion in der Kommission, und zwar nicht nur zu den Artikeln mit Minderheitsanträgen, sondern auch zu den Artikeln, die von der Kommission in die Vorlage eingearbeitet wurden und zu denen kein Minderheitsantrag vorhanden ist. 
-Zuerst zum Antrag der Minderheit Aeschi zu Artikel 4 Absatz 2bis: Dieser Antrag wurde in der Abstimmung in der Kommission mit 16 zu 8 Stimmen abgelehnt. Demnach soll der Zugang zur elektronischen Kommunikation Personen verwehrt sein, welche </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich informiere Sie über die Diskussion in der Kommission, und zwar nicht nur zu den Artikeln mit Minderheitsanträgen, sondern auch zu den Artikeln, die von der Kommission in die Vorlage eingearbeitet wurden und zu denen kein Minderheitsantrag vorhanden ist. 
-Zuerst zum Antrag der Minderheit Aeschi zu Artikel 4 Absatz 2bis: Dieser Antrag wurde in der Abstimmung in der Kommission mit 16 zu 8 Stimmen abgelehnt. Demnach soll der Zugang zur elektronischen Kommunikation Personen verwehrt sein, welche keinen gültigen Aufenthaltsstatus in der Schweiz haben. Die Mehrheit der Kommission ist der Meinung, dass die Verankerung einer solchen Zugangsbeschränkung im Spezialgesetz BISS systemfremd ist. Weder die Zentrale Ausgleichsstelle noch die Durchführungsstellen sind die richtigen Ansprechpartner für den Abgleich des ausländerrechtlichen Status.
-Tatsächlich gibt es Menschen in der Schweiz, welche trotz illegalem Aufenthalt eine AHV-Nummer haben. Grundgedanke der Minderheit war, dass kein Zugang zu Leistungen möglich ist, wenn jemand im Status eines illegalen Aufenthalts hier ist. Da die Versicherten aber die Daten weiterhin auch analog bestellen können, wäre diese Einschränkung des elektronischen Zugriffs nicht wirkungsvoll. Für die Kommissionsmehrheit stand zudem der digitale Austausch im Zentrum und nicht die Prüfung des rechtlichen Aufenthaltsstatus. 
-Zu Artikel 5 Buchstabe abis: Dort ist zwar kein Minderheitsantrag vorhanden, aber ich mache dennoch kurz eine Erläuterung: Die Kommission hat da eingearbeitet, dass den versicherten Personen jährlich automatisch ein einfach verständlicher Auszug aus dem individuellen Konto der AHV zur Verfügung gestellt wird. Sie haben es gehört: Er soll jährlich und automatisch erfolgen und verständlich sein. Es liegt in der Handlungskompetenz des Bundesrates bzw. der Zentralen Ausgleichsstelle, wie das gemacht wird. Gedacht ist, dass alle Versicherten erfahren können, ob sie Beitragslücken haben, und diese gegebenenfalls schnell schliessen können. Dass diese Information zur Verfügung gestellt wird, erscheint der Kommission wichtig. 
-Ich komme zu Artikel 22a, zum Steuerungs- und Mitwirkungsgremium: Dort gibt es einen Antrag der Minderheit de Courten. Der entsprechende Antrag wurde in der Kommission mit 17 zu 8 Stimmen abgelehnt. Bei Artikel 22a wird von der Mehrheit der Umstand berücksichtigt, dass bisher noch zu unklar ist, wer beim BSV, bei der ZAS und bei den Durchführungsstellen genau welche Verantwortung hat. Deshalb will die Kommissionsmehrheit unter dem Abschnitt "Governancebestimmungen" das Steuerungs- und Mitwirkungsgremium verankern, dessen Zusammensetzung benennen und auch dessen Aufgaben aufführen. Sie will diese Massnahme auch aufgrund der Vernehmlassung und den Anhörungen einführen, bei welchen diese als notwendig erachtet wurde. 
-Bei Artikel 22b wurde der entsprechende Antrag der Minderheit de Courten mit 17 zu 8 Stimmen abgelehnt.
-Wie ich bei der Vorstellung des Geschäfts angetönt habe, hat die Kommission auch Punkte aus dem Bericht der Eidgenössischen Finanzkontrolle aufgenommen. Dort wurde reklamiert, dass bei den Durchführungsstellen grosse Intransparenz über die Kosten, einschliesslich der IT-Kosten, herrsche. Deshalb sollen gemäss Mehrheit neu die Verwaltungskosten nach einheitlichem Standard erfasst und ausgewiesen werden. Ergänzend dazu sollen auch Vorgaben zur Standardisierung der Schnittstellen und zur Interoperabilität gemacht werden. Damit werden Datenaustausch, Anbindung der Systeme, Effizienzgewinne und Transparenz möglich. 
-In den Artikeln 37a bis 37c geht es um die Änderung anderer Erlasse, konkret um das ASTG. Dort ist auch kein Minderheitsantrag vorhanden. Es geht um die elektronische Kommunikation der Versicherungen untereinander und mit den Versicherten. Artikel 37a hält die Anforderungen an die Plattform für die elektronische Kommunikation, welche die Versicherungen anbieten müssen, fest.
-Auch zu Artikel 49 Absatz 1bis ist kein Minderheitsantrag vorhanden, aber die Kommission hat hier eine Ergänzung beschlossen. Es geht hier um Verfügungen, welche der Versicherungsträger, zum Beispiel die AHV, IV oder die Militärversicherung (MV), schriftlich erlässt. Da sollen Medienbrüche verhindern werden. Konkret sollen diese Verfügungen der Sozialversicherungen auch elektronisch übermittelt werden können, wenn entweder die Pflicht zur elektronischen Kommunikation besteht oder diese verlangt wird. Gemäss Artikel 37c BISS hat die versicherte Person die Möglichkeit, die elektronische Kommunikation zu verlangen.
-Letztlich informiere ich Sie über die Minderheit Rechsteiner Thomas, übernommen von Hess Lorenz, welche erstmals bei Artikel 50a Absatz 1 Buchstabe b1 AHVG erwähnt wird. Der ursprüngliche Antrag in der Kommission wurde mit 16 zu 8 Stimmen abgelehnt. Die Mehrheit der Kommission will die automatische und vollständige Datenbekanntgabe zwischen AHV, IV, Unfallversicherung und Militärversicherung für die Koordination von Leistungen, die Abklärung der Versicherungspflicht, das Festsetzen der Versicherungspflicht, der Versicherungsprämien oder der Renten nicht ermöglichen. Gemäss der Minderheit ist diese gesetzliche Grundlage notwendig, damit der Austausch möglich ist, da heute die Datenanfrage in dieser Sache einzelfallweise und jeweils mit Begründung erfolgen muss und damit sehr aufwendig ist. Dieser Automatismus ist für die Kommissionsmehrheit aufgrund von Datenschutzbestimmungen noch nicht angebracht.
-Ihre Kommission hat dem BISS sowie den Änderungen im ATSG in der Gesamtabstimmung mit 17 zu 7 Stimmen zugestimmt. Gleichzeitig hat die Kommission auch der Abschreibung von zwei Motionen zugestimmt. Das ist einerseits die Motion 23.4041, "Sozialversicherung. Umfassende und einheitliche Rechtsgrundlage für das elektronische Verfahren schaffen (eATSG)" - BISS ist nun quasi die Umsetzung davon -, andererseits meine Motion 23.4435, "AHV endlich digitalisieren". Aus diesen Gründen bitte ich Sie im Namen der Kommission, die Mehrheitsanträge zu unterstützen, die beiden Motionen abzuschreiben und das Geschäft in der Schlussabstimmung anzunehmen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373974</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baume-Schneider Elisabeth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dans le cadre du traitement du présent projet de loi, plusieurs questions critiques ont été soulevées - je dois bien le dire - de manière légitime. Elles ont été débattues en commission et je peux vous assurer que pour le présent projet de loi un certain nombre de critiques a été pris en considération. 
-Premièrement, pourquoi une nouvelle loi ? Cet aspect a été discuté, débattu et critiqué lors de la consultation aussi bien par les cantons - cela a été dit - que par les organes d'exécution. Je p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dans le cadre du traitement du présent projet de loi, plusieurs questions critiques ont été soulevées - je dois bien le dire - de manière légitime. Elles ont été débattues en commission et je peux vous assurer que pour le présent projet de loi un certain nombre de critiques a été pris en considération. 
-Premièrement, pourquoi une nouvelle loi ? Cet aspect a été discuté, débattu et critiqué lors de la consultation aussi bien par les cantons - cela a été dit - que par les organes d'exécution. Je peux véritablement désormais affirmer que nous avons abordé et examiné de manière approfondie cette question, qui était légitime et nécessaire. Si la plateforme était intégrée dans la LPGA, elle devrait être utilisée par toutes les assurances sociales, y compris les assureurs maladie et - cela a été dit - possiblement par des assureurs privés, ce qui serait complexe. À l'inverse, l'absence de loi spécifique impliquerait d'introduire des références complexes et peu lisibles dans toutes les lois spéciales du premier pilier. 
-La minorité Aeschi demande le renvoi du projet en argumentant qu'une plateforme électronique décentralisée permettrait d'aboutir à une solution plus efficace et moins coûteuse. Néanmoins, le projet prend en considération les enseignements tirés d'autres projets numériques, notamment du dossier électronique du patient. Certaines solutions techniques doivent être gérées de manière centralisée, afin que l'ensemble des assurés, indépendamment de leur lieu de résidence ou encore indépendamment de leur employeur, disposent du même accès à leurs données. La plateforme centrale proposée constitue donc un élément clé du projet.
-Die Idee einer zentralen Plattform beim Bund löst bei den Durchführungsstellen teilweise Ängste aus. Klar ist jedoch, dass das Projekt nicht auf eine Zentralisierung der ersten Säule abzielt. Die dezentrale föderale Organisation der ersten Säule funktioniert gut und soll nicht infrage gestellt werden. Sie muss aber modernisiert werden, um mit den technologischen Entwicklungen Schritt zu halten. Weder das neue Gesetz noch die elektronische Plattform ersetzen zudem die bestehenden IT-Systeme der IV-Stellen und AHV-Ausgleichskassen.
-Ces dernières années, les assurances sociales, comme l'AVS, l'AI ou le régime des APG, ont numérisé un certain nombre de leurs processus. Toutefois, la communication électronique reste encore insuffisante et insuffisamment automatisée et standardisée aujourd'hui. La nouvelle loi fédérale sur les systèmes d'information des assurances (LSIAS) représente ainsi une avancée majeure dans la stratégie numérique de la Confédération et elle fait progresser la numérisation du premier pilier.
-La majorité de votre commission partage cette appréciation et propose ainsi l'entrée en matière sur le projet, par 16 voix contre 8. Une minorité de Courten demande de ne pas entrer en matière, alors qu'une minorité de Aeschi demande le renvoi du projet au Conseil fédéral afin de prendre en considération les demandes des cantons et des caisses cantonales de compensation. La LSIAS crée le cadre nécessaire pour une communication électronique sécurisée et efficace pour l'exécution des assurances sociales du premier pilier. Au coeur du projet figure donc la mise en place d'une plateforme électronique centrale qui est destinée aux offices AI, aux caisses de compensation AVS, aux autres instances administratives - on peut penser aux assurances-accidents ou encore aux services cantonaux des impôts - et surtout et en premier lieu aux assurés, c'est-à-dire à l'ensemble de la population.
-Für die Versicherten bietet die Plattform einen einfachen, sicheren und direkten Zugang zu ihren Daten der ersten Säule. Sie wird von der Zentralen Ausgleichsstelle verwaltet und ermöglicht es, eine automatisierte Simulation ihrer AHV-Rente durchzuführen; denn nur gut informierte Personen können fundierte Entscheidungen treffen.
-Les bénéficiaires de prestations AI ou encore d'allocations pour perte de gains pourront également disposer de la plateforme pour déposer des demandes de remboursement directement en ligne avec un traitement plus rapide. La plateforme permettra enfin aux autorités de transmettre en toute sécurité des documents tels que des décisions et des factures.
-Outre les dispositions prévues dans la LSIAS, le projet prévoit également des modifications de la loi fédérale sur la partie générale du droit des assurances sociales (LPGA). La plus importante concerne la communication électronique. L'ensemble des assurances sociales relevant de la LPGA, donc également l'assurance-chômage, l'assurance-maladie, l'assurance-accidents, seront tenues de communiquer entre elles par voie électronique. Les assurés resteront quant à eux libres de choisir. Ils pourront donc utiliser la nouvelle offre numérique ou alors continuer à échanger avec leur assurance par voie postale.
-Le projet présente également un potentiel d'économies, car il réduit les coûts administratifs grâce à la communication électronique. En effet, aujourd'hui, les fonds de compensation de l'AVS, de l'AI et des APG consacrent chaque année 25 millions de francs en frais postaux, auxquels s'ajoutent environ 10 millions pour couvrir les frais d'administration. Une partie de ces coûts pourra dès lors être économisée.
-Cela a été mentionné également, l'audit de la transformation numérique du premier pilier, réalisé par le Contrôle fédéral des finances, a été critique, disons-le de manière transparente. Je cite un élément qu'il a mentionné ; il parle effectivement de la nécessité de numérisation, en mentionnant qu'elle "ne pourra aboutir que si tous les acteurs concernés, et plus particulièrement l'OFAS et les organes d'exécution, coordonnent leur action dans un esprit de coopération." Grâce aux travaux en commission, cette coopération a été non seulement abordée, mais inscrite désormais dans la loi.
-En conclusion, le projet constitue une étape importante pour la modernisation du premier pilier. Il améliore l'accès des assurés à leurs informations. Ces informations leur appartiennent. Il simplifie également la communication entre les institutions et il rend l'exécution des assurances sociales plus efficace.
-Dès lors, je vous remercie de suivre la majorité, d'entrer en matière et de rejeter les propositions de minorité de Courten et Aeschi.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373986</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La commission a donc examiné de manière approfondie le projet de loi et les discussions ont permis d'aboutir à des adaptations qui permettent d'améliorer l'efficacité et la portée de la plateforme, ainsi que de la numérisation du premier pilier. Néanmoins, je vous proposerai de rejeter les différentes minorités.
-Premièrement, la minorité Aeschi prévoit que les personnes sans statut de séjour valable en Suisse n'auront pas accès à la plateforme. Or, il est important de le préciser : la plateforme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La commission a donc examiné de manière approfondie le projet de loi et les discussions ont permis d'aboutir à des adaptations qui permettent d'améliorer l'efficacité et la portée de la plateforme, ainsi que de la numérisation du premier pilier. Néanmoins, je vous proposerai de rejeter les différentes minorités.
-Premièrement, la minorité Aeschi prévoit que les personnes sans statut de séjour valable en Suisse n'auront pas accès à la plateforme. Or, il est important de le préciser : la plateforme centrale est conçue comme une plateforme purement informative, qui ne crée aucun droit à des prestations. Avec la plateforme, il est uniquement prévu de donner aux assurés un accès numérique facilité à leurs données de prévoyance. L'accès est d'ailleurs déjà limité. Il nécessite une identification par le biais d'une identité électronique reconnue, par exemple le numéro AVS. Dès lors, n'auront accès à la plateforme que les personnes qui ont ou qui avaient une assurance sociale en Suisse. Si ces conditions sont remplies, il est pratiquement impossible, d'un point de vue technique, d'en empêcher l'accès. De plus, la plateforme n'est pas le seul moyen d'accéder aux données de prévoyance ; la personne peut y accéder par le biais des caisses de compensation ou des offices AI cantonaux.
-Pour ces raisons, je vous invite à suivre la majorité et à rejeter la minorité Aeschi.
-Une minorité de Courten propose en outre de renoncer à créer un organe de pilotage et de participation pour les systèmes d'information à l'échelle nationale. Toutefois, la numérisation du premier pilier ne peut fonctionner que si la Confédération, c'est-à-dire l'OFAS et la Centrale de compensation, collabore étroitement et de manière durable avec les organes d'exécution, notamment dans le cadre d'instances communes. Dans ce contexte, des travaux sont en cours afin de clarifier et de préciser, avec l'ensemble des acteurs, les rôles, les compétences et les mécanismes de décision. C'est extrêmement important pour aboutir à des systèmes non seulement qui fonctionnent, mais qui créent aussi de la confiance.
-La disposition proposée par la majorité vise donc à inscrire cette collaboration dans la loi et à lui donner un cadre contraignant bienvenu. Elle correspond en outre à la recommandation formulée dans le rapport du Contrôle fédéral des finances sur la numérisation dans le premier pilier.
-Je vous invite dès lors à suivre la majorité de la commission et à rejeter la proposition de minorité de Courten.
-Une autre minorité de Courten vise, quant à elle, la suppression des règles relatives à la transparence des coûts ainsi qu'à la standardisation et à l'interopérabilité des systèmes d'information. Il s'agit toutefois de conditions essentielles, là aussi, pour que la Confédération puisse exercer efficacement sa fonction de pilotage, mais aussi sa fonction de surveillance. Le Contrôle fédéral des finances a d'ailleurs invité l'OFAS à utiliser de manière plus systématique ces instruments de pilotage existants, notamment en ce qui concerne les coûts informatiques. Là aussi, je vous invite à suivre la majorité de votre commission.
-Enfin, la minorité Rechsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
-Das Anliegen ist nachvollziehbar. Der Antrag der Minderheit würde jedoch unserer Meinung nach zu weit gehen. Es würde der Militär- und der Unfallversicherung Zugang zu allen Daten der ersten Säule gewähren. Wir dürfen nicht vergessen, dass es sich dabei teilweise um besonders sensible Daten handelt, insbesondere um Daten zur Gesundheit oder zur Invalidität. Das BSV hat in Zusammenarbeit mit den betroffenen Versichern ein Projekt lanciert. Ziel ist es, die Datenflüsse zu analysieren und die notwendigen rechtlichen Grundlagen zu klären, um einen gezielten und nachvollziehbaren Datenaustausch zu ermöglichen.
-Cependant, nous l'avons indiqué en commission, ce projet de discussions n'est pas encore suffisamment avancé à l'heure actuelle. J'ai demandé à l'OFAS de mettre la priorité sur ces discussions. Je crois que tout le monde est intéressé à clarifier la nature des données à transmettre pour faciliter et favoriser le travail de concertation entre les assurances, mais aussi pour aller en faveur des assurés. L'objectif est de pouvoir présenter une disposition correspondante, donc d'être pragmatique, en faisant une proposition au Conseil des États.
-Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Rechsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piller Carrard Valérie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notre commission s'est penchée sur les différents articles qui composent ce projet de loi. Nous avons apporté plusieurs adaptations, acceptées à l'unanimité, afin de préciser certains éléments, notamment la collaboration entre l'administration, la Centrale de compensation et les organes d'exécution, comme à l'article 4 alinéa 2ter et à l'article 18, mais aussi pour apporter plus de sécurité juridique dans la gestion des canaux pour permettre des transferts de données de système d'information à s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notre commission s'est penchée sur les différents articles qui composent ce projet de loi. Nous avons apporté plusieurs adaptations, acceptées à l'unanimité, afin de préciser certains éléments, notamment la collaboration entre l'administration, la Centrale de compensation et les organes d'exécution, comme à l'article 4 alinéa 2ter et à l'article 18, mais aussi pour apporter plus de sécurité juridique dans la gestion des canaux pour permettre des transferts de données de système d'information à système d'information, comme à l'article 37a alinéa 2, lettres a, b et c, ou encore à l'article 49, où nous avons modifié l'alinéa 1bis afin de clarifier la communication de décisions qui peuvent être notifiées valablement par voie électronique non seulement aux personnes assurées, mais aussi à l'ensemble des parties, notamment les employeurs.
-En ce qui concerne les différentes propositions de minorité, à l'article 4 alinéa 2bis, la minorité Aeschi propose que l'accès à la plateforme ne soit pas accordé aux personnes résidant en Suisse sans statut de séjour valable. La commission a rejeté cette proposition, par 16 voix contre 8. Elle estime que l'instauration d'une telle restriction d'accès serait contraire au fonctionnement du système, qui est conçu comme une plateforme purement informative. Cette loi ne crée donc aucun droit à des prestations, mais rend simplement transparentes et accessibles les informations qui existent déjà. Aussi, les caisses de compensation ne sont pas les instances compétentes pour vérifier le statut au regard du droit des étrangers. Cette tâche relève de la compétence d'autres autorités.
-Pour ce qui est des propositions de minorité de biffer les articles 22a et 22b, ces deux articles s'inscrivent directement dans les conclusions du rapport du Contrôle fédéral des finances "Audit de la transformation numérique du 1er pilier" qui nous a été présenté en commission en février dernier. Dans ce rapport, plusieurs recommandations avaient été émises, notamment sur la gouvernance qui n'était pas suffisamment claire et sur le manque de transparence en matière de coûts. C'est pourquoi la majorité de la commission propose, à l'article 22a, que l'OFAS mette en place un organe de pilotage permanent à l'échelle nationale pour les systèmes d'information régis par la LSIAS, avec la participation des organismes d'exécution. Cet organe devra notamment définir les normes nationales, les modalités de mise en oeuvre et prioriser les projets.
-À l'article 22b, nous avons intégré les aspects de la transparence, de la standardisation et de l'obligation de rendre compte ; éléments qui faisaient défaut à ce projet de loi. Nous devons disposer en effet de données comparables et saisies uniformément, afin d'identifier les fausses incitations économiques. Il est donc essentiel que l'OFAS collecte ces données et les rende publiques.
-Nous vous invitons donc, pour ces deux articles, à soutenir les propositions de la majorité de la commission, qui ont été acceptées par 17 voix contre 8, et qui sont également soutenues par le Conseil fédéral.
-Concernant la minorité Rechsteiner Thomas à l'article 50a de la loi sur l'AVS, à l'article 97 de la loi sur l'assurance-accidents et à l'article 95a de la loi sur l'assurance militaire, cette proposition de minorité est un concept concernant la communication de données entre les différentes assurances mentionnées en vue de la coordination des prestations, de la détermination de l'assujettissement à l'assurance, de la fixation des primes d'assurance ou de la rente. Pour la minorité, c'est la seule façon d'assurer une communication électronique fluide et sans rupture de média. Pour que cela soit conforme à la loi sur la protection des données, il faut un ancrage légal. La majorité de la commission, qui, d'après ce que j'ai pu entendre, aurait évolué, ne souhaite pas pour le moment donner une carte blanche aux transferts de données, notamment du point de vue de la protection des données. Avec cette proposition de minorité, nous donnons à l'assurance-accidents un accès à l'ensemble des données du premier pilier.
-Pour réglementer cela de manière plus précise, il faudrait clarifier dans la loi quelles données sont transmises grâce à une cartographie des flux de données. Comme expliqué en commission par l'administration, l'examen actuel des flux de données avec les assureurs-accidents et l'assurance militaire prend un certain temps, mais ce délai pourrait suffire pour préciser les flux de données avant l'examen en deuxième lecture. Il vaut donc la peine, dans l'intérêt de la qualité de la loi, d'attendre la cartographie des flux de données, puis de procéder aux adaptations légales nécessaires. Nous avons par conséquent refusé cette proposition de minorité Rechsteiner Thomas, par 16 voix contre 8.
+    <t xml:space="preserve">GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
+Il disavanzo del bilancio straordinario è dovuto soprattutto ai contributi versati ai Cantoni per le persone con statuto di protezione S provenienti dall'Ucraina, 700 milioni, e al contributo unico alle FFS, 850 milioni, compensati in parte da entrate straordinarie della Banca nazionale svizzera.
+L'avanzo dell'amministrazione ordinaria raggiunge 1,2 miliardi di franchi, mentre la regola del freno all'indebitamento avrebbe consentito un deficit di 262 milioni di franchi. Ne risulta quindi un saldo strutturale positivo di 1,4 miliardi, nettamente superiore al valore previsto nel preventivo.
+Le entrate ordinarie superano il budget di 1,9 miliardi e il risultato dell'anno precedente di ben 3,3 miliardi. La crescita è dovuta soprattutto all'imposta federale diretta sulle imprese, che beneficia delle entrate temporanee dal Cantone di Ginevra per circa 1,5 miliardi di franchi.
+Anche l'imposta federale diretta sui redditi aumenta di 0,5 miliardi, mentre l'IVA aumenta di 700 milioni, grazie alla crescita dell'economia nominale e all'effetto ritardato dell'aumento dell'aliquota dal 2024. Le entrate dell'imposta preventiva, invece, risultano inferiori alle attese.
+Le spese totali sono aumentate del 4 percento e ammontano a 87,6 miliardi di franchi. 
+I principali aumenti riguardano la previdenza sociale, le finanze e imposte, i trasporti, l'istruzione e la ricerca e l'esercito.
+Nel 2025 il numero di posti nella Confederazione è cresciuto di 240 unità, più 0,6 per cento, mentre le spese per il personale sono aumentate di 79 milioni di franchi, soprattutto per il rincaro dell'1 per cento.
+Il debito netto scende leggermente a 140 miliardi di franchi. Il conto di ammortamento del debito Covid si riduce per la prima volta di circa 500 milioni, grazie al saldo strutturale positivo e alle entrate straordinarie, e ammonta a 26,3 miliardi di franchi. Il conto di compensazione rimane stabile a circa 20 miliardi di franchi.
+Nella seduta dell'11 e 12 maggio 2026, la commissione ha proceduto all'esame di dettaglio del consuntivo. Le sue quattro sottocommissioni hanno presentato le conclusioni delle rispettive analisi approfondite dei consuntivi dei singoli servizi federali realizzate nel corso del mese di aprile.
+Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla sua commissione i risultati delle tre verifiche relative al Consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del Fondo per l'infrastruttura ferroviaria e quella del Fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
+Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del Fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma ancora irrisolte. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
+Il Controllo federale delle finanze conferma che il consuntivo rispetta le prescrizioni legali e le regole del freno all'indebitamento previste dall'articolo 126 della Costituzione federale. Per questo motivo raccomanda all'Assemblea federale di approvare il conto annuale.
+Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
+La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
+Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
 </t>
   </si>
 </sst>
@@ -240,8 +192,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -608,27 +560,27 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -637,105 +589,22 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5"/>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
         <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6"/>
-      <c r="F6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-06-03
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -144,6 +144,73 @@
 Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
 La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
 Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jauslin Matthias Samuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen Halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
+Die GLP steht für Freiheit, Eigenverantwortung, Innovation und einen starken Rechtsstaat ein. Gerade deshalb unterstützen wir die Revision des Nachrichtendienstgesetzes. Freiheit und Sicherheit sind keine Gegensätze. Freiheit kann nur dort bestehen, wo Menschen sicher leben können, wo demokratische Institutionen geschützt werden und wo der Staat seine grundlegenden Funktionen wahrnehmen kann. Der Staat muss in der Lage sein, Bedrohungen frühzeitig zu erkennen und angemessen darauf zu reagieren.
+Die geopolitische Lage hat sich in den vergangenen Jahren deutlich verschärft. Spätestens seit dem russischen Angriffskrieg gegen die Ukraine ist klar geworden, dass Europa wieder verstärkt im Fokus nachrichtendienstlicher und hybrider Operationen steht. Die Schweiz bildet dabei keine Ausnahme, im Gegenteil: Als international vernetzter Wirtschafts-, Forschungs- und Diplomatiestandort ist sie besonders exponiert. Fremde Nachrichtendienste nutzen die Schweiz als Operationsraum, während gleichzeitig unsere Unternehmen, Hochschulen und Forschungsinstitutionen vermehrt Ziel von Spionageversuchen werden. Wer glaubt, die Schweiz könne sich diesen Entwicklungen entziehen, verkennt die Realität.
+Das angepasste Gesetz schafft die Voraussetzungen dafür, dass der Nachrichtendienst seinen Auftrag auch unter den Bedingungen des digitalen Zeitalters erfüllen kann. Kriminelle und feindliche Akteure nutzen verschlüsselte Kommunikationskanäle, globale Datennetze und moderne Technologien. Ein Nachrichtendienst, der auf Instrumenten des letzten Jahrhunderts basiert, kann diesen Herausforderungen nicht wirksam begegnen. Wer von den Sicherheitsbehörden erwartet, dass sie Gefahren erkennen und verhindern, muss ihnen auch die dafür notwendigen Mittel und Tools zur Verfügung stellen.
+Die Erfahrungen der letzten Jahre haben gezeigt, dass Radikalisierung häufig lange vor einer konkreten Tat sichtbar wird. Sicherheitsbehörden müssen deshalb die Möglichkeit haben, verdächtige Entwicklungen rechtzeitig zu erkennen und Risiken zu beurteilen. Es geht nicht darum, Menschen unter Generalverdacht zu stellen. Es geht darum, konkrete Gefahren frühzeitig zu erkennen.
+Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
+Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
+Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu diesem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wichtig sind auch klare Datenschutzgarantien im Gesetz - insbesondere, wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
+Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
+Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
+Für die GLP ist entscheidend, dass Sicherheit nicht auf Kosten der Freiheit erreicht wird. Die vorliegende Revision ermöglicht eine ausgewogene Balance zwischen wirksamer Gefahrenabwehr und dem Schutz der Grundrechte. Sie stärkt die Handlungsfähigkeit des Staates dort, wo dies notwendig ist, und setzt gleichzeitig klare Grenzen.
+Aus diesen Gründen tritt die GLP-Fraktion auf die Vorlage ein.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addor Jean-Luc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été : dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
+Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front - heureusement d'ailleurs - et les optimistes peuvent donc croire que "ça n'arrivera jamais". Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux ? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
+Le SRC, dans ce pays où l'on n'a pas la culture du renseignement, où l'on se méfie de toute zone grise, doit régater avec des homologues étrangers qui, eux, sont depuis longtemps sur le pied de guerre, et il doit le faire avec des moyens dramatiquement insuffisants et des procédures dont la lourdeur excessive fait parfois que certaines opérations nécessaires et urgentes sont simplement impossibles à mener.
+Pouvons-nous nous payer encore longtemps ce luxe de beau temps ? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
+Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission ? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
+La commission propose à son conseil d'apporter des modifications au projet de loi sur un certain nombre de points. J'en cite quelques-uns. D'abord, une extension des tâches du SRC en matière de recherche d'informations est nécessaire afin de couvrir également les activités d'influence du fait d'États étrangers dirigées contre l'ordre démocratique, le fonctionnement de l'État ou de la société. Il faut également étendre, en particulier, les compétences du service aux évènements relevant de la politique de sécurité qui se produisent dans le cyberespace. Le cyberespace est une notion que la commission a souhaité définir plus précisément en reprenant la formulation figurant dans la cyberstratégie nationale. Afin de rendre la lutte contre le financement du terrorisme et l'espionnage plus efficace, la commission préconise que le SRC puisse, en cas de graves menaces, collecter également des données auprès d'intermédiaires financiers et de négociants au moyen de mesures de recherche soumises à autorisation. Elle propose néanmoins que les conditions de cette obligation de fournir des renseignements soient définies plus clairement dans la loi fédérale sur le renseignement, sur la base des dispositions de la loi sur le blanchiment d'argent, afin de garantir la sécurité du droit.
+La commission estime en outre justifié qu'en cas d'urgence, le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif : si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
+La commission souhaite renforcer davantage la collaboration intercantonale et, dans ce sens, elle propose que les autorités d'exécution cantonales aient l'obligation de s'accorder réciproquement un accès en ligne aux données qu'elles ont obtenues sur la base de la loi sur le renseignement. La commission juge en effet insuffisant l'accès seulement facultatif que propose le Conseil fédéral. Par ailleurs, la commission demande que les services de renseignement cantonaux puissent également transmettre, avec l'accord du SRC, des données qu'ils ont reçues de celui-ci aux polices cantonales dans le cadre de mandats précis.
+La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances. - On voit déjà que c'est simple ! Je m'arrête deux secondes ici : c'est peut-être un objet de réflexion. - Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
+La commission a rejeté toutes les autres propositions d'amendement. À cet égard, le débat s'est cristallisé, entre autres, sur les points qui sont énumérés dans la seconde minorité Chollet, celle qui demande un renvoi du projet au Conseil fédéral.
+Il a d'abord été question de la problématique - je ne dirais pas "phare", mais enfin elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
+Sur ce point, la majorité de la commission, avec le Conseil fédéral d'ailleurs, considère que les dispositions proposées dans ce projet sont conformes à notre ordre juridique, tout en fournissant au SRC les compétences supplémentaires dont celui-ci a besoin pour notre sécurité.
+Un autre élément qui a suscité certains débats : ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, de ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
+Au bilan, la question se pose de savoir si, avec la révision telle que proposée par la commission, qui tient dans un volumineux document de 205 pages, nous aurons simplifié suffisamment les procédures pour garantir au SRC l'efficacité que les décideurs de ce pays attendent de lui, cela dans le respect de la sphère privée des citoyens - c'est évidemment un défi. La question lancinante des effectifs du SRC reste en outre sans la moindre réponse en ces temps d'allègements budgétaires.
+Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
 </sst>
@@ -192,8 +259,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -607,6 +674,64 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-08
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -303,6 +303,31 @@
 Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">375897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260608</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moser Tiana Angelina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
+Die Resolution verdient eine besondere Aufmerksamkeit. Sie stammt nicht nur von einzelnen Organisationen, sondern von denjenigen, die die Folgen der PFAS-Belastung im Interesse und zum Schutz der Bevölkerung bewältigen müssen. Die Brunnenmeister beispielsweise sind zuständig für die Sicherung der Wasserqualität und die Versorgung der Bevölkerung. 
+PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
+Vor diesem Hintergrund ist die Stellungnahme des Bundesrates zu Frage 2 meiner Interpellation besonders bemerkenswert. Der Bundesrat anerkennt ausdrücklich den Nutzen des Human Biomonitoring für die Erfassung der Belastung der Bevölkerung. Genau solche Daten bräuchten wir, um Risiken frühzeitig zu erkennen und entsprechende Entwicklungen zu verfolgen. Umso weniger verständlich ist es, dass ausgerechnet dieses Instrument aus Spargründen eingestellt worden ist. Die Kosten des Human Biomonitoring stehen in keinem Verhältnis zu den Folgekosten der PFAS-Belastung, die sich, Sie haben es gehört, im Milliardenbereich bewegen. Auf das Monitoring zu verzichten, heisst, auf Wissen zu verzichten, das helfen könnte, gesundheitliche Risiken frühzeitig zu erkennen und Schäden zu begrenzen. 
+Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind wie gesagt nur die Beispiele zum Gewässer. 
+Es ist offensichtlich, dass es sich hier um eine schweizweite Herausforderung handelt. Wir stehen bei der PFAS-Thematik erst am Anfang, und gerade deshalb können wir es uns nicht leisten, auf Wissen zu verzichten. Entsprechend wichtig wäre eine Wiederaufnahme des Human Biomonitoring im Rahmen des Aktionsplans zur Reduktion der Ewigkeitschemikalien. Diese Einschätzung wurde im Übrigen auch von der Eidgenössischen Finanzkontrolle 2024 geteilt. Gerade angesichts der gesundheitlichen Risiken und der möglichen Folgekosten sowie der grossen Wissenslücken wäre das eine sehr wichtige Aussage, um auch das Vertrauen der Bevölkerung zu steigern. 
+In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -349,8 +374,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -851,6 +876,35 @@
         <v>46</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-09
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -328,6 +328,27 @@
 In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">376183</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parmelin Guy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
+Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
+C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -374,8 +395,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I9"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -905,6 +926,33 @@
         <v>52</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-11
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -67,17 +67,15 @@
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
 Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
-Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019.
-Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
-Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken. Hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
+Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken - hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
 Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
 Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
-Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf.
-Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
+Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf. Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
 Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
 Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
 Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
@@ -104,8 +102,8 @@
     <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
 Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
-Das ist Steuersubventionitis, eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
-Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Sätze, Befreiungen oder Abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Das ist "Steuersubventionitis", eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte -sätze, -befreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
 Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
 </t>
   </si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-14
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -63,23 +63,26 @@
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Depar</t>
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20.[NB]Februar 2026 darüber orientiert. Am 20.[NB]März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die</t>
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20.[NB]Februar 2026 darüber orientiert. Am 20.[NB]März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11.[NB]und 12.[NB]Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
 Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
-Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
-Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken - hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
-Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
-Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. 
+Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. Budgetiert war ursprünglich ein nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. 
+Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken, hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie wegen des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
+Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent; dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39[NB]202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
 Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf. Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
-Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
+Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. 
+Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
 Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
 Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
-Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
+Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. 
+Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-15
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -72,7 +72,7 @@
 Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. 
 Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. Budgetiert war ursprünglich ein nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. 
 Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken, hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie wegen des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
-Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
+Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundesgesetz über die direkte Bundessteuer, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
 Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent; dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39[NB]202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
@@ -98,16 +98,17 @@
     <t xml:space="preserve">ZH</t>
   </si>
   <si>
-    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "Steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Ei</t>
   </si>
   <si>
-    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "Steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
 Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
 Das ist "Steuersubventionitis", eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
-Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte -sätze, -befreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
-Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Steuersätze, Steuerbefreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. 
+Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
 </t>
   </si>
   <si>
@@ -287,21 +288,21 @@
     <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégique</t>
   </si>
   <si>
-    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été : dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
-Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front - heureusement d'ailleurs - et les optimistes peuvent donc croire que "ça n'arrivera jamais". Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux ? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été[NB]: dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
+Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front, heureusement, d'ailleurs, et les optimistes peuvent donc croire que ça n'arrivera jamais. Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours, d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux[NB]? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
 Le SRC, dans ce pays où l'on n'a pas la culture du renseignement, où l'on se méfie de toute zone grise, doit régater avec des homologues étrangers qui, eux, sont depuis longtemps sur le pied de guerre, et il doit le faire avec des moyens dramatiquement insuffisants et des procédures dont la lourdeur excessive fait parfois que certaines opérations nécessaires et urgentes sont simplement impossibles à mener.
-Pouvons-nous nous payer encore longtemps ce luxe de beau temps ? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
-Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission ? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
+Pouvons-nous nous payer encore longtemps ce luxe de beau temps[NB]? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
+Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission[NB]? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
 La commission propose à son conseil d'apporter des modifications au projet de loi sur un certain nombre de points. J'en cite quelques-uns. D'abord, une extension des tâches du SRC en matière de recherche d'informations est nécessaire afin de couvrir également les activités d'influence du fait d'États étrangers dirigées contre l'ordre démocratique, le fonctionnement de l'État ou de la société. Il faut également étendre, en particulier, les compétences du service aux évènements relevant de la politique de sécurité qui se produisent dans le cyberespace. Le cyberespace est une notion que la commission a souhaité définir plus précisément en reprenant la formulation figurant dans la cyberstratégie nationale. Afin de rendre la lutte contre le financement du terrorisme et l'espionnage plus efficace, la commission préconise que le SRC puisse, en cas de graves menaces, collecter également des données auprès d'intermédiaires financiers et de négociants au moyen de mesures de recherche soumises à autorisation. Elle propose néanmoins que les conditions de cette obligation de fournir des renseignements soient définies plus clairement dans la loi fédérale sur le renseignement, sur la base des dispositions de la loi sur le blanchiment d'argent, afin de garantir la sécurité du droit.
-La commission estime en outre justifié qu'en cas d'urgence, le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif : si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
+La commission estime en outre justifié qu'en cas d'urgence le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif[NB]: si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
 La commission souhaite renforcer davantage la collaboration intercantonale et, dans ce sens, elle propose que les autorités d'exécution cantonales aient l'obligation de s'accorder réciproquement un accès en ligne aux données qu'elles ont obtenues sur la base de la loi sur le renseignement. La commission juge en effet insuffisant l'accès seulement facultatif que propose le Conseil fédéral. Par ailleurs, la commission demande que les services de renseignement cantonaux puissent également transmettre, avec l'accord du SRC, des données qu'ils ont reçues de celui-ci aux polices cantonales dans le cadre de mandats précis.
-La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances. - On voit déjà que c'est simple ! Je m'arrête deux secondes ici : c'est peut-être un objet de réflexion. - Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
+La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances - on voit déjà que c'est simple[NB]; je m'arrête deux secondes ici, c'est peut-être un objet de réflexion. Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
 La commission a rejeté toutes les autres propositions d'amendement. À cet égard, le débat s'est cristallisé, entre autres, sur les points qui sont énumérés dans la seconde minorité Chollet, celle qui demande un renvoi du projet au Conseil fédéral.
-Il a d'abord été question de la problématique - je ne dirais pas "phare", mais enfin elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
+Il a d'abord été question de la problématique - je ne dirais pas "phare", mais, enfin, elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
 Sur ce point, la majorité de la commission, avec le Conseil fédéral d'ailleurs, considère que les dispositions proposées dans ce projet sont conformes à notre ordre juridique, tout en fournissant au SRC les compétences supplémentaires dont celui-ci a besoin pour notre sécurité.
-Un autre élément qui a suscité certains débats : ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, de ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
+Un autre élément qui a suscité certains débats[NB]: ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, que ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
 Au bilan, la question se pose de savoir si, avec la révision telle que proposée par la commission, qui tient dans un volumineux document de 205 pages, nous aurons simplifié suffisamment les procédures pour garantir au SRC l'efficacité que les décideurs de ce pays attendent de lui, cela dans le respect de la sphère privée des citoyens - c'est évidemment un défi. La question lancinante des effectifs du SRC reste en outre sans la moindre réponse en ces temps d'allègements budgétaires.
-Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
+Toujours est-il qu'avec 21 voix contre 4 la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
   <si>
@@ -348,6 +349,39 @@
     <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
 Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
 C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376778</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herzog Eva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Staatsrechnung 2025 des Bundes schliesst mit einem Finanzierungsüberschuss von 259 Millionen Franken. Sie fällt damit deutlich besser aus als erwartet; veranschlagt war ein Defizit von 815 Millionen Franken. Der negative ausserordentliche Finanzierungssaldo von 926 Millionen Franken wurde durch den positiven ordentlichen Finanzierungssaldo von 1,185 Milliarden Franken mehr als ausgeglichen. Dies ist vor allem auf temporär höhere Gewinnsteuereinnahmen aus dem Kanton Genf im Umfang von 1,5 Mil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Staatsrechnung 2025 des Bundes schliesst mit einem Finanzierungsüberschuss von 259 Millionen Franken. Sie fällt damit deutlich besser aus als erwartet; veranschlagt war ein Defizit von 815 Millionen Franken. Der negative ausserordentliche Finanzierungssaldo von 926 Millionen Franken wurde durch den positiven ordentlichen Finanzierungssaldo von 1,185 Milliarden Franken mehr als ausgeglichen. Dies ist vor allem auf temporär höhere Gewinnsteuereinnahmen aus dem Kanton Genf im Umfang von 1,5 Milliarden Franken zurückzuführen. 
+Die ordentlichen Einnahmen fielen insgesamt um 1,9 Milliarden Franken bzw. 2,2 Prozent höher aus als budgetiert und um 3,3 Milliarden Franken höher als im Vorjahr. Zugleich lagen die ordentlichen Ausgaben des Bundes 2025 erstmals seit der Einführung der Schuldenbremse im Jahr 2003 über dem Budgetwert. Dies ist unter anderem auf den Nachtragskredit für Horizon Europe zurückzuführen. Der ordentliche Finanzierungssaldo war positiv. Aus der Differenz ergibt sich ein struktureller Überschuss von 1,4 Milliarden Franken. In diesem Umfang war der ordentliche Finanzierungssaldo höher als von der Schuldenbremse vorgegeben. 
+Nennenswert sind im ausserordentlichen Haushalt die Mehreinnahmen aus der Zusatzausschüttung der Schweizerischen Nationalbank von 333 Millionen Franken und die budgetierte Sonderzuweisung der SNB aus den nicht ausgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Die beiden grössten Posten auf der Ausgabenseite sind die ausserordentlichen Ausgaben für die Schutzsuchenden aus der Ukraine sowie der einmalige Kapitalzuschuss an die SBB von 850 Millionen Franken, die ursprünglich für 2024 budgetiert waren.
+Weitere wichtige Kennzahlen: Erstmals seit der Corona-Pandemie konnte der Fehlbetrag des Amortisationskontos um 500 Millionen Franken reduziert werden. Neu beläuft sich der Fehlbetrag auf 26,3 Milliarden Franken. Das Ausgleichskonto hat unverändert einen positiven Stand von rund 20 Milliarden Franken. Die Nettoverschuldung hat 2025 leicht abgenommen und beträgt neu 140,1 Milliarden Franken. Die Nettoschuldenquote ging ebenfalls zurück, und zwar auf 16,1 Prozent des BIP. 
+Die Finanzkommission erhielt an ihrer Sitzung vom 26. Februar 2026 erste Informationen zum Ergebnis der Staatsrechnung. Anschliessend tagten die Subkommissionen. An der Sitzung vom 18. Mai 2026 hat die Finanzkommission die Rechnung 2025 und den Nachtrag I zum Voranschlag 2026 beraten. Im Gegensatz zur Einnahmenseite gab es auf der Ausgabenseite keine ausserordentlichen Vorkommnisse. Die Departemente sind daran, die beschlossenen Sparmassnahmen umzusetzen. Die Kommission hat zur Kenntnis genommen, dass die Digitalisierung allgemein vorangeht, aber nicht so schnell wie gewünscht, was auch an den Budgetkürzungen seitens des Parlamentes liegt. Weiter wurde berichtet, dass die erstinstanzlich hängigen Asylgesuche rückläufig sind. Ein Abbau der Gesuche war möglich, die Zahlen beim Bundesverwaltungsgericht sind aber weiter angestiegen. Die Verfahrensdauer ist nach wie vor weit weg von der ursprünglichen Zielsetzung im Rahmen der letzten Asylreform.
+Berichtet wurde über die ersten Gespräche mit dem neuen Leiter des Nachrichtendienstes des Bundes und über die höheren Ausgaben beim NDB.
+Thematisiert wurden ebenfalls die Probleme mit dem neuen Auszahlungssystem der Arbeitslosenkasse, Asalfutur. Die Kommission wurde darüber informiert, dass auf Ende März die Rückstände aufgeholt und alles ausbezahlt worden sei.
+Angesprochen wurde auch die Thematik, dass der Kapitalbezug der zweiten Säule nicht in den nationalen Finanzausgleich integriert ist. Die FK-S wird das Thema weiterverfolgen. 
+Informationen hat die Kommission auch erbeten bezüglich der Verhandlungen über die neue Vereinbarung mit der Schweizerischen Nationalbank. Auslöser waren die Aussagen des SNB-Präsidenten von Ende April in den Medien. Er sagte, dass für die SNB eine Eigenkapitalquote von 15 bis 20 Prozent zu tief sei. Aktuell sind es 19 Prozent. Eine Erhöhung würde bedeuten, dass statt einer Verbesserung sogar eine Verschlechterung gegenüber der heutigen Ausschüttungsvereinbarung drohen könnte, was in der Kommission kritisch gesehen wurde. Die Eidgenössische Finanzverwaltung erläuterte der Kommission die Rückstellungspolitik der SNB und bestätigte, dass sich die SNB eine Eigenkapitalquote zwischen 20 und 30 Prozent vorstelle, während andere Zentralbanken viel tiefere Werte hätten; so hätten beispielsweise die Fed oder die Bank of England eine Eigenkapitalquote von 1 Prozent, in Australien und Schweden sei das Eigenkapital negativ, in Singapur liege die Eigenkapitalquote bei 10 Prozent. Wenn die SNB mit ihrer Rückstellungspolitik tatsächlich dieses Ziel verfolge, müssten sich Bund und Kantone keine Hoffnungen auf höhere Ausschüttungen machen. Die Kommission wird das Thema weiterverfolgen, im Wissen, dass die Entscheide beim Bankrat angesiedelt sind. 
+Die Finanzministerin gab der Kommission auch einen Ausblick auf den Voranschlag 2027 und die kommenden Jahre.
+Nach Verabschiedung des EP 27 in beiden Räten ging der Bundesrat am 15. April noch von einem strukturellen Finanzierungsdefizit von 600 Millionen Franken aus und schlug erste mögliche Massnahmen zu dessen Bereinigung vor. An der Sitzung der FK-S vom 18. Mai konnte Bundesrätin Karin Keller-Sutter Entwarnung geben für den Voranschlag 2027, obwohl das Finanzdepartement für 2027 nochmals mit einer Verschlechterung um voraussichtlich rund 400 Millionen Franken rechnet, insbesondere aufgrund von Schätzkorrekturen bei den Sozialversicherungen und der Migration. Grund dafür sind deutliche Verbesserungen bei der Gewinnsteuer für juristische Personen, auch in anderen Kantonen als Genf. Zwar wies die Finanzministerin darauf hin, dass sich dieses ausserordentliche Wachstum auf einige wenige Unternehmen konzentriere. Sie sagte aber auch, dass die positive Entwicklung der Gewinnsteuern über diese Effekte hinaus breit abgestützt sei. Eine Mehrheit der Kantone habe Anfang Mai gemeldet, dass sie höhere Gewinnsteuereinnahmen hätten.
+Die Mehreinnahmen aus Genf waren hier ja schon mehrfach ein Thema, deshalb lediglich noch ein Wort zu ihrer Verbuchung. Die Eidgenössische Finanzkontrolle (EFK) hat verlangt, dass 1,5 Milliarden Franken schon im Jahr 2025 verbucht werden, ich habe diese eingangs erwähnt. 2026 sind es dann 1,3 Milliarden und 2027 noch 400 Millionen Franken. Es wäre auch denkbar gewesen, die Einnahmen über die Jahre zu glätten und kommende Budgets zu entlasten, doch die EFK bot nicht Hand dazu. So warnte die Finanzministerin auch bereits davor, dass die Lage angesichts der weiterhin bestehenden Herausforderungen, insbesondere bei der Armeefinanzierung und der AHV, ab 2028 wieder schwierig werden dürfte.
+Wenn keine zusätzlichen Einnahmen erschlossen werden könnten, würden ab 2028 beträchtliche strukturelle Defizite drohen. Ein Drittel der vom Bundesrat vorgesehenen Erhöhung der Mehrwertsteuer von 0,8 Prozent soll allein das bereits beschlossene Wachstum der Armee finanzieren, also den Aufwuchs auf 1 Prozent des BIP bis 2032. Der Bundesrat wird die Botschaft zur Armeefinanzierung nach der Sommerpause verabschieden. Neben der federführenden SiK wird sich auch die Finanzkommission in einem Mitbericht mit dem Geschäft befassen.
+Die Kommission tagte stets in Anwesenheit von Bundesrätin Karin Keller-Sutter und der Direktorin der Eidgenössischen Finanzverwaltung Sabine D'Amelio-Favez sowie weiteren Mitarbeiterinnen und Mitarbeitern des EFD, und sie tagte teilweise in Anwesenheit des Leiters der Finanzkontrolle Pascal Stirnimann und der zuständigen Mitarbeiterin. Ich danke den Beteiligten für ihre Begleitung unserer Diskussionen und für die guten Auskünfte.
+Nach Kenntnisnahme der Revisionsberichte der Eidgenössischen Finanzkontrolle sowie der Erwägungen und Schlussfolgerungen der Subkommissionen der FK-S beantragt die Kommission einstimmig, die Staatsrechnung 2025, die Sonderrechnungen für den Bahninfrastrukturfonds sowie den Nationalstrassen- und Agglomerationsverkehrsfonds, die Kreditüberschreitungen von 1,86 Milliarden Franken und die Bildung neuer Reserven in Höhe von 569 Millionen Franken zu genehmigen. Zum Schluss geht mein Dank an das Sekretariat der Finanzkommission für die umsichtige Vorbereitung, Organisation und Begleitung der Sitzungen.
 </t>
   </si>
 </sst>
@@ -396,8 +430,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I10"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -954,6 +988,35 @@
         <v>58</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-16
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -161,12 +161,12 @@
     <t xml:space="preserve">AG</t>
   </si>
   <si>
-    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
-Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
-Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen Halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass der Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass der Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
 Die GLP steht für Freiheit, Eigenverantwortung, Innovation und einen starken Rechtsstaat ein. Gerade deshalb unterstützen wir die Revision des Nachrichtendienstgesetzes. Freiheit und Sicherheit sind keine Gegensätze. Freiheit kann nur dort bestehen, wo Menschen sicher leben können, wo demokratische Institutionen geschützt werden und wo der Staat seine grundlegenden Funktionen wahrnehmen kann. Der Staat muss in der Lage sein, Bedrohungen frühzeitig zu erkennen und angemessen darauf zu reagieren.
 Die geopolitische Lage hat sich in den vergangenen Jahren deutlich verschärft. Spätestens seit dem russischen Angriffskrieg gegen die Ukraine ist klar geworden, dass Europa wieder verstärkt im Fokus nachrichtendienstlicher und hybrider Operationen steht. Die Schweiz bildet dabei keine Ausnahme, im Gegenteil: Als international vernetzter Wirtschafts-, Forschungs- und Diplomatiestandort ist sie besonders exponiert. Fremde Nachrichtendienste nutzen die Schweiz als Operationsraum, während gleichzeitig unsere Unternehmen, Hochschulen und Forschungsinstitutionen vermehrt Ziel von Spionageversuchen werden. Wer glaubt, die Schweiz könne sich diesen Entwicklungen entziehen, verkennt die Realität.
 Das angepasste Gesetz schafft die Voraussetzungen dafür, dass der Nachrichtendienst seinen Auftrag auch unter den Bedingungen des digitalen Zeitalters erfüllen kann. Kriminelle und feindliche Akteure nutzen verschlüsselte Kommunikationskanäle, globale Datennetze und moderne Technologien. Ein Nachrichtendienst, der auf Instrumenten des letzten Jahrhunderts basiert, kann diesen Herausforderungen nicht wirksam begegnen. Wer von den Sicherheitsbehörden erwartet, dass sie Gefahren erkennen und verhindern, muss ihnen auch die dafür notwendigen Mittel und Tools zur Verfügung stellen.
@@ -174,8 +174,8 @@
 Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
 Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
 Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
-Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu diesem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
-Wichtig sind auch klare Datenschutzgarantien im Gesetz - insbesondere, wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wichtig sind auch klare Datenschutzgarantien im Gesetz, insbesondere wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
 Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
 Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
 Für die GLP ist entscheidend, dass Sicherheit nicht auf Kosten der Freiheit erreicht wird. Die vorliegende Revision ermöglicht eine ausgewogene Balance zwischen wirksamer Gefahrenabwehr und dem Schutz der Grundrechte. Sie stärkt die Handlungsfähigkeit des Staates dort, wo dies notwendig ist, und setzt gleichzeitig klare Grenzen.
@@ -343,12 +343,12 @@
     <t xml:space="preserve">VD</t>
   </si>
   <si>
-    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
-Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
-C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que, compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que, compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
+Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés[NB]; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
+C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter. Il n'y en a pas beaucoup, mais, de temps en temps, il faut que les choses soient claires.
 </t>
   </si>
   <si>
@@ -382,6 +382,70 @@
 Wenn keine zusätzlichen Einnahmen erschlossen werden könnten, würden ab 2028 beträchtliche strukturelle Defizite drohen. Ein Drittel der vom Bundesrat vorgesehenen Erhöhung der Mehrwertsteuer von 0,8 Prozent soll allein das bereits beschlossene Wachstum der Armee finanzieren, also den Aufwuchs auf 1 Prozent des BIP bis 2032. Der Bundesrat wird die Botschaft zur Armeefinanzierung nach der Sommerpause verabschieden. Neben der federführenden SiK wird sich auch die Finanzkommission in einem Mitbericht mit dem Geschäft befassen.
 Die Kommission tagte stets in Anwesenheit von Bundesrätin Karin Keller-Sutter und der Direktorin der Eidgenössischen Finanzverwaltung Sabine D'Amelio-Favez sowie weiteren Mitarbeiterinnen und Mitarbeitern des EFD, und sie tagte teilweise in Anwesenheit des Leiters der Finanzkontrolle Pascal Stirnimann und der zuständigen Mitarbeiterin. Ich danke den Beteiligten für ihre Begleitung unserer Diskussionen und für die guten Auskünfte.
 Nach Kenntnisnahme der Revisionsberichte der Eidgenössischen Finanzkontrolle sowie der Erwägungen und Schlussfolgerungen der Subkommissionen der FK-S beantragt die Kommission einstimmig, die Staatsrechnung 2025, die Sonderrechnungen für den Bahninfrastrukturfonds sowie den Nationalstrassen- und Agglomerationsverkehrsfonds, die Kreditüberschreitungen von 1,86 Milliarden Franken und die Bildung neuer Reserven in Höhe von 569 Millionen Franken zu genehmigen. Zum Schluss geht mein Dank an das Sekretariat der Finanzkommission für die umsichtige Vorbereitung, Organisation und Begleitung der Sitzungen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377091</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260616</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weichelt Manuela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das vergangene Geschäftsjahr stand im Zeichen eines wichtigen rechtsstaatlichen Jubiläums: 150 Jahre Bundesgericht. Tragen wir Sorge zu unseren Errungenschaften. Respektieren wir die Gewaltenteilung und achten wir unsere Bundesverfassung sowie die Gesetze.
+Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden GPK haben ihre Aufsichtssitzung im April zum Geschäftsbericht traditionsgemäss in Lausanne am Bundesgericht durchgeführt. An der Mai-Sitzung des Plenums der GPK-N haben zudem sowohl de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das vergangene Geschäftsjahr stand im Zeichen eines wichtigen rechtsstaatlichen Jubiläums: 150 Jahre Bundesgericht. Tragen wir Sorge zu unseren Errungenschaften. Respektieren wir die Gewaltenteilung und achten wir unsere Bundesverfassung sowie die Gesetze.
+Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden GPK haben ihre Aufsichtssitzung im April zum Geschäftsbericht traditionsgemäss in Lausanne am Bundesgericht durchgeführt. An der Mai-Sitzung des Plenums der GPK-N haben zudem sowohl der Gerichtspräsident als auch die Subkommission entsprechend informiert.
+Bis auf das Patentgericht haben alle Gerichte einen Geschäftsanstieg zu verzeichnen. Das Bundesgericht hat einen Anstieg von rund 7 Prozent gegenüber dem Vorjahr zu verzeichnen. Dieser im Vergleich zu früheren Jahren geringere Anstieg zeigt, dass die Neuorganisation vor einigen Jahren allmählich Früchte trägt. Die durchschnittliche Verfahrensdauer verkürzte sich um einige Tage. Leicht weniger Beschwerden wurden gutgeheissen. Das Bundesgericht veröffentlichte 213 Urteile, auch, um die Transparenz der Rechtsprechung zu gewährleisten.
+Im Vergleich zum Bundesgericht verfügt das Bundesstrafgericht über eine kurze institutionelle Geschichte. Die Strafkammer konnte die Zahl der hängigen Verfahren reduzieren, hatte aber gleichzeitig mehrere grosse bedeutende Verfahren zu bearbeiten, beispielsweise bezüglich Bestechung fremder Amtsträger im internationalen Handel mit Erdölprodukten.
+Die Beschwerdekammer hatte Ende des Jahres mehr hängige Verfahren. Dies unter anderem aufgrund der Zunahme der Verfahren im Verwaltungsstrafrecht und im Bereich der internationalen Rechtshilfe.
+Die Berufungskammer hatte eine weitere Zunahme der Verfahren zu verzeichnen; diese betrafen das Unternehmensstrafrecht, Geldwäscherei, Insider Tradings, Terrorismus sowie die Bankomatensprengungen.
+Es wurde auch darauf hingewiesen, dass die nebenamtlichen Richterpersonen aufgrund ihrer hauptberuflichen Auslastung zeitlich nicht so flexibel sind, wie es ursprünglich angedacht war.
+Interessant für das Parlament sind auch immer die Hinweise an den Gesetzgeber. So hat das Bundesstrafgericht beispielsweise den EFK-Bericht bezüglich den Einziehungen und Ersatzforderungen nach Artikel 70 ff. StGB ernst genommen. Damit sich der Grundsatz "Strafbares Handeln soll sich nicht lohnen" auch richtig umsetzen lässt, wird angeregt, ein vereinfachtes Vollstreckungsverfahren zu schaffen, damit die Ersatzforderungen schnell eingetrieben werden können. Das ist ein wichtiger Punkt bei der Bekämpfung der Wirtschaftskriminalität.
+Das Bundesverwaltungsgericht verzeichnet erneut einen markanten Anstieg der Geschäftslast. Eine bessere Koordination zwischen dem SEM und dem Bundesverwaltungsgericht wäre mehr als wünschenswert. Es gab 70 neue Stellen beim SEM, aber nur eine Mikroerhöhung des Stellenetats beim Bundesverwaltungsgericht in St. Gallen. Eine bessere Koordination hätte da zu einer besseren Lösung führen können.
+Die durchschnittliche Verfahrensdauer konnte man jedoch reduzieren. Gleichzeitig hat man in St. Gallen aber auch viel in die Digitalisierung investiert. Das Ziel, Papier definitiv beiseite zu lassen, rückt immer näher. Die Spruchkörperbildung soll ab 2027 mit dem System "Diva" durchgeführt werden und den Abteilungspräsidien eine grosse Entlastung bringen.
+Das Bundespatentgericht verzeichnete einen Rückgang an Eingängen. Kein Fall ist länger als zwei Jahre hängig. Der Grund liegt vermutlich in der Bildung des Einheitlichen Patentgerichts (EPG). Dieses erlässt Verbote, die für bis zu 18 Länder gelten, und kann Patente für alle angeschlossenen Länder für ungültig erklären. Die Teilnahme am System steht nur für EU-Staaten offen, hat aber auch Auswirkungen auf die Schweiz.
+Das Bundespatentgericht in der Schweiz hat sich das Ziel gesetzt, das schnellste Gericht in Europa zu werden. Hierfür hat es unter anderem ein beschleunigtes Nichtigkeitsverfahren eingeführt.
+Ich sage noch einige wenige Worte zum Militärkassationsgericht. Dieses gehört nicht zum Bundesgericht, wie Sie wissen, aber auch hier hat die Bundesversammlung die Oberaufsicht. Deshalb erlaube ich mir dazu noch zwei, drei Sätze.
+Die zuständigen Subkommissionen des Ständerates und Nationalrates konnten vom Geschäftsbericht des Militärkassationsgerichtes keine Kenntnis nehmen. Grund: Wir haben keinen erhalten. Das ist unbefriedigend und nicht tolerierbar.
+Einige Worte zur Arbeit in der GPK im Zusammenhang mit den Gerichten: Wir haben einige Motionen und Berichte gemacht. Ich möchte Ihnen ganz kurz den Stand mitteilen:
+1. Die parlamentarische Initiative der GPK, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", ist zurzeit in der RK-S.
+2. Die Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes und der anderen erstinstanzlichen Gerichte wurde von der RK-N im Rahmen einer grösseren Revision behandelt.
+3. Die Motion zur Reorganisation des Bundesstrafgerichtes wurde in der RK-N einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die RK auf den Bericht der GPK von 2022.
+4. Den Bericht zum System der nebenamtlichen Richterinnen und Richter konnte die Subkommission Gerichte in der RK-N vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv werden.
+Ich möchte nicht schliessen, ohne dem Präsidenten des Bundesgerichtes und allen, die zum reibungslosen Funktionieren der Bundesjustiz beitragen, sowie dem Sekretariat der Geschäftsprüfungskommission für ihre Arbeit ganz herzlich zu danken. Es versteht sich von selbst, dass beaufsichtigte Stellen nicht alle Fragen der Aufsicht lieben. Das müssen sie auch nicht. Wir haben alle das gleiche Ziel: eine gut funktionierende und von der Politik unabhängige Justiz. Eine solche ist unabdingbar für eine Demokratie, in der heutigen Zeit mehr denn je.
+Ich bitte Sie, den Geschäftsbericht 2025 des Bundesgerichtes zu genehmigen. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salzmann Werner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
+Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
+Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.
+Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
+Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
+Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
 </t>
   </si>
 </sst>
@@ -430,8 +494,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I12"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1017,6 +1081,64 @@
         <v>64</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-17
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -127,24 +127,24 @@
     <t xml:space="preserve">IT</t>
   </si>
   <si>
-    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
 Il disavanzo del bilancio straordinario è dovuto soprattutto ai contributi versati ai Cantoni per le persone con statuto di protezione S provenienti dall'Ucraina, 700 milioni, e al contributo unico alle FFS, 850 milioni, compensati in parte da entrate straordinarie della Banca nazionale svizzera.
 L'avanzo dell'amministrazione ordinaria raggiunge 1,2 miliardi di franchi, mentre la regola del freno all'indebitamento avrebbe consentito un deficit di 262 milioni di franchi. Ne risulta quindi un saldo strutturale positivo di 1,4 miliardi, nettamente superiore al valore previsto nel preventivo.
 Le entrate ordinarie superano il budget di 1,9 miliardi e il risultato dell'anno precedente di ben 3,3 miliardi. La crescita è dovuta soprattutto all'imposta federale diretta sulle imprese, che beneficia delle entrate temporanee dal Cantone di Ginevra per circa 1,5 miliardi di franchi.
 Anche l'imposta federale diretta sui redditi aumenta di 0,5 miliardi, mentre l'IVA aumenta di 700 milioni, grazie alla crescita dell'economia nominale e all'effetto ritardato dell'aumento dell'aliquota dal 2024. Le entrate dell'imposta preventiva, invece, risultano inferiori alle attese.
-Le spese totali sono aumentate del 4 percento e ammontano a 87,6 miliardi di franchi. 
+Le spese totali sono aumentate del 4 per cento e ammontano a 87,6 miliardi di franchi. 
 I principali aumenti riguardano la previdenza sociale, le finanze e imposte, i trasporti, l'istruzione e la ricerca e l'esercito.
 Nel 2025 il numero di posti nella Confederazione è cresciuto di 240 unità, più 0,6 per cento, mentre le spese per il personale sono aumentate di 79 milioni di franchi, soprattutto per il rincaro dell'1 per cento.
 Il debito netto scende leggermente a 140 miliardi di franchi. Il conto di ammortamento del debito Covid si riduce per la prima volta di circa 500 milioni, grazie al saldo strutturale positivo e alle entrate straordinarie, e ammonta a 26,3 miliardi di franchi. Il conto di compensazione rimane stabile a circa 20 miliardi di franchi.
 Nella seduta dell'11 e 12 maggio 2026, la commissione ha proceduto all'esame di dettaglio del consuntivo. Le sue quattro sottocommissioni hanno presentato le conclusioni delle rispettive analisi approfondite dei consuntivi dei singoli servizi federali realizzate nel corso del mese di aprile.
-Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla sua commissione i risultati delle tre verifiche relative al Consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del Fondo per l'infrastruttura ferroviaria e quella del Fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
-Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del Fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma ancora irrisolte. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
+Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla vostra commissione i risultati delle tre verifiche relative al consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del fondo per l'infrastruttura ferroviaria e quella del fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
+Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma i problemi ancora irrisolti. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
 Il Controllo federale delle finanze conferma che il consuntivo rispetta le prescrizioni legali e le regole del freno all'indebitamento previste dall'articolo 126 della Costituzione federale. Per questo motivo raccomanda all'Assemblea federale di approvare il conto annuale.
 Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
-La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
+La vostra commissione vi propone all'unanimità di approvare il consuntivo 2025 della Confederazione come pure i conti speciali concernenti il fondo per le strade nazionali e il traffico d'agglomerato e il fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
 Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
 </t>
   </si>
@@ -306,6 +306,32 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">375543</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Lieber ein Ende mit Schrecken als ein Schrecken ohne Ende" - ich habe noch eine Motion, die ich von Kollege Glättli geerbt habe und hier kurz vorstelle. Es geht um die Beschaffung des F-35. Sie erinnern sich: Im Februar 2025 informierten die USA die Schweiz schriftlich, dass der vertraglich vereinbarte Festpreis aus ihrer Sicht ein Missverständnis sei. Es zeigte sich: Der Festpreis, der uns ziemlich vehement und über Jahre als solcher verkauft wurde, war keiner und ist den USA gegenüber auch ni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Lieber ein Ende mit Schrecken als ein Schrecken ohne Ende" - ich habe noch eine Motion, die ich von Kollege Glättli geerbt habe und hier kurz vorstelle. Es geht um die Beschaffung des F-35. Sie erinnern sich: Im Februar 2025 informierten die USA die Schweiz schriftlich, dass der vertraglich vereinbarte Festpreis aus ihrer Sicht ein Missverständnis sei. Es zeigte sich: Der Festpreis, der uns ziemlich vehement und über Jahre als solcher verkauft wurde, war keiner und ist den USA gegenüber auch nicht durchsetzbar. Je nach Berechnung können mit dem vom Volk bewilligten Budget nur noch zwischen 24 und 30 Maschinen beschafft werden statt der geplanten und versprochenen 36.
+Zusätzlich steigen die Infrastrukturkosten substanziell. Statt 120 Millionen sollen die Anpassungen der Militärflugplätze mindestens 200 Millionen Franken kosten. Die Eidgenössische Finanzkontrolle hat weitere Projekte von über 50 Millionen Franken identifiziert, die da obendrauf kommen. Das ist nicht ganz die Beschaffung, die uns 2021 verkauft wurde.
+Nun aber zu einer Frage, die zu wenig oft gestellt wird: Wofür braucht die Schweiz ein Kampfflugzeug? Die Hauptaufgabe ist die Luftpolizei, also das Identifizieren, Begleiten und nötigenfalls Abfangen von Flugzeugen im Schweizer Luftraum. Dafür braucht es Verfügbarkeit, Reaktionsgeschwindigkeit und Interoperabilität mit europäischen Partnern. Der F-35 ist als erstes Tarnkappenflugzeug der Geschichte zertifiziert, um Atomwaffen zu tragen. Im Juni 2025 drangen F-35A als erste Flugzeuge in den iranischen Luftraum ein, um Luftabwehrsysteme zu unterdrücken und B2-Bomber beim Angriff auf unterirdische Atomanlagen zu eskortieren. Das ist das Profil des F-35: Erstschlag tief im feindlichen Territorium, sogar mit nuklearer Bestückung und Tarnkappe.
+Die Schweiz ihrerseits eskortiert Privatjets über den Alpen und schützt vor allem Konferenzen in Genf und Davos. Die Stealth-Fähigkeit ist für diese Aufgaben schlicht irrelevant. Europäische Alternativen wie der Eurofighter oder die Rafale beherrschen den Luftpolizeidienst vollständig. Das hat auch ein ehemaliger Bundesrat ganz beeindruckend erlebt, als er von zwei Rafales eskortiert wurde. Offenbar kann dieses Flugzeug Luftpolizei.
+Auch sonst würden beispielsweise Eurofighter, Rafale oder Gripen das, was man sich vom F-35 erhofft, auch können, aber mit mehr operativer Unabhängigkeit. Sie würden auch zur Strategie des Bundesrates passen, künftig 60 Prozent aller Rüstungsbeschaffungen in der Schweiz und 30 Prozent in Europa zu tätigen und eben nur den Rest, 10 Prozent, ausserhalb Europas, sprich: mehr oder weniger in den USA. Eine Grossbeschaffung, die das gesamte Kampfflugzeugbudget exklusiv in die USA leitet, widerspricht diesem Ziel fundamental.
+Der Bundesrat hat die richtige Strategie formuliert und zieht die falschen Konsequenzen. Dazu kommt die operative Abhängigkeit. Die wichtigsten Stärken des F-35, seine Sensorfähigkeiten und seine Vernetzung, hängen direkt von US-amerikanischen Software-Updates und Aktivierungscodes ab. Bei politischer Instabilität in Washington, und von dieser gibt es zur Genüge, könnte der Jet innerhalb weniger Tage unbrauchbar gemacht werden. Das Herz des Jets liegt nicht in Emmen, sondern in Fort Worth.
+Der Bundesrat warnt vor einer Fähigkeitslücke, und auch das nehmen wir ernst. Deshalb fordert die Motion nicht einfach ein Abbrechen ohne Konzept, sondern gleichzeitig die Prüfung europäischer Alternativen und den Aufbau von Kapazitäten zur Drohnenabwehr und bodengestützten Luftverteidigung. Das ist die Richtung, in die Europa ohnehin zieht. Ein Jet, dessen Operabilität von einem unzuverlässigen Partner in Washington abhängt, schützt uns nicht. Er macht uns erpressbar. Die Motion ist aktueller denn je.
+Ich bitte um Zustimmung.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">375897</t>
   </si>
   <si>
@@ -318,14 +344,14 @@
     <t xml:space="preserve">Moser Tiana Angelina</t>
   </si>
   <si>
-    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband, der Fachverband für Wasser, Gas und Wärme, der Schweizerische Berufsfischerverband, der Schweizerische Brunnenmeister-Verband, und der Verband Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband, der Fachverband für Wasser, Gas und Wärme, der Schweizerische Berufsfischerverband, der Schweizerische Brunnenmeister-Verband, und der Verband Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
 Die Resolution verdient eine besondere Aufmerksamkeit. Sie stammt nicht nur von einzelnen Organisationen, sondern von denjenigen, die die Folgen der PFAS-Belastung im Interesse und zum Schutz der Bevölkerung bewältigen müssen. Die Brunnenmeister beispielsweise sind zuständig für die Sicherung der Wasserqualität und die Versorgung der Bevölkerung. 
-PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
+PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig, zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
 Vor diesem Hintergrund ist die Stellungnahme des Bundesrates zu Frage 2 meiner Interpellation besonders bemerkenswert. Der Bundesrat anerkennt ausdrücklich den Nutzen des Human Biomonitoring für die Erfassung der Belastung der Bevölkerung. Genau solche Daten bräuchten wir, um Risiken frühzeitig zu erkennen und entsprechende Entwicklungen zu verfolgen. Umso weniger verständlich ist es, dass ausgerechnet dieses Instrument aus Spargründen eingestellt worden ist. Die Kosten des Human Biomonitoring stehen in keinem Verhältnis zu den Folgekosten der PFAS-Belastung, die sich, Sie haben es gehört, im Milliardenbereich bewegen. Auf das Monitoring zu verzichten, heisst, auf Wissen zu verzichten, das helfen könnte, gesundheitliche Risiken frühzeitig zu erkennen und Schäden zu begrenzen. 
-Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind wie gesagt nur die Beispiele zum Gewässer. 
+Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind, wie gesagt, nur die Beispiele zum Gewässer. 
 Es ist offensichtlich, dass es sich hier um eine schweizweite Herausforderung handelt. Wir stehen bei der PFAS-Thematik erst am Anfang, und gerade deshalb können wir es uns nicht leisten, auf Wissen zu verzichten. Entsprechend wichtig wäre eine Wiederaufnahme des Human Biomonitoring im Rahmen des Aktionsplans zur Reduktion der Ewigkeitschemikalien. Diese Einschätzung wurde im Übrigen auch von der Eidgenössischen Finanzkontrolle 2024 geteilt. Gerade angesichts der gesundheitlichen Risiken und der möglichen Folgekosten sowie der grossen Wissenslücken wäre das eine sehr wichtige Aussage, um auch das Vertrauen der Bevölkerung zu steigern. 
 In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
 </t>
@@ -392,9 +418,6 @@
   </si>
   <si>
     <t xml:space="preserve">Weichelt Manuela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
   </si>
   <si>
     <t xml:space="preserve">ZG</t>
@@ -446,6 +469,37 @@
 Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
 Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
 Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377387</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binder-Keller Marianne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden Geschäftsprüfungskommissionen, also des Nationalrates und des Ständerates, tagen in der Regel gemeinsam. Traditionellerweise findet die Sitzung, in welcher sie den Geschäftsbericht des Bundesgerichtes diskutieren und zur Kenntnis nehmen, am Bundesgericht in Lausanne statt; dies - nebenbei bemerkt - in einem Raum mit ikonischen Bildern. Eines zeigt die archaische Szene des salomonischen Urteils und bringt mich jedes Mal ins Grübeln, wenn </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden Geschäftsprüfungskommissionen, also des Nationalrates und des Ständerates, tagen in der Regel gemeinsam. Traditionellerweise findet die Sitzung, in welcher sie den Geschäftsbericht des Bundesgerichtes diskutieren und zur Kenntnis nehmen, am Bundesgericht in Lausanne statt; dies - nebenbei bemerkt - in einem Raum mit ikonischen Bildern. Eines zeigt die archaische Szene des salomonischen Urteils und bringt mich jedes Mal ins Grübeln, wenn ich ein Urteil wieder einmal als salomonisch loben will. Da kommen zwei Frauen zu Salomon mit einem Kind, beide behaupten, es sei ihres. König Salomon befiehlt, das Kind mit einem Schwert auseinanderzuhauen, damit jede Frau ihre Hälfte bekäme. Die eine Frau sagte dann, man solle es der anderen geben, damit das Kind überlebe. Voilà, da hat Salomon gemerkt, dass das die richtige Mutter ist. Wenn Sie also das Wort "salomonisch" bei einem Urteil verwenden, geht das auf diese Geschichte zurück. 
+Anwesend am 22. April 2026 in Lausanne war der Bundesgerichtspräsident, verschiedene weitere Mitglieder des Bundesgerichtes, die Präsidentinnen und Präsidenten der erstinstanzlichen Gerichte und weitere Mitglieder. In ihrer Plenarsitzung im Mai 2026 hat auch die Geschäftsprüfungskommission den Bericht zur Kenntnis genommen, der ihr dann auch vom Bundesgericht vorgestellt wurde.
+Zur Einordnung der Aufgaben der Geschäftsprüfungskommissionen gegenüber dem Bundesgericht: Die Bundesversammlung übt die Oberaufsicht über das Bundesgericht, die oberste gerichtliche Instanz der Eidgenossenschaft, aus. Das heisst, sie übt die Oberaufsicht über die Geschäftsführung des Bundesgerichtes aus, selbstverständlich geht es nicht um die Wertung von Urteilen. Das Bundesgericht übt seinerseits die Aufsicht über das Bundesstrafgericht, das Bundesverwaltungsgericht und das Bundespatentgericht aus, wobei das Bundesgericht nach wie vor nicht über die Befugnisse und Mittel verfügt, um in persönlichen Angelegenheiten umfassend einzugreifen. Wie die jüngsten Ereignisse jedoch zeigen, bereiten bestimmte Fälle nach wie vor Probleme. Wir werden bei der Prüfung des Geschäftsberichtes des Jahres 2026 darauf zurückkommen müssen.
+Im Jahr 2025 haben die verschiedenen Kammern des Bundesgerichtes über 7883 Fälle entschieden, was rund 7 Prozent mehr als dem Wert des Vorjahres entspricht; im Jahr 2024 wurden 7351 Fälle entschieden. Dieser geringere Anstieg als zuvor zeigt, dass die 2020 eingeleitete Reorganisation der Kammern allmählich Früchte trägt. Die durchschnittliche Verfahrensdauer verkürzte sich um einige Tage. Leicht weniger Beschwerden wurden gutgeheissen. Das Bundesgericht veröffentlichte 213 Urteile, auch um die Transparenz der Rechtsprechung zu gewährleisten. All dies ersehen Sie im Detail im Bericht des Bundesgerichtes. 
+Zu den erstinstanzlichen Gerichten: Das Bundesstrafgericht verzeichnete im Jahr 2025 insgesamt einen Anstieg der Eingänge auf 686 neue Fälle gegenüber 619 im Jahr 2024. Die Erledigungsquote blieb stabil bei 93 Prozent statt 94 Prozent im Jahr 2024. Die Strafkammer hatte mehrere bedeutende Verfahren zu bearbeiten, beispielsweise bezüglich Bestechung fremder Amtsträger im internationalen Handel mit Erdölprodukten. Die Beschwerdekammer hatte Ende des Jahres mehr hängige Verfahren, dies unter anderem aufgrund der Zunahme der Verfahren im Verwaltungsstrafrecht und im Bereich der internationalen Rechtshilfe. Die Berufungskammer hatte eine weitere Zunahme der Verfahren zu verzeichnen. Diese betrafen das Unternehmensstrafrecht, Geldwäscherei, Insiderhandel, Terrorismus sowie die Bankomatsprengungen. 
+Es wurde auch darauf hingewiesen, dass die nebenamtlichen Richterpersonen aufgrund ihrer hauptberuflichen Auslastung zeitlich nicht so flexibel sind, wie es ursprünglich angedacht war. 
+Interessant für das Parlament sind auch immer die Hinweise an den Gesetzgeber, die wir unterdessen auch noch direkt den Sachbereichskommissionen mitteilen. So hat das Bundesstrafgericht beispielsweise den EFK-Bericht bezüglich der Einziehungen und Ersatzforderungen nach Artikel 70 StGB ernst genommen. Damit sich der Grundsatz "Strafbares Handeln soll sich nicht lohnen" auch richtig umsetzen lässt, wird angeregt, ein vereinfachtes Vollstreckungsverfahren zu schaffen, damit die Ersatzforderungen schnell eingetrieben werden können. Das ist ein wichtiger Punkt bei der Bekämpfung der Wirtschaftskriminalität.
+Das Bundesverwaltungsgericht verzeichnet erneut einen markanten Anstieg der Geschäftslast. Eine bessere Koordination zwischen dem SEM und dem Bundesverwaltungsgericht wäre wünschenswert. Es gab 70 neue Stellen beim SEM, aber nur eine Mikroerhöhung des Stellenetats beim Bundesverwaltungsgericht in St. Gallen. Eine bessere Koordination hätte da, wie betont, zu einer besseren Lösung führen können. Die durchschnittliche Verfahrensdauer konnte man jedoch reduzieren. Gleichzeitig hat man in St. Gallen auch viel in die Digitalisierung investiert. Das Ziel, Papier definitiv beiseitezulassen, rückt näher.
+Das Bundespatentgericht verzeichnete einen Rückgang an Eingängen. Kein Fall ist länger als zwei Jahre hängig. Der Grund liegt vermutlich in der Bildung des Einheitlichen Patentgerichtes. Dieses erlässt Verbote, die für bis zu 18 Länder gelten, und kann Patente für alle angeschlossenen Länder für ungültig erklären. Die Teilnahme am System steht nur EU-Staaten offen, das System hat aber auch Auswirkungen auf die Schweiz. Das Bundespatentgericht hat sich zum Ziel gesetzt, das schnellste Gericht in Europa zu werden. Hierfür hat es unter anderem ein beschleunigtes Nichtigkeitsverfahren eingeführt.
+Einige Worte noch zur Arbeit in der Geschäftsprüfungskommission im Zusammenhang mit den Gerichten: Wir haben einige Vorstösse und Berichte ausgearbeitet. Ganz kurz zum Stand: 
+Erstens hat die GPK-S die parlamentarische Initiative 25.401, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", eingereicht. Dieser Vorstoss, dieses Anliegen liegt zurzeit in der Kommission für Rechtsfragen des Ständerates. Die Motion 22.4250, "Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes, des Bundesverwaltungsgerichtes und des Bundesstrafgerichtes", wurde von der Kommission für Rechtsfragen des Nationalrates im Rahmen einer grösseren Revision behandelt. Die Motion 25.4395 der RK-S, "Reorganisation des Bundesstrafgerichtes", wurde ebenfalls in der Kommission für Rechtsfragen des Nationalrates einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die Kommission für Rechtsfragen auf den Bericht der GPK aus dem Jahre 2022. Weiter konnte die GPK-Subkommission Gerichte/BA den Bericht zum System der nebenamtlichen Richterinnen und Richter in der Kommission für Rechtsfragen des Nationalrates vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv wird.
+Letztlich sei daran erinnert, dass das Bundesgericht im Jahr 2025 sein 150-jähriges Bestehen feierte. Zu diesem Anlass wurden unter anderem ein wissenschaftliches Kolloquium, eine Festschrift, eine offizielle Feier sowie Tage der offenen Tür mit etwa zweitausend Besuchern organisiert. 
+Ich möchte, Herr Bundesgerichtspräsident, diesen Bericht nicht abschliessen, ohne Ihre Arbeit zu verdanken, die gute Zusammenarbeit mit den Bundesbehörden und auch die Arbeit Ihres Sekretariats, unter anderem im Zusammenhang mit der Tätigkeit unserer Kommission.
 </t>
   </si>
 </sst>
@@ -494,8 +548,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I14"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1004,16 +1058,16 @@
         <v>48</v>
       </c>
       <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
@@ -1033,17 +1087,19 @@
         <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9"/>
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="H9" t="s">
         <v>57</v>
@@ -1060,19 +1116,17 @@
         <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
-        <v>49</v>
-      </c>
+      <c r="E10"/>
       <c r="F10" t="s">
         <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
         <v>63</v>
@@ -1089,42 +1143,42 @@
         <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
         <v>67</v>
       </c>
       <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
         <v>68</v>
-      </c>
-      <c r="F11" t="s">
-        <v>69</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
       </c>
       <c r="H11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" t="s">
         <v>70</v>
-      </c>
-      <c r="I11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
         <v>72</v>
       </c>
-      <c r="B12" t="s">
-        <v>66</v>
-      </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
         <v>74</v>
@@ -1137,6 +1191,64 @@
       </c>
       <c r="I12" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-06-18
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -460,16 +460,10 @@
     <t xml:space="preserve">BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
-Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
-Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.
-Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
-Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
-Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
-</t>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir beschaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.</t>
   </si>
   <si>
     <t xml:space="preserve">377387</t>
@@ -500,6 +494,106 @@
 Erstens hat die GPK-S die parlamentarische Initiative 25.401, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", eingereicht. Dieser Vorstoss, dieses Anliegen liegt zurzeit in der Kommission für Rechtsfragen des Ständerates. Die Motion 22.4250, "Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes, des Bundesverwaltungsgerichtes und des Bundesstrafgerichtes", wurde von der Kommission für Rechtsfragen des Nationalrates im Rahmen einer grösseren Revision behandelt. Die Motion 25.4395 der RK-S, "Reorganisation des Bundesstrafgerichtes", wurde ebenfalls in der Kommission für Rechtsfragen des Nationalrates einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die Kommission für Rechtsfragen auf den Bericht der GPK aus dem Jahre 2022. Weiter konnte die GPK-Subkommission Gerichte/BA den Bericht zum System der nebenamtlichen Richterinnen und Richter in der Kommission für Rechtsfragen des Nationalrates vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv wird.
 Letztlich sei daran erinnert, dass das Bundesgericht im Jahr 2025 sein 150-jähriges Bestehen feierte. Zu diesem Anlass wurden unter anderem ein wissenschaftliches Kolloquium, eine Festschrift, eine offizielle Feier sowie Tage der offenen Tür mit etwa zweitausend Besuchern organisiert. 
 Ich möchte, Herr Bundesgerichtspräsident, diesen Bericht nicht abschliessen, ohne Ihre Arbeit zu verdanken, die gute Zusammenarbeit mit den Bundesbehörden und auch die Arbeit Ihres Sekretariats, unter anderem im Zusammenhang mit der Tätigkeit unserer Kommission.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377942</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fässler Daniel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. 
+Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. 
+Zur Detailberatung: Ich mache zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. 
+Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. 
+Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. 
+Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. 
+Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 
+1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 
+2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 
+3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. 
+Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dittli Josef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Postulat geht direkt auf unseren umfassenden Untersuchungsbericht vom 30. Januar 2026 zur Aufsicht und Steuerung der Ruag MRO zurück. Lassen Sie mich kurz rekapitulieren, worum es in dieser Untersuchung ging.
+Im Jahre 2023 beabsichtigte die Ruag MRO, 96 Leopard-1-Panzer nach Deutschland zu verkaufen. Die frühere Ruag Schweiz AG hatte die bereits seit Längerem ausser Dienst stehenden Panzer 2016 einer Agentur des italienischen Verteidigungsministeriums abgekauft. Sie wurden sodann in Itali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Postulat geht direkt auf unseren umfassenden Untersuchungsbericht vom 30. Januar 2026 zur Aufsicht und Steuerung der Ruag MRO zurück. Lassen Sie mich kurz rekapitulieren, worum es in dieser Untersuchung ging.
+Im Jahre 2023 beabsichtigte die Ruag MRO, 96 Leopard-1-Panzer nach Deutschland zu verkaufen. Die frühere Ruag Schweiz AG hatte die bereits seit Längerem ausser Dienst stehenden Panzer 2016 einer Agentur des italienischen Verteidigungsministeriums abgekauft. Sie wurden sodann in Italien gelagert. Bei diesem Geschäft traten Ungereimtheiten zutage. In der Folge veröffentlichte die Eidgenössische Finanzkontrolle in den Jahren 2024 und 2025 vier Berichte, die Mängel in der Compliance und Führung innerhalb der Ruag MRO, aber auch Probleme in der Aufsicht und Steuerung der Ruag MRO durch den Eigner, den Bund, aufzeigten.
+Unsere Kommission hat diese Vorfälle vertieft analysiert und festgestellt, dass die Probleme struktureller Natur sind. Die GPK richtete total sechs Empfehlungen zur Führung und Steuerung der Ruag MRO an den Bundesrat und beantragt dem Ständerat nun eben auch die Annahme dieses Postulates. Wir wollen damit den Bundesrat beauftragen, ergebnisoffen zu prüfen, ob die Corporate Governance des Bundes und das heutige duale Steuerungsmodell noch eine angemessene Wahrnehmung der Eignerinteressen erlauben. Er soll insbesondere prüfen, ob Anpassungen am aktuellen System nötig sind. Zudem soll er mögliche Alternativen, wie die Einsetzung einer einzigen zentralen Stelle für die Vorbereitung und Koordination aller eignerpolitischen Geschäfte zuhanden des Bundesrates, prüfen.
+Das heutige Modell birgt folgende Herausforderung. Das VBS ist nicht nur Miteigentümer, sondern auch der mit Abstand grösste Kunde der Ruag MRO. Die Eidgenössische Finanzverwaltung hingegen ist in dieser Kundenbeziehung nicht involviert und konzentriert sich rein auf die Finanzen. Dadurch entsteht ein Informationsgefälle. Die Eidgenössische Finanzverwaltung hat oft keinen Einblick in operative Sachverhalte, was das Risiko von blinden Flecken, etwa bei der Compliance, erhöht. Die GPK sieht daher möglichen Handlungsbedarf und identifiziert vier Schwachstellen des aktuellen Systems:
+1. Eine fehlende ganzheitliche Sicht: Da sich das VBS auf die Fachsicht und die Eidgenössische Finanzverwaltung auf die Finanzen fokussiert, fehlt oft eine kritische, ressortübergreifende Betrachtung.
+2. Uneinheitliche Umsetzung: Jedes Departement führt seine Unternehmen etwas anders. Eine bundesweite, einheitliche Linie fehlt.
+3. Komplexität: Die Betriebe sind hochkomplex und agieren am Markt. Übergeordnete Themen wie Governance oder Korruptionsbekämpfung erfordern gebündelte Expertise.
+4. Interessenkonflikte: Fachdepartemente sind oft Eigner, Kunde, Subventionsgeber und Regulator in Personalunion. Dies gefährdet eine objektive Aufsicht.
+Dies ganz kurz in etwa die Begründung des Postulates.
+Der Bundesrat beantragt die Ablehnung dieses Postulates. Seine Begründung ist vor allem formal. Man habe die Corporate Governance bereits 2018 und 2019 analysiert. Das Modell funktioniere gut, und mit dem neuen Artikel 24a der Regierungs- und Verwaltungsorganisationsverordnung (RVOV) sei die Aufgabenteilung nun rechtlich verankert. Ein Bericht bringe keine neuen Erkenntnisse.
+Die GPK-S teilt diese wohlwollende Sicht des Bundesrates nicht. Zu behaupten, die Ausgangslage habe sich seit 2019 nicht verändert, blendet die Realität aus. Die gravierenden Mängel bei der Ruag MRO, das Versagen bei den Compliance-Strukturen und die Intransparenz bei der Lagerverwaltung sind reale Befunde aus den Jahren 2024 und 2025. Sie traten also trotz der alten Berichte und trotz der neuen Verordnungstexte auf. Eine formale Aufgabenteilung auf dem Papier nützt uns nichts, wenn sie in der Praxis scheitert.
+Im Namen der GPK-S bitte ich Sie deshalb, das Postulat anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mühlemann Benjamin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Vorstoss von Kollege Regazzi verlangt einen Bericht zur Wirksamkeit, Zielgenauigkeit und volkswirtschaftlichen Wirkung von Bundessubventionen. Es geht insbesondere um die Fragen, welche Subventionen ihre Ziele erreichen, wo Fehlanreize oder Mitnahmeeffekte bestehen, wo Wettbewerbsverzerrungen entstehen können und wo Verbesserungen und allenfalls auch Reduktionen möglich wären.
+Ich finde, das ist ein sinnvoller und angemessener Auftrag, und deshalb beantrage ich Ihnen ebenfalls, das Postulat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Vorstoss von Kollege Regazzi verlangt einen Bericht zur Wirksamkeit, Zielgenauigkeit und volkswirtschaftlichen Wirkung von Bundessubventionen. Es geht insbesondere um die Fragen, welche Subventionen ihre Ziele erreichen, wo Fehlanreize oder Mitnahmeeffekte bestehen, wo Wettbewerbsverzerrungen entstehen können und wo Verbesserungen und allenfalls auch Reduktionen möglich wären.
+Ich finde, das ist ein sinnvoller und angemessener Auftrag, und deshalb beantrage ich Ihnen ebenfalls, das Postulat anzunehmen.
+Wir haben von Herrn Regazzi gehört, welches Instrumentarium bereits existiert. Darauf verweist auch der Bundesrat in seiner ablehnenden Stellungnahme. Nun ist das heutige Verfahren im Kern so angelegt: Die zuständigen Ämter nehmen zunächst eine Selbstbeurteilung vor. Die Eidgenössische Finanzverwaltung überprüft danach, ob die rechtlichen Grundlagen und die Subventionspraxis mit den Grundsätzen des Subventionsgesetzes übereinstimmen, und die Ergebnisse und allfällige Massnahmen werden dann im Rahmen der Staatsrechnung, bei entsprechenden Botschaften zu Finanzbeschlüssen oder bei Botschaften zu gesetzlichen Grundlagen ausgewiesen. Also, im Grundsatz ist das sicher ein wertvoller Prozess. Man muss dieses Instrument auch überhaupt nicht infrage stellen. Aber gerade weil dieses Instrument heute bereits besteht, sollten wir genauer hinschauen, um zu sehen, wie gut es tatsächlich wirkt.
+Die Eidgenössische Finanzkontrolle (EFK) hat dazu kürzlich einen sehr relevanten Bericht veröffentlicht, und ich melde mich genau deshalb zu Wort, damit dieser Bericht eine gewisse Öffentlichkeit erhält und nicht einfach in einer Schublade verschwindet. Dieser Bericht trägt den Titel "Prüfung des Prozesses und des Nutzens der periodischen Subventionsüberprüfung". Der Bericht ist vom Januar dieses Jahres.
+Die EFK kommt darin zu einem differenzierten Befund. Sie sagt nicht, dass das Verfahren nutzlos sei, im Gegenteil. Die periodische Überprüfung hat eine gewisse präventive Wirkung. Sie sensibilisiert die Verwaltungseinheiten für die Anforderungen des Subventionsgesetzes, und auch der administrative Aufwand wird von der EFK nicht als unverhältnismässig dargestellt. Aber die EFK zeigt ebenso klar auf, dass im Hinblick auf die eigentliche Steuerung der Bundessubventionen die Wirkung bisher zu gering ist. Das ist ein wichtiger Punkt, denn wir haben die Zahlen jetzt schon zwei-, dreimal gehört. Es geht bei diesem Volumen von 48 Milliarden Franken, das bereitgestellt wird, nicht um einen Randbereich des Bundeshaushalts. Die EFK nennt drei Punkte, die aus meiner Sicht für die heutige Diskussion ganz besonders wichtig sind. 
+Zum ersten Punkt: Die Überprüfung ist eben nicht vollständig. Die Finanzverwaltung stützt sich bei der Auswahl der zu prüfenden Subventionen auf die Ausgabenkredite. Bestimmte Formen von Subventionen werden dadurch nicht oder nicht systematisch erfasst. Dazu gehören etwa unentgeltliche oder vergünstigte Leistungen des Bundes. Dazu gehören Subventionen über Fonds oder Institutionen, die im Auftrag des Bundes handeln, sowie Steuervergünstigungen. Die EFK hält fest, dass die Finanzverwaltung über keine abschliessende Übersicht dieser Subventionsformen verfügt und auch das entsprechende Volumen nicht kennt. 
+Zum zweiten Punkt, der bemängelt wird: Die Ämter melden im Rahmen ihrer Selbstbeurteilung Abweichungen von den Grundsätzen des Subventionsgesetzes in der Regel nicht von sich aus. Die Finanzverwaltung kann zwar noch Probleme identifizieren und dann auch Massnahmen vorschlagen, aber diese Massnahmen werden in der Regel im Konsens mit den betroffenen Verwaltungseinheiten vereinbart, auch um eine Eskalation zu vermeiden. 
+Zum dritten Punkt, den die EFK bemängelt: Die finanziellen Auswirkungen bleiben bisher sehr, sehr bescheiden. Die EFK stellt fest, dass zwischen 2014 und 2024 nur vier Fälle identifiziert wurden, in denen Massnahmen zur Streichung einer Subvention oder zu einer effektiven Einsparung geführt haben. Das Einsparvolumen betrug insgesamt 2,3 Millionen Franken pro Jahr. Bei einem Subventionsvolumen von 48 Milliarden Franken ist das ja eigentlich nichts. 
+Persönlich komme ich zum Schluss, dass in der periodischen Subventionsüberprüfung Potenzial liegt, das heute nicht genügend ausgeschöpft wird. Genau hier setzt das Postulat Regazzi an. Er verlangt nicht, dass Subventionen pauschal infrage gestellt werden; das wäre auch nicht sachgerecht. Aber es braucht eine saubere Unterscheidung. Wir müssen wissen, welche Subventionen noch ihre Ziele erreichen, welche noch gerechtfertigt sind, welche allenfalls angepasst werden müssen. Wir müssen auch wissen, wo Mitnahmeeffekte da sind, wo Fehlanreize gesetzt werden und wo der Mitteleinsatz nicht mehr im Verhältnis zur Wirkung steht. 
+Es ist also sinnvoll, heute die Grundlagen für eine nächste Prüfung, die zweifelsohne stattfinden wird, zu verbessern. Es geht nicht darum, jetzt sofort ein neues, grosses Entlastungspaket zu schnüren. Es geht darum, im ordentlichen Prozess früher, systematischer und wirksamer zu erkennen, wo Handlungsbedarf besteht. Wenn wir in Zukunft grössere Sparrunden und hektische Entlastungsprogramme vermeiden wollen, dann müssen wir im Tagesgeschäft besser steuern. Die periodische Subventionsüberprüfung ist dafür ein geeignetes Instrument, aber, ich habe den Bericht der EFK erwähnt, eben noch kein genügend wirksames Instrument. Das Postulat Regazzi ist deshalb ein sachlicher und moderater Beitrag, um hier weiterzukommen. 
+Ich bitte Sie, dieses Postulat anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gapany Johanna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En voyant le vote de la commission, je me doute qu'il y a un vrai malaise autour de ce programme. Il y a autant de membres de la commission qui se sont abstenus que de membres qui se sont opposés à l'initiative de notre collègue Stark. Ce débat n'est donc pas totalement inutile vu ce résultat. Et même si on est tous d'accord, je crois, sur la nécessité de récolter et de traiter des données, la méthode pose problème. Personne, dans cette salle, ne conteste la nécessité d'un suivi sérieux, crédibl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En voyant le vote de la commission, je me doute qu'il y a un vrai malaise autour de ce programme. Il y a autant de membres de la commission qui se sont abstenus que de membres qui se sont opposés à l'initiative de notre collègue Stark. Ce débat n'est donc pas totalement inutile vu ce résultat. Et même si on est tous d'accord, je crois, sur la nécessité de récolter et de traiter des données, la méthode pose problème. Personne, dans cette salle, ne conteste la nécessité d'un suivi sérieux, crédible aussi, de l'utilisation des produits phytosanitaires. En fait, c'est ce qu'on avait défendu devant la population, et la population a massivement refusé les initiatives dont on parle et dont on parlait précédemment. Le suivi se fait d'ailleurs déjà et il se fera encore demain ; il se fera sans doute encore plus demain. Les produits utilisés sont beaucoup plus contrôlés que du temps de nos parents, c'est un fait. Ils le sont aussi beaucoup plus en Suisse que dans la plupart des autres pays dans le monde.
+Personne ne conteste non plus que notre agriculture doit pouvoir démontrer ses efforts, sa responsabilité et sa capacité à évoluer. Au contraire, on veut - et on le voit aussi quand on lit les perspectives de la politique agricole 2030 -, une agriculture moderne, capable de nourrir la population en utilisant le progrès. Alors, ce qu'on exige de l'agriculture, on doit être capable de l'appliquer aussi à l'administration fédérale : de la modernité, de l'efficacité et un système qui fonctionne dans la pratique. C'est tout simplement ce que demande notre collègue Stark.
+On parle aussi de surcharge bureaucratique, avec le Digiflux dans sa version actuelle. Ce n'est pas seulement un terme à la mode, cette surcharge bureaucratique. C'est un vrai fléau et un vrai frein à la production alimentaire, alors que déjà aujourd'hui, on parle de pénurie dans certains domaines. Personne ici - en tout cas j'imagine - ne pense d'ailleurs que les agriculteurs ou les PME s'ennuient au point qu'il faut leur donner du travail supplémentaire. La pression est déjà suffisante, entre la hausse généralisée des coûts, la multiplication des normes, les exigences administratives aussi, qui sont toujours plus nombreuses. On peut dire sans caricaturer que ceux qui nous nourrissent passent gentiment plus de temps devant leur ordinateur que sur le tracteur.
+Et sur ce constat, on vient ajouter une couche supplémentaire, sans gain pour la production. C'est d'autant plus un problème que c'est contraire à un principe qu'on avait voulu dans ce Parlement, le principe "once only", selon lequel chaque donnée doit être introduite une seule fois dans un système. C'est un principe de bon sens, un principe d'efficacité, et aujourd'hui, avec la version actuelle du Digiflux, clairement, on ne le met pas en oeuvre.
+Et puis, il y a un autre élément qui est quand même important : le Contrôle fédéral des finances a lui-même rendu un rapport et il a fait sept recommandations concrètes. Ce rapport était très clairement critique : il a relevé des lacunes dans le pilotage du projet, dans la clarté des bénéfices attendus et dans l'utilisation des données. Pour un projet dont le budget est quand même d'environ 16 millions de francs, quand on reçoit ce genre de remarques, notamment sur les lacunes au niveau du pilotage, mais aussi au niveau des bénéfices attendus, on ne peut pas simplement en prendre connaissance et passer à autre chose. C'est non seulement une question technique, mais c'est aussi une question de confiance. Celles et ceux qui livrent ces données doivent avoir la garantie que les données sensibles concernant leur activité, concernant leurs clients, soient traitées de manière transparente, avec une base légale claire et dans un objectif qui est précisément défini. Cette confiance est élémentaire si on veut que les acteurs du terrain adhèrent à ce système.
+La proposition de notre collègue Stark va précisément dans cette direction, et c'est la raison pour laquelle je la soutiens. Je la soutiens d'autant plus qu'elle ne remet pas en question les engagements de l'agriculture. Elle vise un système plus pragmatique, plus proportionné et utilisable aussi dans la pratique ; un système qui est compatible avec une agriculture moderne, qui respecte ses engagements environnementaux, mais sans être étouffée par des charges administratives dont les bénéfices ne sont pas clairs, comme l'a dit le Contrôle fédéral des finances.
+Je vous remercie pour votre attention et j'espère vous voir soutenir cette initiative parlementaire ainsi que l'initiative du canton de Berne en y donnant suite.
 </t>
   </si>
 </sst>
@@ -548,8 +642,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I18" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I18"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1251,6 +1345,122 @@
         <v>87</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>97</v>
+      </c>
+      <c r="I16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
+      </c>
+      <c r="I17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-19
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -174,7 +174,7 @@
 Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
 Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
 Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
-Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen, zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
 Wichtig sind auch klare Datenschutzgarantien im Gesetz, insbesondere wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
 Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
 Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
@@ -512,17 +512,7 @@
     <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. 
-Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. 
-Zur Detailberatung: Ich mache zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. 
-Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. 
-Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. 
-Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. 
-Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 
-1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 
-2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 
-3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. 
-Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. Zur Detailberatung: Ich mache jetzt in einem einzigen Votum zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-09-15
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -85,6 +85,72 @@
     <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir ? C'est la question centrale de cette motion. Son point de départ est concret : une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, la destination des sommes récupérées relève pleinement de notre responsabilité politique, car cet argent a été financé par les assurés, par leurs primes, mais également par leur franchise et leur quote-part. Le Conseil fédéral estime que ma motion est inutile. Selon son avis, les sommes récupérées améliorent le résultat technique des assureurs et peuvent ainsi contribuer à réduire les primes, mais une possibilité de baisse future n'est pas une garantie de restitution. Lorsqu'un assuré a personnellement supporté une partie d'une facture, ensuite corrigée, où apparaît cette correction ? Comment sa participation est-elle recalculée ? Comment s'assure-t-on que la somme correspondante lui revient ? Pour les montants financés collectivement par les primes, comment démontre-t-on qu'ils bénéficient effectivement aux assurés, au lieu de simplement alimenter les réserves ? Voilà les questions auxquelles il faut répondre.
 L'interdiction de distribuer des bénéfices invoquée par le Conseil fédéral ne suffit pas. Elle ne démontre ni à qui les montants récupérés bénéficient, ni quand, ni comment. Une écriture comptable favorable à l'assureur ne prouve pas à elle seule une restitution à l'assuré. Cette motion s'inscrit dans la continuité de mon travail parlementaire, notamment de la motion 24.3060 sur le contrôle des finances des caisses-maladie. Rabais, rétrocessions ou remboursements de prestations : les mécanismes diffèrent, mais l'exigence demeure. Nous devons pouvoir tracer l'argent et vérifier qu'il bénéficie à ceux qui financent l'assurance obligatoire. Les travaux du Contrôle fédéral des finances renforcent cette exigence de transparence et de contrôle. Les médecins qui assurent les consultations le soir et le week-end rendent un service indispensable et les assureurs doivent appliquer les décisions judiciaires, mais il reste à garantir que les conséquences financières soient correctement répercutées jusqu'aux assurés. La récupération de l'argent ne doit pas être la dernière étape. Sa restitution doit être l'objectif. Les assurés paient leurs primes, leur franchise et leur quote-part. Ces obligations sont précises et leurs échéances aussi. Ils sont en droit d'attendre la même précision lorsqu'une somme doit leur revenir.
 Je vous demande donc d'adopter cette motion pour garantir une traçabilité des montants récupérés, la correction des participations individuelles concernées et une répercussion effective au bénéfice des assurés. Au-delà de cette taxe de 40 francs, nous défendons un principe essentiel : l'argent récupéré dans l'assurance obligatoire doit bénéficier aux assurés de manière concrète, transparente et vérifiable.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">419015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260915</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chollet Clarence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifie pas continuer comme si rien ne s'était passé au sein du DDPS.
+Au moment où ce Parlement s'apprête à voter 3,4 milliards de francs supplémentaires, dont 394 millions pour le F-35A, une question s'impose : pouvons-nous encore avoir confiance dans la manière dont le DDPS conduit ses grands projets d'armement ? La semaine dernière, la Commission de gestion nous a donné quelques éléments de réponse qui sont accablants. Pendant des années, on nous a répété que le prix du F-35A était fixe. Il ne l'est pas. On nous a affirmé que la Suisse avait négocié une garantie particulière avec les États-Unis. Cette garantie n'existe pas. Des doutes avaient été exprimés par le Contrôle fédéral des finances, mais ils n'ont pas conduit à l'examen critique qui aurait été nécessaire. Le service juridique d'Armasuisse, pourtant compétent en la matière, n'a pratiquement pas participé à la négociation de ce contrat. Seules quelques personnes impliquées dans le dossier ont lu le contrat dans son intégralité. Comme si cela ne suffisait pas, la Commission de gestion constate que certains documents n'ont même pas été archivés conformément aux règles.
+Nous ne parlons pas de l'achat de quelques véhicules de service. Nous parlons du plus grand projet d'acquisition militaire de l'histoire récente de notre pays. Pourtant, à chaque nouvelle révélation, le même constat s'impose : manque de conduite, manque de contrôle, manque de transparence. Et maintenant, le Parlement doit octroyer 394 millions supplémentaires, non pour améliorer la sécurité de la Suisse, mais pour essayer de sauver 30 avions sur les 36 que le Conseil fédéral voulait acquérir. Faut-il avaler cette couleuvre tranquillement ? Nous ne le pensons pas.
+Il faut savoir s'arrêter lorsqu'un projet déraille. Le projet F-35A a largement dépassé ce stade, d'autant plus que notre opposition au F-35A n'a jamais été uniquement financière. Nous avons toujours contesté le choix de cet appareil, un avion extrêmement complexe dépendant des États-Unis pour son exploitation et son évolution, conçu pour opérer au sein d'un dispositif militaire intégré qui n'est pas celui de la Suisse. Aujourd'hui, à ces critiques stratégiques s'ajoute un fiasco dans la conduite de son acquisition.
+Il y a également une contradiction plus fondamentale dans la politique que nous menons. Nous parlons de sécurité comme si elle se mesurait au nombre de milliards de francs consacrés à l'armement, mais la sécurité de la Suisse ne commence pas lorsqu'un missile franchit notre frontière. Elle commence bien avant. Elle se construit lorsque nous empêchons les conflits de naître et de s'étendre, lorsque nous défendons le droit international, lorsque nous investissons dans la coopération internationale, dans la diplomatie et dans la promotion de la paix, lorsque nous luttons contre le dérèglement climatique qui multiplie les crises et les déplacements des populations, lorsque nous renforçons notre capacité à faire face aux cyberattaques, à la désinformation et aux nouveaux risques liés à l'intelligence artificielle. C'est cela aussi la politique de sécurité. Dans ces domaines, la tendance est exactement inverse. Alors que l'objectif de 1 pour cent du PIB pour l'armée doit être atteint toujours plus rapidement, la part consacrée à la coopération internationale recule. Toujours plus pour réagir aux conflits, toujours moins pour contribuer à les prévenir : ce déséquilibre est une erreur stratégique. Nous le répétons : le groupe des Verts ne nie pas la détérioration de la situation sécuritaire. Au contraire, c'est précisément parce que les ressources sont limitées et que les menaces augmentent que nous devons les investir là où elles apportent réellement davantage de sécurité, c'est-à-dire dans la cyberdéfense, dans la résilience de nos infrastructures et dans la coopération internationale et la diplomatie, mais pas obstinément dans un projet de F-35A dont chaque nouveau chapitre vient confirmer les erreurs du précédent.
+La sécurité ne se mesure pas au prix du matériel que nous achetons. Elle se mesure à notre capacité à identifier les menaces, à faire les bons choix et à utiliser intelligemment les moyens à disposition. Sur ce dernier élément, le dossier F-35A devrait nous inciter à une certaine humilité. Notre groupe entrera donc en matière sur les arrêtés fédéraux 1 et 2, tout en les examinant de manière critique. Mais concernant l'arrêté fédéral 3 et les 394 millions de francs supplémentaires destinés au F-35A, notre position est claire : après les erreurs, les dissimulations, les approximations et les défaillances de conduite révélées dans ce dossier, notre réponse ne peut pas être de mettre à nouveau simplement 394 millions sur la table. 
+Nous refuserons donc l'entrée en matière sur l'arrêté fédéral 3.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">418941</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Würth Benedikt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5. März 2026 in der abgeänderten Fassung an.
+Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5. März 2026 in der abgeänderten Fassung an.
+Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585, "Aktionsplan zur Reduktion der Belastung von Mensch und Umwelt durch langlebige Chemikalien". Diesen Bericht haben wir in der Kommission ebenfalls einlässlich diskutiert. Auf dessen Basis haben wir zahlreiche Zusatzfragen an die Verwaltung übermittelt, in Kenntnis der Antworten haben wir dann die vorliegenden Vorstösse behandelt. Es geht hier nur um die Vorstösse im Zuständigkeitsbereich des EDI, also um die Motion Michel Matthias, die Motion Vincenz und um die Motion Rechsteiner Thomas. Es gibt dann noch weitere Motionen, die im Zuständigkeitsbereich des UVEK sind: die Motionen Moser, Graf Maya, Crevoisier Crelier, Silberschmidt und Mühlemann. Ich sage das darum, weil wir in der Kommission alle als Gesamtpaket angeschaut haben. Wir sagten insgesamt, dass eigentlich alle Themen, die in diesen Motionen adressiert werden, bereits von der Motion 25.3421 der UREK-S umfasst sind, weshalb wir alle diese Motionen zur Ablehnung empfehlen. Auch die Verwaltung sagte klar, dass im Grunde genommen alle Themen bereits jetzt in Bearbeitung seien und grundsätzlich keine neuen Vorstösse mehr erforderlich seien; auch der Bundesrat beantragt alle diese Vorstösse zur Ablehnung.
+Wie sieht nun grosso modo die Pipeline aus? Was ist in diesem Bereich in Bearbeitung? Der Bund wird im kommenden Herbst die Vernehmlassung im Rahmen der Umsetzung der Motion Maret Marianne 22.3929, "Festlegung von PFAS-spezifischen Werten in Verordnungen", eröffnen. Verbindliche Grenzwerte für Aushub und Abfall werden Teil der entsprechenden Vorlage sein. Im Winter wird die Verwaltung dann Grenzwerte für den Boden festlegen.
+Wir haben auch die Frage der Steuerung dieses ganzen Themas diskutiert. Der Bundesrat hat zwar nicht einen formellen bundesrätlichen Ausschuss für PFAS eingesetzt, aber es finden regelmässige Treffen zum Thema Pflanzenschutzmittel zwischen der Vorsteherin des EDI und den Vorstehern von WBF und UVEK statt. In diesem Rahmen werden auch die Themen rund um PFAS diskutiert. Auf Ebene der Verwaltung gibt es eine Projektorganisation, welche insbesondere die Umsetzung des Postulates Moser an die Hand nimmt. In dieser Projektorganisation arbeiten die genannten Departemente und auch die Kantone eng zusammen.
+Möglicherweise haben Sie auch von den Beschlüssen des Bundesrates vom 27. Mai 2026 Kenntnis genommen. Damit wurde die Vernehmlassung zur erwähnten Motion 25.3421 der UREK-S ausgelöst. PFAS-Betriebe sollen mehr Zeit für eine Produktionsumstellung erhalten und währenddessen weiterhin ein wirtschaftliches Auskommen erzielen können - das war ein Kernelement dieser Motion. Gleichzeitig beschloss der Bundesrat, PFAS-belastete Betriebe in Härtefällen finanziell zu unterstützen. Diesbezüglich gab es eine Aussprache, und bis März 2027 soll ein Entwurf für ein zeitlich begrenztes Spezialgesetz in die Vernehmlassung gehen. Es ist damit zu rechnen, dass im Jahr 2028 hier Rechtsgrundlagen bestehen werden.
+Parallel dazu hat das BLV - nicht der Bundesrat - eine Weisung erlassen, um den einheitlichen Vollzug der PFAS-Höchstgehalte durch die Kantone sicherzustellen - ich werde noch darauf zu sprechen kommen. Das hat wahrscheinlich mehr Probleme geschaffen als gelöst.
+In der Kommission wurde im Wesentlichen die Frage diskutiert, wie mit den belasteten Böden umzugehen ist. Da wir uns im Bereich des Altlastenrechtes befinden, stellen sich Fragen der Sanierung, des Verursacherprinzips sowie der Finanzierung.
+Wie erwähnt, beabsichtigt das BAFU, im Zuge der Umsetzung der Motion Maret Marianne entsprechende Grenzwerte zu definieren. In der Vergangenheit fand dazu eine Diskussion mit der Branche statt. Ursprünglich waren die entsprechenden Werte sehr tief angesetzt, was zu erheblichen Problemen führte. Mittlerweile wurden diese Grenzwerte erhöht und sind nach Aussage der Verwaltung toxikologisch weiterhin vertretbar. Zudem wird ein Spezialgesetz für betriebliche Härtefälle geschaffen.
+Insbesondere stellt sich natürlich auch die Frage, wie rein technisch mit diesen belasteten Böden umzugehen ist. Man kann diese Böden nicht einfach vollumfänglich von PFAS befreien, da sonst kein Humus mehr vorhanden wäre und der Boden tot ist. Man befindet sich im Prinzip in einer erheblichen Zwickmühle.
+Auch die bereits erwähnte Finanzierung ist komplex. Eigentlich wäre der Vasa-Fonds das Instrument, um die Sanierung von Altlasten zu alimentieren und zu finanzieren. Dieser ist jedoch nicht für solche Situationen ausgerichtet, da bei mit Klärschlamm belasteten Böden kein Anspruch auf Mittel des Vasa-Fonds besteht. Dies ist ein nach wie vor ungelöstes Problem. Die EFK hat der Verwaltung im Rahmen einer Querschnittprüfung empfohlen, Abklärungen zum Verursacherprinzip durchzuführen; diese laufen derzeit. Das Verursacherprinzip muss im Umweltrecht sehr unmittelbar sein. Seine Anwendung ist im Falle von Belastungen, deren Ursachen zwanzig oder dreissig Jahre zurückliegen, relativ schwierig, weshalb die Verursacher oftmals nicht mehr direkt belangt werden können. Die Kommission hat jedoch verlangt, dass ihr die Resultate der Abklärungen zum Verursacherprinzip wieder unterbreitet werden. Dies stellt eine weitere Pendenz in diesem Kontext dar.
+Summa summarum: Vieles befindet sich in der Pipeline, weshalb es nicht sinnvoll ist, neue Vorstösse zu überweisen. Deshalb haben wir die Motionen Rechsteiner Thomas 25.3906 sowie Vincenz 25.3902 jeweils mit 10 zu 2 Stimmen abgelehnt. Die Motion Michel Matthias 25.3866 wurde einstimmig abgelehnt, da es sich dabei um einen gleichlautenden Vorstoss handelt und insofern keine materielle Änderung im Raum steht. Alle weiteren Vorstösse werden voraussichtlich am 1. Oktober im Rat behandelt. Ich werde Ihnen dann im Wesentlichen wieder kurz und bündig die gleiche Ausgangslage darlegen bzw. mich kurzfassen, um mich nicht zu wiederholen.
+Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen an die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
+Namens der Kommission bitte ich Sie, auf die drei erwähnten Vorstösse nicht einzutreten bzw. diese abzulehnen.
 </t>
   </si>
 </sst>
@@ -133,8 +199,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I3" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -517,6 +583,64 @@
         <v>22</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-16
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -151,6 +151,43 @@
 Summa summarum: Vieles befindet sich in der Pipeline, weshalb es nicht sinnvoll ist, neue Vorstösse zu überweisen. Deshalb haben wir die Motionen Rechsteiner Thomas 25.3906 sowie Vincenz 25.3902 jeweils mit 10 zu 2 Stimmen abgelehnt. Die Motion Michel Matthias 25.3866 wurde einstimmig abgelehnt, da es sich dabei um einen gleichlautenden Vorstoss handelt und insofern keine materielle Änderung im Raum steht. Alle weiteren Vorstösse werden voraussichtlich am 1. Oktober im Rat behandelt. Ich werde Ihnen dann im Wesentlichen wieder kurz und bündig die gleiche Ausgangslage darlegen bzw. mich kurzfassen, um mich nicht zu wiederholen.
 Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen an die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
 Namens der Kommission bitte ich Sie, auf die drei erwähnten Vorstösse nicht einzutreten bzw. diese abzulehnen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">419420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260916</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revaz Estelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités : vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités : vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en situation de handicap est donc un véritable sujet de société. Cela concerne près d'une personne sur cinq dans notre pays et, à ce titre, nous concerne toutes et tous.
+L'initiative pour l'inclusion traduit un constat et une impatience. Le constat, c'est que malgré les progrès accomplis, la Suisse accuse encore un retard important dans la mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées. L'impatience, parfaitement compréhensible, est celle des personnes concernées et de leurs organisations qui attendent des avancées concrètes depuis trop longtemps.
+L'initiative nous rappelle ainsi le chemin qu'il reste à parcourir pour faire de l'inclusion une réalité. Elle demande l'égalité de droit et de fait des personnes en situation de handicap dans tous les domaines de la vie. Elle vise notamment à garantir le libre choix du logement et à inscrire dans la Constitution un droit à des mesures de soutien et d'adaptation.
+La majorité de la commission comprend ces préoccupations, mais estime que la modification constitutionnelle proposée n'est pas adéquate. Celle-ci n'apporterait en effet pas d'amélioration significative par rapport au droit actuel et soulèverait des difficultés de mise en oeuvre. La commission propose donc de rejeter l'initiative, par 16 voix contre 8.
+La majorité de votre commission rejoint cependant les auteurs de l'initiative sur un point essentiel : il est nécessaire d'agir. Elle salue donc le contre-projet indirect proposé par le Conseil fédéral et, par 17 voix contre 8, a décidé d'entrer en matière. Une minorité propose de ne pas entrer en matière. Si cette proposition est rejetée, la même minorité demande le renvoi du projet au Conseil fédéral et formule plusieurs pistes de modifications.
+Nous avons mené de longues discussions sur la portée du contre-projet indirect. Pour les auteurs de l'initiative comme pour la majorité de votre commission, il contient beaucoup de dispositions déclaratoires et peu de mesures concrètes. La majorité de votre commission a donc souhaité renforcer le contre-projet indirect et s'éloigner d'une loi essentiellement programmatique, en agissant dans les domaines essentiels de la vie quotidienne. Il ne s'agit pas d'inventer de nouveaux droits, mais de permettre aux personnes en situation de handicap de bénéficier concrètement des mêmes droits et des mêmes possibilités que les autres. Enfin, la commission a souhaité clarifier les responsabilités et renforcer la coordination avec les cantons, qui jouent un rôle central dans la mise en oeuvre de nombreuses mesures.
+Afin d'avoir une vision globale des mesures en faveur de l'égalité des personnes en situation de handicap, la commission a décidé, à l'unanimité, d'examiner l'objet 25.020 "Loi sur l'égalité pour les handicapés. Modification" en parallèle de la loi sur l'inclusion qui constitue le contre-projet indirect du Conseil fédéral à l'initiative. Elle a en revanche décidé, par 14 voix contre 10 et 1 abstention, de traiter séparément la question des langues des signes dans une loi spécifique. Ce sera l'objet de l'initiative parlementaire 26.404 qui vous sera très prochainement soumise.
+Des mesures concrètes ont ainsi été proposées autour de quatre axes : le libre choix du logement, l'intégration sur le marché du travail, la participation à la vie culturelle, aux loisirs et au sport, ainsi que les prestations d'assistance. Pour agir dans ces différents domaines, votre commission a travaillé sur pas moins de sept lois différentes : la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, la loi fédérale sur des mesures de promotion civile de la paix et de renforcement des droits de l'homme, la loi fédérale sur l'assurance-invalidité, la loi fédérale sur l'élimination des inégalités frappant les personnes handicapées, la loi sur les langues, la loi sur l'organisation du gouvernement et de l'administration et, enfin, la loi fédérale sur l'encouragement des hautes écoles et la coordination dans le domaine suisse des hautes écoles.
+Étant donné l'organisation du débat et le temps limité dont dispose la commission pour vous présenter les dizaines de propositions qui sont encore en discussion, je vais passer dès maintenant à l'examen de détail sans m'appesantir sur les points qui n'ont pas rencontré d'opposition.
+Je commence donc par la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, aussi appelée loi sur l'inclusion (LIncl), et je commence à l'article 2. 
+La loi sur l'inclusion est une loi-cadre qui doit donner une orientation politique claire. Par 14 voix contre 8 et 3 abstentions, votre commission propose donc de renforcer cet article sans lui donner une portée juridique qu'il ne pourrait avoir. Une minorité souhaite aller plus loin, tandis qu'une autre préfère s'en tenir à la proposition du Conseil fédéral. 
+À l'article 3, votre commission a souhaité clarifier la relation avec le droit cantonal, mais aussi mentionner explicitement l'importance de la collaboration entre la Confédération et les cantons. Convaincue qu'il est important de réaffirmer la nécessité d'agir, votre commission, par 12 voix contre 11, a accepté cet ajout. Une minorité s'y oppose. 
+À l'article 5, l'objectif est simple : faire en sorte que la stratégie nationale de mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées (CDPH) ne reste pas un document d'intention, mais débouche sur des mesures concrètes. Par 11 voix contre 8 et 5 abstentions, la majorité de votre commission souhaite renforcer les objectifs en matière d'autodétermination, de liberté de choix et de participation à la vie sociale. Une minorité souhaite suivre le Conseil fédéral. 
+À l'article 6 alinéas 4 et 5, il s'agit d'inscrire les projets pilotes dans la loi. Ces derniers permettent de tester concrètement les mesures prévues dans la stratégie et les plans d'action et d'identifier celles qui fonctionnent. Ces modifications ont été adoptées par 13 voix contre 10 et 2 abstentions. Il n'y a pas de proposition de minorité. 
+À l'article 8, la majorité souhaite impliquer les personnes en situation de handicap dès l'élaboration de la stratégie et des plans d'action. Leur expérience permet d'identifier les besoins en amont et d'éviter des corrections qui seraient ultérieurement plus coûteuses. Cette proposition a été adoptée par 13 voix contre 8 et 3 abstentions. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
+À l'article 11, la majorité souhaite renforcer l'autonomie des personnes en situation de handicap dans le choix de leur logement. Pour cela, elle propose notamment d'améliorer l'information et la coordination ; un élément également relevé par le Contrôle fédéral des finances. Ces modifications ont été adoptées par 14 voix contre 10. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
+À l'article 11a, l'objectif est de renforcer l'autonomie économique des personnes en situation de handicap en facilitant leur accès au marché du travail. Leur potentiel reste insuffisamment exploité, alors que la Suisse manque de main-d'oeuvre qualifiée et que l'assurance-invalidité (AI) fait face à des difficultés financières. Par 16 voix contre 8, votre commission a accepté cette proposition. 
+À l'article 11b, il s'agit de favoriser la participation des personnes en situation de handicap à la vie culturelle, aux loisirs, au sport et aux activités politiques. Par 14 voix contre 11, la majorité de votre commission souhaite inscrire cet objectif dans la loi sans que cela entraîne automatiquement de nouvelles dépenses. Une minorité la juge inopportune. 
+À l'article 11c, l'objectif est de renforcer la liberté de choix des personnes en situation de handicap en adaptant mieux les prestations d'assistance à leur réalité de vie et en améliorant leur coordination. Par 13 voix contre 11 et 1 abstention, votre commission veut inscrire cette orientation dans la loi. Une minorité estime qu'elle fait doublon avec les travaux annoncés concernant l'AI. 
+À l'article 12, l'objectif est de disposer de données fiables sur l'accessibilité des bâtiments, des installations et des logements. Ces données sont indispensables pour identifier les besoins et agir de manière ciblée. Par 13 voix contre 9 et 3 abstentions, la majorité de votre commission a décidé d'inscrire cet ajout dans la loi. Une minorité veut s'en tenir à la version du Conseil fédéral. 
+La majorité de votre commission souhaite également introduire une section 4a sur les mesures transitoires. À l'article 12a, elle propose un délai de 8 ans pour la mise en oeuvre de la loi par la Confédération et les cantons. Au regard des délais prévus dans d'autres lois, ce délai lui paraît à la fois réaliste et nécessaire. Elle souhaite également mettre l'accent sur le libre choix du logement qui est au coeur de l'initiative populaire. Cette proposition a été adoptée par 17 voix contre 6. Une minorité s'y oppose. 
+Je continuerai au milieu du bloc 2 pour vous rendre compte en détail des autres modifications des autres actes, puisque, comme je vous l'ai dit, on a travaillé sur sept lois différentes. Il y a donc encore du travail sur la planche.
 </t>
   </si>
 </sst>
@@ -199,8 +236,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -641,6 +678,35 @@
         <v>37</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-21
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -62,7 +62,7 @@
     <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà é</t>
   </si>
   <si>
-    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà épuisées. Les personnes concernées peuvent demander à leur assureur-maladie le remboursement du montant différentiel. Si les assurés ne font pas valoir activement leur avoir auprès de la caisse-maladie, les assureurs peuvent renoncer à un remboursement lorsque celui-ci engendrerait une charge disproportionnée. Tel est le cas, par exemple, lorsque les assurés ne peuvent pas être contactés malgré des efforts avérés, ou encore en présence de montants minimes lorsque les frais de traitement excèdent les montants à rembourser. Lorsque les restitutions ne sont pas utilisées pour réduire la participation aux coûts, elles diminuent le coût des prestations. Cela améliore le résultat actuariel global et conduit, au final, à des primes moins élevées. Néanmoins j'en conviens, Monsieur le conseiller national, ce qui compte, c'est la traçabilité des montants et la transparence - nous l'avons vu également dans le rapport du Contrôle fédéral des finances. Par votre motion, vous demandez plus de transparence et de traçabilité. Le Conseil fédéral estime que les restitutions doivent bénéficier aux personnes assurées, tout comme vous, mais il estime que la LAMal le permet d'ores et déjà.
+    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà épuisées. Les personnes concernées peuvent demander à leur assureur-maladie le remboursement du montant différentiel. Si les assurés ne font pas valoir activement leur avoir auprès de la caisse-maladie, les assureurs peuvent renoncer à un remboursement lorsque celui-ci engendrerait une charge disproportionnée. Tel est le cas, par exemple, lorsque les assurés ne peuvent pas être contactés malgré des efforts avérés, ou encore en présence de montants minimes lorsque les frais de traitement excèdent les montants à rembourser. Lorsque les restitutions ne sont pas utilisées pour réduire la participation aux coûts, elles diminuent le coût des prestations. Cela améliore le résultat actuariel global et conduit, au final, à des primes moins élevées. Néanmoins, j'en conviens, Monsieur le conseiller national, ce qui compte, c'est la traçabilité des montants et la transparence - nous l'avons vu également dans le rapport du Contrôle fédéral des finances. Par votre motion, vous demandez plus de transparence et de traçabilité. Le Conseil fédéral estime que les restitutions doivent bénéficier aux personnes assurées, tout comme vous, mais il estime que la LAMal le permet d'ores et déjà.
 C'est pourquoi il demande le rejet de la motion.
 </t>
   </si>
@@ -83,7 +83,7 @@
   </si>
   <si>
     <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir ? C'est la question centrale de cette motion. Son point de départ est concret : une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, la destination des sommes récupérées relève pleinement de notre responsabilité politique, car cet argent a été financé par les assurés, par leurs primes, mais également par leur franchise et leur quote-part. Le Conseil fédéral estime que ma motion est inutile. Selon son avis, les sommes récupérées améliorent le résultat technique des assureurs et peuvent ainsi contribuer à réduire les primes, mais une possibilité de baisse future n'est pas une garantie de restitution. Lorsqu'un assuré a personnellement supporté une partie d'une facture, ensuite corrigée, où apparaît cette correction ? Comment sa participation est-elle recalculée ? Comment s'assure-t-on que la somme correspondante lui revient ? Pour les montants financés collectivement par les primes, comment démontre-t-on qu'ils bénéficient effectivement aux assurés, au lieu de simplement alimenter les réserves ? Voilà les questions auxquelles il faut répondre.
-L'interdiction de distribuer des bénéfices invoquée par le Conseil fédéral ne suffit pas. Elle ne démontre ni à qui les montants récupérés bénéficient, ni quand, ni comment. Une écriture comptable favorable à l'assureur ne prouve pas à elle seule une restitution à l'assuré. Cette motion s'inscrit dans la continuité de mon travail parlementaire, notamment de la motion 24.3060 sur le contrôle des finances des caisses-maladie. Rabais, rétrocessions ou remboursements de prestations : les mécanismes diffèrent, mais l'exigence demeure. Nous devons pouvoir tracer l'argent et vérifier qu'il bénéficie à ceux qui financent l'assurance obligatoire. Les travaux du Contrôle fédéral des finances renforcent cette exigence de transparence et de contrôle. Les médecins qui assurent les consultations le soir et le week-end rendent un service indispensable et les assureurs doivent appliquer les décisions judiciaires, mais il reste à garantir que les conséquences financières soient correctement répercutées jusqu'aux assurés. La récupération de l'argent ne doit pas être la dernière étape. Sa restitution doit être l'objectif. Les assurés paient leurs primes, leur franchise et leur quote-part. Ces obligations sont précises et leurs échéances aussi. Ils sont en droit d'attendre la même précision lorsqu'une somme doit leur revenir.
+L'interdiction de distribuer des bénéfices invoquée par le Conseil fédéral ne suffit pas. Elle ne démontre ni à qui les montants récupérés bénéficient, ni quand, ni comment. Une écriture comptable favorable à l'assureur ne prouve pas à elle seule une restitution à l'assuré. Cette motion s'inscrit dans la continuité de mon travail parlementaire, notamment de la motion 24.3060 sur le contrôle des finances des caisses-maladie. Rabais, rétrocessions ou remboursements de prestations, les mécanismes diffèrent, mais l'exigence demeure. Nous devons pouvoir tracer l'argent et vérifier qu'il bénéficie à ceux qui financent l'assurance obligatoire. Les travaux du Contrôle fédéral des finances renforcent cette exigence de transparence et de contrôle. Les médecins qui assurent les consultations le soir et le week-end rendent un service indispensable et les assureurs doivent appliquer les décisions judiciaires, mais il reste à garantir que les conséquences financières soient correctement répercutées jusqu'aux assurés. La récupération de l'argent ne doit pas être la dernière étape. Sa restitution doit être l'objectif. Les assurés paient leurs primes, leur franchise et leur quote-part. Ces obligations sont précises et leurs échéances aussi. Ils sont en droit d'attendre la même précision lorsqu'une somme doit leur revenir.
 Je vous demande donc d'adopter cette motion pour garantir une traçabilité des montants récupérés, la correction des participations individuelles concernées et une répercussion effective au bénéfice des assurés. Au-delà de cette taxe de 40 francs, nous défendons un principe essentiel : l'argent récupéré dans l'assurance obligatoire doit bénéficier aux assurés de manière concrète, transparente et vérifiable.
 </t>
   </si>
@@ -188,6 +188,50 @@
 À l'article 12, l'objectif est de disposer de données fiables sur l'accessibilité des bâtiments, des installations et des logements. Ces données sont indispensables pour identifier les besoins et agir de manière ciblée. Par 13 voix contre 9 et 3 abstentions, la majorité de votre commission a décidé d'inscrire cet ajout dans la loi. Une minorité veut s'en tenir à la version du Conseil fédéral. 
 La majorité de votre commission souhaite également introduire une section 4a sur les mesures transitoires. À l'article 12a, elle propose un délai de 8 ans pour la mise en oeuvre de la loi par la Confédération et les cantons. Au regard des délais prévus dans d'autres lois, ce délai lui paraît à la fois réaliste et nécessaire. Elle souhaite également mettre l'accent sur le libre choix du logement qui est au coeur de l'initiative populaire. Cette proposition a été adoptée par 17 voix contre 6. Une minorité s'y oppose. 
 Je continuerai au milieu du bloc 2 pour vous rendre compte en détail des autres modifications des autres actes, puisque, comme je vous l'ai dit, on a travaillé sur sept lois différentes. Il y a donc encore du travail sur la planche.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260921</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rossi Viktor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, wo wir noch besser werden können und müssen.
+Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut, dass </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, wo wir noch besser werden können und müssen.
+Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut, dass die EFK teilweise auch positive Aspekte feststellt, auch wenn diese in den Auseinandersetzungen mit den Berichten manchmal etwas untergehen. So erlaube ich mir zu erwähnen, dass die überwiegende Mehrheit der IKT-Projekte mit Erfolg abgeschlossen werden. In den letzten zwei Jahren haben wir in der Bundesverwaltung rund 200 Projekte mit einem Budget von über 400 000 Franken abgeschlossen, und rund 85 Prozent dieser Projekte wurden sowohl in der Zeit wie auch im Budget abgeschlossen. Aber nochmals, ich gehe mit Ihnen und auch mit der EFK einig: Das darf nicht unsere Ambition und unser Anspruch sein, da müssen wir besser werden.
+Ich versuche, die eine oder andere Frage zu beantworten. Ich werde, wie von Ihnen angeboten, dann sehr gerne noch schriftlich auf die verschiedenen Fragen eingehen.
+Zum Projektleiterpool: Sie haben es erwähnt, 2014 forderten zwei gleichlautende Motionen der Finanzkommissionen beider Räte, dass der Bundesrat einen Projektleiterpool für Schlüsselprojektleiter aufbaut. Dieser Pool besteht aus drei Personen. Wenn wir alle 21 laufenden Schlüsselprojekte abdecken und auch für neue Schlüsselprojekte bereit sein möchten, dann müssten wir den Pool auf mindestens 25 Personen ausweiten. Das wäre eine massive Aufstockung gegenüber heute. Deshalb werden diese Leistungen teilweise von externen Personen wahrgenommen oder die Positionen durch bundesverwaltungsinterne Mitarbeitende besetzt.
+Ich komme zu den Assessments. Hier ist die Bundeskanzlei im Sinne einer übergreifenden Koordination der digitalen Transformation bei Schlüsselprojekten aktiv Folgendes angegangen: Wir haben in den vergangenen zwei Jahren bei rund 14 Grossprojekten ein Assessment durchgeführt. Ich bin der Meinung, das hat Wirkung gezeigt. In rund zwei Drittel der Fälle hat die Bundeskanzlei Empfehlungen abgegeben oder Bedingungen gestellt. Hauptsächlich ging es dabei um Konkretisierungen der Kontrollmechanismen oder um die Forderung, die unabhängige Qualitätssicherung rascher zu besetzen und nicht erst nach Ablauf der Initialisierungsphase.
+Zur Begleitung der Projekte in der Initialisierungsphase: Das ist auch aus meiner Sicht und aus Sicht des Bundesrates wichtig und richtig, und das ist auch entsprechend aufgesetzt. Die Bundeskanzlei wird dem Bundesrat bis Ende dieses Jahres Grundlagen zur Weiterentwicklung der Gouvernanz der digitalen Transformation vorlegen. Ein Kernstück dieser Weiterentwicklung bildet die Erteilung der Kompetenz an die Bundeskanzlei, in der Initialisierungsphase Synergieprüfungen durchzuführen, damit sichergestellt ist, dass in neuen Vorhaben nicht plötzlich Dinge beschafft oder entwickelt werden, die wir bereits im Einsatz haben. Ein Beispiel, das Sie wahrscheinlich kennen, ist das mittlerweile schweizweit im Einsatz stehende Behördenlogin Agov. In dem Sinn und Geist versuchen wir auch hier vorwärts zu machen, um Kosten und Zeit zu sparen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salzmann Werner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich nur teilweise davon befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
+Zur Antwort 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie andererseits zu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich nur teilweise davon befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
+Zur Antwort 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie andererseits zur Unterstützung der Departemente beiziehen zu können. Haben die Departemente diese Möglichkeit genutzt? Wenn ja, welche Projektprobleme konnten nachweislich verhindert werden? Wie wird konkret gemessen, ob der Expertenpool die Mängel in der Initialisierungsphase reduziert hat? Gibt es Kennzahlen zu Projekten mit oder ohne Poolunterstützung? 
+Zur Antwort 2: Die Möglichkeit, Projektassessments durchzuführen, gibt es seit 2015. Eine Bilanz sollte daher über die Projekte gezogen werden, die sich jetzt in der Realisierungsphase befinden. Dazu habe ich folgende Nachfragen: Werden die richtigen Themen und Risiken im Assessment untersucht? Würden Sie sagen, dass ein Projekt ohne Assessment häufiger in Schwierigkeiten gerät? Wenn ja, warum? Gehen die Prüfer genügend auf die Besonderheiten des jeweiligen Projektes ein? Wie fundiert und aussagekräftig sind die Ergebnisse des Assessments aus Ihrer Sicht? Werden die Erkenntnisse aus den Assessments auch für andere Projekte genutzt? Lernt die Organisation aus wiederkehrenden Erkenntnissen und Problemen des Assessments? 
+Zur Antwort 3: Die ursprüngliche Frage zielt auf eine obligatorische Begleitung der Projektteams, das heisst, auf Übungsebene und nicht auf Steuerungsebene hin. Wurden somit unabhängig von der Synergieprüfung Modelle geprüft oder pilotiert, die die Projektteams während der Initialisierungsphase begleiten oder beraten? 
+Zum Schluss stellen sich für mich noch generelle Fragen, zu denen ich gerne eine Antwort hätte, nämlich: Warum greifen bestehende Instrumente nicht? Welche Massnahmen sind erforderlich, wenn sich bereits 2016 erkannte Probleme wiederholen? Wenn die Instrumente funktionieren, warum benötigen wir sie nach 10 Jahren noch in nahezu unveränderter Form? Woran lässt sich objektiv erkennen, dass diese Instrumente nicht nur zusätzliche Kontrolle erzeugen, sondern dass sich die Qualität der Projekte tatsächlich verbessert hat? 
+Die Eidgenössische Finanzkontrolle weist regelmässig auf diese Schwachstellen in grossen IKT-Vorhaben der Bundesverwaltung hin. Ein wesentlicher Teil dieser Feststellung deutet darauf hin, dass grundlegende Voraussetzungen bereits in der Projektinitialisierung unzureichend geklärt und vorbereitet wurden. Mir geht es darum, dass wir hier einen merklichen Fortschritt erzielen und IKT-Projekte in der Bundesverwaltung von Anfang an auf den richtigen Weg bringen. Daher, sehr geehrter Herr Bundeskanzler, wäre ich Ihnen dankbar, wenn Sie meine Fragen heute, aber auch schriftlich beantworten können. Besten Dank.
 </t>
   </si>
 </sst>
@@ -236,8 +280,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -707,6 +751,62 @@
         <v>42</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7"/>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-22
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -79,12 +79,12 @@
     <t xml:space="preserve">GE</t>
   </si>
   <si>
-    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir ? C'est la question centrale de cette motion. Son point de départ est concret : une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir ? C'est la question centrale de cette motion. Son point de départ est concret : une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, la destination des sommes récupérées relève pleinement de notre responsabilité politique, car cet argent a été financé par les assurés, par leurs primes, mais également par leur franchise et leur quote-part. Le Conseil fédéral estime que ma motion est inutile. Selon son avis, les sommes récupérées améliorent le résultat technique des assureurs et peuvent ainsi contribuer à réduire les primes, mais une possibilité de baisse future n'est pas une garantie de restitution. Lorsqu'un assuré a personnellement supporté une partie d'une facture, ensuite corrigée, où apparaît cette correction ? Comment sa participation est-elle recalculée ? Comment s'assure-t-on que la somme correspondante lui revient ? Pour les montants financés collectivement par les primes, comment démontre-t-on qu'ils bénéficient effectivement aux assurés, au lieu de simplement alimenter les réserves ? Voilà les questions auxquelles il faut répondre.
+    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir[NB]? C'est la question centrale de cette motion. Son point de départ est concret[NB]: une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En reva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir[NB]? C'est la question centrale de cette motion. Son point de départ est concret[NB]: une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, la destination des sommes récupérées relève pleinement de notre responsabilité politique, car cet argent a été financé par les assurés, par leurs primes, mais également par leur franchise et leur quote-part. Le Conseil fédéral estime que ma motion est inutile. Selon son avis, les sommes récupérées améliorent le résultat technique des assureurs et peuvent ainsi contribuer à réduire les primes, mais une possibilité de baisse future n'est pas une garantie de restitution. Lorsqu'un assuré a personnellement supporté une partie d'une facture, ensuite corrigée, où apparaît cette correction[NB]? Comment sa participation est-elle recalculée[NB]? Comment s'assure-t-on que la somme correspondante lui revient[NB]? Pour les montants financés collectivement par les primes, comment démontre-t-on qu'ils bénéficient effectivement aux assurés, au lieu de simplement alimenter les réserves[NB]? Voilà les questions auxquelles il faut répondre.
 L'interdiction de distribuer des bénéfices invoquée par le Conseil fédéral ne suffit pas. Elle ne démontre ni à qui les montants récupérés bénéficient, ni quand, ni comment. Une écriture comptable favorable à l'assureur ne prouve pas à elle seule une restitution à l'assuré. Cette motion s'inscrit dans la continuité de mon travail parlementaire, notamment de la motion 24.3060 sur le contrôle des finances des caisses-maladie. Rabais, rétrocessions ou remboursements de prestations, les mécanismes diffèrent, mais l'exigence demeure. Nous devons pouvoir tracer l'argent et vérifier qu'il bénéficie à ceux qui financent l'assurance obligatoire. Les travaux du Contrôle fédéral des finances renforcent cette exigence de transparence et de contrôle. Les médecins qui assurent les consultations le soir et le week-end rendent un service indispensable et les assureurs doivent appliquer les décisions judiciaires, mais il reste à garantir que les conséquences financières soient correctement répercutées jusqu'aux assurés. La récupération de l'argent ne doit pas être la dernière étape. Sa restitution doit être l'objectif. Les assurés paient leurs primes, leur franchise et leur quote-part. Ces obligations sont précises et leurs échéances aussi. Ils sont en droit d'attendre la même précision lorsqu'une somme doit leur revenir.
-Je vous demande donc d'adopter cette motion pour garantir une traçabilité des montants récupérés, la correction des participations individuelles concernées et une répercussion effective au bénéfice des assurés. Au-delà de cette taxe de 40 francs, nous défendons un principe essentiel : l'argent récupéré dans l'assurance obligatoire doit bénéficier aux assurés de manière concrète, transparente et vérifiable.
+Je vous demande donc d'adopter cette motion pour garantir une traçabilité des montants récupérés, la correction des participations individuelles concernées et une répercussion effective au bénéfice des assurés. Au-delà de cette taxe de 40 francs, nous défendons un principe essentiel[NB]: l'argent récupéré dans l'assurance obligatoire doit bénéficier aux assurés de manière concrète, transparente et vérifiable.
 </t>
   </si>
   <si>
@@ -232,6 +232,48 @@
 Zur Antwort 3: Die ursprüngliche Frage zielt auf eine obligatorische Begleitung der Projektteams, das heisst, auf Übungsebene und nicht auf Steuerungsebene hin. Wurden somit unabhängig von der Synergieprüfung Modelle geprüft oder pilotiert, die die Projektteams während der Initialisierungsphase begleiten oder beraten? 
 Zum Schluss stellen sich für mich noch generelle Fragen, zu denen ich gerne eine Antwort hätte, nämlich: Warum greifen bestehende Instrumente nicht? Welche Massnahmen sind erforderlich, wenn sich bereits 2016 erkannte Probleme wiederholen? Wenn die Instrumente funktionieren, warum benötigen wir sie nach 10 Jahren noch in nahezu unveränderter Form? Woran lässt sich objektiv erkennen, dass diese Instrumente nicht nur zusätzliche Kontrolle erzeugen, sondern dass sich die Qualität der Projekte tatsächlich verbessert hat? 
 Die Eidgenössische Finanzkontrolle weist regelmässig auf diese Schwachstellen in grossen IKT-Vorhaben der Bundesverwaltung hin. Ein wesentlicher Teil dieser Feststellung deutet darauf hin, dass grundlegende Voraussetzungen bereits in der Projektinitialisierung unzureichend geklärt und vorbereitet wurden. Mir geht es darum, dass wir hier einen merklichen Fortschritt erzielen und IKT-Projekte in der Bundesverwaltung von Anfang an auf den richtigen Weg bringen. Daher, sehr geehrter Herr Bundeskanzler, wäre ich Ihnen dankbar, wenn Sie meine Fragen heute, aber auch schriftlich beantworten können. Besten Dank.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420614</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ettlin Erich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Artikel 22a und 22b greifen Empfehlungen aus dem Bericht der Eidgenössischen Finanzkontrolle auf. In Artikel 22a wird ein Steuerungs- und Mitwirkungsgremium verankert, dessen Zusammensetzung benannt und dessen Aufgaben aufgeführt. Der Nationalrat hat die Bestimmung mit 131 zu 62 Stimmen angenommen. Ihre Kommission ist dem einstimmig gefolgt.
+Artikel 23b schreibt verbindliche Vorgaben zur Standardisierung der Schnittstellen, zur Interoperabilität und zur Verfassung der Verwaltungs- und IT-Kos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Artikel 22a und 22b greifen Empfehlungen aus dem Bericht der Eidgenössischen Finanzkontrolle auf. In Artikel 22a wird ein Steuerungs- und Mitwirkungsgremium verankert, dessen Zusammensetzung benannt und dessen Aufgaben aufgeführt. Der Nationalrat hat die Bestimmung mit 131 zu 62 Stimmen angenommen. Ihre Kommission ist dem einstimmig gefolgt.
+Artikel 23b schreibt verbindliche Vorgaben zur Standardisierung der Schnittstellen, zur Interoperabilität und zur Verfassung der Verwaltungs- und IT-Kosten vor. Auch diese Bestimmung wurde vom Nationalrat mit 131 zu 62 Stimmen und von unserer Kommission einstimmig angenommen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420637</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ausgangspunkt für dieses Postulat war ein Prüfbericht der Eidgenössischen Finanzkontrolle mit dem Titel "Evaluation der Mechanismen zur angemessenen Verwendung bildgebender Verfahren in der Medizin". Dieser Bericht stammt von Januar 2025. Darin ist festgehalten, mit einzelnen Beispielen, wie oft bildgebende Verfahren angewendet werden, teilweise zu oft, was natürlich Kostenfolgen hat.
+Ihre Kommission hat diesen Bericht an der Sitzung vom 25./26. Juni beraten und einstimmig beschlossen, das vorli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ausgangspunkt für dieses Postulat war ein Prüfbericht der Eidgenössischen Finanzkontrolle mit dem Titel "Evaluation der Mechanismen zur angemessenen Verwendung bildgebender Verfahren in der Medizin". Dieser Bericht stammt von Januar 2025. Darin ist festgehalten, mit einzelnen Beispielen, wie oft bildgebende Verfahren angewendet werden, teilweise zu oft, was natürlich Kostenfolgen hat.
+Ihre Kommission hat diesen Bericht an der Sitzung vom 25./26. Juni beraten und einstimmig beschlossen, das vorliegende Postulat einzureichen. Sie möchte mit dem Postulat beim Bundesrat Informationen zu verschiedenen Punkten einholen, Sie sehen die Auflistung: Wie viele Geräte sind vorhanden? Für was werden sie verwendet? Welche Kriterien müssen erfüllt sein, damit ein Gerät überhaupt angewendet wird? Werden die WZW-Kriterien angewendet? Haben sie auch einen Nutzen? Prüfen die Versicherer richtig? 
+Mit diesem Wissen möchten wir dann den Bericht der EFK sozusagen in politische Arbeit umsetzen. Wir müssen hier mehr wissen. Das ist der Grund für das Postulat. Es war, wie gesagt, in der Kommission unbestritten. 
+Ich bitte Sie daher, der Kommission zu folgen und dieses Postulat anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420571</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Contrôle fédéral des finances a publié un rapport en 2025 qui met en évidence le poids et l'existence de coûts potentiellement inutiles dans ce domaine. Le Conseil fédéral soutient le postulat de votre commission. Le domaine de l'imagerie médicale doit donc continuer à être suivi attentivement, afin que d'éventuelles évolutions problématiques soient identifiées rapidement et puissent surtout être corrigées.
 </t>
   </si>
 </sst>
@@ -280,8 +322,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -807,6 +849,91 @@
         <v>52</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11"/>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-23
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -103,15 +103,15 @@
     <t xml:space="preserve">NE</t>
   </si>
   <si>
-    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifie pas continuer comme si rien ne s'était passé au sein du DDPS.
-Au moment où ce Parlement s'apprête à voter 3,4 milliards de francs supplémentaires, dont 394 millions pour le F-35A, une question s'impose : pouvons-nous encore avoir confiance dans la manière dont le DDPS conduit ses grands projets d'armement ? La semaine dernière, la Commission de gestion nous a donné quelques éléments de réponse qui sont accablants. Pendant des années, on nous a répété que le prix du F-35A était fixe. Il ne l'est pas. On nous a affirmé que la Suisse avait négocié une garantie particulière avec les États-Unis. Cette garantie n'existe pas. Des doutes avaient été exprimés par le Contrôle fédéral des finances, mais ils n'ont pas conduit à l'examen critique qui aurait été nécessaire. Le service juridique d'Armasuisse, pourtant compétent en la matière, n'a pratiquement pas participé à la négociation de ce contrat. Seules quelques personnes impliquées dans le dossier ont lu le contrat dans son intégralité. Comme si cela ne suffisait pas, la Commission de gestion constate que certains documents n'ont même pas été archivés conformément aux règles.
-Nous ne parlons pas de l'achat de quelques véhicules de service. Nous parlons du plus grand projet d'acquisition militaire de l'histoire récente de notre pays. Pourtant, à chaque nouvelle révélation, le même constat s'impose : manque de conduite, manque de contrôle, manque de transparence. Et maintenant, le Parlement doit octroyer 394 millions supplémentaires, non pour améliorer la sécurité de la Suisse, mais pour essayer de sauver 30 avions sur les 36 que le Conseil fédéral voulait acquérir. Faut-il avaler cette couleuvre tranquillement ? Nous ne le pensons pas.
-Il faut savoir s'arrêter lorsqu'un projet déraille. Le projet F-35A a largement dépassé ce stade, d'autant plus que notre opposition au F-35A n'a jamais été uniquement financière. Nous avons toujours contesté le choix de cet appareil, un avion extrêmement complexe dépendant des États-Unis pour son exploitation et son évolution, conçu pour opérer au sein d'un dispositif militaire intégré qui n'est pas celui de la Suisse. Aujourd'hui, à ces critiques stratégiques s'ajoute un fiasco dans la conduite de son acquisition.
-Il y a également une contradiction plus fondamentale dans la politique que nous menons. Nous parlons de sécurité comme si elle se mesurait au nombre de milliards de francs consacrés à l'armement, mais la sécurité de la Suisse ne commence pas lorsqu'un missile franchit notre frontière. Elle commence bien avant. Elle se construit lorsque nous empêchons les conflits de naître et de s'étendre, lorsque nous défendons le droit international, lorsque nous investissons dans la coopération internationale, dans la diplomatie et dans la promotion de la paix, lorsque nous luttons contre le dérèglement climatique qui multiplie les crises et les déplacements des populations, lorsque nous renforçons notre capacité à faire face aux cyberattaques, à la désinformation et aux nouveaux risques liés à l'intelligence artificielle. C'est cela aussi la politique de sécurité. Dans ces domaines, la tendance est exactement inverse. Alors que l'objectif de 1 pour cent du PIB pour l'armée doit être atteint toujours plus rapidement, la part consacrée à la coopération internationale recule. Toujours plus pour réagir aux conflits, toujours moins pour contribuer à les prévenir : ce déséquilibre est une erreur stratégique. Nous le répétons : le groupe des Verts ne nie pas la détérioration de la situation sécuritaire. Au contraire, c'est précisément parce que les ressources sont limitées et que les menaces augmentent que nous devons les investir là où elles apportent réellement davantage de sécurité, c'est-à-dire dans la cyberdéfense, dans la résilience de nos infrastructures et dans la coopération internationale et la diplomatie, mais pas obstinément dans un projet de F-35A dont chaque nouveau chapitre vient confirmer les erreurs du précédent.
-La sécurité ne se mesure pas au prix du matériel que nous achetons. Elle se mesure à notre capacité à identifier les menaces, à faire les bons choix et à utiliser intelligemment les moyens à disposition. Sur ce dernier élément, le dossier F-35A devrait nous inciter à une certaine humilité. Notre groupe entrera donc en matière sur les arrêtés fédéraux 1 et 2, tout en les examinant de manière critique. Mais concernant l'arrêté fédéral 3 et les 394 millions de francs supplémentaires destinés au F-35A, notre position est claire : après les erreurs, les dissimulations, les approximations et les défaillances de conduite révélées dans ce dossier, notre réponse ne peut pas être de mettre à nouveau simplement 394 millions sur la table. 
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles, et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles, et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifie pas continuer comme si rien ne s'était passé au sein du DDPS.
+Au moment où ce Parlement s'apprête à voter 3,4 milliards de francs supplémentaires, dont 394 millions pour le F-35A, une question s'impose[NB]: pouvons-nous encore avoir confiance dans la manière dont le DDPS conduit ses grands projets d'armement[NB]? La semaine dernière, la Commission de gestion nous a donné quelques éléments de réponse qui sont accablants. Pendant des années, on nous a répété que le prix du F-35A était fixe. Il ne l'est pas. On nous a affirmé que la Suisse avait négocié une garantie particulière avec les États-Unis. Cette garantie n'existe pas. Des doutes avaient été exprimés par le Contrôle fédéral des finances, mais ils n'ont pas conduit à l'examen critique qui aurait été nécessaire. Le service juridique d'Armasuisse, pourtant compétent en la matière, n'a pratiquement pas participé à la négociation de ce contrat. Seules quelques personnes impliquées dans le dossier ont lu le contrat dans son intégralité. Comme si cela ne suffisait pas, la Commission de gestion constate que certains documents n'ont même pas été archivés conformément aux règles.
+Nous ne parlons pas de l'achat de quelques véhicules de service. Nous parlons du plus grand projet d'acquisition militaire de l'histoire récente de notre pays. Pourtant, à chaque nouvelle révélation, le même constat s'impose[NB]: manque de conduite, manque de contrôle, manque de transparence. Et maintenant, le Parlement doit octroyer 394 millions de francs supplémentaires, non pour améliorer la sécurité de la Suisse, mais pour essayer de sauver 30 avions sur les 36 que le Conseil fédéral voulait acquérir. Faut-il avaler cette couleuvre tranquillement[NB]? Nous ne le pensons pas.
+Il faut savoir s'arrêter lorsqu'un projet déraille. Le projet F-35A a largement dépassé ce stade, d'autant plus que notre opposition au F-35A n'a jamais été uniquement financière. Nous avons toujours contesté le choix de cet appareil, un avion extrêmement complexe, dépendant des États-Unis pour son exploitation et son évolution, conçu pour opérer au sein d'un dispositif militaire intégré qui n'est pas celui de la Suisse. Aujourd'hui, à ces critiques stratégiques s'ajoute un fiasco dans la conduite de son acquisition.
+Il y a également une contradiction plus fondamentale dans la politique que nous menons. Nous parlons de sécurité comme si elle se mesurait au nombre de milliards de francs consacrés à l'armement, mais la sécurité de la Suisse ne commence pas lorsqu'un missile franchit notre frontière. Elle commence bien avant. Elle se construit lorsque nous empêchons les conflits de naître et de s'étendre, lorsque nous défendons le droit international, lorsque nous investissons dans la coopération internationale, dans la diplomatie et dans la promotion de la paix, lorsque nous luttons contre le dérèglement climatique qui multiplie les crises et les déplacements des populations, lorsque nous renforçons notre capacité à faire face aux cyberattaques, à la désinformation et aux nouveaux risques liés à l'intelligence artificielle. C'est cela aussi la politique de sécurité. Dans ces domaines, la tendance est exactement inverse. Alors que l'objectif de 1 pour cent du PIB pour l'armée doit être atteint toujours plus rapidement, la part consacrée à la coopération internationale recule. Toujours plus pour réagir aux conflits, toujours moins pour contribuer à les prévenir[NB]: ce déséquilibre est une erreur stratégique. Nous le répétons[NB]: le groupe des Verts ne nie pas la détérioration de la situation sécuritaire. Au contraire, c'est précisément parce que les ressources sont limitées et que les menaces augmentent que nous devons les investir là où elles apportent réellement davantage de sécurité, c'est-à-dire dans la cyberdéfense, dans la résilience de nos infrastructures et dans la coopération internationale et la diplomatie, mais pas obstinément dans un projet de F-35A dont chaque nouveau chapitre vient confirmer les erreurs du précédent.
+La sécurité ne se mesure pas au prix du matériel que nous achetons. Elle se mesure à notre capacité à identifier les menaces, à faire les bons choix et à utiliser intelligemment les moyens à disposition. Sur ce dernier élément, le dossier F-35A devrait nous inciter à une certaine humilité. Notre groupe entrera donc en matière sur les arrêtés fédéraux 1 et 2, tout en les examinant de manière critique. Mais concernant l'arrêté fédéral 3 et les 394 millions de francs supplémentaires destinés au F-35A, notre position est claire[NB]: après les erreurs, les dissimulations, les approximations et les défaillances de conduite révélées dans ce dossier, notre réponse ne peut pas être de mettre à nouveau simplement 394 millions de francs sur la table. 
 Nous refuserons donc l'entrée en matière sur l'arrêté fédéral 3.
 </t>
   </si>
@@ -274,6 +274,61 @@
   </si>
   <si>
     <t xml:space="preserve">Le Contrôle fédéral des finances a publié un rapport en 2025 qui met en évidence le poids et l'existence de coûts potentiellement inutiles dans ce domaine. Le Conseil fédéral soutient le postulat de votre commission. Le domaine de l'imagerie médicale doit donc continuer à être suivi attentivement, afin que d'éventuelles évolutions problématiques soient identifiées rapidement et puissent surtout être corrigées.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420874</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260923</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schnyder Markus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wir sprechen wieder einmal über das Gesetz über die Mobilitätsdateninfrastruktur (MODIG). Wir haben bereits mehrfach über dieses Thema diskutiert. Heute darf ich zu meinen Minderheitsanträgen auf Nichteintreten auf den Bundesbeschluss 1 sowie auf Nichteintreten auf den Bundesbeschluss 2 sprechen. Zudem spreche ich für die Fraktion. Ich hätte also fast unbegrenzt Zeit zur Verfügung, ich werde diese allerdings nicht beanspruchen. Ich könnte auch einfach nochmals das erste Votum vorlesen, das mache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wir sprechen wieder einmal über das Gesetz über die Mobilitätsdateninfrastruktur (MODIG). Wir haben bereits mehrfach über dieses Thema diskutiert. Heute darf ich zu meinen Minderheitsanträgen auf Nichteintreten auf den Bundesbeschluss 1 sowie auf Nichteintreten auf den Bundesbeschluss 2 sprechen. Zudem spreche ich für die Fraktion. Ich hätte also fast unbegrenzt Zeit zur Verfügung, ich werde diese allerdings nicht beanspruchen. Ich könnte auch einfach nochmals das erste Votum vorlesen, das mache ich allerdings nicht. Dennoch möchte ich darauf hinweisen, dass der Ständerat bzw. die ständerätliche Kommission für Verkehr und Fernmeldewesen sich in Hinblick auf dieses Geschäft mit 8 zu 3 Stimmen für Nichteintreten entschieden hat. Der Ständerat selbst hat beim Bundesbeschluss 1 mit 25 zu 20 Stimmen und beim Bundesbeschluss 2 sogar mit 27 zu 17 Stimmen für Nichteintreten gestimmt.
+Die Fehler dieser Vorlage sind offensichtlich, bei diesem Punkt werde ich mich wiederholen. Das Gesetz hat nämlich einen grundsätzlichen Konstruktionsfehler, der sich in der Detailberatung nicht aufheben lässt: Die Datenlieferung basiert auf einer gewissen Freiwilligkeit. Das heisst, nur diejenigen müssen Daten liefern, die das wollen, ausgenommen sind Transportunternehmen, die konzessioniert oder subventioniert sind. Wenn Sie nun aber nur die Daten bekommen, die diese Unternehmen liefern wollen, dann werden Sie von Anfang an ein unvollständiges Bild der Daten haben. Wenn Sie ein unvollständiges Bild haben, dann wird das dazu führen, dass Sie keine schlauen Massnahmen daraus ableiten können. Entweder werden in der Folge Fehlinvestitionen geplant, wenn nämlich aufgrund des falschen Bildes eine falsche Einschätzung oder Beurteilung vorgenommen wird, oder es entstehen Doppelspurigkeiten, wenn zum Beispiel konzessionierte Unternehmen ihre Daten offenlegen und dann irgendein privater Anbieter der Meinung ist, das könnte eine interessante Strecke sein. Das kann zu Doppelspurigkeiten führen und dazu, dass die konzessionierten Unternehmen weniger Geld verdienen.
+Das zweite Problem ist das unterschiedliche Verständnis dieser Vorlage. Bereits in der Kommission hat sich gezeigt, dass es unterschiedliche Meinungen dazu gibt, was das Gesetz genau bewirken soll. Die links-grüne Ratshälfte hat bereits in der Kommissionsdebatte immer wieder versucht, aus diesem Gesetz irgendein Lenkungsgesetz zu machen oder zumindest den Modalsplit zugunsten des ÖV zu ändern. Das ist aber nicht die Idee dieser Vorlage. Es geht wirklich nur darum, Daten zu sammeln. Diese Daten sind dann aber bereits das dritte Problem. Es hat sich auch in der Kommissionsdebatte gezeigt, dass der Datenschutz sehr anspruchsvoll ist. Wie das in der Praxis gehandhabt werden soll, wenn jede Person, die transportiert wird, ihr Einverständnis geben muss, dass ihre Daten weitergeleitet werden können, wurde nicht abschliessend geklärt.
+Das vierte Problem - wahrscheinlich das Hauptproblem - sind die Kosten. Wir sprechen hier von 86 Millionen Franken für vier Jahre. Sie wissen, dass wir in diesem Rat ein Entlastungspaket beschlossen haben, und zeitgleich wollen wir 86 Millionen Franken für einen bekanntermassen sehr kleinen Nutzen ausgeben. Ich bin ehrlicherweise überrascht, dass die EFK ihre Meinung dazu nicht kundgetan hat, mittlerweile ist das ja Standard. Nun kann man sagen, dass die Finanzierung mit Geldern aus dem NAF und dem BIF passieren würde. Sie wissen aber ebenfalls, dass wir das Projekt Verkehr '45 haben, und die Ansprüche an diese beiden Fonds fast unermesslich hoch sind - das Geld hingegen nicht entsprechend vorhanden ist.
+Ich möchte auch darauf hinweisen, dass wir in der ersten Runde nicht eingetreten sind, dass wir aber einen Rückweisungsantrag gestellt haben mit der Aufforderung, die Vorlage müsse nutzerfinanziert sein. Das wollten Sie damals nicht, und nun ist diese Vorlage im Ständerat halt gescheitert.
+Ich bitte Sie, ebenfalls für Nichteintreten zu stimmen. Das Fazit ist klar: Die Vorlage bringt sehr wenig bis nichts, kostet hingegen sehr viel. Der Ständerat hat das bemerkt; ich hoffe, Sie haben es auch bemerkt. Stimmen Sie den Anträgen der Minderheit zu.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420917</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imark Christian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigentlich wollte ich nichts sagen, aber jetzt muss ich, da einiges gesagt wurde, das nicht ganz korrekt ist. Einfach an alle, die in diesem Saal die Dekarbonisierung vorantreiben wollen; an alle, die nicht nur ein grünes Etikett haben, sondern wirklich etwas für die Dekarbonisierung tun wollen: Stimmen Sie der Minderheit Heimgartner zu! Dann schaffen Sie Rechtssicherheit, damit die Elektrifizierung im Schwerverkehr auch für kleine Betriebe beschleunigt wird. Hier können Sie zeigen, dass Ihnen d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigentlich wollte ich nichts sagen, aber jetzt muss ich, da einiges gesagt wurde, das nicht ganz korrekt ist. Einfach an alle, die in diesem Saal die Dekarbonisierung vorantreiben wollen; an alle, die nicht nur ein grünes Etikett haben, sondern wirklich etwas für die Dekarbonisierung tun wollen: Stimmen Sie der Minderheit Heimgartner zu! Dann schaffen Sie Rechtssicherheit, damit die Elektrifizierung im Schwerverkehr auch für kleine Betriebe beschleunigt wird. Hier können Sie zeigen, dass Ihnen die Dekarbonisierung wirklich wichtig ist. 
+Dann muss ich noch Folgendes korrigieren: Herr Roth hat gesagt oder so getan, als ob wir hier den Schwerverkehr subventionieren würden. Herr Roth, ich weiss nicht, ob Ihnen bewusst ist - Sie sind gar nicht mehr da, ich spreche Sie trotzdem an und tue so, als ob Sie noch im Saal sitzen würden -, woher die Gelder der LSVA kommen. Der Schwerverkehr bezahlt jedes Jahr 1,7 Milliarden Franken, die für Schienenverbindungen ausgegeben werden können. Würde die Eidgenössische Finanzkontrolle, wie sie es kürzlich getan hat, das Kosten-Nutzen-Verhältnis der Schiene genau unter die Lupe nehmen, und würden wir unsere Entscheidungen so fällen, dass das Kosten-Nutzen-Verhältnis im Schienenverkehr massgeblich wäre, würde in diesem Land wohl kaum mehr ein Zug fahren. Das Geld kommt vom Schwerverkehr, und wir sprechen hier nicht von Subventionen, sondern wir sprechen von Investitionssicherheiten, damit auch Ihre Ziele der Dekarbonisierung erfüllt werden können. 
+Noch eine letzte Bemerkung: Es wurde von der Rückverlagerung auf die Strasse gesprochen. Auch das haben wir kürzlich in diesem Rat diskutiert, als wir das Gütertransportgesetz mit einer Mitte-Links-Mehrheit verabschiedet haben. Das Gesetz müssen wir bald wieder korrigieren, weil eine Rückverlagerung auf die Strasse stattfindet. Es passiert das, was wir vorausgesagt haben, nämlich dass der Einzelwagenladungsverkehr nicht mehr funktionstüchtig ist. Auch hier müssen wir leider bald wieder korrigieren, weil die Mitte-Links-Mehrheit nicht das bringt, was sie versprochen hat.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">420951</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weichelt Manuela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geschätzter Kollege Wyssmann, Sie haben jetzt wieder mal darüber gewettert, was Swissmedic alles schlecht mache. Kennen Sie den Bericht der EFK, der besagt, dass Swissmedic konkurrenzfähig zu international führenden Zulassungsbehörden sei? Wir haben etwas Verspätung, weil die Firmen ihre Gesuche rund 200 Tage nach der Einreichung bei der Europäischen Arzneimittelagentur einreichen. Das hat überhaupt nichts mit Swissmedic zu tun. Was sagen Sie zu diesem Bericht?
 </t>
   </si>
 </sst>
@@ -322,8 +377,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I14"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -934,6 +989,93 @@
         <v>63</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-24
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà é</t>
   </si>
   <si>
-    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà épuisées. Les personnes concernées peuvent demander à leur assureur-maladie le remboursement du montant différentiel. Si les assurés ne font pas valoir activement leur avoir auprès de la caisse-maladie, les assureurs peuvent renoncer à un remboursement lorsque celui-ci engendrerait une charge disproportionnée. Tel est le cas, par exemple, lorsque les assurés ne peuvent pas être contactés malgré des efforts avérés, ou encore en présence de montants minimes lorsque les frais de traitement excèdent les montants à rembourser. Lorsque les restitutions ne sont pas utilisées pour réduire la participation aux coûts, elles diminuent le coût des prestations. Cela améliore le résultat actuariel global et conduit, au final, à des primes moins élevées. Néanmoins, j'en conviens, Monsieur le conseiller national, ce qui compte, c'est la traçabilité des montants et la transparence - nous l'avons vu également dans le rapport du Contrôle fédéral des finances. Par votre motion, vous demandez plus de transparence et de traçabilité. Le Conseil fédéral estime que les restitutions doivent bénéficier aux personnes assurées, tout comme vous, mais il estime que la LAMal le permet d'ores et déjà.
+    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà épuisées. Les personnes concernées peuvent demander à leur assureur-maladie le remboursement du montant différentiel. Si les assurés ne font pas valoir activement leur avoir auprès de la caisse-maladie, les assureurs peuvent renoncer à un remboursement lorsque celui-ci engendrerait une charge disproportionnée. Tel est le cas, par exemple, lorsque les assurés ne peuvent pas être contactés malgré des efforts avérés, ou encore en présence de montants minimes lorsque les frais de traitement excèdent les montants à rembourser. Lorsque les restitutions ne sont pas utilisées pour réduire la participation aux coûts, elles diminuent le coût des prestations. Cela améliore le résultat actuariel global et conduit, au final, à des primes moins élevées. Néanmoins, j'en conviens, Monsieur le conseiller national, ce qui compte, c'est la traçabilité des montants et la transparence - nous l'avons vu également dans le rapport du Contrôle fédéral des finances. Par votre motion, vous demandez plus de transparence et de traçabilité. Le Conseil fédéral estime que les restitutions doivent bénéficier aux personnes assurées, tout comme vous, mais il estime que la LAMal le permet d'ores et déjà. [GZ]
 C'est pourquoi il demande le rejet de la motion.
 </t>
   </si>
@@ -141,15 +141,15 @@
     <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5. März 2026 in der abgeänderten Fassung an.
 Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585, "Aktionsplan zur Reduktion der Belastung von Mensch und Umwelt durch langlebige Chemikalien". Diesen Bericht haben wir in der Kommission ebenfalls einlässlich diskutiert. Auf dessen Basis haben wir zahlreiche Zusatzfragen an die Verwaltung übermittelt, in Kenntnis der Antworten haben wir dann die vorliegenden Vorstösse behandelt. Es geht hier nur um die Vorstösse im Zuständigkeitsbereich des EDI, also um die Motion Michel Matthias, die Motion Vincenz und um die Motion Rechsteiner Thomas. Es gibt dann noch weitere Motionen, die im Zuständigkeitsbereich des UVEK sind: die Motionen Moser, Graf Maya, Crevoisier Crelier, Silberschmidt und Mühlemann. Ich sage das darum, weil wir in der Kommission alle als Gesamtpaket angeschaut haben. Wir sagten insgesamt, dass eigentlich alle Themen, die in diesen Motionen adressiert werden, bereits von der Motion 25.3421 der UREK-S umfasst sind, weshalb wir alle diese Motionen zur Ablehnung empfehlen. Auch die Verwaltung sagte klar, dass im Grunde genommen alle Themen bereits jetzt in Bearbeitung seien und grundsätzlich keine neuen Vorstösse mehr erforderlich seien; auch der Bundesrat beantragt alle diese Vorstösse zur Ablehnung.
 Wie sieht nun grosso modo die Pipeline aus? Was ist in diesem Bereich in Bearbeitung? Der Bund wird im kommenden Herbst die Vernehmlassung im Rahmen der Umsetzung der Motion Maret Marianne 22.3929, "Festlegung von PFAS-spezifischen Werten in Verordnungen", eröffnen. Verbindliche Grenzwerte für Aushub und Abfall werden Teil der entsprechenden Vorlage sein. Im Winter wird die Verwaltung dann Grenzwerte für den Boden festlegen.
-Wir haben auch die Frage der Steuerung dieses ganzen Themas diskutiert. Der Bundesrat hat zwar nicht einen formellen bundesrätlichen Ausschuss für PFAS eingesetzt, aber es finden regelmässige Treffen zum Thema Pflanzenschutzmittel zwischen der Vorsteherin des EDI und den Vorstehern von WBF und UVEK statt. In diesem Rahmen werden auch die Themen rund um PFAS diskutiert. Auf Ebene der Verwaltung gibt es eine Projektorganisation, welche insbesondere die Umsetzung des Postulates Moser an die Hand nimmt. In dieser Projektorganisation arbeiten die genannten Departemente und auch die Kantone eng zusammen.
+Wir haben auch die Frage der Steuerung dieses ganzen Themas diskutiert. Der Bundesrat hat zwar nicht einen formellen bundesrätlichen Ausschuss für PFAS eingesetzt, aber es finden regelmässige Treffen zum Thema Pflanzenschutzmittel zwischen der Vorsteherin des EDI und den Vorstehern von WBF und UVEK statt. In diesem Rahmen werden auch die Themen rund um PFAS diskutiert. Auf Ebene der Verwaltung gibt es eine Projektorganisation, welche insbesondere die Umsetzung des Postulates Moser in die Hand nimmt. In dieser Projektorganisation arbeiten die genannten Departemente und auch die Kantone eng zusammen.
 Möglicherweise haben Sie auch von den Beschlüssen des Bundesrates vom 27. Mai 2026 Kenntnis genommen. Damit wurde die Vernehmlassung zur erwähnten Motion 25.3421 der UREK-S ausgelöst. PFAS-Betriebe sollen mehr Zeit für eine Produktionsumstellung erhalten und währenddessen weiterhin ein wirtschaftliches Auskommen erzielen können - das war ein Kernelement dieser Motion. Gleichzeitig beschloss der Bundesrat, PFAS-belastete Betriebe in Härtefällen finanziell zu unterstützen. Diesbezüglich gab es eine Aussprache, und bis März 2027 soll ein Entwurf für ein zeitlich begrenztes Spezialgesetz in die Vernehmlassung gehen. Es ist damit zu rechnen, dass im Jahr 2028 hier Rechtsgrundlagen bestehen werden.
-Parallel dazu hat das BLV - nicht der Bundesrat - eine Weisung erlassen, um den einheitlichen Vollzug der PFAS-Höchstgehalte durch die Kantone sicherzustellen - ich werde noch darauf zu sprechen kommen. Das hat wahrscheinlich mehr Probleme geschaffen als gelöst.
+Parallel dazu hat das Bundesamt für Lebensmittelsicherheit und Veterinärwesen - nicht der Bundesrat - eine Weisung erlassen, um den einheitlichen Vollzug der PFAS-Höchstgehalte durch die Kantone sicherzustellen. Ich werde noch darauf zu sprechen kommen. Das hat wahrscheinlich mehr Probleme geschaffen als gelöst.
 In der Kommission wurde im Wesentlichen die Frage diskutiert, wie mit den belasteten Böden umzugehen ist. Da wir uns im Bereich des Altlastenrechtes befinden, stellen sich Fragen der Sanierung, des Verursacherprinzips sowie der Finanzierung.
 Wie erwähnt, beabsichtigt das BAFU, im Zuge der Umsetzung der Motion Maret Marianne entsprechende Grenzwerte zu definieren. In der Vergangenheit fand dazu eine Diskussion mit der Branche statt. Ursprünglich waren die entsprechenden Werte sehr tief angesetzt, was zu erheblichen Problemen führte. Mittlerweile wurden diese Grenzwerte erhöht und sind nach Aussage der Verwaltung toxikologisch weiterhin vertretbar. Zudem wird ein Spezialgesetz für betriebliche Härtefälle geschaffen.
 Insbesondere stellt sich natürlich auch die Frage, wie rein technisch mit diesen belasteten Böden umzugehen ist. Man kann diese Böden nicht einfach vollumfänglich von PFAS befreien, da sonst kein Humus mehr vorhanden wäre und der Boden tot ist. Man befindet sich im Prinzip in einer erheblichen Zwickmühle.
-Auch die bereits erwähnte Finanzierung ist komplex. Eigentlich wäre der Vasa-Fonds das Instrument, um die Sanierung von Altlasten zu alimentieren und zu finanzieren. Dieser ist jedoch nicht für solche Situationen ausgerichtet, da bei mit Klärschlamm belasteten Böden kein Anspruch auf Mittel des Vasa-Fonds besteht. Dies ist ein nach wie vor ungelöstes Problem. Die EFK hat der Verwaltung im Rahmen einer Querschnittprüfung empfohlen, Abklärungen zum Verursacherprinzip durchzuführen; diese laufen derzeit. Das Verursacherprinzip muss im Umweltrecht sehr unmittelbar sein. Seine Anwendung ist im Falle von Belastungen, deren Ursachen zwanzig oder dreissig Jahre zurückliegen, relativ schwierig, weshalb die Verursacher oftmals nicht mehr direkt belangt werden können. Die Kommission hat jedoch verlangt, dass ihr die Resultate der Abklärungen zum Verursacherprinzip wieder unterbreitet werden. Dies stellt eine weitere Pendenz in diesem Kontext dar.
+Auch die bereits erwähnte Finanzierung ist komplex. Eigentlich wäre der Vasa-Fonds das Instrument, um die Sanierung von Altlasten zu alimentieren und zu finanzieren. Dieser ist jedoch nicht für solche Situationen ausgerichtet, da bei mit Klärschlamm belasteten Böden kein Anspruch auf Mittel des Vasa-Fonds besteht. Dies ist ein nach wie vor ungelöstes Problem. Die Eidgenössische Finanzkontrolle hat der Verwaltung im Rahmen einer Querschnittprüfung empfohlen, Abklärungen zum Verursacherprinzip durchzuführen; diese laufen derzeit. Das Verursacherprinzip muss im Umweltrecht sehr unmittelbar sein. Seine Anwendung ist im Falle von Belastungen, deren Ursachen zwanzig oder dreissig Jahre zurückliegen, relativ schwierig, weshalb die Verursacher oftmals nicht mehr direkt belangt werden können. Die Kommission hat jedoch verlangt, dass ihr die Resultate der Abklärungen zum Verursacherprinzip wieder unterbreitet werden. Dies stellt eine weitere Pendenz in diesem Kontext dar.
 Summa summarum: Vieles befindet sich in der Pipeline, weshalb es nicht sinnvoll ist, neue Vorstösse zu überweisen. Deshalb haben wir die Motionen Rechsteiner Thomas 25.3906 sowie Vincenz 25.3902 jeweils mit 10 zu 2 Stimmen abgelehnt. Die Motion Michel Matthias 25.3866 wurde einstimmig abgelehnt, da es sich dabei um einen gleichlautenden Vorstoss handelt und insofern keine materielle Änderung im Raum steht. Alle weiteren Vorstösse werden voraussichtlich am 1. Oktober im Rat behandelt. Ich werde Ihnen dann im Wesentlichen wieder kurz und bündig die gleiche Ausgangslage darlegen bzw. mich kurzfassen, um mich nicht zu wiederholen.
-Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen an die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
+Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen in die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
 Namens der Kommission bitte ich Sie, auf die drei erwähnten Vorstösse nicht einzutreten bzw. diese abzulehnen.
 </t>
   </si>

</xml_diff>

<commit_message>
Update debates data - 2026-09-25
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -134,22 +134,23 @@
     <t xml:space="preserve">DE</t>
   </si>
   <si>
-    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5. März 2026 in der abgeänderten Fassung an.
-Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5. März 2026 in der abgeänderten Fassung an.
-Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585, "Aktionsplan zur Reduktion der Belastung von Mensch und Umwelt durch langlebige Chemikalien". Diesen Bericht haben wir in der Kommission ebenfalls einlässlich diskutiert. Auf dessen Basis haben wir zahlreiche Zusatzfragen an die Verwaltung übermittelt, in Kenntnis der Antworten haben wir dann die vorliegenden Vorstösse behandelt. Es geht hier nur um die Vorstösse im Zuständigkeitsbereich des EDI, also um die Motion Michel Matthias, die Motion Vincenz und um die Motion Rechsteiner Thomas. Es gibt dann noch weitere Motionen, die im Zuständigkeitsbereich des UVEK sind: die Motionen Moser, Graf Maya, Crevoisier Crelier, Silberschmidt und Mühlemann. Ich sage das darum, weil wir in der Kommission alle als Gesamtpaket angeschaut haben. Wir sagten insgesamt, dass eigentlich alle Themen, die in diesen Motionen adressiert werden, bereits von der Motion 25.3421 der UREK-S umfasst sind, weshalb wir alle diese Motionen zur Ablehnung empfehlen. Auch die Verwaltung sagte klar, dass im Grunde genommen alle Themen bereits jetzt in Bearbeitung seien und grundsätzlich keine neuen Vorstösse mehr erforderlich seien; auch der Bundesrat beantragt alle diese Vorstösse zur Ablehnung.
+    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5.[NB]März 2026 in der abgeänderten Fassung an.
+Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die UREK Ihres Rates behandelt dieses Thema seit bald zwei Jahren; es ist ein sehr komplexes Thema. Wir haben umfassende Anhörungen gemacht. Aus diesen Anhörungen ist auch die bekannte Motion 25.3421 entstanden, eine sehr umfassende Kommissionsmotion, die auch vom Bundesrat zur Annahme empfohlen wurde. Der Nationalrat änderte sie leicht ab, unser Rat nahm sie am 5.[NB]März 2026 in der abgeänderten Fassung an.
+Parallel dazu arbeitete der Bundesrat am Bericht in Erfüllung des Postulates Moser 22.4585, "Aktionsplan zur Reduktion der Belastung von Mensch und Umwelt durch langlebige Chemikalien". Diesen Bericht haben wir in der Kommission ebenfalls einlässlich diskutiert. Auf dessen Basis haben wir zahlreiche Zusatzfragen an die Verwaltung übermittelt, in Kenntnis der Antworten haben wir dann die vorliegenden Vorstösse behandelt. Es geht hier nur um die Vorstösse im Zuständigkeitsbereich des EDI, also um die Motion Michel Matthias, die Motion Vincenz und die Motion Rechsteiner Thomas. Es gibt dann noch weitere Motionen, die im Zuständigkeitsbereich des UVEK sind: die Motionen Moser, Graf Maya, Crevoisier Crelier, Silberschmidt und Mühlemann. Ich sage das darum, weil wir in der Kommission alle als Gesamtpaket angeschaut haben. Wir sagten insgesamt, dass eigentlich alle Themen, die in diesen Motionen adressiert werden, bereits von der Motion 25.3421 der UREK-S umfasst sind, weshalb wir alle diese Motionen zur Ablehnung empfehlen. Auch die Verwaltung sagte klar, dass im Grunde genommen alle Themen bereits jetzt in Bearbeitung seien und grundsätzlich keine neuen Vorstösse mehr erforderlich seien; auch der Bundesrat beantragt alle diese Vorstösse zur Ablehnung.
 Wie sieht nun grosso modo die Pipeline aus? Was ist in diesem Bereich in Bearbeitung? Der Bund wird im kommenden Herbst die Vernehmlassung im Rahmen der Umsetzung der Motion Maret Marianne 22.3929, "Festlegung von PFAS-spezifischen Werten in Verordnungen", eröffnen. Verbindliche Grenzwerte für Aushub und Abfall werden Teil der entsprechenden Vorlage sein. Im Winter wird die Verwaltung dann Grenzwerte für den Boden festlegen.
-Wir haben auch die Frage der Steuerung dieses ganzen Themas diskutiert. Der Bundesrat hat zwar nicht einen formellen bundesrätlichen Ausschuss für PFAS eingesetzt, aber es finden regelmässige Treffen zum Thema Pflanzenschutzmittel zwischen der Vorsteherin des EDI und den Vorstehern von WBF und UVEK statt. In diesem Rahmen werden auch die Themen rund um PFAS diskutiert. Auf Ebene der Verwaltung gibt es eine Projektorganisation, welche insbesondere die Umsetzung des Postulates Moser in die Hand nimmt. In dieser Projektorganisation arbeiten die genannten Departemente und auch die Kantone eng zusammen.
-Möglicherweise haben Sie auch von den Beschlüssen des Bundesrates vom 27. Mai 2026 Kenntnis genommen. Damit wurde die Vernehmlassung zur erwähnten Motion 25.3421 der UREK-S ausgelöst. PFAS-Betriebe sollen mehr Zeit für eine Produktionsumstellung erhalten und währenddessen weiterhin ein wirtschaftliches Auskommen erzielen können - das war ein Kernelement dieser Motion. Gleichzeitig beschloss der Bundesrat, PFAS-belastete Betriebe in Härtefällen finanziell zu unterstützen. Diesbezüglich gab es eine Aussprache, und bis März 2027 soll ein Entwurf für ein zeitlich begrenztes Spezialgesetz in die Vernehmlassung gehen. Es ist damit zu rechnen, dass im Jahr 2028 hier Rechtsgrundlagen bestehen werden.
+Wir haben auch die Frage der Steuerung dieses ganzen Themas diskutiert. Der Bundesrat hat zwar nicht einen formellen bundesrätlichen Ausschuss für PFAS eingesetzt, aber es finden regelmässige Treffen zum Thema Pflanzenschutzmittel zwischen der Vorsteherin des EDI und den Vorstehern von WBF und UVEK statt. In diesem Rahmen werden auch die Themen rund um PFAS diskutiert. Auf Ebene der Verwaltung gibt es eine Projektorganisation, welche insbesondere die Umsetzung des Postulates Moser an die Hand nimmt. In dieser Projektorganisation arbeiten die genannten Departemente und auch die Kantone eng zusammen.
+Möglicherweise haben Sie auch von den Beschlüssen des Bundesrates vom 27.[NB]Mai 2026 Kenntnis genommen. Damit wurde die Vernehmlassung zur erwähnten Motion 25.3421 der UREK-S ausgelöst. PFAS-Betriebe sollen mehr Zeit für eine Produktionsumstellung erhalten und währenddessen weiterhin ein wirtschaftliches Auskommen erzielen können; das war ein Kernelement dieser Motion. Gleichzeitig beschloss der Bundesrat, PFAS-belastete Betriebe in Härtefällen finanziell zu unterstützen. Diesbezüglich gab es eine Aussprache, und bis März 2027 soll ein Entwurf für ein zeitlich begrenztes Spezialgesetz in die Vernehmlassung gehen. Es ist damit zu rechnen, dass im Jahr 2028 hier Rechtsgrundlagen bestehen werden.
 Parallel dazu hat das Bundesamt für Lebensmittelsicherheit und Veterinärwesen - nicht der Bundesrat - eine Weisung erlassen, um den einheitlichen Vollzug der PFAS-Höchstgehalte durch die Kantone sicherzustellen. Ich werde noch darauf zu sprechen kommen. Das hat wahrscheinlich mehr Probleme geschaffen als gelöst.
 In der Kommission wurde im Wesentlichen die Frage diskutiert, wie mit den belasteten Böden umzugehen ist. Da wir uns im Bereich des Altlastenrechtes befinden, stellen sich Fragen der Sanierung, des Verursacherprinzips sowie der Finanzierung.
 Wie erwähnt, beabsichtigt das BAFU, im Zuge der Umsetzung der Motion Maret Marianne entsprechende Grenzwerte zu definieren. In der Vergangenheit fand dazu eine Diskussion mit der Branche statt. Ursprünglich waren die entsprechenden Werte sehr tief angesetzt, was zu erheblichen Problemen führte. Mittlerweile wurden diese Grenzwerte erhöht und sind nach Aussage der Verwaltung toxikologisch weiterhin vertretbar. Zudem wird ein Spezialgesetz für betriebliche Härtefälle geschaffen.
 Insbesondere stellt sich natürlich auch die Frage, wie rein technisch mit diesen belasteten Böden umzugehen ist. Man kann diese Böden nicht einfach vollumfänglich von PFAS befreien, da sonst kein Humus mehr vorhanden wäre und der Boden tot ist. Man befindet sich im Prinzip in einer erheblichen Zwickmühle.
-Auch die bereits erwähnte Finanzierung ist komplex. Eigentlich wäre der Vasa-Fonds das Instrument, um die Sanierung von Altlasten zu alimentieren und zu finanzieren. Dieser ist jedoch nicht für solche Situationen ausgerichtet, da bei mit Klärschlamm belasteten Böden kein Anspruch auf Mittel des Vasa-Fonds besteht. Dies ist ein nach wie vor ungelöstes Problem. Die Eidgenössische Finanzkontrolle hat der Verwaltung im Rahmen einer Querschnittprüfung empfohlen, Abklärungen zum Verursacherprinzip durchzuführen; diese laufen derzeit. Das Verursacherprinzip muss im Umweltrecht sehr unmittelbar sein. Seine Anwendung ist im Falle von Belastungen, deren Ursachen zwanzig oder dreissig Jahre zurückliegen, relativ schwierig, weshalb die Verursacher oftmals nicht mehr direkt belangt werden können. Die Kommission hat jedoch verlangt, dass ihr die Resultate der Abklärungen zum Verursacherprinzip wieder unterbreitet werden. Dies stellt eine weitere Pendenz in diesem Kontext dar.
-Summa summarum: Vieles befindet sich in der Pipeline, weshalb es nicht sinnvoll ist, neue Vorstösse zu überweisen. Deshalb haben wir die Motionen Rechsteiner Thomas 25.3906 sowie Vincenz 25.3902 jeweils mit 10 zu 2 Stimmen abgelehnt. Die Motion Michel Matthias 25.3866 wurde einstimmig abgelehnt, da es sich dabei um einen gleichlautenden Vorstoss handelt und insofern keine materielle Änderung im Raum steht. Alle weiteren Vorstösse werden voraussichtlich am 1. Oktober im Rat behandelt. Ich werde Ihnen dann im Wesentlichen wieder kurz und bündig die gleiche Ausgangslage darlegen bzw. mich kurzfassen, um mich nicht zu wiederholen.
-Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen in die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
+Auch die bereits erwähnte Finanzierung ist komplex. Eigentlich wäre der Vasa-Fonds das Instrument, um die Sanierung von Altlasten zu alimentieren und zu finanzieren. Dieser ist jedoch nicht für solche Situationen ausgerichtet, da bei mit Klärschlamm belasteten Böden kein Anspruch auf Mittel des Vasa-Fonds besteht. Dies ist ein nach wie vor ungelöstes Problem. 
+Die Eidgenössische Finanzkontrolle hat der Verwaltung im Rahmen einer Querschnittprüfung empfohlen, Abklärungen zum Verursacherprinzip durchzuführen; diese laufen derzeit. Das Verursacherprinzip muss im Umweltrecht sehr unmittelbar sein. Seine Anwendung ist im Falle von Belastungen, deren Ursachen zwanzig oder dreissig Jahre zurückliegen, relativ schwierig, weshalb die Verursacher oftmals nicht mehr direkt belangt werden können. Die Kommission hat jedoch verlangt, dass ihr die Resultate der Abklärungen zum Verursacherprinzip wieder unterbreitet werden. Dies stellt eine weitere Pendenz in diesem Kontext dar.
+Summa summarum: Vieles befindet sich in der Pipeline, weshalb es nicht sinnvoll ist, neue Vorstösse zu überweisen. Deshalb haben wir die Motionen Rechsteiner Thomas 25.3906 sowie Vincenz 25.3902 jeweils mit 10 zu 2 Stimmen abgelehnt. Die Motion Michel Matthias 25.3866 wurde einstimmig abgelehnt, da es sich dabei um einen gleichlautenden Vorstoss handelt und insofern keine materielle Änderung im Raum steht. Alle weiteren Vorstösse werden voraussichtlich am 1.[NB]Oktober im Rat behandelt. Ich werde Ihnen dann im Wesentlichen wieder kurz und bündig die gleiche Ausgangslage darlegen bzw. mich kurzfassen, um mich nicht zu wiederholen.
+Eine Schlussbemerkung: Wir sind der Meinung, dass die seinerzeitige Motion 25.3421 der UREK-S nach wie vor eine gute Grundlage darstellt. Wir erwarten, dass der Bundesrat die entsprechenden Massnahmen an die Hand nimmt sowie regulatorische Anpassungen vornimmt. Es besteht kein Grund, weitere Vorstösse einzureichen oder zu überweisen. Ebenso gibt es keinen Grund für einen überhasteten Vollzug, solange der Auftrag des Parlamentes noch nicht umgesetzt ist. Dies ist ein Thema des nächsten Vorstosses, das ich dort weiter erläutern werde.
 Namens der Kommission bitte ich Sie, auf die drei erwähnten Vorstösse nicht einzutreten bzw. diese abzulehnen.
 </t>
   </si>

</xml_diff>

<commit_message>
Update debates data - 2026-09-28
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -164,25 +164,25 @@
     <t xml:space="preserve">Revaz Estelle</t>
   </si>
   <si>
-    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités : vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en si</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités : vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en situation de handicap est donc un véritable sujet de société. Cela concerne près d'une personne sur cinq dans notre pays et, à ce titre, nous concerne toutes et tous.
-L'initiative pour l'inclusion traduit un constat et une impatience. Le constat, c'est que malgré les progrès accomplis, la Suisse accuse encore un retard important dans la mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées. L'impatience, parfaitement compréhensible, est celle des personnes concernées et de leurs organisations qui attendent des avancées concrètes depuis trop longtemps.
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités[NB]: vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités[NB]: vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en situation de handicap est donc un véritable sujet de société. Cela concerne près d'une personne sur cinq dans notre pays et, à ce titre, nous concerne toutes et tous.
+L'initiative pour l'inclusion traduit un constat et une impatience. Le constat, c'est que, malgré les progrès accomplis, la Suisse accuse encore un retard important dans la mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées. L'impatience, parfaitement compréhensible, est celle des personnes concernées et de leurs organisations qui attendent des avancées concrètes depuis trop longtemps.
 L'initiative nous rappelle ainsi le chemin qu'il reste à parcourir pour faire de l'inclusion une réalité. Elle demande l'égalité de droit et de fait des personnes en situation de handicap dans tous les domaines de la vie. Elle vise notamment à garantir le libre choix du logement et à inscrire dans la Constitution un droit à des mesures de soutien et d'adaptation.
 La majorité de la commission comprend ces préoccupations, mais estime que la modification constitutionnelle proposée n'est pas adéquate. Celle-ci n'apporterait en effet pas d'amélioration significative par rapport au droit actuel et soulèverait des difficultés de mise en oeuvre. La commission propose donc de rejeter l'initiative, par 16 voix contre 8.
-La majorité de votre commission rejoint cependant les auteurs de l'initiative sur un point essentiel : il est nécessaire d'agir. Elle salue donc le contre-projet indirect proposé par le Conseil fédéral et, par 17 voix contre 8, a décidé d'entrer en matière. Une minorité propose de ne pas entrer en matière. Si cette proposition est rejetée, la même minorité demande le renvoi du projet au Conseil fédéral et formule plusieurs pistes de modifications.
+La majorité de votre commission rejoint cependant les auteurs de l'initiative sur un point essentiel[NB]: il est nécessaire d'agir. Elle salue donc le contre-projet indirect proposé par le Conseil fédéral et, par 17 voix contre 8, a décidé d'entrer en matière. Une minorité propose de ne pas entrer en matière. Si cette proposition est rejetée, la même minorité demande le renvoi du projet au Conseil fédéral et formule plusieurs pistes de modifications.
 Nous avons mené de longues discussions sur la portée du contre-projet indirect. Pour les auteurs de l'initiative comme pour la majorité de votre commission, il contient beaucoup de dispositions déclaratoires et peu de mesures concrètes. La majorité de votre commission a donc souhaité renforcer le contre-projet indirect et s'éloigner d'une loi essentiellement programmatique, en agissant dans les domaines essentiels de la vie quotidienne. Il ne s'agit pas d'inventer de nouveaux droits, mais de permettre aux personnes en situation de handicap de bénéficier concrètement des mêmes droits et des mêmes possibilités que les autres. Enfin, la commission a souhaité clarifier les responsabilités et renforcer la coordination avec les cantons, qui jouent un rôle central dans la mise en oeuvre de nombreuses mesures.
-Afin d'avoir une vision globale des mesures en faveur de l'égalité des personnes en situation de handicap, la commission a décidé, à l'unanimité, d'examiner l'objet 25.020 "Loi sur l'égalité pour les handicapés. Modification" en parallèle de la loi sur l'inclusion qui constitue le contre-projet indirect du Conseil fédéral à l'initiative. Elle a en revanche décidé, par 14 voix contre 10 et 1 abstention, de traiter séparément la question des langues des signes dans une loi spécifique. Ce sera l'objet de l'initiative parlementaire 26.404 qui vous sera très prochainement soumise.
-Des mesures concrètes ont ainsi été proposées autour de quatre axes : le libre choix du logement, l'intégration sur le marché du travail, la participation à la vie culturelle, aux loisirs et au sport, ainsi que les prestations d'assistance. Pour agir dans ces différents domaines, votre commission a travaillé sur pas moins de sept lois différentes : la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, la loi fédérale sur des mesures de promotion civile de la paix et de renforcement des droits de l'homme, la loi fédérale sur l'assurance-invalidité, la loi fédérale sur l'élimination des inégalités frappant les personnes handicapées, la loi sur les langues, la loi sur l'organisation du gouvernement et de l'administration et, enfin, la loi fédérale sur l'encouragement des hautes écoles et la coordination dans le domaine suisse des hautes écoles.
+Afin d'avoir une vision globale des mesures en faveur de l'égalité des personnes en situation de handicap, la commission a décidé, à l'unanimité, d'examiner l'objet 25.020 "Loi sur l'égalité pour les handicapés. Modification" en parallèle à la loi sur l'inclusion qui constitue le contre-projet indirect du Conseil fédéral à l'initiative. Elle a en revanche décidé, par 14 voix contre 10 et 1 abstention, de traiter séparément la question des langues des signes dans une loi spécifique. Ce sera l'objet de l'initiative parlementaire 26.404 qui vous sera très prochainement soumise.
+Des mesures concrètes ont ainsi été proposées autour de quatre axes[NB]: le libre choix du logement, l'intégration sur le marché du travail, la participation à la vie culturelle, aux loisirs et au sport, ainsi que les prestations d'assistance. Pour agir dans ces différents domaines, votre commission a travaillé sur pas moins de sept lois différentes[NB]: la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, la loi fédérale sur des mesures de promotion civile de la paix et de renforcement des droits de l'homme, la loi fédérale sur l'assurance-invalidité, la loi fédérale sur l'élimination des inégalités frappant les personnes handicapées, la loi sur les langues, la loi sur l'organisation du gouvernement et de l'administration et, enfin, la loi fédérale sur l'encouragement des hautes écoles et la coordination dans le domaine suisse des hautes écoles.
 Étant donné l'organisation du débat et le temps limité dont dispose la commission pour vous présenter les dizaines de propositions qui sont encore en discussion, je vais passer dès maintenant à l'examen de détail sans m'appesantir sur les points qui n'ont pas rencontré d'opposition.
 Je commence donc par la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, aussi appelée loi sur l'inclusion (LIncl), et je commence à l'article 2. 
 La loi sur l'inclusion est une loi-cadre qui doit donner une orientation politique claire. Par 14 voix contre 8 et 3 abstentions, votre commission propose donc de renforcer cet article sans lui donner une portée juridique qu'il ne pourrait avoir. Une minorité souhaite aller plus loin, tandis qu'une autre préfère s'en tenir à la proposition du Conseil fédéral. 
 À l'article 3, votre commission a souhaité clarifier la relation avec le droit cantonal, mais aussi mentionner explicitement l'importance de la collaboration entre la Confédération et les cantons. Convaincue qu'il est important de réaffirmer la nécessité d'agir, votre commission, par 12 voix contre 11, a accepté cet ajout. Une minorité s'y oppose. 
-À l'article 5, l'objectif est simple : faire en sorte que la stratégie nationale de mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées (CDPH) ne reste pas un document d'intention, mais débouche sur des mesures concrètes. Par 11 voix contre 8 et 5 abstentions, la majorité de votre commission souhaite renforcer les objectifs en matière d'autodétermination, de liberté de choix et de participation à la vie sociale. Une minorité souhaite suivre le Conseil fédéral. 
+À l'article 5, l'objectif est simple[NB]: faire en sorte que la stratégie nationale de mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées (CDPH) ne reste pas un document d'intention, mais débouche sur des mesures concrètes. Par 11 voix contre 8 et 5 abstentions, la majorité de votre commission souhaite renforcer les objectifs en matière d'autodétermination, de liberté de choix et de participation à la vie sociale. Une minorité souhaite suivre le Conseil fédéral. 
 À l'article 6 alinéas 4 et 5, il s'agit d'inscrire les projets pilotes dans la loi. Ces derniers permettent de tester concrètement les mesures prévues dans la stratégie et les plans d'action et d'identifier celles qui fonctionnent. Ces modifications ont été adoptées par 13 voix contre 10 et 2 abstentions. Il n'y a pas de proposition de minorité. 
 À l'article 8, la majorité souhaite impliquer les personnes en situation de handicap dès l'élaboration de la stratégie et des plans d'action. Leur expérience permet d'identifier les besoins en amont et d'éviter des corrections qui seraient ultérieurement plus coûteuses. Cette proposition a été adoptée par 13 voix contre 8 et 3 abstentions. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
-À l'article 11, la majorité souhaite renforcer l'autonomie des personnes en situation de handicap dans le choix de leur logement. Pour cela, elle propose notamment d'améliorer l'information et la coordination ; un élément également relevé par le Contrôle fédéral des finances. Ces modifications ont été adoptées par 14 voix contre 10. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
+À l'article 11, la majorité souhaite renforcer l'autonomie des personnes en situation de handicap dans le choix de leur logement. Pour cela, elle propose notamment d'améliorer l'information et la coordination[NB]; un élément également relevé par le Contrôle fédéral des finances. Ces modifications ont été adoptées par 14 voix contre 10. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
 À l'article 11a, l'objectif est de renforcer l'autonomie économique des personnes en situation de handicap en facilitant leur accès au marché du travail. Leur potentiel reste insuffisamment exploité, alors que la Suisse manque de main-d'oeuvre qualifiée et que l'assurance-invalidité (AI) fait face à des difficultés financières. Par 16 voix contre 8, votre commission a accepté cette proposition. 
 À l'article 11b, il s'agit de favoriser la participation des personnes en situation de handicap à la vie culturelle, aux loisirs, au sport et aux activités politiques. Par 14 voix contre 11, la majorité de votre commission souhaite inscrire cet objectif dans la loi sans que cela entraîne automatiquement de nouvelles dépenses. Une minorité la juge inopportune. 
 À l'article 11c, l'objectif est de renforcer la liberté de choix des personnes en situation de handicap en adaptant mieux les prestations d'assistance à leur réalité de vie et en améliorant leur coordination. Par 13 voix contre 11 et 1 abstention, votre commission veut inscrire cette orientation dans la loi. Une minorité estime qu'elle fait doublon avec les travaux annoncés concernant l'AI. 
@@ -330,6 +330,32 @@
   </si>
   <si>
     <t xml:space="preserve">Geschätzter Kollege Wyssmann, Sie haben jetzt wieder mal darüber gewettert, was Swissmedic alles schlecht mache. Kennen Sie den Bericht der EFK, der besagt, dass Swissmedic konkurrenzfähig zu international führenden Zulassungsbehörden sei? Wir haben etwas Verspätung, weil die Firmen ihre Gesuche rund 200 Tage nach der Einreichung bei der Europäischen Arzneimittelagentur einreichen. Das hat überhaupt nichts mit Swissmedic zu tun. Was sagen Sie zu diesem Bericht?
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">421379</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260928</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Bundesgesetz über die Krankenversicherung sieht vor, dass Leistungserbringer, die beim Medikamentenkauf Vergünstigungen erhalten, diese grundsätzlich an die Versicherer bzw. an die Prämienzahlenden weitergeben müssen. Die Transparenzpflicht gemäss Heilmittelgesetz verlangt zudem, dass gewährte Vergünstigungen auszuweisen und den zuständigen Behörden auf Verlangen offenzulegen sind. 
+Für die Aufsicht über die Einhaltung dieser gesetzlichen Bestimmungen ist seit 2020 das Bundesamt für Gesundhe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Bundesgesetz über die Krankenversicherung sieht vor, dass Leistungserbringer, die beim Medikamentenkauf Vergünstigungen erhalten, diese grundsätzlich an die Versicherer bzw. an die Prämienzahlenden weitergeben müssen. Die Transparenzpflicht gemäss Heilmittelgesetz verlangt zudem, dass gewährte Vergünstigungen auszuweisen und den zuständigen Behörden auf Verlangen offenzulegen sind. 
+Für die Aufsicht über die Einhaltung dieser gesetzlichen Bestimmungen ist seit 2020 das Bundesamt für Gesundheit (BAG) zuständig. Das BAG muss sicherstellen, dass Vergünstigungen an die Versicherer bzw. die Versicherten weitergegeben werden. Die Eidgenössische Finanzkontrolle hat 2026 die Aufsicht des BAG bezüglich Weitergabepflicht von Vergünstigungen bei der Medikamentenabgabe überprüft und kommt zum Schluss, dass diese noch kaum wirksam ist. Der Bundesrat erwartet von allen beteiligten Akteuren, dass der rechtliche Rahmen eingehalten wird. Das BAG wird die EFK-Empfehlungen gemäss dem Prüfbericht vom 10. April 2026 zur verbesserten Weitergabe von Vergünstigungen fristgerecht umsetzen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">421388</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merci beaucoup pour votre question complémentaire. En fait, il ne s'agit pas de la question de la responsabilité de 5, 10 ou 12 personnes qui travaillent à l'OFSP. Comme je l'ai indiqué, la base légale demande que l'OFSP contrôle, mais demande aussi que les personnes mettent les données à disposition et que les caisses-maladie contrôlent ces données. Le Contrôle fédéral des finances a estimé que le contrôle, du côté de l'OFSP, était insuffisant et qu'on devait maintenant mettre plus de priorités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merci beaucoup pour votre question complémentaire. En fait, il ne s'agit pas de la question de la responsabilité de 5, 10 ou 12 personnes qui travaillent à l'OFSP. Comme je l'ai indiqué, la base légale demande que l'OFSP contrôle, mais demande aussi que les personnes mettent les données à disposition et que les caisses-maladie contrôlent ces données. Le Contrôle fédéral des finances a estimé que le contrôle, du côté de l'OFSP, était insuffisant et qu'on devait maintenant mettre plus de priorités pour arriver à une situation conforme à la loi, à savoir que les rabais doivent être mis à disposition des assurances et, en particulier, des assurés. Il ne s'agit pas de dire qui est responsable en matière de personnes. Ce que je m'engage à faire, c'est que l'OFSP, désormais, mette la priorité sur la mission qui consiste à mieux ou à plus contrôler par rapport à ces rabais.
+Ich habe Ihre Frage genau verstanden, aber ich werde Ihnen nicht sagen können - ich kann es gar nicht -, ob es zwei, drei oder zehn Personen sind, die verantwortlich sind, denn es geht hier nicht um eine Verantwortung einzelner Personen. Das BAG muss diese Kontrolle von Gesetzes wegen durchführen, und wir werden sie auch durchführen. Aber man kann nicht sagen, bestimmte Personen hätten ihre Aufgabe nicht gemacht oder so; nein, sicher nicht. Wir können darüber noch stundenlang diskutieren. Es gibt keine Verantwortung einzelner Personen. 
 </t>
   </si>
 </sst>
@@ -378,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I16"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1077,6 +1103,60 @@
         <v>78</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15"/>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-30
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -356,6 +356,36 @@
   <si>
     <t xml:space="preserve">Merci beaucoup pour votre question complémentaire. En fait, il ne s'agit pas de la question de la responsabilité de 5, 10 ou 12 personnes qui travaillent à l'OFSP. Comme je l'ai indiqué, la base légale demande que l'OFSP contrôle, mais demande aussi que les personnes mettent les données à disposition et que les caisses-maladie contrôlent ces données. Le Contrôle fédéral des finances a estimé que le contrôle, du côté de l'OFSP, était insuffisant et qu'on devait maintenant mettre plus de priorités pour arriver à une situation conforme à la loi, à savoir que les rabais doivent être mis à disposition des assurances et, en particulier, des assurés. Il ne s'agit pas de dire qui est responsable en matière de personnes. Ce que je m'engage à faire, c'est que l'OFSP, désormais, mette la priorité sur la mission qui consiste à mieux ou à plus contrôler par rapport à ces rabais.
 Ich habe Ihre Frage genau verstanden, aber ich werde Ihnen nicht sagen können - ich kann es gar nicht -, ob es zwei, drei oder zehn Personen sind, die verantwortlich sind, denn es geht hier nicht um eine Verantwortung einzelner Personen. Das BAG muss diese Kontrolle von Gesetzes wegen durchführen, und wir werden sie auch durchführen. Aber man kann nicht sagen, bestimmte Personen hätten ihre Aufgabe nicht gemacht oder so; nein, sicher nicht. Wir können darüber noch stundenlang diskutieren. Es gibt keine Verantwortung einzelner Personen. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keller-Sutter Karin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben es gehört: Mit der Immobilienbotschaft 2026 beantragt der Bundesrat neun Verpflichtungskredite in der Höhe von insgesamt 773,8 Millionen Franken. Lassen Sie mich kurz auf die einzelnen Projekte eingehen. 
+Ich beginne mit dem Umbau und der Sanierung des Verwaltungsgebäudes an der Bundesgasse 32 in Bern. Es liegt in unmittelbarer Nähe der Bundeshäuser und wurde bisher durch das EDA genutzt. Nach dem Umzug des EDA nach Zollikofen soll das Gebäude in einen neuen Lebenszyklus überführt werd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben es gehört: Mit der Immobilienbotschaft 2026 beantragt der Bundesrat neun Verpflichtungskredite in der Höhe von insgesamt 773,8 Millionen Franken. Lassen Sie mich kurz auf die einzelnen Projekte eingehen. 
+Ich beginne mit dem Umbau und der Sanierung des Verwaltungsgebäudes an der Bundesgasse 32 in Bern. Es liegt in unmittelbarer Nähe der Bundeshäuser und wurde bisher durch das EDA genutzt. Nach dem Umzug des EDA nach Zollikofen soll das Gebäude in einen neuen Lebenszyklus überführt werden. Vier heutige Standorte der Bundeskanzlei sollen dort zusammengeführt werden. Dies ermöglicht betriebliche Synergien und erhöht die Flächeneffizienz um rund 30 Prozent. Hierfür wird ein Verpflichtungskredit von 24,6 Millionen Franken beantragt. 
+Für die Sanierung und Erweiterung der Nationalbibliothek in Bern beantragt der Bundesrat einen Verpflichtungskredit von 211,7 Millionen Franken. Das aus den 1930er-Jahren stammende Gebäude an der Hallwylstrasse in Bern ist ein bedeutender Zeuge des "Neuen Bauens" und entsprechend denkmalpflegerisch geschützt. Mit der umfassenden Sanierung und Erweiterung wird das Gebäude in einen neuen Lebenszyklus überführt. Die statischen Mängel werden beseitigt und die raumklimatischen Verhältnisse den heutigen Anforderungen an die Aufbewahrung von Kulturgütern angepasst.
+Ich komme zum Gebäude an der Monbijoustrasse 40 in Bern. Es wurde in den 1950er-Jahren als Verwaltungsgebäude für die damalige Oberzolldirektion der Eidgenössischen Zollverwaltung erstellt. Das schützenswerte Gebäude von nationaler Bedeutung wurde seit dem Bau nie umfassend saniert. Sowohl Statik als auch Fassaden sowie Haus- und Sicherheitstechnik weisen einen grossen Instandsetzungsbedarf auf.
+Das Gebäude soll künftig gemischt genutzt werden, als Büro- und Bildungsgebäude der Eidgenössischen Hochschule für Berufsbildung, der Eidgenössischen Finanzkontrolle, der Oberaufsichtskommission Berufliche Vorsorge sowie der Eidgenössischen Spielbankenkommission.
+Dann zur Gesamtsanierung der Botschaft in London: Diese zählt zu den weltweit bedeutendsten Vertretungen der Schweiz. Mit der geplanten Gesamtsanierung wird ein nachhaltiger Gebäudebetrieb für den nächsten Lebenszyklus sichergestellt. Durch räumliche Anpassungen werden Funktionsabläufe optimiert. Gleichzeitig kann eine Portfoliobereinigung erfolgen: Die drei weiteren Standorte der Eidgenossenschaft in London können in das Botschaftsgebäude integriert werden. Hierfür werden 96 Millionen Franken beantragt. Der Betrag ist auch deshalb relativ hoch, weil 20 Millionen Franken Mehrwertsteuer fällig werden. 
+Dann haben wir das Vorhaben in Magglingen: Für den Neubau des Unterkunfts- und Ausbildungsgebäudes für das Kompetenzzentrum Sport der Armee in Magglingen beantragt der Bundesrat einen Verpflichtungskredit über 30,9 Millionen Franken. Der Armeesport und die Spitzensportförderung der Armee haben sich am Standort Magglingen etabliert. Die Unterkunftsmöglichkeiten für den Armeesport sind jedoch knapp bemessen und genügen nicht. 2021 hat das Parlament bereits einen Verpflichtungskredit über 27 Millionen Franken für den Neubau des Unterkunfts- und Ausbildungsgebäudes genehmigt. Dieses Projekt stiess jedoch auf Widerstand bei einem Teil der Gemeinde und der Bevölkerung. Das Projekt konnte jetzt überarbeitet und angepasst werden. Es ist so, dass der 2021 bewilligte Verpflichtungskredit unbenutzt abgerechnet werden konnte.
+Dann haben wir das Projekt "Neubau Magazin des Bundesarchivs". Hier geht es darum, dass das Bundesarchiv seinen gesetzlichen Auftrag sicherstellen kann. Es benötigt zusätzliche Archivflächen. Das Bundesarchiv nutzt heute unter anderem Lagerkapazitäten in einem Tiefmagazin der Nationalbibliothek in Bern. Da diese die entsprechenden Flächen nun selbst benötigt, müssen die eigenen Flächen des Bundesarchivs ausgeweitet werden. Wir sprechen von einem Verpflichtungskredit von 73,6 Millionen Franken.
+Dann gibt es noch weitere Immobilienvorhaben. Dazu gehören unter anderem Ausgaben von bis zu 10 Millionen Franken für bauliche Massnahmen, Ausgaben für nicht planbare oder dringliche Liegenschaftskäufe sowie Ausgaben für Projektierungen. Für diese weiteren Immobilienvorhaben wird ein Sammelkredit von 170 Millionen Franken beantragt.
+Dann gibt es das Projekt "Basel, Stücki Park, Zumiete Stützpunkt regionale Führung Zoll Nord, Lokalebene Basel Nord und Basel Mitte". In der Region Zoll Nord sollen 18 heutige Standorte in Basel in unmittelbarer Nähe der Grenze zu einem gemeinsamen Stützpunkt zusammengeführt werden. Dieser dient zudem als Ersatzstandort für die ab 2030 wegfallenden Flächen bei der Gemeinschaftszollanlage Basel/Weil-Autobahn in Deutschland, die am Ende des Lebenszyklus ist. Da die Eidgenossenschaft über keine geeignete Parzelle in der Region verfügt und auf dem Markt keine solche erworben werden konnte, sollen die entsprechenden Flächen im Stücki Park angemietet werden. Hier geht es um einen Verpflichtungskredit von 56,8 Millionen Franken.
+Dann zum umstrittensten Projekt, "Zumiete und Mieterausbau Besuchs- und Informationszentrum des Parlamentes", in Bern: Das ist das letzte Vorhaben der Immobilienbotschaft. Hier wird ein Verpflichtungskredit von 44,2 Millionen Franken für die Zumiete und den Mieterausbau des Besuchs- und Informationszentrums des Parlamentes am Bundesplatz 2 vis-à-vis des Bundeshauses in Bern beantragt.
+Der Verpflichtungskredit umfasst die Anmiete über zwölf Jahre sowie den Mieterausbau. Der Mietvertrag kann bei Ablauf der festen Mietdauer zweimal um je fünf Jahre verlängert werden.
+Der guten Ordnung halber möchte ich im Namen des Bundesrates darauf hinweisen, dass dieses Vorhaben weder finanziert ist noch dem aktuellen Grundsatz der Immobilienpolitik des Bundesrates entspricht. Entsprechend müsste das Parlament sowohl den vorliegenden Verpflichtungskredit wie auch eine entsprechende Plafonderhöhung im Voranschlag 2027 genehmigen, ansonsten kann dieses Projekt nicht umgesetzt werden. Zu den beiden Minderheitsanträgen und zu den Voten der Fraktionen zu diesem Projekt wird die Delegierte der Verwaltungsdelegation der Bundesversammlung, Frau Nationalrätin Rumy, Stellung nehmen.
+Ich bitte Sie, auf die Vorlage zur Immobilienbotschaft 2026 einzutreten und dieser zuzustimmen.
 </t>
   </si>
 </sst>
@@ -404,8 +434,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I17" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I17"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1157,6 +1187,33 @@
         <v>85</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17"/>
+      <c r="F17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" t="s">
+        <v>89</v>
+      </c>
+      <c r="I17" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-10-01
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -204,16 +204,16 @@
     <t xml:space="preserve">BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, wo wir noch besser werden können und müssen.
-Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut, dass </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, wo wir noch besser werden können und müssen.
-Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut, dass die EFK teilweise auch positive Aspekte feststellt, auch wenn diese in den Auseinandersetzungen mit den Berichten manchmal etwas untergehen. So erlaube ich mir zu erwähnen, dass die überwiegende Mehrheit der IKT-Projekte mit Erfolg abgeschlossen werden. In den letzten zwei Jahren haben wir in der Bundesverwaltung rund 200 Projekte mit einem Budget von über 400 000 Franken abgeschlossen, und rund 85 Prozent dieser Projekte wurden sowohl in der Zeit wie auch im Budget abgeschlossen. Aber nochmals, ich gehe mit Ihnen und auch mit der EFK einig: Das darf nicht unsere Ambition und unser Anspruch sein, da müssen wir besser werden.
+    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, bei denen wir noch besser werden können und müssen.
+Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich schicke voraus, dass es mir wahrscheinlich nicht möglich sein wird, alle diese Fragen hier direkt mündlich zu beantworten. Aber ich möchte unterstreichen, Herr Ständerat Salzmann: Ihre Fragen, die Themen, die Sie in Ihrer Interpellation ansprechen, sind wichtig, und der Bundesrat sowie ich als Bundeskanzler nehmen sie sehr ernst. Die EFK muss und soll den Finger auf Dinge legen, bei denen wir noch besser werden können und müssen.
+Ich erlaube mir trotzdem, kurz zu erwähnen, dass es mich freut, dass die EFK teilweise auch positive Aspekte feststellt, auch wenn diese in den Auseinandersetzungen mit den Berichten manchmal etwas untergehen. So erlaube ich mir zu erwähnen, dass die überwiegende Mehrheit der IKT-Projekte mit Erfolg abgeschlossen wird. In den letzten zwei Jahren haben wir in der Bundesverwaltung rund 200 Projekte mit einem Budget von über 400 000 Franken abgeschlossen, und rund 85 Prozent dieser Projekte wurden sowohl in der Zeit wie auch im Budget abgeschlossen. Aber nochmals, ich gehe mit Ihnen und auch mit der EFK einig: Das darf nicht unsere Ambition und unser Anspruch sein, da müssen wir besser werden.
 Ich versuche, die eine oder andere Frage zu beantworten. Ich werde, wie von Ihnen angeboten, dann sehr gerne noch schriftlich auf die verschiedenen Fragen eingehen.
-Zum Projektleiterpool: Sie haben es erwähnt, 2014 forderten zwei gleichlautende Motionen der Finanzkommissionen beider Räte, dass der Bundesrat einen Projektleiterpool für Schlüsselprojektleiter aufbaut. Dieser Pool besteht aus drei Personen. Wenn wir alle 21 laufenden Schlüsselprojekte abdecken und auch für neue Schlüsselprojekte bereit sein möchten, dann müssten wir den Pool auf mindestens 25 Personen ausweiten. Das wäre eine massive Aufstockung gegenüber heute. Deshalb werden diese Leistungen teilweise von externen Personen wahrgenommen oder die Positionen durch bundesverwaltungsinterne Mitarbeitende besetzt.
+Zum Projektleiterpool: Sie haben es erwähnt, 2012 forderten zwei gleichlautende Motionen der Finanzkommissionen beider Räte, dass der Bundesrat einen Projektleiterpool für Schlüsselprojekte aufbaut. Dieser Pool besteht aus drei Personen. Wenn wir alle 21 laufenden Schlüsselprojekte abdecken und auch für neue Schlüsselprojekte bereit sein möchten, dann müssten wir den Pool auf mindestens 25 Personen ausweiten. Das wäre eine massive Aufstockung gegenüber heute. Deshalb werden diese Leistungen teilweise von externen Personen wahrgenommen oder die Positionen durch bundesverwaltungsinterne Mitarbeitende besetzt.
 Ich komme zu den Assessments. Hier ist die Bundeskanzlei im Sinne einer übergreifenden Koordination der digitalen Transformation bei Schlüsselprojekten aktiv Folgendes angegangen: Wir haben in den vergangenen zwei Jahren bei rund 14 Grossprojekten ein Assessment durchgeführt. Ich bin der Meinung, das hat Wirkung gezeigt. In rund zwei Drittel der Fälle hat die Bundeskanzlei Empfehlungen abgegeben oder Bedingungen gestellt. Hauptsächlich ging es dabei um Konkretisierungen der Kontrollmechanismen oder um die Forderung, die unabhängige Qualitätssicherung rascher zu besetzen und nicht erst nach Ablauf der Initialisierungsphase.
-Zur Begleitung der Projekte in der Initialisierungsphase: Das ist auch aus meiner Sicht und aus Sicht des Bundesrates wichtig und richtig, und das ist auch entsprechend aufgesetzt. Die Bundeskanzlei wird dem Bundesrat bis Ende dieses Jahres Grundlagen zur Weiterentwicklung der Gouvernanz der digitalen Transformation vorlegen. Ein Kernstück dieser Weiterentwicklung bildet die Erteilung der Kompetenz an die Bundeskanzlei, in der Initialisierungsphase Synergieprüfungen durchzuführen, damit sichergestellt ist, dass in neuen Vorhaben nicht plötzlich Dinge beschafft oder entwickelt werden, die wir bereits im Einsatz haben. Ein Beispiel, das Sie wahrscheinlich kennen, ist das mittlerweile schweizweit im Einsatz stehende Behördenlogin Agov. In dem Sinn und Geist versuchen wir auch hier vorwärts zu machen, um Kosten und Zeit zu sparen.
+Zur Begleitung der Projekte in der Initialisierungsphase: Das ist auch aus meiner Sicht und aus Sicht des Bundesrates wichtig und richtig, und das ist auch entsprechend aufgesetzt. Die Bundeskanzlei wird dem Bundesrat bis Ende dieses Jahres Grundlagen zur Weiterentwicklung der Gouvernanz der digitalen Transformation vorlegen. Ein Kernstück dieser Weiterentwicklung bildet die Erteilung der Kompetenz an die Bundeskanzlei, in der Initialisierungsphase Synergieprüfungen durchzuführen, damit sichergestellt ist, dass in neuen Vorhaben nicht plötzlich Dinge beschafft oder entwickelt werden, die wir bereits im Einsatz haben. Ein Beispiel, das Sie wahrscheinlich kennen, ist das mittlerweile schweizweit im Einsatz stehende Behördenlogin Agov. In dem Sinn und Geist versuchen wir auch hier, vorwärtszumachen, um Kosten und Zeit zu sparen.
 </t>
   </si>
   <si>
@@ -223,16 +223,16 @@
     <t xml:space="preserve">Salzmann Werner</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich nur teilweise davon befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
-Zur Antwort 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie andererseits zu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich nur teilweise davon befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
-Zur Antwort 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie andererseits zur Unterstützung der Departemente beiziehen zu können. Haben die Departemente diese Möglichkeit genutzt? Wenn ja, welche Projektprobleme konnten nachweislich verhindert werden? Wie wird konkret gemessen, ob der Expertenpool die Mängel in der Initialisierungsphase reduziert hat? Gibt es Kennzahlen zu Projekten mit oder ohne Poolunterstützung? 
-Zur Antwort 2: Die Möglichkeit, Projektassessments durchzuführen, gibt es seit 2015. Eine Bilanz sollte daher über die Projekte gezogen werden, die sich jetzt in der Realisierungsphase befinden. Dazu habe ich folgende Nachfragen: Werden die richtigen Themen und Risiken im Assessment untersucht? Würden Sie sagen, dass ein Projekt ohne Assessment häufiger in Schwierigkeiten gerät? Wenn ja, warum? Gehen die Prüfer genügend auf die Besonderheiten des jeweiligen Projektes ein? Wie fundiert und aussagekräftig sind die Ergebnisse des Assessments aus Ihrer Sicht? Werden die Erkenntnisse aus den Assessments auch für andere Projekte genutzt? Lernt die Organisation aus wiederkehrenden Erkenntnissen und Problemen des Assessments? 
-Zur Antwort 3: Die ursprüngliche Frage zielt auf eine obligatorische Begleitung der Projektteams, das heisst, auf Übungsebene und nicht auf Steuerungsebene hin. Wurden somit unabhängig von der Synergieprüfung Modelle geprüft oder pilotiert, die die Projektteams während der Initialisierungsphase begleiten oder beraten? 
-Zum Schluss stellen sich für mich noch generelle Fragen, zu denen ich gerne eine Antwort hätte, nämlich: Warum greifen bestehende Instrumente nicht? Welche Massnahmen sind erforderlich, wenn sich bereits 2016 erkannte Probleme wiederholen? Wenn die Instrumente funktionieren, warum benötigen wir sie nach 10 Jahren noch in nahezu unveränderter Form? Woran lässt sich objektiv erkennen, dass diese Instrumente nicht nur zusätzliche Kontrolle erzeugen, sondern dass sich die Qualität der Projekte tatsächlich verbessert hat? 
-Die Eidgenössische Finanzkontrolle weist regelmässig auf diese Schwachstellen in grossen IKT-Vorhaben der Bundesverwaltung hin. Ein wesentlicher Teil dieser Feststellung deutet darauf hin, dass grundlegende Voraussetzungen bereits in der Projektinitialisierung unzureichend geklärt und vorbereitet wurden. Mir geht es darum, dass wir hier einen merklichen Fortschritt erzielen und IKT-Projekte in der Bundesverwaltung von Anfang an auf den richtigen Weg bringen. Daher, sehr geehrter Herr Bundeskanzler, wäre ich Ihnen dankbar, wenn Sie meine Fragen heute, aber auch schriftlich beantworten können. Besten Dank.
+    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich davon nur teilweise befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
+Zur Antwort auf Frage 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie ander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich davon nur teilweise befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
+Zur Antwort auf Frage 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie andererseits zur Unterstützung der Departemente beiziehen zu können. Haben die Departemente diese Möglichkeit genutzt? Wenn ja, welche Projektprobleme konnten nachweislich verhindert werden? Wie wird konkret gemessen, ob der Expertenpool die Mängel in der Initialisierungsphase reduziert hat? Gibt es Kennzahlen zu Projekten mit und zu Projekten ohne Poolunterstützung? 
+Zur Antwort auf Frage 2: Die Möglichkeit, Projektassessments durchzuführen, gibt es seit 2015. Eine Bilanz sollte daher über die Projekte gezogen werden, die sich jetzt in der Realisierungsphase befinden. Dazu habe ich folgende Nachfragen: Werden die richtigen Themen und Risiken im Assessment untersucht? Würden Sie sagen, dass ein Projekt ohne Assessment häufiger in Schwierigkeiten gerät? Wenn ja, warum? Gehen die Prüfer genügend auf die Besonderheiten des jeweiligen Projektes ein? Wie fundiert und aussagekräftig sind die Ergebnisse des Assessments aus Ihrer Sicht? Werden die Erkenntnisse aus den Assessments auch für andere Projekte genutzt? Lernt die Organisation aus wiederkehrenden Erkenntnissen und Problemen des Assessments? 
+Zur Antwort auf Frage 3: Die ursprüngliche Frage zielt auf eine obligatorische Begleitung der Projektteams, das heisst auf Übungsebene und nicht auf Steuerungsebene, hin. Wurden somit unabhängig von der Synergieprüfung Modelle geprüft oder pilotiert, die die Projektteams während der Initialisierungsphase begleiten oder beraten? 
+Zum Schluss stellen sich für mich noch generelle Fragen, zu denen ich gerne eine Antwort hätte, nämlich: Warum greifen bestehende Instrumente nicht? Welche Massnahmen sind erforderlich, wenn sich bereits 2016 erkannte Probleme wiederholen? Wenn die Instrumente funktionieren, warum benötigen wir sie nach 10 Jahren noch in nahezu unveränderter Form? Woran lässt sich objektiv erkennen, dass diese Instrumente nicht nur zusätzliche Kontrolle erzeugen, sondern sich die Qualität der Projekte tatsächlich verbessert hat? 
+Die Eidgenössische Finanzkontrolle weist regelmässig auf diese Schwachstellen in grossen IKT-Vorhaben der Bundesverwaltung hin. Ein wesentlicher Teil dieser Feststellung deutet darauf hin, dass grundlegende Voraussetzungen bereits in der Projektinitialisierung unzureichend geklärt und vorbereitet wurden. Mir geht es darum, dass wir hier einen merklichen Fortschritt erzielen und IKT-Projekte in der Bundesverwaltung von Anfang an auf den richtigen Weg bringen. Daher, sehr geehrter Herr Bundeskanzler, wäre ich Ihnen dankbar, wenn Sie meine Fragen heute oder auch schriftlich beantworten könnten. Besten Dank.
 </t>
   </si>
   <si>
@@ -386,6 +386,40 @@
 Der Verpflichtungskredit umfasst die Anmiete über zwölf Jahre sowie den Mieterausbau. Der Mietvertrag kann bei Ablauf der festen Mietdauer zweimal um je fünf Jahre verlängert werden.
 Der guten Ordnung halber möchte ich im Namen des Bundesrates darauf hinweisen, dass dieses Vorhaben weder finanziert ist noch dem aktuellen Grundsatz der Immobilienpolitik des Bundesrates entspricht. Entsprechend müsste das Parlament sowohl den vorliegenden Verpflichtungskredit wie auch eine entsprechende Plafonderhöhung im Voranschlag 2027 genehmigen, ansonsten kann dieses Projekt nicht umgesetzt werden. Zu den beiden Minderheitsanträgen und zu den Voten der Fraktionen zu diesem Projekt wird die Delegierte der Verwaltungsdelegation der Bundesversammlung, Frau Nationalrätin Rumy, Stellung nehmen.
 Ich bitte Sie, auf die Vorlage zur Immobilienbotschaft 2026 einzutreten und dieser zuzustimmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour cet article 41, il y a lieu de distinguer les lettres a et b des lettres c et d. Aux lettres a et b, la proposition de la majorité de la commission correspond sur le fond au droit en vigueur ainsi qu'au projet du Conseil fédéral. Elle est donc en ordre et peut être acceptée.
+Par contre, la disposition prévue à la lettre c met en oeuvre la recommandation du Contrôle fédéral des finances qui vise à fixer des objectifs pour les contrôles des produits. Il est également important que le Conseil </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour cet article 41, il y a lieu de distinguer les lettres a et b des lettres c et d. Aux lettres a et b, la proposition de la majorité de la commission correspond sur le fond au droit en vigueur ainsi qu'au projet du Conseil fédéral. Elle est donc en ordre et peut être acceptée.
+Par contre, la disposition prévue à la lettre c met en oeuvre la recommandation du Contrôle fédéral des finances qui vise à fixer des objectifs pour les contrôles des produits. Il est également important que le Conseil fédéral dispose de la compétence prévue, car l'article 58 du projet de loi stipule que les autorités fédérales collaborent avec des services et institutions étrangers et internationaux spécialisés et assument les tâches découlant des traités internationaux. Cette nouvelle compétence vise à garantir que la Suisse puisse participer à des programmes de contrôle coordonnés sur la base d'accords internationaux. Par ailleurs, diverses crises alimentaires survenues par le passé - on peut penser à la céréulide ou encore aux salmonelles dans le fromage - ont montré que l'autorité de surveillance doit pouvoir orienter davantage qu'aujourd'hui l'application des mesures cantonales visant à les combattre. Si cette disposition est biffée, le Conseil fédéral se retrouvera dépourvu des instruments nécessaires notamment dans le cadre de la gestion des crises. Cette disposition doit donc être maintenue.
+Concernant la lettre d, pour lutter efficacement contre la criminalité alimentaire, il est indispensable de pouvoir intervenir de manière coordonnée et efficace dans des cas où l'on soupçonne des infractions systématiques à la législation sur les denrées alimentaires résultant de pratiques frauduleuses ou trompeuses. On peut penser à l'affaire de la viande de cheval en 2013. Aujourd'hui, les pratiques frauduleuses ou trompeuses ne se limitent souvent pas à un seul canton, elles s'étendent à l'ensemble de la Suisse, voire revêtent une dimension internationale. C'est pourquoi le Conseil fédéral doit pouvoir contraindre les autorités cantonales chargées de l'exécution à signaler les cas concernés à l'Office fédéral de la sécurité alimentaire et des affaires vétérinaires. Cette disposition doit donc également être maintenue.
+Je vous invite dès lors, et vous en remercie, à suivre la minorité Crevoisier Crelier pour les lettres c et d.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crevoisier Crelier Mathilde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À l'article 41, la majorité entend entraver les compétences du Conseil fédéral en matière de contrôle des denrées alimentaires en biffant les lettres c et d. Ainsi, contrairement au projet présenté, le Conseil fédéral ne pourrait plus décider de réaliser des contrôles de catégories de produits dans le cadre de programmes d'analyse.
+Je rappelle que la lettre c met en oeuvre les recommandations du Contrôle fédéral des finances, qui visent à fixer des objectifs pour la réalisation de contrôles de p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À l'article 41, la majorité entend entraver les compétences du Conseil fédéral en matière de contrôle des denrées alimentaires en biffant les lettres c et d. Ainsi, contrairement au projet présenté, le Conseil fédéral ne pourrait plus décider de réaliser des contrôles de catégories de produits dans le cadre de programmes d'analyse.
+Je rappelle que la lettre c met en oeuvre les recommandations du Contrôle fédéral des finances, qui visent à fixer des objectifs pour la réalisation de contrôles de produits. Le fait que le Conseil fédéral disposera de cette compétence à l'avenir est important ; d'autant plus important que l'article 58 de la loi sur les denrées alimentaires prévoit que les autorités fédérales collaborent "avec les institutions et organes spécialisés étrangers et internationaux". Cette nouvelle compétence permet de garantir que la Suisse participe à des programmes de contrôle coordonnés, par exemple le programme national d'analyse et de détection de substances étrangères. Il s'agit aussi de lutter contre les fraudes et d'essayer de combattre la criminalité liée aux denrées alimentaires. Pour ce faire, il est important de pouvoir agir de façon coordonnée en cas de soupçons d'infraction.
+Ainsi, en biffant la lettre d, c'est-à-dire en privant le Conseil fédéral de la possibilité d'obliger les autorités cantonales d'exécution de signaler des cas manifestes et graves de fraude ou d'infraction à la loi sur les denrées alimentaires, on entrave cette collaboration et cette possibilité d'avoir un signalement fluide, un flux fluide d'informations.
+Ainsi, je vous invite à en rester à la version du Conseil fédéral en adoptant la proposition de la minorité.
 </t>
   </si>
 </sst>
@@ -434,8 +468,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I17" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I19" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I19"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1214,6 +1248,62 @@
         <v>90</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" t="s">
+        <v>93</v>
+      </c>
+      <c r="I18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
+        <v>97</v>
+      </c>
+      <c r="I19" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-10-02
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -41,10 +41,82 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
+    <t xml:space="preserve">418692</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260914</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baume-Schneider Elisabeth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà é</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La motion charge le Conseil fédéral de veiller à ce que le remboursement de la taxe d'urgence revienne aux assurés et ne soit pas versé dans les réserves des caisses-maladie. La LAMal autorise les assureurs à réclamer la restitution de prestations indûment versées. Des demandes de restitution qui aboutissent et qui peuvent être individualisées réduisent la participation aux coûts de l'assuré - on peut penser à la franchise ou à la quote-part -, mais pour autant que celles-ci ne soient pas déjà épuisées. Les personnes concernées peuvent demander à leur assureur-maladie le remboursement du montant différentiel. Si les assurés ne font pas valoir activement leur avoir auprès de la caisse-maladie, les assureurs peuvent renoncer à un remboursement lorsque celui-ci engendrerait une charge disproportionnée. Tel est le cas, par exemple, lorsque les assurés ne peuvent pas être contactés malgré des efforts avérés, ou encore en présence de montants minimes lorsque les frais de traitement excèdent les montants à rembourser. Lorsque les restitutions ne sont pas utilisées pour réduire la participation aux coûts, elles diminuent le coût des prestations. Cela améliore le résultat actuariel global et conduit, au final, à des primes moins élevées. Néanmoins, j'en conviens, Monsieur le conseiller national, ce qui compte, c'est la traçabilité des montants et la transparence - nous l'avons vu également dans le rapport du Contrôle fédéral des finances. Par votre motion, vous demandez plus de transparence et de traçabilité. Le Conseil fédéral estime que les restitutions doivent bénéficier aux personnes assurées, tout comme vous, mais il estime que la LAMal le permet d'ores et déjà. [GZ]
+C'est pourquoi il demande le rejet de la motion.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">418734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bläsi Thomas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir[NB]? C'est la question centrale de cette motion. Son point de départ est concret[NB]: une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En reva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorsqu'un assureur récupère une somme versée pour une prestation, à qui cet argent doit-il revenir[NB]? C'est la question centrale de cette motion. Son point de départ est concret[NB]: une taxe d'urgence d'environ 40 francs facturée pour certaines consultations en dehors des heures ordinaires et une décision du Tribunal fédéral à la suite de laquelle des assureurs demandent le remboursement de montants auparavant pris en charge. Cette décision judiciaire n'est pas l'objet de notre débat. En revanche, la destination des sommes récupérées relève pleinement de notre responsabilité politique, car cet argent a été financé par les assurés, par leurs primes, mais également par leur franchise et leur quote-part. Le Conseil fédéral estime que ma motion est inutile. Selon son avis, les sommes récupérées améliorent le résultat technique des assureurs et peuvent ainsi contribuer à réduire les primes, mais une possibilité de baisse future n'est pas une garantie de restitution. Lorsqu'un assuré a personnellement supporté une partie d'une facture, ensuite corrigée, où apparaît cette correction[NB]? Comment sa participation est-elle recalculée[NB]? Comment s'assure-t-on que la somme correspondante lui revient[NB]? Pour les montants financés collectivement par les primes, comment démontre-t-on qu'ils bénéficient effectivement aux assurés, au lieu de simplement alimenter les réserves[NB]? Voilà les questions auxquelles il faut répondre.
+L'interdiction de distribuer des bénéfices invoquée par le Conseil fédéral ne suffit pas. Elle ne démontre ni à qui les montants récupérés bénéficient, ni quand, ni comment. Une écriture comptable favorable à l'assureur ne prouve pas à elle seule une restitution à l'assuré. Cette motion s'inscrit dans la continuité de mon travail parlementaire, notamment de la motion 24.3060 sur le contrôle des finances des caisses-maladie. Rabais, rétrocessions ou remboursements de prestations, les mécanismes diffèrent, mais l'exigence demeure. Nous devons pouvoir tracer l'argent et vérifier qu'il bénéficie à ceux qui financent l'assurance obligatoire. Les travaux du Contrôle fédéral des finances renforcent cette exigence de transparence et de contrôle. Les médecins qui assurent les consultations le soir et le week-end rendent un service indispensable et les assureurs doivent appliquer les décisions judiciaires, mais il reste à garantir que les conséquences financières soient correctement répercutées jusqu'aux assurés. La récupération de l'argent ne doit pas être la dernière étape. Sa restitution doit être l'objectif. Les assurés paient leurs primes, leur franchise et leur quote-part. Ces obligations sont précises et leurs échéances aussi. Ils sont en droit d'attendre la même précision lorsqu'une somme doit leur revenir.
+Je vous demande donc d'adopter cette motion pour garantir une traçabilité des montants récupérés, la correction des participations individuelles concernées et une répercussion effective au bénéfice des assurés. Au-delà de cette taxe de 40 francs, nous défendons un principe essentiel[NB]: l'argent récupéré dans l'assurance obligatoire doit bénéficier aux assurés de manière concrète, transparente et vérifiable.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">419015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260915</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chollet Clarence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles, et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La situation sécuritaire en Europe s'est profondément dégradée, nous ne le contestons pas. Nous ne contestons pas non plus la nécessité d'adapter les capacités de notre armée aux menaces actuelles, et nous saluons le fait que le Conseil fédéral mette davantage l'accent sur les menaces les plus probables, les attaques à distance, les drones, les cyberattaques ou encore la guerre électronique. Mais reconnaître la nécessité d'agir ne signifie pas signer des chèques en blanc. Surtout, cela ne signifie pas continuer comme si rien ne s'était passé au sein du DDPS.
+Au moment où ce Parlement s'apprête à voter 3,4 milliards de francs supplémentaires, dont 394 millions pour le F-35A, une question s'impose[NB]: pouvons-nous encore avoir confiance dans la manière dont le DDPS conduit ses grands projets d'armement[NB]? La semaine dernière, la Commission de gestion nous a donné quelques éléments de réponse qui sont accablants. Pendant des années, on nous a répété que le prix du F-35A était fixe. Il ne l'est pas. On nous a affirmé que la Suisse avait négocié une garantie particulière avec les États-Unis. Cette garantie n'existe pas. Des doutes avaient été exprimés par le Contrôle fédéral des finances, mais ils n'ont pas conduit à l'examen critique qui aurait été nécessaire. Le service juridique d'Armasuisse, pourtant compétent en la matière, n'a pratiquement pas participé à la négociation de ce contrat. Seules quelques personnes impliquées dans le dossier ont lu le contrat dans son intégralité. Comme si cela ne suffisait pas, la Commission de gestion constate que certains documents n'ont même pas été archivés conformément aux règles.
+Nous ne parlons pas de l'achat de quelques véhicules de service. Nous parlons du plus grand projet d'acquisition militaire de l'histoire récente de notre pays. Pourtant, à chaque nouvelle révélation, le même constat s'impose[NB]: manque de conduite, manque de contrôle, manque de transparence. Et maintenant, le Parlement doit octroyer 394 millions de francs supplémentaires, non pour améliorer la sécurité de la Suisse, mais pour essayer de sauver 30 avions sur les 36 que le Conseil fédéral voulait acquérir. Faut-il avaler cette couleuvre tranquillement[NB]? Nous ne le pensons pas.
+Il faut savoir s'arrêter lorsqu'un projet déraille. Le projet F-35A a largement dépassé ce stade, d'autant plus que notre opposition au F-35A n'a jamais été uniquement financière. Nous avons toujours contesté le choix de cet appareil, un avion extrêmement complexe, dépendant des États-Unis pour son exploitation et son évolution, conçu pour opérer au sein d'un dispositif militaire intégré qui n'est pas celui de la Suisse. Aujourd'hui, à ces critiques stratégiques s'ajoute un fiasco dans la conduite de son acquisition.
+Il y a également une contradiction plus fondamentale dans la politique que nous menons. Nous parlons de sécurité comme si elle se mesurait au nombre de milliards de francs consacrés à l'armement, mais la sécurité de la Suisse ne commence pas lorsqu'un missile franchit notre frontière. Elle commence bien avant. Elle se construit lorsque nous empêchons les conflits de naître et de s'étendre, lorsque nous défendons le droit international, lorsque nous investissons dans la coopération internationale, dans la diplomatie et dans la promotion de la paix, lorsque nous luttons contre le dérèglement climatique qui multiplie les crises et les déplacements des populations, lorsque nous renforçons notre capacité à faire face aux cyberattaques, à la désinformation et aux nouveaux risques liés à l'intelligence artificielle. C'est cela aussi la politique de sécurité. Dans ces domaines, la tendance est exactement inverse. Alors que l'objectif de 1 pour cent du PIB pour l'armée doit être atteint toujours plus rapidement, la part consacrée à la coopération internationale recule. Toujours plus pour réagir aux conflits, toujours moins pour contribuer à les prévenir[NB]: ce déséquilibre est une erreur stratégique. Nous le répétons[NB]: le groupe des Verts ne nie pas la détérioration de la situation sécuritaire. Au contraire, c'est précisément parce que les ressources sont limitées et que les menaces augmentent que nous devons les investir là où elles apportent réellement davantage de sécurité, c'est-à-dire dans la cyberdéfense, dans la résilience de nos infrastructures et dans la coopération internationale et la diplomatie, mais pas obstinément dans un projet de F-35A dont chaque nouveau chapitre vient confirmer les erreurs du précédent.
+La sécurité ne se mesure pas au prix du matériel que nous achetons. Elle se mesure à notre capacité à identifier les menaces, à faire les bons choix et à utiliser intelligemment les moyens à disposition. Sur ce dernier élément, le dossier F-35A devrait nous inciter à une certaine humilité. Notre groupe entrera donc en matière sur les arrêtés fédéraux 1 et 2, tout en les examinant de manière critique. Mais concernant l'arrêté fédéral 3 et les 394 millions de francs supplémentaires destinés au F-35A, notre position est claire[NB]: après les erreurs, les dissimulations, les approximations et les défaillances de conduite révélées dans ce dossier, notre réponse ne peut pas être de mettre à nouveau simplement 394 millions de francs sur la table. 
+Nous refuserons donc l'entrée en matière sur l'arrêté fédéral[NB]3.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">418941</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20260915</t>
   </si>
   <si>
     <t xml:space="preserve">S</t>
@@ -83,6 +155,43 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">419420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260916</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revaz Estelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités[NB]: vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'initiative populaire "pour l'égalité des personnes handicapées (initiative pour l'inclusion)" a été déposée en septembre 2024. Près de 20 pour cent de la population suisse vit avec un handicap. Pourtant, seuls 5 pour cent perçoivent une prestation de l'assurance-invalidité (AI), dont 2,7 pour cent une rente. Il est donc essentiel de distinguer ces réalités[NB]: vivre avec un handicap ne signifie pas forcément bénéficier de l'AI, et encore moins percevoir une rente. L'inclusion des personnes en situation de handicap est donc un véritable sujet de société. Cela concerne près d'une personne sur cinq dans notre pays et, à ce titre, nous concerne toutes et tous.
+L'initiative pour l'inclusion traduit un constat et une impatience. Le constat, c'est que, malgré les progrès accomplis, la Suisse accuse encore un retard important dans la mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées. L'impatience, parfaitement compréhensible, est celle des personnes concernées et de leurs organisations qui attendent des avancées concrètes depuis trop longtemps.
+L'initiative nous rappelle ainsi le chemin qu'il reste à parcourir pour faire de l'inclusion une réalité. Elle demande l'égalité de droit et de fait des personnes en situation de handicap dans tous les domaines de la vie. Elle vise notamment à garantir le libre choix du logement et à inscrire dans la Constitution un droit à des mesures de soutien et d'adaptation.
+La majorité de la commission comprend ces préoccupations, mais estime que la modification constitutionnelle proposée n'est pas adéquate. Celle-ci n'apporterait en effet pas d'amélioration significative par rapport au droit actuel et soulèverait des difficultés de mise en oeuvre. La commission propose donc de rejeter l'initiative, par 16 voix contre[NB]8.
+La majorité de votre commission rejoint cependant les auteurs de l'initiative sur un point essentiel[NB]: il est nécessaire d'agir. Elle salue donc le contre-projet indirect proposé par le Conseil fédéral et, par 17 voix contre 8, a décidé d'entrer en matière. Une minorité propose de ne pas entrer en matière. Si cette proposition est rejetée, la même minorité demande le renvoi du projet au Conseil fédéral et formule plusieurs pistes de modifications.
+Nous avons mené de longues discussions sur la portée du contre-projet indirect. Pour les auteurs de l'initiative comme pour la majorité de votre commission, il contient beaucoup de dispositions déclaratoires et peu de mesures concrètes. La majorité de votre commission a donc souhaité renforcer le contre-projet indirect et s'éloigner d'une loi essentiellement programmatique, en agissant dans les domaines essentiels de la vie quotidienne. Il ne s'agit pas d'inventer de nouveaux droits, mais de permettre aux personnes en situation de handicap de bénéficier concrètement des mêmes droits et des mêmes possibilités que les autres. Enfin, la commission a souhaité clarifier les responsabilités et renforcer la coordination avec les cantons, qui jouent un rôle central dans la mise en oeuvre de nombreuses mesures.
+Afin d'avoir une vision globale des mesures en faveur de l'égalité des personnes en situation de handicap, la commission a décidé, à l'unanimité, d'examiner l'objet 25.020 "Loi sur l'égalité pour les handicapés. Modification" en parallèle à la loi sur l'inclusion qui constitue le contre-projet indirect du Conseil fédéral à l'initiative. Elle a en revanche décidé, par 14 voix contre 10 et 1 abstention, de traiter séparément la question des langues des signes dans une loi spécifique. Ce sera l'objet de l'initiative parlementaire 26.404 qui vous sera très prochainement soumise.
+Des mesures concrètes ont ainsi été proposées autour de quatre axes[NB]: le libre choix du logement, l'intégration sur le marché du travail, la participation à la vie culturelle, aux loisirs et au sport, ainsi que les prestations d'assistance. Pour agir dans ces différents domaines, votre commission a travaillé sur pas moins de sept lois différentes[NB]: la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, la loi fédérale sur des mesures de promotion civile de la paix et de renforcement des droits de l'homme, la loi fédérale sur l'assurance-invalidité, la loi fédérale sur l'élimination des inégalités frappant les personnes handicapées, la loi sur les langues, la loi sur l'organisation du gouvernement et de l'administration et, enfin, la loi fédérale sur l'encouragement des hautes écoles et la coordination dans le domaine suisse des hautes écoles.
+Étant donné l'organisation du débat et le temps limité dont dispose la commission pour vous présenter les dizaines de propositions qui sont encore en discussion, je vais passer dès maintenant à l'examen de détail sans m'appesantir sur les points qui n'ont pas rencontré d'opposition.
+Je commence donc par la loi fédérale sur l'encouragement de l'inclusion des personnes handicapées, aussi appelée loi sur l'inclusion (LIncl), et je commence à l'article[NB]2. 
+La loi sur l'inclusion est une loi-cadre qui doit donner une orientation politique claire. Par 14 voix contre 8 et 3 abstentions, votre commission propose donc de renforcer cet article sans lui donner une portée juridique qu'il ne pourrait avoir. Une minorité souhaite aller plus loin, tandis qu'une autre préfère s'en tenir à la proposition du Conseil fédéral. 
+À l'article 3, votre commission a souhaité clarifier la relation avec le droit cantonal, mais aussi mentionner explicitement l'importance de la collaboration entre la Confédération et les cantons. Convaincue qu'il est important de réaffirmer la nécessité d'agir, votre commission, par 12 voix contre 11, a accepté cet ajout. Une minorité s'y oppose. 
+À l'article 5, l'objectif est simple[NB]: faire en sorte que la stratégie nationale de mise en oeuvre de la Convention de l'ONU relative aux droits des personnes handicapées (CDPH) ne reste pas un document d'intention, mais débouche sur des mesures concrètes. Par 11 voix contre 8 et 5 abstentions, la majorité de votre commission souhaite renforcer les objectifs en matière d'autodétermination, de liberté de choix et de participation à la vie sociale. Une minorité souhaite suivre le Conseil fédéral. 
+À l'article 6 alinéas 4 et 5, il s'agit d'inscrire les projets pilotes dans la loi. Ces derniers permettent de tester concrètement les mesures prévues dans la stratégie et les plans d'action et d'identifier celles qui fonctionnent. Ces modifications ont été adoptées par 13 voix contre 10 et 2 abstentions. Il n'y a pas de proposition de minorité. 
+À l'article 8, la majorité souhaite impliquer les personnes en situation de handicap dès l'élaboration de la stratégie et des plans d'action. Leur expérience permet d'identifier les besoins en amont et d'éviter des corrections qui seraient ultérieurement plus coûteuses. Cette proposition a été adoptée par 13 voix contre 8 et 3 abstentions. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
+À l'article 11, la majorité souhaite renforcer l'autonomie des personnes en situation de handicap dans le choix de leur logement. Pour cela, elle propose notamment d'améliorer l'information et la coordination[NB]; un élément également relevé par le Contrôle fédéral des finances. Ces modifications ont été adoptées par 14 voix contre[NB]10. Une minorité souhaite s'en tenir au projet du Conseil fédéral. 
+À l'article 11a, l'objectif est de renforcer l'autonomie économique des personnes en situation de handicap en facilitant leur accès au marché du travail. Leur potentiel reste insuffisamment exploité, alors que la Suisse manque de main-d'oeuvre qualifiée et que l'assurance-invalidité (AI) fait face à des difficultés financières. Par 16 voix contre 8, votre commission a accepté cette proposition. 
+À l'article 11b, il s'agit de favoriser la participation des personnes en situation de handicap à la vie culturelle, aux loisirs, au sport et aux activités politiques. Par 14 voix contre 11, la majorité de votre commission souhaite inscrire cet objectif dans la loi sans que cela entraîne automatiquement de nouvelles dépenses. Une minorité la juge inopportune. 
+À l'article 11c, l'objectif est de renforcer la liberté de choix des personnes en situation de handicap en adaptant mieux les prestations d'assistance à leur réalité de vie et en améliorant leur coordination. Par 13 voix contre 11 et 1 abstention, votre commission veut inscrire cette orientation dans la loi. Une minorité estime qu'elle fait doublon avec les travaux annoncés concernant l'AI. 
+À l'article 12, l'objectif est de disposer de données fiables sur l'accessibilité des bâtiments, des installations et des logements. Ces données sont indispensables pour identifier les besoins et agir de manière ciblée. Par 13 voix contre 9 et 3 abstentions, la majorité de votre commission a décidé d'inscrire cet ajout dans la loi. Une minorité veut s'en tenir à la version du Conseil fédéral. 
+La majorité de votre commission souhaite également introduire une section 4a sur les mesures transitoires. À l'article 12a, elle propose un délai de 8 ans pour la mise en oeuvre de la loi par la Confédération et les cantons. Au regard des délais prévus dans d'autres lois, ce délai lui paraît à la fois réaliste et nécessaire. Elle souhaite également mettre l'accent sur le libre choix du logement qui est au coeur de l'initiative populaire. Cette proposition a été adoptée par 17 voix contre[NB]6. Une minorité s'y oppose. 
+Je continuerai au milieu du bloc 2 pour vous rendre compte en détail des autres modifications des autres actes, puisque, comme je vous l'ai dit, on a travaillé sur sept lois différentes. Il y a donc encore du travail sur la planche.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">420080</t>
   </si>
   <si>
@@ -114,9 +223,6 @@
     <t xml:space="preserve">Salzmann Werner</t>
   </si>
   <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ich danke dem Bundesrat für die Antworten. Leider bin ich davon nur teilweise befriedigt. Deshalb erlaube ich mir heute, nachzufragen. 
 Zur Antwort auf Frage 1: Die Frage, wie der Bundesrat den Einsatz der Expertenpools beurteilt, da es weiterhin zu Versäumnissen in der Initialisierungsphase kommt, wurde meines Erachtens nicht beantwortet. Die beiden Motionen 12.3986 und 12.3987 sahen vor, die Personen aus dem Projektleiterpool einerseits für komplexe Informatikprojekte einzusetzen und sie ander</t>
   </si>
@@ -165,13 +271,17 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">420571</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Contrôle fédéral des finances a publié un rapport en 2025 qui met en évidence le poids et l'existence de coûts potentiellement inutiles dans ce domaine. Le Conseil fédéral soutient le postulat de votre commission. Le domaine de l'imagerie médicale doit donc continuer à être suivi attentivement, afin que d'éventuelles évolutions problématiques soient identifiées rapidement et puissent surtout être corrigées.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">420874</t>
   </si>
   <si>
     <t xml:space="preserve">20260923</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
   </si>
   <si>
     <t xml:space="preserve">Schnyder Markus</t>
@@ -216,9 +326,6 @@
     <t xml:space="preserve">Weichelt Manuela</t>
   </si>
   <si>
-    <t xml:space="preserve">G</t>
-  </si>
-  <si>
     <t xml:space="preserve">ZG</t>
   </si>
   <si>
@@ -230,12 +337,6 @@
   </si>
   <si>
     <t xml:space="preserve">20260928</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baume-Schneider Elisabeth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JU</t>
   </si>
   <si>
     <t xml:space="preserve">Das Bundesgesetz über die Krankenversicherung sieht vor, dass Leistungserbringer, die beim Medikamentenkauf Vergünstigungen erhalten, diese grundsätzlich an die Versicherer bzw. an die Prämienzahlenden weitergeben müssen. Die Transparenzpflicht gemäss Heilmittelgesetz verlangt zudem, dass gewährte Vergünstigungen auszuweisen und den zuständigen Behörden auf Verlangen offenzulegen sind. 
@@ -244,6 +345,17 @@
   <si>
     <t xml:space="preserve">Das Bundesgesetz über die Krankenversicherung sieht vor, dass Leistungserbringer, die beim Medikamentenkauf Vergünstigungen erhalten, diese grundsätzlich an die Versicherer bzw. an die Prämienzahlenden weitergeben müssen. Die Transparenzpflicht gemäss Heilmittelgesetz verlangt zudem, dass gewährte Vergünstigungen auszuweisen und den zuständigen Behörden auf Verlangen offenzulegen sind. 
 Für die Aufsicht über die Einhaltung dieser gesetzlichen Bestimmungen ist seit 2020 das Bundesamt für Gesundheit (BAG) zuständig. Das BAG muss sicherstellen, dass Vergünstigungen an die Versicherer bzw. die Versicherten weitergegeben werden. Die Eidgenössische Finanzkontrolle hat 2026 die Aufsicht des BAG bezüglich Weitergabepflicht von Vergünstigungen bei der Medikamentenabgabe überprüft und kommt zum Schluss, dass diese noch kaum wirksam ist. Der Bundesrat erwartet von allen beteiligten Akteuren, dass der rechtliche Rahmen eingehalten wird. Das BAG wird die EFK-Empfehlungen gemäss dem Prüfbericht vom 10. April 2026 zur verbesserten Weitergabe von Vergünstigungen fristgerecht umsetzen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">421388</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merci beaucoup pour votre question complémentaire. En fait, il ne s'agit pas de la question de la responsabilité de 5, 10 ou 12 personnes qui travaillent à l'OFSP. Comme je l'ai indiqué, la base légale demande que l'OFSP contrôle, mais demande aussi que les personnes mettent les données à disposition et que les caisses-maladie contrôlent ces données. Le Contrôle fédéral des finances a estimé que le contrôle, du côté de l'OFSP, était insuffisant et qu'on devait maintenant mettre plus de priorités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merci beaucoup pour votre question complémentaire. En fait, il ne s'agit pas de la question de la responsabilité de 5, 10 ou 12 personnes qui travaillent à l'OFSP. Comme je l'ai indiqué, la base légale demande que l'OFSP contrôle, mais demande aussi que les personnes mettent les données à disposition et que les caisses-maladie contrôlent ces données. Le Contrôle fédéral des finances a estimé que le contrôle, du côté de l'OFSP, était insuffisant et qu'on devait maintenant mettre plus de priorités pour arriver à une situation conforme à la loi, à savoir que les rabais doivent être mis à disposition des assurances et, en particulier, des assurés. Il ne s'agit pas de dire qui est responsable en matière de personnes. Ce que je m'engage à faire, c'est que l'OFSP, désormais, mette la priorité sur la mission qui consiste à mieux ou à plus contrôler par rapport à ces rabais.
+Ich habe Ihre Frage genau verstanden, aber ich werde Ihnen nicht sagen können - ich kann es gar nicht -, ob es zwei, drei oder zehn Personen sind, die verantwortlich sind, denn es geht hier nicht um eine Verantwortung einzelner Personen. Das BAG muss diese Kontrolle von Gesetzes wegen durchführen, und wir werden sie auch durchführen. Aber man kann nicht sagen, bestimmte Personen hätten ihre Aufgabe nicht gemacht oder so; nein, sicher nicht. Wir können darüber noch stundenlang diskutieren. Es gibt keine Verantwortung einzelner Personen. 
 </t>
   </si>
   <si>
@@ -302,6 +414,37 @@
 Artikel 156 des Parlamentsgesetzes reicht nicht aus, zumal dieser Artikel ursprünglich nur auf die PUK bezogen war, rein deklaratorisch ist und nach meinem Kenntnisstand im Falle einer nicht wahrheitsgemässen Auskunft durch Bundesrat oder Bundesverwaltung auch noch nie zu einer Konsequenz geführt hat. 
 Man wird mir entgegnen, mein Anliegen sei doch selbstverständlich. Ja, das sollte es sein. Aber die F-35-Affäre zeigt, dass es in der Praxis offensichtlich nicht selbstverständlich ist. Eine allgemeine Informationspflicht reicht nicht, wenn nicht garantiert ist, dass diese Information nach bestem Wissen und Gewissen auch stimmt. Die Wahrheitspflicht hat einen Massstab verdient, an dem sich Regierung und Verwaltung messen lassen müssen und an dem sich unsere Aufsicht orientieren kann.
 Ohne verlässliche Informationen kann das Parlament seine Aufgabe als Gesetzgeber und Oberaufsicht nicht wahrnehmen. Wahrheit ist in einer Demokratie die Grundlage einer jeden Entscheidung. Der Bundesrat muss dem Parlament die Wahrheit sagen, und zwar nicht aus Anstand, sondern weil es das Gesetz verlangt und dieses Gesetz notfalls auch durchgesetzt werden kann. Ich bitte Sie, dieser Selbstverständlichkeit Nachdruck zu verleihen und der parlamentarischen Initiative Folge zu geben.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour cet article 41, il y a lieu de distinguer les lettres a et b des lettres c et d. Aux lettres a et b, la proposition de la majorité de la commission correspond sur le fond au droit en vigueur ainsi qu'au projet du Conseil fédéral. Elle est donc en ordre et peut être acceptée.
+Par contre, la disposition prévue à la lettre c met en oeuvre la recommandation du Contrôle fédéral des finances qui vise à fixer des objectifs pour les contrôles des produits. Il est également important que le Conseil </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour cet article 41, il y a lieu de distinguer les lettres a et b des lettres c et d. Aux lettres a et b, la proposition de la majorité de la commission correspond sur le fond au droit en vigueur ainsi qu'au projet du Conseil fédéral. Elle est donc en ordre et peut être acceptée.
+Par contre, la disposition prévue à la lettre c met en oeuvre la recommandation du Contrôle fédéral des finances qui vise à fixer des objectifs pour les contrôles des produits. Il est également important que le Conseil fédéral dispose de la compétence prévue, car l'article 58 du projet de loi stipule que les autorités fédérales collaborent avec des services et institutions étrangers et internationaux spécialisés et assument les tâches découlant des traités internationaux. Cette nouvelle compétence vise à garantir que la Suisse puisse participer à des programmes de contrôle coordonnés sur la base d'accords internationaux. Par ailleurs, diverses crises alimentaires survenues par le passé - on peut penser à la céréulide ou encore aux salmonelles dans le fromage - ont montré que l'autorité de surveillance doit pouvoir orienter davantage qu'aujourd'hui l'application des mesures cantonales visant à les combattre. Si cette disposition est biffée, le Conseil fédéral se retrouvera dépourvu des instruments nécessaires notamment dans le cadre de la gestion des crises. Cette disposition doit donc être maintenue.
+Concernant la lettre d, pour lutter efficacement contre la criminalité alimentaire, il est indispensable de pouvoir intervenir de manière coordonnée et efficace dans des cas où l'on soupçonne des infractions systématiques à la législation sur les denrées alimentaires résultant de pratiques frauduleuses ou trompeuses. On peut penser à l'affaire de la viande de cheval en 2013. Aujourd'hui, les pratiques frauduleuses ou trompeuses ne se limitent souvent pas à un seul canton, elles s'étendent à l'ensemble de la Suisse, voire revêtent une dimension internationale. C'est pourquoi le Conseil fédéral doit pouvoir contraindre les autorités cantonales chargées de l'exécution à signaler les cas concernés à l'Office fédéral de la sécurité alimentaire et des affaires vétérinaires. Cette disposition doit donc également être maintenue.
+Je vous invite dès lors, et vous en remercie, à suivre la minorité Crevoisier Crelier pour les lettres c et d.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crevoisier Crelier Mathilde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À l'article 41, la majorité entend entraver les compétences du Conseil fédéral en matière de contrôle des denrées alimentaires en biffant les lettres c et d. Ainsi, contrairement au projet présenté, le Conseil fédéral ne pourrait plus décider de réaliser des contrôles de catégories de produits dans le cadre de programmes d'analyse.
+Je rappelle que la lettre c met en oeuvre les recommandations du Contrôle fédéral des finances, qui visent à fixer des objectifs pour la réalisation de contrôles de p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À l'article 41, la majorité entend entraver les compétences du Conseil fédéral en matière de contrôle des denrées alimentaires en biffant les lettres c et d. Ainsi, contrairement au projet présenté, le Conseil fédéral ne pourrait plus décider de réaliser des contrôles de catégories de produits dans le cadre de programmes d'analyse.
+Je rappelle que la lettre c met en oeuvre les recommandations du Contrôle fédéral des finances, qui visent à fixer des objectifs pour la réalisation de contrôles de produits. Le fait que le Conseil fédéral disposera de cette compétence à l'avenir est important ; d'autant plus important que l'article 58 de la loi sur les denrées alimentaires prévoit que les autorités fédérales collaborent "avec les institutions et organes spécialisés étrangers et internationaux". Cette nouvelle compétence permet de garantir que la Suisse participe à des programmes de contrôle coordonnés, par exemple le programme national d'analyse et de détection de substances étrangères. Il s'agit aussi de lutter contre les fraudes et d'essayer de combattre la criminalité liée aux denrées alimentaires. Pour ce faire, il est important de pouvoir agir de façon coordonnée en cas de soupçons d'infraction.
+Ainsi, en biffant la lettre d, c'est-à-dire en privant le Conseil fédéral de la possibilité d'obliger les autorités cantonales d'exécution de signaler des cas manifestes et graves de fraude ou d'infraction à la loi sur les denrées alimentaires, on entrave cette collaboration et cette possibilité d'avoir un signalement fluide, un flux fluide d'informations.
+Ainsi, je vous invite à en rester à la version du Conseil fédéral en adoptant la proposition de la minorité.
 </t>
   </si>
 </sst>
@@ -350,8 +493,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I20" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I20"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -691,55 +834,55 @@
       <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2"/>
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
         <v>20</v>
       </c>
-      <c r="E3"/>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
         <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -751,244 +894,468 @@
         <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="E6" t="s">
-        <v>13</v>
-      </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="E7"/>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10"/>
-      <c r="F10" t="s">
-        <v>58</v>
-      </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
         <v>14</v>
       </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
         <v>66</v>
       </c>
-      <c r="B12" t="s">
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="G12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="I12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
         <v>11</v>
       </c>
-      <c r="F12" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>70</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="D13" t="s">
         <v>71</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15"/>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17"/>
+      <c r="F17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" t="s">
+        <v>89</v>
+      </c>
+      <c r="I17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" t="s">
+        <v>94</v>
+      </c>
+      <c r="G18" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" t="s">
+        <v>95</v>
+      </c>
+      <c r="I18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" t="s">
+        <v>101</v>
+      </c>
+      <c r="E20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>